<commit_message>
RE-043.1: adaptador real Personal Capacity Facts, genérico por patrimonio
</commit_message>
<xml_diff>
--- a/data/raw/personal_capacity_facts.xlsx
+++ b/data/raw/personal_capacity_facts.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="302" uniqueCount="143">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="326" uniqueCount="152">
   <si>
     <t xml:space="preserve">PERSONAL CAPACITY FACTS — Notas de uso</t>
   </si>
@@ -237,7 +237,7 @@
     <t xml:space="preserve">% Otros</t>
   </si>
   <si>
-    <t xml:space="preserve">Valoración cualitativa</t>
+    <t xml:space="preserve">Valoración cualitativa (concentración de ingresos)</t>
   </si>
   <si>
     <t xml:space="preserve">Pendiente</t>
@@ -282,6 +282,12 @@
     <t xml:space="preserve">% Liquidez</t>
   </si>
   <si>
+    <t xml:space="preserve">Valoración cualitativa (concentración de cartera)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RE-043.1 -- añadido para que el adaptador tenga una celda que leer; no hay umbral numérico de concentración acordado, es juicio del operador, no un cálculo</t>
+  </si>
+  <si>
     <t xml:space="preserve">5. RESTRICCIONES DE HORIZONTE CONOCIDO</t>
   </si>
   <si>
@@ -294,6 +300,12 @@
     <t xml:space="preserve">Confirmado — solo liquidez y Fondo Monetario, sin vencimientos</t>
   </si>
   <si>
+    <t xml:space="preserve">Próximo evento con necesidad de liquidez conocida</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RE-043.1 -- solo 'Ninguno conocido' se lee como favorable; en blanco el adaptador lo trata como no medido, nunca como favorable por defecto</t>
+  </si>
+  <si>
     <t xml:space="preserve">6. RESTRICCIONES FISCALES / OPERATIVAS</t>
   </si>
   <si>
@@ -303,6 +315,12 @@
     <t xml:space="preserve">Venta 2026, pendiente de compensar</t>
   </si>
   <si>
+    <t xml:space="preserve">Restricciones fiscales pendientes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RE-043.1 -- la minusvalía de arriba es favorable (reduce impuesto futuro), no una restricción; esta celda es para cualquier restricción fiscal/operativa aparte. Solo 'Ninguna conocida' se lee como favorable, en blanco = no medido</t>
+  </si>
+  <si>
     <t xml:space="preserve">PERSONAL CAPACITY FACTS — AML (patrimonio de tus padres)</t>
   </si>
   <si>
@@ -420,6 +438,9 @@
     <t xml:space="preserve">% TEF</t>
   </si>
   <si>
+    <t xml:space="preserve">RE-043.1 -- añadido para que el adaptador tenga una celda que leer; no hay umbral numérico de concentración acordado, es juicio del operador, no un cálculo. Nota: Iberdrola es 66% de la sub-cartera de Acciones pero solo ~8,4% del patrimonio total -- la concentración relevante depende de a qué nivel se mida</t>
+  </si>
+  <si>
     <t xml:space="preserve">Depósito Myinvestor — vencimiento</t>
   </si>
   <si>
@@ -447,10 +468,16 @@
     <t xml:space="preserve">Vence en breve — primer candidato a nutrir el Fondo Monetario</t>
   </si>
   <si>
+    <t xml:space="preserve">RE-043.1 -- los vencimientos de depósitos de arriba son liquidez entrante, no una necesidad de gasto -- no cuentan aquí. Solo 'Ninguno conocido' se lee como favorable, en blanco = no medido</t>
+  </si>
+  <si>
     <t xml:space="preserve">Planes de Pensiones — excluidos permanentemente</t>
   </si>
   <si>
     <t xml:space="preserve">Legalmente ilíquidos salvo jubilación/paro larga duración/enfermedad grave. Rescate tributa como rendimiento del trabajo — sumado a las pensiones, marginal cercano al 50%. No se van a tocar: destino, herencia para Armando y su hermana. No cuentan como pólvora seca ni liquidez bajo ningún escenario operativo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RE-043.1 -- la exclusión de Planes de Pensiones de arriba ya está gestionada y documentada; esta celda es para cualquier restricción fiscal/operativa adicional no capturada todavía. Solo 'Ninguna conocida' se lee como favorable, en blanco = no medido</t>
   </si>
 </sst>
 </file>
@@ -1055,7 +1082,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D57"/>
+  <dimension ref="A1:D60"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40"/>
@@ -1630,76 +1657,118 @@
       </c>
       <c r="D49" s="9"/>
     </row>
-    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="5" t="s">
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="B51" s="6"/>
-      <c r="C51" s="6"/>
-      <c r="D51" s="6"/>
+      <c r="B50" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="C50" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="D50" s="9" t="s">
+        <v>87</v>
+      </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="7" t="s">
+      <c r="A52" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="B52" s="6"/>
+      <c r="C52" s="6"/>
+      <c r="D52" s="6"/>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="B52" s="7" t="s">
+      <c r="B53" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="C52" s="7" t="s">
+      <c r="C53" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="D52" s="7" t="s">
+      <c r="D53" s="7" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="3" t="s">
-        <v>87</v>
-      </c>
-      <c r="B53" s="4" t="s">
-        <v>88</v>
-      </c>
-      <c r="C53" s="9" t="s">
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="B54" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="C54" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="D53" s="9" t="s">
-        <v>89</v>
+      <c r="D54" s="9" t="s">
+        <v>91</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="5" t="s">
-        <v>90</v>
-      </c>
-      <c r="B55" s="6"/>
-      <c r="C55" s="6"/>
-      <c r="D55" s="6"/>
-    </row>
-    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="7" t="s">
+      <c r="A55" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="B55" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="C55" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="D55" s="9" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="B57" s="6"/>
+      <c r="C57" s="6"/>
+      <c r="D57" s="6"/>
+    </row>
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="B56" s="7" t="s">
+      <c r="B58" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="C56" s="7" t="s">
+      <c r="C58" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="D56" s="7" t="s">
+      <c r="D58" s="7" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="B57" s="8" t="n">
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="B59" s="8" t="n">
         <v>-215092</v>
       </c>
-      <c r="C57" s="9" t="s">
+      <c r="C59" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="D57" s="9" t="s">
-        <v>92</v>
+      <c r="D59" s="9" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A60" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="B60" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="C60" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="D60" s="9" t="s">
+        <v>98</v>
       </c>
     </row>
   </sheetData>
@@ -1718,7 +1787,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D68"/>
+  <dimension ref="A1:D72"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44"/>
@@ -1729,7 +1798,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1765,7 +1834,7 @@
         <v>31</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1779,12 +1848,12 @@
         <v>31</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="B7" s="10" t="n">
         <f aca="false">B6-B5</f>
@@ -1794,7 +1863,7 @@
         <v>36</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1808,7 +1877,7 @@
         <v>31</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1860,7 +1929,7 @@
         <v>36</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1871,36 +1940,36 @@
         <v>54375</v>
       </c>
       <c r="C13" s="9" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="D13" s="9"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="B14" s="8" t="n">
         <v>60000</v>
       </c>
       <c r="C14" s="9" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="D14" s="9" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="B15" s="8" t="n">
         <v>85000</v>
       </c>
       <c r="C15" s="9" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="D15" s="9" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1914,7 +1983,7 @@
         <v>31</v>
       </c>
       <c r="D16" s="9" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1981,7 +2050,7 @@
         <v>36</v>
       </c>
       <c r="D21" s="9" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2057,7 +2126,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="3" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="B30" s="8" t="n">
         <v>60000</v>
@@ -2066,12 +2135,12 @@
         <v>31</v>
       </c>
       <c r="D30" s="9" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="3" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="B31" s="8" t="n">
         <v>20000</v>
@@ -2096,7 +2165,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="3" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
       <c r="B33" s="11" t="n">
         <f aca="false">B30/B32</f>
@@ -2109,7 +2178,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="3" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="B34" s="11" t="n">
         <f aca="false">B31/B32</f>
@@ -2125,13 +2194,13 @@
         <v>71</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="C35" s="9" t="s">
         <v>31</v>
       </c>
       <c r="D35" s="9" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2158,63 +2227,63 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="3" t="s">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="B39" s="8" t="n">
         <v>2183088.49</v>
       </c>
       <c r="C39" s="9" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="D39" s="9"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="3" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="B40" s="8" t="n">
         <v>1157519.11</v>
       </c>
       <c r="C40" s="9" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="D40" s="9" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="3" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="B41" s="8" t="n">
         <v>538013.75</v>
       </c>
       <c r="C41" s="9" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="D41" s="9"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="3" t="s">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="B42" s="8" t="n">
         <v>139351.5</v>
       </c>
       <c r="C42" s="9" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="D42" s="9"/>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="3" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="B43" s="8" t="n">
         <v>199375</v>
       </c>
       <c r="C43" s="9" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="D43" s="9"/>
     </row>
@@ -2233,7 +2302,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="3" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="B45" s="11" t="n">
         <f aca="false">B39/B44</f>
@@ -2246,7 +2315,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="3" t="s">
-        <v>121</v>
+        <v>127</v>
       </c>
       <c r="B46" s="11" t="n">
         <f aca="false">B40/B44</f>
@@ -2259,7 +2328,7 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="3" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="B47" s="11" t="n">
         <f aca="false">B41/B44</f>
@@ -2285,7 +2354,7 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="3" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
       <c r="B49" s="11" t="n">
         <f aca="false">B43/B44</f>
@@ -2298,48 +2367,48 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="2" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="3" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
       <c r="B52" s="8" t="n">
         <v>356040</v>
       </c>
       <c r="C52" s="9" t="s">
-        <v>126</v>
+        <v>132</v>
       </c>
       <c r="D52" s="9"/>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="3" t="s">
-        <v>127</v>
+        <v>133</v>
       </c>
       <c r="B53" s="8" t="n">
         <v>125804.4</v>
       </c>
       <c r="C53" s="9" t="s">
-        <v>126</v>
+        <v>132</v>
       </c>
       <c r="D53" s="9"/>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="3" t="s">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="B54" s="8" t="n">
         <v>56169.35</v>
       </c>
       <c r="C54" s="9" t="s">
-        <v>126</v>
+        <v>132</v>
       </c>
       <c r="D54" s="9"/>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="3" t="s">
-        <v>129</v>
+        <v>135</v>
       </c>
       <c r="B55" s="11" t="n">
         <f aca="false">B52/B41</f>
@@ -2352,7 +2421,7 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="3" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="B56" s="11" t="n">
         <f aca="false">B53/B41</f>
@@ -2365,7 +2434,7 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="3" t="s">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="B57" s="11" t="n">
         <f aca="false">B54/B41</f>
@@ -2376,118 +2445,160 @@
       </c>
       <c r="D57" s="9"/>
     </row>
-    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A59" s="5" t="s">
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="B59" s="6"/>
-      <c r="C59" s="6"/>
-      <c r="D59" s="6"/>
+      <c r="B58" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="C58" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="D58" s="9" t="s">
+        <v>138</v>
+      </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A60" s="7" t="s">
+      <c r="A60" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="B60" s="6"/>
+      <c r="C60" s="6"/>
+      <c r="D60" s="6"/>
+    </row>
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="B60" s="7" t="s">
+      <c r="B61" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="C60" s="7" t="s">
+      <c r="C61" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="D60" s="7" t="s">
+      <c r="D61" s="7" t="s">
         <v>29</v>
-      </c>
-    </row>
-    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="3" t="s">
-        <v>132</v>
-      </c>
-      <c r="B61" s="4" t="s">
-        <v>133</v>
-      </c>
-      <c r="C61" s="9" t="s">
-        <v>134</v>
-      </c>
-      <c r="D61" s="9" t="s">
-        <v>135</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="3" t="s">
-        <v>136</v>
-      </c>
-      <c r="B62" s="15" t="n">
+        <v>139</v>
+      </c>
+      <c r="B62" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="C62" s="9" t="s">
+        <v>141</v>
+      </c>
+      <c r="D62" s="9" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A63" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="B63" s="15" t="n">
         <f aca="true">DATE(2026,9,29)-TODAY()</f>
         <v>50</v>
       </c>
-      <c r="C62" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="D62" s="9"/>
-    </row>
-    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A63" s="3" t="s">
-        <v>137</v>
-      </c>
-      <c r="B63" s="4" t="s">
-        <v>138</v>
-      </c>
       <c r="C63" s="9" t="s">
-        <v>134</v>
-      </c>
-      <c r="D63" s="9" t="s">
-        <v>139</v>
-      </c>
+        <v>36</v>
+      </c>
+      <c r="D63" s="9"/>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="3" t="s">
-        <v>136</v>
-      </c>
-      <c r="B64" s="15" t="n">
+        <v>144</v>
+      </c>
+      <c r="B64" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="C64" s="9" t="s">
+        <v>141</v>
+      </c>
+      <c r="D64" s="9" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="B65" s="15" t="n">
         <f aca="true">DATE(2026,8,26)-TODAY()</f>
         <v>16</v>
       </c>
-      <c r="C64" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="D64" s="9" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A66" s="5" t="s">
-        <v>90</v>
-      </c>
-      <c r="B66" s="6"/>
-      <c r="C66" s="6"/>
-      <c r="D66" s="6"/>
+      <c r="C65" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="D65" s="9" t="s">
+        <v>147</v>
+      </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A67" s="7" t="s">
+      <c r="A67" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="B67" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="C67" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="D67" s="9" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A69" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="B69" s="6"/>
+      <c r="C69" s="6"/>
+      <c r="D69" s="6"/>
+    </row>
+    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A70" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="B67" s="7" t="s">
+      <c r="B70" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="C67" s="7" t="s">
+      <c r="C70" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="D67" s="7" t="s">
+      <c r="D70" s="7" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="68" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A68" s="3" t="s">
-        <v>141</v>
-      </c>
-      <c r="B68" s="8" t="n">
+    <row r="71" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A71" s="3" t="s">
+        <v>149</v>
+      </c>
+      <c r="B71" s="8" t="n">
         <v>1157519.11</v>
       </c>
-      <c r="C68" s="9" t="s">
+      <c r="C71" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="D68" s="9" t="s">
-        <v>142</v>
+      <c r="D71" s="9" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A72" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="B72" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="C72" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="D72" s="9" t="s">
+        <v>151</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
RE-043.2: resolver Pendientes restantes, primer resultado ADEQUATE
</commit_message>
<xml_diff>
--- a/data/raw/personal_capacity_facts.xlsx
+++ b/data/raw/personal_capacity_facts.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="326" uniqueCount="152">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="333" uniqueCount="158">
   <si>
     <t xml:space="preserve">PERSONAL CAPACITY FACTS — Notas de uso</t>
   </si>
@@ -138,6 +138,15 @@
     <t xml:space="preserve">Negativo = déficit que la cartera debe poder cubrir</t>
   </si>
   <si>
+    <t xml:space="preserve">Objetivo declarado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cerrar el gap con ingresos pasivos recurrentes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confirmado 2026-08-10 -- históricamente cubierto de sobra con ingresos de consultoría (variables, no 'ciertos y conocidos', por eso excluidos de 'Ingresos recurrentes anuales'), pero el objetivo es cerrar los 7.000€/año con fuentes pasivas predecibles, no seguir dependiendo de la consultoría. Contexto, no una de las nueve categorías del gate.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Colchón de seguridad mínimo (intocable)</t>
   </si>
   <si>
@@ -240,10 +249,10 @@
     <t xml:space="preserve">Valoración cualitativa (concentración de ingresos)</t>
   </si>
   <si>
-    <t xml:space="preserve">Pendiente</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ninguna fuente domina; dividendos ETF (38%) tienen correlación parcial con el ciclo de mercado</t>
+    <t xml:space="preserve">Adecuado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confirmado 2026-08-10 -- distribución correcta, ninguna fuente domina; dividendos ETF (38%) tienen correlación parcial con el ciclo de mercado. La preocupación real de Armando no es concentración sino cerrar el gap de 7.000€/año con ingresos pasivos -- ver 'Objetivo declarado' arriba</t>
   </si>
   <si>
     <t xml:space="preserve">4. CONCENTRACIÓN DE CARTERA</t>
@@ -285,7 +294,7 @@
     <t xml:space="preserve">Valoración cualitativa (concentración de cartera)</t>
   </si>
   <si>
-    <t xml:space="preserve">RE-043.1 -- añadido para que el adaptador tenga una celda que leer; no hay umbral numérico de concentración acordado, es juicio del operador, no un cálculo</t>
+    <t xml:space="preserve">Confirmado por Armando 2026-08-10 -- 69,5% en un único índice (SP500) considerado concentración aceptable dado que es un índice diversificado de 500 compañías, no una apuesta individual</t>
   </si>
   <si>
     <t xml:space="preserve">5. RESTRICCIONES DE HORIZONTE CONOCIDO</t>
@@ -303,7 +312,10 @@
     <t xml:space="preserve">Próximo evento con necesidad de liquidez conocida</t>
   </si>
   <si>
-    <t xml:space="preserve">RE-043.1 -- solo 'Ninguno conocido' se lee como favorable; en blanco el adaptador lo trata como no medido, nunca como favorable por defecto</t>
+    <t xml:space="preserve">Ninguno conocido</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confirmado 2026-08-10</t>
   </si>
   <si>
     <t xml:space="preserve">6. RESTRICCIONES FISCALES / OPERATIVAS</t>
@@ -312,13 +324,16 @@
     <t xml:space="preserve">Minusvalía pendiente de compensar (TEF)</t>
   </si>
   <si>
-    <t xml:space="preserve">Venta 2026, pendiente de compensar</t>
+    <t xml:space="preserve">Venta 2026. Crédito fiscal favorable, no una restricción -- 4 años para compensar vía plusvalías (confirmado por Armando 2026-08-10); si no se generan plusvalías suficientes en ese plazo, el crédito caduca sin usarse</t>
   </si>
   <si>
     <t xml:space="preserve">Restricciones fiscales pendientes</t>
   </si>
   <si>
-    <t xml:space="preserve">RE-043.1 -- la minusvalía de arriba es favorable (reduce impuesto futuro), no una restricción; esta celda es para cualquier restricción fiscal/operativa aparte. Solo 'Ninguna conocida' se lee como favorable, en blanco = no medido</t>
+    <t xml:space="preserve">Ninguna conocida</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confirmado 2026-08-10 -- la minusvalía de arriba es la única cuestión fiscal conocida, y es favorable, no restrictiva</t>
   </si>
   <si>
     <t xml:space="preserve">PERSONAL CAPACITY FACTS — AML (patrimonio de tus padres)</t>
@@ -378,9 +393,6 @@
     <t xml:space="preserve">% Dividendos</t>
   </si>
   <si>
-    <t xml:space="preserve">Adecuado</t>
-  </si>
-  <si>
     <t xml:space="preserve">Fuente dominante (pensión pública) es la más estable posible; ingreso total muy por encima del gasto</t>
   </si>
   <si>
@@ -438,7 +450,7 @@
     <t xml:space="preserve">% TEF</t>
   </si>
   <si>
-    <t xml:space="preserve">RE-043.1 -- añadido para que el adaptador tenga una celda que leer; no hay umbral numérico de concentración acordado, es juicio del operador, no un cálculo. Nota: Iberdrola es 66% de la sub-cartera de Acciones pero solo ~8,4% del patrimonio total -- la concentración relevante depende de a qué nivel se mida</t>
+    <t xml:space="preserve">Confirmado 2026-08-10 -- foco en USA/SP500 es la tesis de partida del SOP, no un riesgo a corregir. Verificado en '02. Fondos Myinvestor': Vanguard US500 87,2% + Fidelity S&amp;P500 0,4% (mismo índice, dos proveedores) + iShares Developed World 4,0%. Iberdrola 66% de la sub-cartera de Acciones mas solo 8,4% del patrimonio total, con función de renta vía dividendos, no de crecimiento</t>
   </si>
   <si>
     <t xml:space="preserve">Depósito Myinvestor — vencimiento</t>
@@ -468,7 +480,7 @@
     <t xml:space="preserve">Vence en breve — primer candidato a nutrir el Fondo Monetario</t>
   </si>
   <si>
-    <t xml:space="preserve">RE-043.1 -- los vencimientos de depósitos de arriba son liquidez entrante, no una necesidad de gasto -- no cuentan aquí. Solo 'Ninguno conocido' se lee como favorable, en blanco = no medido</t>
+    <t xml:space="preserve">Confirmado 2026-08-10. Los vencimientos de depósitos de arriba son liquidez entrante, no una necesidad de gasto -- no cuentan aquí.</t>
   </si>
   <si>
     <t xml:space="preserve">Planes de Pensiones — excluidos permanentemente</t>
@@ -477,7 +489,13 @@
     <t xml:space="preserve">Legalmente ilíquidos salvo jubilación/paro larga duración/enfermedad grave. Rescate tributa como rendimiento del trabajo — sumado a las pensiones, marginal cercano al 50%. No se van a tocar: destino, herencia para Armando y su hermana. No cuentan como pólvora seca ni liquidez bajo ningún escenario operativo.</t>
   </si>
   <si>
-    <t xml:space="preserve">RE-043.1 -- la exclusión de Planes de Pensiones de arriba ya está gestionada y documentada; esta celda es para cualquier restricción fiscal/operativa adicional no capturada todavía. Solo 'Ninguna conocida' se lee como favorable, en blanco = no medido</t>
+    <t xml:space="preserve">Manual (confirmado por Armando 2026-08-10)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Crédito fiscal favorable, no una restricción -- 4 años para compensar vía plusvalías; si no se generan plusvalías suficientes en ese plazo, el crédito caduca sin usarse</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confirmado 2026-08-10 -- la exclusión de Planes de Pensiones y la minusvalía TEF de arriba son las únicas cuestiones fiscales conocidas; ninguna de las dos es una restricción activa</t>
   </si>
 </sst>
 </file>
@@ -1082,7 +1100,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D60"/>
+  <dimension ref="A1:D61"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40"/>
@@ -1165,64 +1183,65 @@
       <c r="A8" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="B8" s="8" t="n">
-        <v>30000</v>
+      <c r="B8" s="4" t="s">
+        <v>39</v>
       </c>
       <c r="C8" s="9" t="s">
         <v>31</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B9" s="8" t="n">
-        <v>70000</v>
+        <v>30000</v>
       </c>
       <c r="C9" s="9" t="s">
         <v>31</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B10" s="8" t="n">
-        <v>120000</v>
+        <v>70000</v>
       </c>
       <c r="C10" s="9" t="s">
         <v>31</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="B11" s="10" t="n">
-        <f aca="false">B8+B9</f>
-        <v>100000</v>
+        <v>45</v>
+      </c>
+      <c r="B11" s="8" t="n">
+        <v>120000</v>
       </c>
       <c r="C11" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="D11" s="9"/>
+        <v>31</v>
+      </c>
+      <c r="D11" s="9" t="s">
+        <v>46</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B12" s="10" t="n">
-        <f aca="false">B8+B10</f>
-        <v>150000</v>
+        <f aca="false">B9+B10</f>
+        <v>100000</v>
       </c>
       <c r="C12" s="9" t="s">
         <v>36</v>
@@ -1231,52 +1250,52 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="B13" s="8" t="n">
-        <v>83100</v>
+        <v>48</v>
+      </c>
+      <c r="B13" s="10" t="n">
+        <f aca="false">B9+B11</f>
+        <v>150000</v>
       </c>
       <c r="C13" s="9" t="s">
-        <v>47</v>
-      </c>
-      <c r="D13" s="9" t="s">
-        <v>48</v>
-      </c>
+        <v>36</v>
+      </c>
+      <c r="D13" s="9"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
         <v>49</v>
       </c>
       <c r="B14" s="8" t="n">
-        <v>89230.77</v>
+        <v>83100</v>
       </c>
       <c r="C14" s="9" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="D14" s="9" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="B15" s="10" t="n">
-        <f aca="false">SUM(B13:B14)</f>
-        <v>172330.77</v>
+        <v>52</v>
+      </c>
+      <c r="B15" s="8" t="n">
+        <v>89230.77</v>
       </c>
       <c r="C15" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="D15" s="9"/>
+        <v>50</v>
+      </c>
+      <c r="D15" s="9" t="s">
+        <v>53</v>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B16" s="10" t="n">
-        <f aca="false">B15-B8</f>
-        <v>142330.77</v>
+        <f aca="false">SUM(B14:B15)</f>
+        <v>172330.77</v>
       </c>
       <c r="C16" s="9" t="s">
         <v>36</v>
@@ -1285,11 +1304,11 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B17" s="10" t="n">
-        <f aca="false">B15-B11</f>
-        <v>72330.77</v>
+        <f aca="false">B16-B9</f>
+        <v>142330.77</v>
       </c>
       <c r="C17" s="9" t="s">
         <v>36</v>
@@ -1298,121 +1317,122 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B18" s="10" t="n">
-        <f aca="false">B15-B12</f>
-        <v>22330.77</v>
+        <f aca="false">B16-B12</f>
+        <v>72330.77</v>
       </c>
       <c r="C18" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="D18" s="9" t="s">
-        <v>55</v>
-      </c>
+      <c r="D18" s="9"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B19" s="10" t="n">
-        <f aca="false">B16-B9</f>
-        <v>72330.77</v>
+        <f aca="false">B16-B13</f>
+        <v>22330.77</v>
       </c>
       <c r="C19" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="D19" s="9"/>
+      <c r="D19" s="9" t="s">
+        <v>58</v>
+      </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B20" s="10" t="n">
-        <f aca="false">B16-B10</f>
+        <f aca="false">B17-B10</f>
+        <v>72330.77</v>
+      </c>
+      <c r="C20" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="D20" s="9"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="B21" s="10" t="n">
+        <f aca="false">B17-B11</f>
         <v>22330.77</v>
       </c>
-      <c r="C20" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="D20" s="9"/>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="B22" s="6"/>
-      <c r="C22" s="6"/>
-      <c r="D22" s="6"/>
+      <c r="C21" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="D21" s="9"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="7" t="s">
+      <c r="A23" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="B23" s="6"/>
+      <c r="C23" s="6"/>
+      <c r="D23" s="6"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="B23" s="7" t="s">
+      <c r="B24" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="C23" s="7" t="s">
+      <c r="C24" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="D23" s="7" t="s">
+      <c r="D24" s="7" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="B24" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="C24" s="9" t="s">
-        <v>61</v>
-      </c>
-      <c r="D24" s="9" t="s">
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="3" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="5" t="s">
+      <c r="B25" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="B26" s="6"/>
-      <c r="C26" s="6"/>
-      <c r="D26" s="6"/>
+      <c r="C25" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="D25" s="9" t="s">
+        <v>65</v>
+      </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="7" t="s">
+      <c r="A27" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="B27" s="6"/>
+      <c r="C27" s="6"/>
+      <c r="D27" s="6"/>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="B27" s="7" t="s">
+      <c r="B28" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="C27" s="7" t="s">
+      <c r="C28" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="D27" s="7" t="s">
+      <c r="D28" s="7" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="B28" s="8" t="n">
-        <v>6000</v>
-      </c>
-      <c r="C28" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="D28" s="9"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="3" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B29" s="8" t="n">
-        <v>5000</v>
+        <v>6000</v>
       </c>
       <c r="C29" s="9" t="s">
         <v>31</v>
@@ -1421,10 +1441,10 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="3" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B30" s="8" t="n">
-        <v>2000</v>
+        <v>5000</v>
       </c>
       <c r="C30" s="9" t="s">
         <v>31</v>
@@ -1433,24 +1453,23 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="3" t="s">
-        <v>67</v>
-      </c>
-      <c r="B31" s="10" t="n">
-        <f aca="false">SUM(B28:B30)</f>
-        <v>13000</v>
+        <v>69</v>
+      </c>
+      <c r="B31" s="8" t="n">
+        <v>2000</v>
       </c>
       <c r="C31" s="9" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="D31" s="9"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="B32" s="11" t="n">
-        <f aca="false">B28/B31</f>
-        <v>0.461538461538462</v>
+        <v>70</v>
+      </c>
+      <c r="B32" s="10" t="n">
+        <f aca="false">SUM(B29:B31)</f>
+        <v>13000</v>
       </c>
       <c r="C32" s="9" t="s">
         <v>36</v>
@@ -1459,11 +1478,11 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="3" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B33" s="11" t="n">
-        <f aca="false">B29/B31</f>
-        <v>0.384615384615385</v>
+        <f aca="false">B29/B32</f>
+        <v>0.461538461538462</v>
       </c>
       <c r="C33" s="9" t="s">
         <v>36</v>
@@ -1472,11 +1491,11 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="3" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B34" s="11" t="n">
-        <f aca="false">B30/B31</f>
-        <v>0.153846153846154</v>
+        <f aca="false">B30/B32</f>
+        <v>0.384615384615385</v>
       </c>
       <c r="C34" s="9" t="s">
         <v>36</v>
@@ -1485,133 +1504,133 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="B35" s="4" t="s">
-        <v>72</v>
+        <v>73</v>
+      </c>
+      <c r="B35" s="11" t="n">
+        <f aca="false">B31/B32</f>
+        <v>0.153846153846154</v>
       </c>
       <c r="C35" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="D35" s="9"/>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="B36" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="C36" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="D35" s="9" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="B37" s="6"/>
-      <c r="C37" s="6"/>
-      <c r="D37" s="6"/>
+      <c r="D36" s="9" t="s">
+        <v>76</v>
+      </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="7" t="s">
+      <c r="A38" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="B38" s="6"/>
+      <c r="C38" s="6"/>
+      <c r="D38" s="6"/>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="B38" s="7" t="s">
+      <c r="B39" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="C38" s="7" t="s">
+      <c r="C39" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="D38" s="7" t="s">
+      <c r="D39" s="7" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="B39" s="8" t="n">
-        <v>872837.88</v>
-      </c>
-      <c r="C39" s="9" t="s">
-        <v>47</v>
-      </c>
-      <c r="D39" s="9"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="3" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B40" s="8" t="n">
-        <v>89230.77</v>
+        <v>872837.88</v>
       </c>
       <c r="C40" s="9" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="D40" s="9"/>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B41" s="8" t="n">
-        <v>111570.37</v>
+        <v>89230.77</v>
       </c>
       <c r="C41" s="9" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="D41" s="9"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="3" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B42" s="8" t="n">
-        <v>100000</v>
+        <v>111570.37</v>
       </c>
       <c r="C42" s="9" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="D42" s="9"/>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="3" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B43" s="8" t="n">
+        <v>100000</v>
+      </c>
+      <c r="C43" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="D43" s="9"/>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="B44" s="8" t="n">
         <v>83100</v>
       </c>
-      <c r="C43" s="9" t="s">
-        <v>47</v>
-      </c>
-      <c r="D43" s="9"/>
-    </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="12" t="s">
-        <v>80</v>
-      </c>
-      <c r="B44" s="13" t="n">
-        <f aca="false">SUM(B39:B43)</f>
+      <c r="C44" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="D44" s="9"/>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="12" t="s">
+        <v>83</v>
+      </c>
+      <c r="B45" s="13" t="n">
+        <f aca="false">SUM(B40:B44)</f>
         <v>1256739.02</v>
       </c>
-      <c r="C44" s="14" t="s">
-        <v>36</v>
-      </c>
-      <c r="D44" s="14"/>
-    </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="3" t="s">
-        <v>81</v>
-      </c>
-      <c r="B45" s="11" t="n">
-        <f aca="false">B39/B44</f>
-        <v>0.694525964507731</v>
-      </c>
-      <c r="C45" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="D45" s="9"/>
+      <c r="C45" s="14" t="s">
+        <v>36</v>
+      </c>
+      <c r="D45" s="14"/>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="3" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B46" s="11" t="n">
-        <f aca="false">B40/B44</f>
-        <v>0.0710018297991575</v>
+        <f aca="false">B40/B45</f>
+        <v>0.694525964507731</v>
       </c>
       <c r="C46" s="9" t="s">
         <v>36</v>
@@ -1620,11 +1639,11 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="3" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B47" s="11" t="n">
-        <f aca="false">B41/B44</f>
-        <v>0.0887776763707074</v>
+        <f aca="false">B41/B45</f>
+        <v>0.0710018297991575</v>
       </c>
       <c r="C47" s="9" t="s">
         <v>36</v>
@@ -1633,11 +1652,11 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="3" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B48" s="11" t="n">
-        <f aca="false">B42/B44</f>
-        <v>0.0795710154682712</v>
+        <f aca="false">B42/B45</f>
+        <v>0.0887776763707074</v>
       </c>
       <c r="C48" s="9" t="s">
         <v>36</v>
@@ -1646,11 +1665,11 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="3" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B49" s="11" t="n">
-        <f aca="false">B43/B44</f>
-        <v>0.0661235138541334</v>
+        <f aca="false">B43/B45</f>
+        <v>0.0795710154682712</v>
       </c>
       <c r="C49" s="9" t="s">
         <v>36</v>
@@ -1659,52 +1678,51 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="B50" s="4" t="s">
-        <v>72</v>
+        <v>88</v>
+      </c>
+      <c r="B50" s="11" t="n">
+        <f aca="false">B44/B45</f>
+        <v>0.0661235138541334</v>
       </c>
       <c r="C50" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="D50" s="9"/>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="B51" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="C51" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="D50" s="9" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="5" t="s">
-        <v>88</v>
-      </c>
-      <c r="B52" s="6"/>
-      <c r="C52" s="6"/>
-      <c r="D52" s="6"/>
+      <c r="D51" s="9" t="s">
+        <v>90</v>
+      </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="7" t="s">
+      <c r="A53" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="B53" s="6"/>
+      <c r="C53" s="6"/>
+      <c r="D53" s="6"/>
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="B53" s="7" t="s">
+      <c r="B54" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="C53" s="7" t="s">
+      <c r="C54" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="D53" s="7" t="s">
+      <c r="D54" s="7" t="s">
         <v>29</v>
-      </c>
-    </row>
-    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="B54" s="4" t="s">
-        <v>90</v>
-      </c>
-      <c r="C54" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="D54" s="9" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1712,63 +1730,77 @@
         <v>92</v>
       </c>
       <c r="B55" s="4" t="s">
-        <v>72</v>
+        <v>93</v>
       </c>
       <c r="C55" s="9" t="s">
         <v>31</v>
       </c>
       <c r="D55" s="9" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="5" t="s">
         <v>94</v>
       </c>
-      <c r="B57" s="6"/>
-      <c r="C57" s="6"/>
-      <c r="D57" s="6"/>
+    </row>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="B56" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="C56" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="D56" s="9" t="s">
+        <v>97</v>
+      </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="7" t="s">
+      <c r="A58" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="B58" s="6"/>
+      <c r="C58" s="6"/>
+      <c r="D58" s="6"/>
+    </row>
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="B58" s="7" t="s">
+      <c r="B59" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="C58" s="7" t="s">
+      <c r="C59" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="D58" s="7" t="s">
+      <c r="D59" s="7" t="s">
         <v>29</v>
-      </c>
-    </row>
-    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A59" s="3" t="s">
-        <v>95</v>
-      </c>
-      <c r="B59" s="8" t="n">
-        <v>-215092</v>
-      </c>
-      <c r="C59" s="9" t="s">
-        <v>47</v>
-      </c>
-      <c r="D59" s="9" t="s">
-        <v>96</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="3" t="s">
-        <v>97</v>
-      </c>
-      <c r="B60" s="4" t="s">
-        <v>72</v>
+        <v>99</v>
+      </c>
+      <c r="B60" s="8" t="n">
+        <v>-215092</v>
       </c>
       <c r="C60" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="D60" s="9" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="B61" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="C61" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="D60" s="9" t="s">
-        <v>98</v>
+      <c r="D61" s="9" t="s">
+        <v>103</v>
       </c>
     </row>
   </sheetData>
@@ -1787,7 +1819,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D72"/>
+  <dimension ref="A1:D73"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44"/>
@@ -1798,7 +1830,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1834,7 +1866,7 @@
         <v>31</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1848,12 +1880,12 @@
         <v>31</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="B7" s="10" t="n">
         <f aca="false">B6-B5</f>
@@ -1863,12 +1895,12 @@
         <v>36</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="B8" s="8" t="n">
         <v>125000</v>
@@ -1877,12 +1909,12 @@
         <v>31</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="B9" s="8" t="n">
         <v>125000</v>
@@ -1894,7 +1926,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="B10" s="8" t="n">
         <v>175000</v>
@@ -1906,7 +1938,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="B11" s="10" t="n">
         <f aca="false">B8+B9</f>
@@ -1919,7 +1951,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="B12" s="10" t="n">
         <f aca="false">B8+B10</f>
@@ -1929,52 +1961,52 @@
         <v>36</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="B13" s="8" t="n">
         <v>54375</v>
       </c>
       <c r="C13" s="9" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="D13" s="9"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="B14" s="8" t="n">
         <v>60000</v>
       </c>
       <c r="C14" s="9" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="D14" s="9" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="B15" s="8" t="n">
         <v>85000</v>
       </c>
       <c r="C15" s="9" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="D15" s="9" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="3" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="B16" s="8" t="n">
         <v>0</v>
@@ -1983,12 +2015,12 @@
         <v>31</v>
       </c>
       <c r="D16" s="9" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="B17" s="10" t="n">
         <f aca="false">SUM(B13:B16)</f>
@@ -2001,7 +2033,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="B18" s="10" t="n">
         <f aca="false">B17-B8</f>
@@ -2014,7 +2046,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="B19" s="10" t="n">
         <f aca="false">B17-B11</f>
@@ -2027,7 +2059,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="B20" s="10" t="n">
         <f aca="false">B17-B12</f>
@@ -2040,7 +2072,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="3" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="B21" s="10" t="n">
         <f aca="false">B18-B9</f>
@@ -2050,12 +2082,12 @@
         <v>36</v>
       </c>
       <c r="D21" s="9" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="3" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="B22" s="10" t="n">
         <f aca="false">B18-B10</f>
@@ -2068,7 +2100,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="5" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="B24" s="6"/>
       <c r="C24" s="6"/>
@@ -2090,21 +2122,21 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="3" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="C26" s="9" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="D26" s="9" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="5" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="B28" s="6"/>
       <c r="C28" s="6"/>
@@ -2126,7 +2158,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="3" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="B30" s="8" t="n">
         <v>60000</v>
@@ -2135,12 +2167,12 @@
         <v>31</v>
       </c>
       <c r="D30" s="9" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="3" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="B31" s="8" t="n">
         <v>20000</v>
@@ -2152,7 +2184,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="3" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="B32" s="10" t="n">
         <f aca="false">SUM(B30:B31)</f>
@@ -2165,7 +2197,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="3" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
       <c r="B33" s="11" t="n">
         <f aca="false">B30/B32</f>
@@ -2178,7 +2210,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="3" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="B34" s="11" t="n">
         <f aca="false">B31/B32</f>
@@ -2191,21 +2223,21 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="3" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>118</v>
+        <v>75</v>
       </c>
       <c r="C35" s="9" t="s">
         <v>31</v>
       </c>
       <c r="D35" s="9" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="5" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="B37" s="6"/>
       <c r="C37" s="6"/>
@@ -2227,69 +2259,69 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="3" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="B39" s="8" t="n">
         <v>2183088.49</v>
       </c>
       <c r="C39" s="9" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="D39" s="9"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="3" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="B40" s="8" t="n">
         <v>1157519.11</v>
       </c>
       <c r="C40" s="9" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="D40" s="9" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="3" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="B41" s="8" t="n">
         <v>538013.75</v>
       </c>
       <c r="C41" s="9" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="D41" s="9"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="3" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="B42" s="8" t="n">
         <v>139351.5</v>
       </c>
       <c r="C42" s="9" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="D42" s="9"/>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="3" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="B43" s="8" t="n">
         <v>199375</v>
       </c>
       <c r="C43" s="9" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="D43" s="9"/>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="12" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="B44" s="13" t="n">
         <f aca="false">SUM(B39:B43)</f>
@@ -2302,7 +2334,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="3" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="B45" s="11" t="n">
         <f aca="false">B39/B44</f>
@@ -2315,7 +2347,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="3" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="B46" s="11" t="n">
         <f aca="false">B40/B44</f>
@@ -2328,7 +2360,7 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="3" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="B47" s="11" t="n">
         <f aca="false">B41/B44</f>
@@ -2341,7 +2373,7 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="3" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="B48" s="11" t="n">
         <f aca="false">B42/B44</f>
@@ -2354,7 +2386,7 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="3" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="B49" s="11" t="n">
         <f aca="false">B43/B44</f>
@@ -2367,48 +2399,48 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="2" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="3" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="B52" s="8" t="n">
         <v>356040</v>
       </c>
       <c r="C52" s="9" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="D52" s="9"/>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="3" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="B53" s="8" t="n">
         <v>125804.4</v>
       </c>
       <c r="C53" s="9" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="D53" s="9"/>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="3" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="B54" s="8" t="n">
         <v>56169.35</v>
       </c>
       <c r="C54" s="9" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="D54" s="9"/>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="3" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="B55" s="11" t="n">
         <f aca="false">B52/B41</f>
@@ -2421,7 +2453,7 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="3" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="B56" s="11" t="n">
         <f aca="false">B53/B41</f>
@@ -2434,7 +2466,7 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="3" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="B57" s="11" t="n">
         <f aca="false">B54/B41</f>
@@ -2447,21 +2479,21 @@
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="3" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="B58" s="4" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="C58" s="9" t="s">
         <v>31</v>
       </c>
       <c r="D58" s="9" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="5" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="B60" s="6"/>
       <c r="C60" s="6"/>
@@ -2483,21 +2515,21 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="3" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="B62" s="4" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="C62" s="9" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="D62" s="9" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="3" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="B63" s="15" t="n">
         <f aca="true">DATE(2026,9,29)-TODAY()</f>
@@ -2510,21 +2542,21 @@
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="3" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="B64" s="4" t="s">
+        <v>149</v>
+      </c>
+      <c r="C64" s="9" t="s">
         <v>145</v>
       </c>
-      <c r="C64" s="9" t="s">
-        <v>141</v>
-      </c>
       <c r="D64" s="9" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="3" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="B65" s="15" t="n">
         <f aca="true">DATE(2026,8,26)-TODAY()</f>
@@ -2534,26 +2566,26 @@
         <v>36</v>
       </c>
       <c r="D65" s="9" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="3" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="B67" s="4" t="s">
-        <v>72</v>
+        <v>96</v>
       </c>
       <c r="C67" s="9" t="s">
         <v>31</v>
       </c>
       <c r="D67" s="9" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="5" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="B69" s="6"/>
       <c r="C69" s="6"/>
@@ -2575,7 +2607,7 @@
     </row>
     <row r="71" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A71" s="3" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="B71" s="8" t="n">
         <v>1157519.11</v>
@@ -2584,21 +2616,35 @@
         <v>31</v>
       </c>
       <c r="D71" s="9" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="3" t="s">
-        <v>97</v>
-      </c>
-      <c r="B72" s="4" t="s">
-        <v>72</v>
+        <v>99</v>
+      </c>
+      <c r="B72" s="8" t="n">
+        <v>-162000</v>
       </c>
       <c r="C72" s="9" t="s">
+        <v>155</v>
+      </c>
+      <c r="D72" s="9" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A73" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="B73" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="C73" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="D72" s="9" t="s">
-        <v>151</v>
+      <c r="D73" s="9" t="s">
+        <v>157</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
RE-043.2: aclarar etiqueta Liquidez en concentración de cartera (excluye FM)
</commit_message>
<xml_diff>
--- a/data/raw/personal_capacity_facts.xlsx
+++ b/data/raw/personal_capacity_facts.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="333" uniqueCount="158">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="335" uniqueCount="160">
   <si>
     <t xml:space="preserve">PERSONAL CAPACITY FACTS — Notas de uso</t>
   </si>
@@ -270,7 +270,10 @@
     <t xml:space="preserve">Pisos</t>
   </si>
   <si>
-    <t xml:space="preserve">Liquidez</t>
+    <t xml:space="preserve">Liquidez (excluido FM)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No confundir con 'Liquidez total actual' de la sección 1, que sí incluye el Fondo Monetario (172.330,77€) -- aquí el FM va aparte como clase de activo propia</t>
   </si>
   <si>
     <t xml:space="preserve">Total patrimonio</t>
@@ -288,7 +291,7 @@
     <t xml:space="preserve">% Pisos</t>
   </si>
   <si>
-    <t xml:space="preserve">% Liquidez</t>
+    <t xml:space="preserve">% Liquidez (excl. FM)</t>
   </si>
   <si>
     <t xml:space="preserve">Valoración cualitativa (concentración de cartera)</t>
@@ -411,7 +414,10 @@
     <t xml:space="preserve">ETF (Aristócratas)</t>
   </si>
   <si>
-    <t xml:space="preserve">Liquidez + Depósitos</t>
+    <t xml:space="preserve">Liquidez + Depósitos (excluido FM)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No confundir con 'Liquidez total actual' de la sección 1 -- hoy coinciden porque el FM de AML aún está a 0€, pero dejarán de coincidir en cuanto el FM se nutra de los depósitos al vencer</t>
   </si>
   <si>
     <t xml:space="preserve">% Fondos RV</t>
@@ -1609,11 +1615,13 @@
       <c r="C44" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="D44" s="9"/>
+      <c r="D44" s="9" t="s">
+        <v>83</v>
+      </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="12" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B45" s="13" t="n">
         <f aca="false">SUM(B40:B44)</f>
@@ -1626,7 +1634,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="3" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B46" s="11" t="n">
         <f aca="false">B40/B45</f>
@@ -1639,7 +1647,7 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="3" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B47" s="11" t="n">
         <f aca="false">B41/B45</f>
@@ -1652,7 +1660,7 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="3" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B48" s="11" t="n">
         <f aca="false">B42/B45</f>
@@ -1665,7 +1673,7 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="3" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B49" s="11" t="n">
         <f aca="false">B43/B45</f>
@@ -1678,7 +1686,7 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="3" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B50" s="11" t="n">
         <f aca="false">B44/B45</f>
@@ -1691,7 +1699,7 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="3" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B51" s="4" t="s">
         <v>75</v>
@@ -1700,12 +1708,12 @@
         <v>31</v>
       </c>
       <c r="D51" s="9" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="5" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B53" s="6"/>
       <c r="C53" s="6"/>
@@ -1727,35 +1735,35 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="3" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B55" s="4" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C55" s="9" t="s">
         <v>31</v>
       </c>
       <c r="D55" s="9" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="3" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B56" s="4" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C56" s="9" t="s">
         <v>31</v>
       </c>
       <c r="D56" s="9" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="5" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B58" s="6"/>
       <c r="C58" s="6"/>
@@ -1777,7 +1785,7 @@
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="3" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B60" s="8" t="n">
         <v>-215092</v>
@@ -1786,21 +1794,21 @@
         <v>50</v>
       </c>
       <c r="D60" s="9" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="3" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B61" s="4" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C61" s="9" t="s">
         <v>31</v>
       </c>
       <c r="D61" s="9" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
   </sheetData>
@@ -1830,7 +1838,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1866,7 +1874,7 @@
         <v>31</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1880,12 +1888,12 @@
         <v>31</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B7" s="10" t="n">
         <f aca="false">B6-B5</f>
@@ -1895,7 +1903,7 @@
         <v>36</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1909,7 +1917,7 @@
         <v>31</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1961,7 +1969,7 @@
         <v>36</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1972,36 +1980,36 @@
         <v>54375</v>
       </c>
       <c r="C13" s="9" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D13" s="9"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B14" s="8" t="n">
         <v>60000</v>
       </c>
       <c r="C14" s="9" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D14" s="9" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B15" s="8" t="n">
         <v>85000</v>
       </c>
       <c r="C15" s="9" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D15" s="9" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2015,7 +2023,7 @@
         <v>31</v>
       </c>
       <c r="D16" s="9" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2082,7 +2090,7 @@
         <v>36</v>
       </c>
       <c r="D21" s="9" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2158,7 +2166,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="3" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B30" s="8" t="n">
         <v>60000</v>
@@ -2167,12 +2175,12 @@
         <v>31</v>
       </c>
       <c r="D30" s="9" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="3" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B31" s="8" t="n">
         <v>20000</v>
@@ -2197,7 +2205,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="3" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="B33" s="11" t="n">
         <f aca="false">B30/B32</f>
@@ -2210,7 +2218,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="3" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="B34" s="11" t="n">
         <f aca="false">B31/B32</f>
@@ -2232,7 +2240,7 @@
         <v>31</v>
       </c>
       <c r="D35" s="9" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2259,69 +2267,71 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="3" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B39" s="8" t="n">
         <v>2183088.49</v>
       </c>
       <c r="C39" s="9" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D39" s="9"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="3" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B40" s="8" t="n">
         <v>1157519.11</v>
       </c>
       <c r="C40" s="9" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D40" s="9" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="3" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B41" s="8" t="n">
         <v>538013.75</v>
       </c>
       <c r="C41" s="9" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D41" s="9"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="3" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B42" s="8" t="n">
         <v>139351.5</v>
       </c>
       <c r="C42" s="9" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D42" s="9"/>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="3" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B43" s="8" t="n">
         <v>199375</v>
       </c>
       <c r="C43" s="9" t="s">
-        <v>111</v>
-      </c>
-      <c r="D43" s="9"/>
+        <v>112</v>
+      </c>
+      <c r="D43" s="9" t="s">
+        <v>131</v>
+      </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="12" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B44" s="13" t="n">
         <f aca="false">SUM(B39:B43)</f>
@@ -2334,7 +2344,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="3" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B45" s="11" t="n">
         <f aca="false">B39/B44</f>
@@ -2347,7 +2357,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="3" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B46" s="11" t="n">
         <f aca="false">B40/B44</f>
@@ -2360,7 +2370,7 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="3" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B47" s="11" t="n">
         <f aca="false">B41/B44</f>
@@ -2373,7 +2383,7 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="3" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B48" s="11" t="n">
         <f aca="false">B42/B44</f>
@@ -2386,7 +2396,7 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="3" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="B49" s="11" t="n">
         <f aca="false">B43/B44</f>
@@ -2399,48 +2409,48 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="2" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="3" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B52" s="8" t="n">
         <v>356040</v>
       </c>
       <c r="C52" s="9" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="D52" s="9"/>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="3" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B53" s="8" t="n">
         <v>125804.4</v>
       </c>
       <c r="C53" s="9" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="D53" s="9"/>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="3" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B54" s="8" t="n">
         <v>56169.35</v>
       </c>
       <c r="C54" s="9" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="D54" s="9"/>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="3" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B55" s="11" t="n">
         <f aca="false">B52/B41</f>
@@ -2453,7 +2463,7 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="3" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="B56" s="11" t="n">
         <f aca="false">B53/B41</f>
@@ -2466,7 +2476,7 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="3" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B57" s="11" t="n">
         <f aca="false">B54/B41</f>
@@ -2479,7 +2489,7 @@
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="3" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B58" s="4" t="s">
         <v>75</v>
@@ -2488,12 +2498,12 @@
         <v>31</v>
       </c>
       <c r="D58" s="9" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="5" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B60" s="6"/>
       <c r="C60" s="6"/>
@@ -2515,21 +2525,21 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="3" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="B62" s="4" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="C62" s="9" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="D62" s="9" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="3" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="B63" s="15" t="n">
         <f aca="true">DATE(2026,9,29)-TODAY()</f>
@@ -2542,21 +2552,21 @@
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="3" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B64" s="4" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="C64" s="9" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="D64" s="9" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="3" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="B65" s="15" t="n">
         <f aca="true">DATE(2026,8,26)-TODAY()</f>
@@ -2566,26 +2576,26 @@
         <v>36</v>
       </c>
       <c r="D65" s="9" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="3" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B67" s="4" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C67" s="9" t="s">
         <v>31</v>
       </c>
       <c r="D67" s="9" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="5" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B69" s="6"/>
       <c r="C69" s="6"/>
@@ -2607,7 +2617,7 @@
     </row>
     <row r="71" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A71" s="3" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="B71" s="8" t="n">
         <v>1157519.11</v>
@@ -2616,35 +2626,35 @@
         <v>31</v>
       </c>
       <c r="D71" s="9" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="3" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B72" s="8" t="n">
         <v>-162000</v>
       </c>
       <c r="C72" s="9" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D72" s="9" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="3" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B73" s="4" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C73" s="9" t="s">
         <v>31</v>
       </c>
       <c r="D73" s="9" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
cosmetic: wrap_text on all cells across project xlsx files
</commit_message>
<xml_diff>
--- a/data/raw/personal_capacity_facts.xlsx
+++ b/data/raw/personal_capacity_facts.xlsx
@@ -634,69 +634,81 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="19">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="167" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -954,139 +966,139 @@
   <dimension ref="A1:B24"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="38"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="70"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="70"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="s">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="4" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="2" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="3" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="4" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="3" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="4" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="2" t="s">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="3" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="3" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="B10" s="4" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="3" t="s">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="B11" s="3" t="s">
+      <c r="B11" s="4" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="3" t="s">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="B12" s="3" t="s">
+      <c r="B12" s="4" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="2" t="s">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="B14" s="3" t="s">
+      <c r="B14" s="4" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="2" t="s">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="B16" s="3" t="s">
+      <c r="B16" s="4" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="2" t="s">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="3" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="3" t="s">
+      <c r="A19" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="B19" s="3" t="s">
+      <c r="B19" s="4" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="3" t="s">
+      <c r="A20" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="B20" s="3" t="s">
+      <c r="B20" s="4" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="3" t="s">
+      <c r="A21" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="B21" s="3" t="s">
+      <c r="B21" s="4" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="3" t="s">
+      <c r="A22" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="B22" s="3" t="s">
+      <c r="B22" s="4" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="3" t="s">
+      <c r="A23" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="B23" s="3" t="s">
+      <c r="B23" s="4" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="3" t="s">
+      <c r="A24" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="B24" s="3" t="s">
+      <c r="B24" s="4" t="s">
         <v>23</v>
       </c>
     </row>
@@ -1109,705 +1121,705 @@
   <dimension ref="A1:D61"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="46"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="5" t="s">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="B3" s="6"/>
-      <c r="C3" s="6"/>
-      <c r="D3" s="6"/>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="7" t="s">
+      <c r="B3" s="7"/>
+      <c r="C3" s="7"/>
+      <c r="D3" s="7"/>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="B4" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="C4" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="D4" s="7" t="s">
+      <c r="D4" s="8" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="B5" s="8" t="n">
+      <c r="B5" s="9" t="n">
         <v>20000</v>
       </c>
-      <c r="C5" s="9" t="s">
+      <c r="C5" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="D5" s="9" t="s">
+      <c r="D5" s="10" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="3" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="B6" s="8" t="n">
+      <c r="B6" s="9" t="n">
         <v>13000</v>
       </c>
-      <c r="C6" s="9" t="s">
+      <c r="C6" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="D6" s="9" t="s">
+      <c r="D6" s="10" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="3" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="B7" s="10" t="n">
+      <c r="B7" s="11" t="n">
         <f aca="false">B6-B5</f>
         <v>-7000</v>
       </c>
-      <c r="C7" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="D7" s="9" t="s">
+      <c r="C7" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="D7" s="10" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="3" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="C8" s="9" t="s">
+      <c r="C8" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="D8" s="9" t="s">
+      <c r="D8" s="10" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3" t="s">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="B9" s="8" t="n">
+      <c r="B9" s="9" t="n">
         <v>30000</v>
       </c>
-      <c r="C9" s="9" t="s">
+      <c r="C9" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="D9" s="9" t="s">
+      <c r="D9" s="10" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="3" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="B10" s="8" t="n">
+      <c r="B10" s="9" t="n">
         <v>70000</v>
       </c>
-      <c r="C10" s="9" t="s">
+      <c r="C10" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="D10" s="9" t="s">
+      <c r="D10" s="10" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="3" t="s">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="B11" s="8" t="n">
+      <c r="B11" s="9" t="n">
         <v>120000</v>
       </c>
-      <c r="C11" s="9" t="s">
+      <c r="C11" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="D11" s="9" t="s">
+      <c r="D11" s="10" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="3" t="s">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="B12" s="10" t="n">
+      <c r="B12" s="11" t="n">
         <f aca="false">B9+B10</f>
         <v>100000</v>
       </c>
-      <c r="C12" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="D12" s="9"/>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="3" t="s">
+      <c r="C12" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="D12" s="12"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="B13" s="10" t="n">
+      <c r="B13" s="11" t="n">
         <f aca="false">B9+B11</f>
         <v>150000</v>
       </c>
-      <c r="C13" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="D13" s="9"/>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="3" t="s">
+      <c r="C13" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="D13" s="12"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="B14" s="8" t="n">
+      <c r="B14" s="9" t="n">
         <v>83100</v>
       </c>
-      <c r="C14" s="9" t="s">
+      <c r="C14" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="D14" s="9" t="s">
+      <c r="D14" s="10" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="3" t="s">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="B15" s="8" t="n">
+      <c r="B15" s="9" t="n">
         <v>89230.77</v>
       </c>
-      <c r="C15" s="9" t="s">
+      <c r="C15" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="D15" s="9" t="s">
+      <c r="D15" s="10" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="3" t="s">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="B16" s="10" t="n">
+      <c r="B16" s="11" t="n">
         <f aca="false">SUM(B14:B15)</f>
         <v>172330.77</v>
       </c>
-      <c r="C16" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="D16" s="9"/>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="3" t="s">
+      <c r="C16" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="D16" s="12"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="B17" s="10" t="n">
+      <c r="B17" s="11" t="n">
         <f aca="false">B16-B9</f>
         <v>142330.77</v>
       </c>
-      <c r="C17" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="D17" s="9"/>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="3" t="s">
+      <c r="C17" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="D17" s="12"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="B18" s="10" t="n">
+      <c r="B18" s="11" t="n">
         <f aca="false">B16-B12</f>
         <v>72330.77</v>
       </c>
-      <c r="C18" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="D18" s="9"/>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="3" t="s">
+      <c r="C18" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="D18" s="12"/>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="B19" s="10" t="n">
+      <c r="B19" s="11" t="n">
         <f aca="false">B16-B13</f>
         <v>22330.77</v>
       </c>
-      <c r="C19" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="D19" s="9" t="s">
+      <c r="C19" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="D19" s="10" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="3" t="s">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="B20" s="10" t="n">
+      <c r="B20" s="11" t="n">
         <f aca="false">B17-B10</f>
         <v>72330.77</v>
       </c>
-      <c r="C20" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="D20" s="9"/>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="3" t="s">
+      <c r="C20" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="D20" s="12"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="B21" s="10" t="n">
+      <c r="B21" s="11" t="n">
         <f aca="false">B17-B11</f>
         <v>22330.77</v>
       </c>
-      <c r="C21" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="D21" s="9"/>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="5" t="s">
+      <c r="C21" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="D21" s="12"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="B23" s="6"/>
-      <c r="C23" s="6"/>
-      <c r="D23" s="6"/>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="7" t="s">
+      <c r="B23" s="7"/>
+      <c r="C23" s="7"/>
+      <c r="D23" s="7"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="B24" s="7" t="s">
+      <c r="B24" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="C24" s="7" t="s">
+      <c r="C24" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="D24" s="7" t="s">
+      <c r="D24" s="8" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="3" t="s">
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="B25" s="4" t="s">
+      <c r="B25" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="C25" s="9" t="s">
+      <c r="C25" s="10" t="s">
         <v>64</v>
       </c>
-      <c r="D25" s="9" t="s">
+      <c r="D25" s="10" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="5" t="s">
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="B27" s="6"/>
-      <c r="C27" s="6"/>
-      <c r="D27" s="6"/>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="7" t="s">
+      <c r="B27" s="7"/>
+      <c r="C27" s="7"/>
+      <c r="D27" s="7"/>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="B28" s="7" t="s">
+      <c r="B28" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="C28" s="7" t="s">
+      <c r="C28" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="D28" s="7" t="s">
+      <c r="D28" s="8" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="3" t="s">
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="B29" s="8" t="n">
+      <c r="B29" s="9" t="n">
         <v>6000</v>
       </c>
-      <c r="C29" s="9" t="s">
+      <c r="C29" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="D29" s="9"/>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="3" t="s">
+      <c r="D29" s="12"/>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="B30" s="8" t="n">
+      <c r="B30" s="9" t="n">
         <v>5000</v>
       </c>
-      <c r="C30" s="9" t="s">
+      <c r="C30" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="D30" s="9"/>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="3" t="s">
+      <c r="D30" s="12"/>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="B31" s="8" t="n">
+      <c r="B31" s="9" t="n">
         <v>2000</v>
       </c>
-      <c r="C31" s="9" t="s">
+      <c r="C31" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="D31" s="9"/>
-    </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="3" t="s">
+      <c r="D31" s="12"/>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="B32" s="10" t="n">
+      <c r="B32" s="11" t="n">
         <f aca="false">SUM(B29:B31)</f>
         <v>13000</v>
       </c>
-      <c r="C32" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="D32" s="9"/>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="3" t="s">
+      <c r="C32" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="D32" s="12"/>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="B33" s="11" t="n">
+      <c r="B33" s="13" t="n">
         <f aca="false">B29/B32</f>
         <v>0.461538461538462</v>
       </c>
-      <c r="C33" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="D33" s="9"/>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="3" t="s">
+      <c r="C33" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="D33" s="12"/>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="B34" s="11" t="n">
+      <c r="B34" s="13" t="n">
         <f aca="false">B30/B32</f>
         <v>0.384615384615385</v>
       </c>
-      <c r="C34" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="D34" s="9"/>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="3" t="s">
+      <c r="C34" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="D34" s="12"/>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="B35" s="11" t="n">
+      <c r="B35" s="13" t="n">
         <f aca="false">B31/B32</f>
         <v>0.153846153846154</v>
       </c>
-      <c r="C35" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="D35" s="9"/>
-    </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="3" t="s">
+      <c r="C35" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="D35" s="12"/>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="B36" s="4" t="s">
+      <c r="B36" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="C36" s="9" t="s">
+      <c r="C36" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="D36" s="9" t="s">
+      <c r="D36" s="10" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="5" t="s">
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="B38" s="6"/>
-      <c r="C38" s="6"/>
-      <c r="D38" s="6"/>
-    </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="7" t="s">
+      <c r="B38" s="7"/>
+      <c r="C38" s="7"/>
+      <c r="D38" s="7"/>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="B39" s="7" t="s">
+      <c r="B39" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="C39" s="7" t="s">
+      <c r="C39" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="D39" s="7" t="s">
+      <c r="D39" s="8" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="3" t="s">
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="B40" s="8" t="n">
+      <c r="B40" s="9" t="n">
         <v>872837.88</v>
       </c>
-      <c r="C40" s="9" t="s">
+      <c r="C40" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="D40" s="9"/>
-    </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="3" t="s">
+      <c r="D40" s="12"/>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="B41" s="8" t="n">
+      <c r="B41" s="9" t="n">
         <v>89230.77</v>
       </c>
-      <c r="C41" s="9" t="s">
+      <c r="C41" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="D41" s="9"/>
-    </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="3" t="s">
+      <c r="D41" s="12"/>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="B42" s="8" t="n">
+      <c r="B42" s="9" t="n">
         <v>111570.37</v>
       </c>
-      <c r="C42" s="9" t="s">
+      <c r="C42" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="D42" s="9"/>
-    </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="3" t="s">
+      <c r="D42" s="12"/>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="B43" s="8" t="n">
+      <c r="B43" s="9" t="n">
         <v>100000</v>
       </c>
-      <c r="C43" s="9" t="s">
+      <c r="C43" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="D43" s="9"/>
-    </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="3" t="s">
+      <c r="D43" s="12"/>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A44" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="B44" s="8" t="n">
+      <c r="B44" s="9" t="n">
         <v>83100</v>
       </c>
-      <c r="C44" s="9" t="s">
+      <c r="C44" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="D44" s="9" t="s">
+      <c r="D44" s="10" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="12" t="s">
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A45" s="14" t="s">
         <v>84</v>
       </c>
-      <c r="B45" s="13" t="n">
+      <c r="B45" s="15" t="n">
         <f aca="false">SUM(B40:B44)</f>
         <v>1256739.02</v>
       </c>
-      <c r="C45" s="14" t="s">
-        <v>36</v>
-      </c>
-      <c r="D45" s="14"/>
-    </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="3" t="s">
+      <c r="C45" s="16" t="s">
+        <v>36</v>
+      </c>
+      <c r="D45" s="17"/>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A46" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="B46" s="11" t="n">
+      <c r="B46" s="13" t="n">
         <f aca="false">B40/B45</f>
         <v>0.694525964507731</v>
       </c>
-      <c r="C46" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="D46" s="9"/>
-    </row>
-    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="3" t="s">
+      <c r="C46" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="D46" s="12"/>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A47" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="B47" s="11" t="n">
+      <c r="B47" s="13" t="n">
         <f aca="false">B41/B45</f>
         <v>0.0710018297991575</v>
       </c>
-      <c r="C47" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="D47" s="9"/>
-    </row>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="3" t="s">
+      <c r="C47" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="D47" s="12"/>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A48" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="B48" s="11" t="n">
+      <c r="B48" s="13" t="n">
         <f aca="false">B42/B45</f>
         <v>0.0887776763707074</v>
       </c>
-      <c r="C48" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="D48" s="9"/>
-    </row>
-    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="3" t="s">
+      <c r="C48" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="D48" s="12"/>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A49" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="B49" s="11" t="n">
+      <c r="B49" s="13" t="n">
         <f aca="false">B43/B45</f>
         <v>0.0795710154682712</v>
       </c>
-      <c r="C49" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="D49" s="9"/>
-    </row>
-    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="3" t="s">
+      <c r="C49" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="D49" s="12"/>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A50" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="B50" s="11" t="n">
+      <c r="B50" s="13" t="n">
         <f aca="false">B44/B45</f>
         <v>0.0661235138541334</v>
       </c>
-      <c r="C50" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="D50" s="9"/>
-    </row>
-    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="3" t="s">
+      <c r="C50" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="D50" s="12"/>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A51" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="B51" s="4" t="s">
+      <c r="B51" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="C51" s="9" t="s">
+      <c r="C51" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="D51" s="9" t="s">
+      <c r="D51" s="10" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="5" t="s">
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A53" s="6" t="s">
         <v>92</v>
       </c>
-      <c r="B53" s="6"/>
-      <c r="C53" s="6"/>
-      <c r="D53" s="6"/>
-    </row>
-    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="7" t="s">
+      <c r="B53" s="7"/>
+      <c r="C53" s="7"/>
+      <c r="D53" s="7"/>
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A54" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="B54" s="7" t="s">
+      <c r="B54" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="C54" s="7" t="s">
+      <c r="C54" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="D54" s="7" t="s">
+      <c r="D54" s="8" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="3" t="s">
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A55" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="B55" s="4" t="s">
+      <c r="B55" s="5" t="s">
         <v>94</v>
       </c>
-      <c r="C55" s="9" t="s">
+      <c r="C55" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="D55" s="9" t="s">
+      <c r="D55" s="10" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="3" t="s">
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A56" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="B56" s="4" t="s">
+      <c r="B56" s="5" t="s">
         <v>97</v>
       </c>
-      <c r="C56" s="9" t="s">
+      <c r="C56" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="D56" s="9" t="s">
+      <c r="D56" s="10" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="5" t="s">
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A58" s="6" t="s">
         <v>99</v>
       </c>
-      <c r="B58" s="6"/>
-      <c r="C58" s="6"/>
-      <c r="D58" s="6"/>
-    </row>
-    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A59" s="7" t="s">
+      <c r="B58" s="7"/>
+      <c r="C58" s="7"/>
+      <c r="D58" s="7"/>
+    </row>
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A59" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="B59" s="7" t="s">
+      <c r="B59" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="C59" s="7" t="s">
+      <c r="C59" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="D59" s="7" t="s">
+      <c r="D59" s="8" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A60" s="3" t="s">
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A60" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="B60" s="8" t="n">
+      <c r="B60" s="9" t="n">
         <v>-215092</v>
       </c>
-      <c r="C60" s="9" t="s">
+      <c r="C60" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="D60" s="9" t="s">
+      <c r="D60" s="10" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="3" t="s">
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A61" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="B61" s="4" t="s">
+      <c r="B61" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="C61" s="9" t="s">
+      <c r="C61" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="D61" s="9" t="s">
+      <c r="D61" s="10" t="s">
         <v>104</v>
       </c>
     </row>
@@ -1830,830 +1842,830 @@
   <dimension ref="A1:D73"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="50"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="50"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="5" t="s">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="B3" s="6"/>
-      <c r="C3" s="6"/>
-      <c r="D3" s="6"/>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="7" t="s">
+      <c r="B3" s="7"/>
+      <c r="C3" s="7"/>
+      <c r="D3" s="7"/>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="B4" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="C4" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="D4" s="7" t="s">
+      <c r="D4" s="8" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="B5" s="8" t="n">
+      <c r="B5" s="9" t="n">
         <v>32500</v>
       </c>
-      <c r="C5" s="9" t="s">
+      <c r="C5" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="D5" s="9" t="s">
+      <c r="D5" s="10" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="3" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="B6" s="8" t="n">
+      <c r="B6" s="9" t="n">
         <v>80000</v>
       </c>
-      <c r="C6" s="9" t="s">
+      <c r="C6" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="D6" s="9" t="s">
+      <c r="D6" s="10" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="3" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="B7" s="10" t="n">
+      <c r="B7" s="11" t="n">
         <f aca="false">B6-B5</f>
         <v>47500</v>
       </c>
-      <c r="C7" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="D7" s="9" t="s">
+      <c r="C7" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="D7" s="10" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="3" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="B8" s="8" t="n">
+      <c r="B8" s="9" t="n">
         <v>125000</v>
       </c>
-      <c r="C8" s="9" t="s">
+      <c r="C8" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="D8" s="9" t="s">
+      <c r="D8" s="10" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3" t="s">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="B9" s="8" t="n">
+      <c r="B9" s="9" t="n">
         <v>125000</v>
       </c>
-      <c r="C9" s="9" t="s">
+      <c r="C9" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="D9" s="9"/>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="3" t="s">
+      <c r="D9" s="12"/>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="B10" s="8" t="n">
+      <c r="B10" s="9" t="n">
         <v>175000</v>
       </c>
-      <c r="C10" s="9" t="s">
+      <c r="C10" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="D10" s="9"/>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="3" t="s">
+      <c r="D10" s="12"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="B11" s="10" t="n">
+      <c r="B11" s="11" t="n">
         <f aca="false">B8+B9</f>
         <v>250000</v>
       </c>
-      <c r="C11" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="D11" s="9"/>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="3" t="s">
+      <c r="C11" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="D11" s="12"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="B12" s="10" t="n">
+      <c r="B12" s="11" t="n">
         <f aca="false">B8+B10</f>
         <v>300000</v>
       </c>
-      <c r="C12" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="D12" s="9" t="s">
+      <c r="C12" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="D12" s="10" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="3" t="s">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="B13" s="8" t="n">
+      <c r="B13" s="9" t="n">
         <v>54375</v>
       </c>
-      <c r="C13" s="9" t="s">
+      <c r="C13" s="10" t="s">
         <v>112</v>
       </c>
-      <c r="D13" s="9"/>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="3" t="s">
+      <c r="D13" s="12"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="4" t="s">
         <v>113</v>
       </c>
-      <c r="B14" s="8" t="n">
+      <c r="B14" s="9" t="n">
         <v>60000</v>
       </c>
-      <c r="C14" s="9" t="s">
+      <c r="C14" s="10" t="s">
         <v>112</v>
       </c>
-      <c r="D14" s="9" t="s">
+      <c r="D14" s="10" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="3" t="s">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="4" t="s">
         <v>115</v>
       </c>
-      <c r="B15" s="8" t="n">
+      <c r="B15" s="9" t="n">
         <v>85000</v>
       </c>
-      <c r="C15" s="9" t="s">
+      <c r="C15" s="10" t="s">
         <v>112</v>
       </c>
-      <c r="D15" s="9" t="s">
+      <c r="D15" s="10" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="3" t="s">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="B16" s="8" t="n">
+      <c r="B16" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="C16" s="9" t="s">
+      <c r="C16" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="D16" s="9" t="s">
+      <c r="D16" s="10" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="3" t="s">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="B17" s="10" t="n">
+      <c r="B17" s="11" t="n">
         <f aca="false">SUM(B13:B16)</f>
         <v>199375</v>
       </c>
-      <c r="C17" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="D17" s="9"/>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="3" t="s">
+      <c r="C17" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="D17" s="12"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="B18" s="10" t="n">
+      <c r="B18" s="11" t="n">
         <f aca="false">B17-B8</f>
         <v>74375</v>
       </c>
-      <c r="C18" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="D18" s="9"/>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="3" t="s">
+      <c r="C18" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="D18" s="12"/>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="B19" s="10" t="n">
+      <c r="B19" s="11" t="n">
         <f aca="false">B17-B11</f>
         <v>-50625</v>
       </c>
-      <c r="C19" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="D19" s="9"/>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="3" t="s">
+      <c r="C19" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="D19" s="12"/>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="B20" s="10" t="n">
+      <c r="B20" s="11" t="n">
         <f aca="false">B17-B12</f>
         <v>-100625</v>
       </c>
-      <c r="C20" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="D20" s="9"/>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="3" t="s">
+      <c r="C20" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="D20" s="12"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="B21" s="10" t="n">
+      <c r="B21" s="11" t="n">
         <f aca="false">B18-B9</f>
         <v>-50625</v>
       </c>
-      <c r="C21" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="D21" s="9" t="s">
+      <c r="C21" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="D21" s="10" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="3" t="s">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="B22" s="10" t="n">
+      <c r="B22" s="11" t="n">
         <f aca="false">B18-B10</f>
         <v>-100625</v>
       </c>
-      <c r="C22" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="D22" s="9"/>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="5" t="s">
+      <c r="C22" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="D22" s="12"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="B24" s="6"/>
-      <c r="C24" s="6"/>
-      <c r="D24" s="6"/>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="7" t="s">
+      <c r="B24" s="7"/>
+      <c r="C24" s="7"/>
+      <c r="D24" s="7"/>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="B25" s="7" t="s">
+      <c r="B25" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="C25" s="7" t="s">
+      <c r="C25" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="D25" s="7" t="s">
+      <c r="D25" s="8" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="3" t="s">
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="B26" s="4" t="s">
+      <c r="B26" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="C26" s="9" t="s">
+      <c r="C26" s="10" t="s">
         <v>64</v>
       </c>
-      <c r="D26" s="9" t="s">
+      <c r="D26" s="10" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="5" t="s">
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="B28" s="6"/>
-      <c r="C28" s="6"/>
-      <c r="D28" s="6"/>
-    </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="7" t="s">
+      <c r="B28" s="7"/>
+      <c r="C28" s="7"/>
+      <c r="D28" s="7"/>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="B29" s="7" t="s">
+      <c r="B29" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="C29" s="7" t="s">
+      <c r="C29" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="D29" s="7" t="s">
+      <c r="D29" s="8" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="3" t="s">
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="4" t="s">
         <v>119</v>
       </c>
-      <c r="B30" s="8" t="n">
+      <c r="B30" s="9" t="n">
         <v>60000</v>
       </c>
-      <c r="C30" s="9" t="s">
+      <c r="C30" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="D30" s="9" t="s">
+      <c r="D30" s="10" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="3" t="s">
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="4" t="s">
         <v>121</v>
       </c>
-      <c r="B31" s="8" t="n">
+      <c r="B31" s="9" t="n">
         <v>20000</v>
       </c>
-      <c r="C31" s="9" t="s">
+      <c r="C31" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="D31" s="9"/>
-    </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="3" t="s">
+      <c r="D31" s="12"/>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="B32" s="10" t="n">
+      <c r="B32" s="11" t="n">
         <f aca="false">SUM(B30:B31)</f>
         <v>80000</v>
       </c>
-      <c r="C32" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="D32" s="9"/>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="3" t="s">
+      <c r="C32" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="D32" s="12"/>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="4" t="s">
         <v>122</v>
       </c>
-      <c r="B33" s="11" t="n">
+      <c r="B33" s="13" t="n">
         <f aca="false">B30/B32</f>
         <v>0.75</v>
       </c>
-      <c r="C33" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="D33" s="9"/>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="3" t="s">
+      <c r="C33" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="D33" s="12"/>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="4" t="s">
         <v>123</v>
       </c>
-      <c r="B34" s="11" t="n">
+      <c r="B34" s="13" t="n">
         <f aca="false">B31/B32</f>
         <v>0.25</v>
       </c>
-      <c r="C34" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="D34" s="9"/>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="3" t="s">
+      <c r="C34" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="D34" s="12"/>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="B35" s="4" t="s">
+      <c r="B35" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="C35" s="9" t="s">
+      <c r="C35" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="D35" s="9" t="s">
+      <c r="D35" s="10" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="5" t="s">
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="B37" s="6"/>
-      <c r="C37" s="6"/>
-      <c r="D37" s="6"/>
-    </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="7" t="s">
+      <c r="B37" s="7"/>
+      <c r="C37" s="7"/>
+      <c r="D37" s="7"/>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="B38" s="7" t="s">
+      <c r="B38" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="C38" s="7" t="s">
+      <c r="C38" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="D38" s="7" t="s">
+      <c r="D38" s="8" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="3" t="s">
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="B39" s="8" t="n">
+      <c r="B39" s="9" t="n">
         <v>2183088.49</v>
       </c>
-      <c r="C39" s="9" t="s">
+      <c r="C39" s="10" t="s">
         <v>112</v>
       </c>
-      <c r="D39" s="9"/>
-    </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="3" t="s">
+      <c r="D39" s="12"/>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="4" t="s">
         <v>126</v>
       </c>
-      <c r="B40" s="8" t="n">
+      <c r="B40" s="9" t="n">
         <v>1157519.11</v>
       </c>
-      <c r="C40" s="9" t="s">
+      <c r="C40" s="10" t="s">
         <v>112</v>
       </c>
-      <c r="D40" s="9" t="s">
+      <c r="D40" s="10" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="3" t="s">
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="4" t="s">
         <v>128</v>
       </c>
-      <c r="B41" s="8" t="n">
+      <c r="B41" s="9" t="n">
         <v>538013.75</v>
       </c>
-      <c r="C41" s="9" t="s">
+      <c r="C41" s="10" t="s">
         <v>112</v>
       </c>
-      <c r="D41" s="9"/>
-    </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="3" t="s">
+      <c r="D41" s="12"/>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="4" t="s">
         <v>129</v>
       </c>
-      <c r="B42" s="8" t="n">
+      <c r="B42" s="9" t="n">
         <v>139351.5</v>
       </c>
-      <c r="C42" s="9" t="s">
+      <c r="C42" s="10" t="s">
         <v>112</v>
       </c>
-      <c r="D42" s="9"/>
-    </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="3" t="s">
+      <c r="D42" s="12"/>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="4" t="s">
         <v>130</v>
       </c>
-      <c r="B43" s="8" t="n">
+      <c r="B43" s="9" t="n">
         <v>199375</v>
       </c>
-      <c r="C43" s="9" t="s">
+      <c r="C43" s="10" t="s">
         <v>112</v>
       </c>
-      <c r="D43" s="9" t="s">
+      <c r="D43" s="10" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="12" t="s">
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A44" s="14" t="s">
         <v>84</v>
       </c>
-      <c r="B44" s="13" t="n">
+      <c r="B44" s="15" t="n">
         <f aca="false">SUM(B39:B43)</f>
         <v>4217347.85</v>
       </c>
-      <c r="C44" s="14" t="s">
-        <v>36</v>
-      </c>
-      <c r="D44" s="14"/>
-    </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="3" t="s">
+      <c r="C44" s="16" t="s">
+        <v>36</v>
+      </c>
+      <c r="D44" s="17"/>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A45" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="B45" s="11" t="n">
+      <c r="B45" s="13" t="n">
         <f aca="false">B39/B44</f>
         <v>0.517644872475957</v>
       </c>
-      <c r="C45" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="D45" s="9"/>
-    </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="3" t="s">
+      <c r="C45" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="D45" s="12"/>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A46" s="4" t="s">
         <v>133</v>
       </c>
-      <c r="B46" s="11" t="n">
+      <c r="B46" s="13" t="n">
         <f aca="false">B40/B44</f>
         <v>0.274466122115111</v>
       </c>
-      <c r="C46" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="D46" s="9"/>
-    </row>
-    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="3" t="s">
+      <c r="C46" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="D46" s="12"/>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A47" s="4" t="s">
         <v>134</v>
       </c>
-      <c r="B47" s="11" t="n">
+      <c r="B47" s="13" t="n">
         <f aca="false">B41/B44</f>
         <v>0.127571585066193</v>
       </c>
-      <c r="C47" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="D47" s="9"/>
-    </row>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="3" t="s">
+      <c r="C47" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="D47" s="12"/>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A48" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="B48" s="11" t="n">
+      <c r="B48" s="13" t="n">
         <f aca="false">B42/B44</f>
         <v>0.0330424487038697</v>
       </c>
-      <c r="C48" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="D48" s="9"/>
-    </row>
-    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="3" t="s">
+      <c r="C48" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="D48" s="12"/>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A49" s="4" t="s">
         <v>135</v>
       </c>
-      <c r="B49" s="11" t="n">
+      <c r="B49" s="13" t="n">
         <f aca="false">B43/B44</f>
         <v>0.0472749716388701</v>
       </c>
-      <c r="C49" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="D49" s="9"/>
-    </row>
-    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="2" t="s">
+      <c r="C49" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="D49" s="12"/>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A51" s="3" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="3" t="s">
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A52" s="4" t="s">
         <v>137</v>
       </c>
-      <c r="B52" s="8" t="n">
+      <c r="B52" s="9" t="n">
         <v>356040</v>
       </c>
-      <c r="C52" s="9" t="s">
+      <c r="C52" s="10" t="s">
         <v>138</v>
       </c>
-      <c r="D52" s="9"/>
-    </row>
-    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="3" t="s">
+      <c r="D52" s="12"/>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A53" s="4" t="s">
         <v>139</v>
       </c>
-      <c r="B53" s="8" t="n">
+      <c r="B53" s="9" t="n">
         <v>125804.4</v>
       </c>
-      <c r="C53" s="9" t="s">
+      <c r="C53" s="10" t="s">
         <v>138</v>
       </c>
-      <c r="D53" s="9"/>
-    </row>
-    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="3" t="s">
+      <c r="D53" s="12"/>
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A54" s="4" t="s">
         <v>140</v>
       </c>
-      <c r="B54" s="8" t="n">
+      <c r="B54" s="9" t="n">
         <v>56169.35</v>
       </c>
-      <c r="C54" s="9" t="s">
+      <c r="C54" s="10" t="s">
         <v>138</v>
       </c>
-      <c r="D54" s="9"/>
-    </row>
-    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="3" t="s">
+      <c r="D54" s="12"/>
+    </row>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A55" s="4" t="s">
         <v>141</v>
       </c>
-      <c r="B55" s="11" t="n">
+      <c r="B55" s="13" t="n">
         <f aca="false">B52/B41</f>
         <v>0.661767473414945</v>
       </c>
-      <c r="C55" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="D55" s="9"/>
-    </row>
-    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="3" t="s">
+      <c r="C55" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="D55" s="12"/>
+    </row>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A56" s="4" t="s">
         <v>142</v>
       </c>
-      <c r="B56" s="11" t="n">
+      <c r="B56" s="13" t="n">
         <f aca="false">B53/B41</f>
         <v>0.233831198552082</v>
       </c>
-      <c r="C56" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="D56" s="9"/>
-    </row>
-    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="3" t="s">
+      <c r="C56" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="D56" s="12"/>
+    </row>
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A57" s="4" t="s">
         <v>143</v>
       </c>
-      <c r="B57" s="11" t="n">
+      <c r="B57" s="13" t="n">
         <f aca="false">B54/B41</f>
         <v>0.104401328032973</v>
       </c>
-      <c r="C57" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="D57" s="9"/>
-    </row>
-    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="3" t="s">
+      <c r="C57" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="D57" s="12"/>
+    </row>
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A58" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="B58" s="4" t="s">
+      <c r="B58" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="C58" s="9" t="s">
+      <c r="C58" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="D58" s="9" t="s">
+      <c r="D58" s="10" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A60" s="5" t="s">
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A60" s="6" t="s">
         <v>92</v>
       </c>
-      <c r="B60" s="6"/>
-      <c r="C60" s="6"/>
-      <c r="D60" s="6"/>
-    </row>
-    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="7" t="s">
+      <c r="B60" s="7"/>
+      <c r="C60" s="7"/>
+      <c r="D60" s="7"/>
+    </row>
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A61" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="B61" s="7" t="s">
+      <c r="B61" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="C61" s="7" t="s">
+      <c r="C61" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="D61" s="7" t="s">
+      <c r="D61" s="8" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="3" t="s">
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A62" s="4" t="s">
         <v>145</v>
       </c>
-      <c r="B62" s="4" t="s">
+      <c r="B62" s="5" t="s">
         <v>146</v>
       </c>
-      <c r="C62" s="9" t="s">
+      <c r="C62" s="10" t="s">
         <v>147</v>
       </c>
-      <c r="D62" s="9" t="s">
+      <c r="D62" s="10" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A63" s="3" t="s">
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A63" s="4" t="s">
         <v>149</v>
       </c>
-      <c r="B63" s="15" t="n">
+      <c r="B63" s="18" t="n">
         <f aca="true">DATE(2026,9,29)-TODAY()</f>
-        <v>50</v>
-      </c>
-      <c r="C63" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="D63" s="9"/>
-    </row>
-    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A64" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="C63" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="D63" s="12"/>
+    </row>
+    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A64" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="B64" s="4" t="s">
+      <c r="B64" s="5" t="s">
         <v>151</v>
       </c>
-      <c r="C64" s="9" t="s">
+      <c r="C64" s="10" t="s">
         <v>147</v>
       </c>
-      <c r="D64" s="9" t="s">
+      <c r="D64" s="10" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A65" s="3" t="s">
+    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A65" s="4" t="s">
         <v>149</v>
       </c>
-      <c r="B65" s="15" t="n">
+      <c r="B65" s="18" t="n">
         <f aca="true">DATE(2026,8,26)-TODAY()</f>
-        <v>16</v>
-      </c>
-      <c r="C65" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="D65" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C65" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="D65" s="10" t="s">
         <v>153</v>
       </c>
     </row>
-    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A67" s="3" t="s">
+    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A67" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="B67" s="4" t="s">
+      <c r="B67" s="5" t="s">
         <v>97</v>
       </c>
-      <c r="C67" s="9" t="s">
+      <c r="C67" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="D67" s="9" t="s">
+      <c r="D67" s="10" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A69" s="5" t="s">
+    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A69" s="6" t="s">
         <v>99</v>
       </c>
-      <c r="B69" s="6"/>
-      <c r="C69" s="6"/>
-      <c r="D69" s="6"/>
-    </row>
-    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A70" s="7" t="s">
+      <c r="B69" s="7"/>
+      <c r="C69" s="7"/>
+      <c r="D69" s="7"/>
+    </row>
+    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A70" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="B70" s="7" t="s">
+      <c r="B70" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="C70" s="7" t="s">
+      <c r="C70" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="D70" s="7" t="s">
+      <c r="D70" s="8" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A71" s="3" t="s">
+      <c r="A71" s="4" t="s">
         <v>155</v>
       </c>
-      <c r="B71" s="8" t="n">
+      <c r="B71" s="9" t="n">
         <v>1157519.11</v>
       </c>
-      <c r="C71" s="9" t="s">
+      <c r="C71" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="D71" s="9" t="s">
+      <c r="D71" s="10" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A72" s="3" t="s">
+    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A72" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="B72" s="8" t="n">
+      <c r="B72" s="9" t="n">
         <v>-162000</v>
       </c>
-      <c r="C72" s="9" t="s">
+      <c r="C72" s="10" t="s">
         <v>157</v>
       </c>
-      <c r="D72" s="9" t="s">
+      <c r="D72" s="10" t="s">
         <v>158</v>
       </c>
     </row>
-    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A73" s="3" t="s">
+    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A73" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="B73" s="4" t="s">
+      <c r="B73" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="C73" s="9" t="s">
+      <c r="C73" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="D73" s="9" t="s">
+      <c r="D73" s="10" t="s">
         <v>159</v>
       </c>
     </row>

</xml_diff>

<commit_message>
CONSTITUTION v1.4: pestañas Cajas + Proyecciones en personal_capacity_facts.xlsx (clasificación 3 cajas AMS/AML y proyección Caja Motor 5/10/15a bajo hipótesis base v1)
</commit_message>
<xml_diff>
--- a/data/raw/personal_capacity_facts.xlsx
+++ b/data/raw/personal_capacity_facts.xlsx
@@ -1,16 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
-  <fileVersion appName="Calc"/>
+  <fileVersion appName="Calc" lowestEdited="4"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="600" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="Notas" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="AMS" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="AML" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="Cajas" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="Proyecciones" sheetId="5" state="visible" r:id="rId7"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -22,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="335" uniqueCount="160">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="417" uniqueCount="212">
   <si>
     <t xml:space="preserve">PERSONAL CAPACITY FACTS — Notas de uso</t>
   </si>
@@ -502,6 +504,162 @@
   </si>
   <si>
     <t xml:space="preserve">Confirmado 2026-08-10 -- la exclusión de Planes de Pensiones y la minusvalía TEF de arriba son las únicas cuestiones fiscales conocidas; ninguna de las dos es una restricción activa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CLASIFICACIÓN EN LAS TRES CAJAS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nivel 3, CONSTITUTION.md Sección 2 — Seguridad / Motor / Rentas Pasivas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AMS — patrimonio propio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Caja</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Partida</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Origen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Seguridad</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AMS!B41</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AMS!B44</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Subtotal Seguridad</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Motor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AMS!B40</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Subtotal Motor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rentas Pasivas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AMS!B42</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AMS!B43</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Subtotal Rentas Pasivas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOTAL AMS (3 cajas)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Diferencia vs. Total patrimonio AMS (control)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Debe ser 0€. Si no lo es, hay una partida nueva en AMS sección 4 sin clasificar aquí.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AML — patrimonio de tus padres</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AML!B43</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AML!B39</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bloqueado operativamente (ilíquido salvo jubilación/paro larga duración/enfermedad grave; destino: herencia). Clasificado en Motor por composición de activo (mayoritariamente RV), confirmado por Armando 2026-08-13.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Función declarada de renta vía dividendos, no de crecimiento (ver AML!D58). Confirmado por Armando 2026-08-13.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AML!B42</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOTAL AML (3 cajas)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Diferencia vs. Total patrimonio AML (control)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Debe ser 0€. Si no lo es, hay una partida nueva en AML sección 4 sin clasificar aquí.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Clasificación fijada por Armando el 2026-08-13, sobre la tabla de cajas de CONSTITUTION.md Sección 2, Nivel 3 (Seguridad: liquidez/depósitos/monetarios · Motor: fondo indexado S&amp;P 500 y otras inversiones a largo plazo · Rentas Pasivas: JGPI, inmobiliario, oro).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PROYECCIÓN CAJA MOTOR — HIPÓTESIS BASE v1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ilustrativa, no un objetivo. X/Y/Z por necesidad patrimonial: CONSTITUTION.md Sección 6, Pendiente.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hipótesis de rentabilidad (CONSTITUTION.md Sección 2)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rentabilidad real anualizada</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hipótesis base v1 — CONSTITUTION.md Sección 2. Serie total return real de Shiller (data/raw/shiller.xlsx), dividendos reinvertidos, CAGR de la serie completa. No se ajusta automáticamente por CAPE ni por el Research Engine — editar solo tras actualización explícita de la Constitución.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rentabilidad nominal anualizada (aprox.)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Derivada de la rentabilidad real + inflación media histórica de la serie Shiller (~2,15%/año). Misma gobernanza que la fila anterior.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Base — Caja Motor (hoja 'Cajas')</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AMS — Caja Motor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cajas!C10 (subtotal Motor)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AML — Caja Motor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cajas!C25 (subtotal Motor, incluye Planes de Pensiones bloqueados)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Proyección AMS — Caja Motor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Horizonte</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Real</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nominal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5 años</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10 años</t>
+  </si>
+  <si>
+    <t xml:space="preserve">15 años</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Proyección AML — Caja Motor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Proyección de puro interés compuesto sobre el saldo actual de Caja Motor. No es el objetivo X/Y/Z (todavía sin definir) — sirve para comparar, una vez fijado ese objetivo, si la trayectoria real va camino de cumplirlo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AML incluye Planes de Pensiones, operativamente bloqueados (ver hoja 'Cajas', nota en D24).</t>
   </si>
 </sst>
 </file>
@@ -514,7 +672,7 @@
     <numFmt numFmtId="166" formatCode="0.0%"/>
     <numFmt numFmtId="167" formatCode="0"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="11">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -569,6 +727,21 @@
       <i val="true"/>
       <sz val="9"/>
       <color rgb="FF666666"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF666666"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -634,7 +807,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="28">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -709,6 +882,42 @@
     </xf>
     <xf numFmtId="167" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -2555,7 +2764,7 @@
       </c>
       <c r="B63" s="18" t="n">
         <f aca="true">DATE(2026,9,29)-TODAY()</f>
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="C63" s="10" t="s">
         <v>36</v>
@@ -2582,7 +2791,7 @@
       </c>
       <c r="B65" s="18" t="n">
         <f aca="true">DATE(2026,8,26)-TODAY()</f>
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C65" s="10" t="s">
         <v>36</v>
@@ -2667,6 +2876,618 @@
       </c>
       <c r="D73" s="10" t="s">
         <v>159</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:D33"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="60"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="19" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="20" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="21" t="s">
+        <v>162</v>
+      </c>
+      <c r="B4" s="22"/>
+      <c r="C4" s="22"/>
+      <c r="D4" s="22"/>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="23" t="s">
+        <v>163</v>
+      </c>
+      <c r="B5" s="23" t="s">
+        <v>164</v>
+      </c>
+      <c r="C5" s="23" t="s">
+        <v>27</v>
+      </c>
+      <c r="D5" s="23" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="24" t="s">
+        <v>166</v>
+      </c>
+      <c r="B6" s="24" t="str">
+        <f aca="false">AMS!A41</f>
+        <v>Fondo Monetario</v>
+      </c>
+      <c r="C6" s="25" t="n">
+        <f aca="false">AMS!B41</f>
+        <v>89230.77</v>
+      </c>
+      <c r="D6" s="20" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="24" t="s">
+        <v>166</v>
+      </c>
+      <c r="B7" s="24" t="str">
+        <f aca="false">AMS!A44</f>
+        <v>Liquidez (excluido FM)</v>
+      </c>
+      <c r="C7" s="25" t="n">
+        <f aca="false">AMS!B44</f>
+        <v>83100</v>
+      </c>
+      <c r="D7" s="20" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="26" t="s">
+        <v>169</v>
+      </c>
+      <c r="B8" s="24"/>
+      <c r="C8" s="25" t="n">
+        <f aca="false">SUM(C6:C7)</f>
+        <v>172330.77</v>
+      </c>
+      <c r="D8" s="20"/>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="24" t="s">
+        <v>170</v>
+      </c>
+      <c r="B9" s="24" t="str">
+        <f aca="false">AMS!A40</f>
+        <v>SP500 (fondos indexados)</v>
+      </c>
+      <c r="C9" s="25" t="n">
+        <f aca="false">AMS!B40</f>
+        <v>872837.88</v>
+      </c>
+      <c r="D9" s="20" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="26" t="s">
+        <v>172</v>
+      </c>
+      <c r="B10" s="24"/>
+      <c r="C10" s="25" t="n">
+        <f aca="false">C9</f>
+        <v>872837.88</v>
+      </c>
+      <c r="D10" s="20"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="24" t="s">
+        <v>173</v>
+      </c>
+      <c r="B11" s="24" t="str">
+        <f aca="false">AMS!A42</f>
+        <v>ETF</v>
+      </c>
+      <c r="C11" s="25" t="n">
+        <f aca="false">AMS!B42</f>
+        <v>111570.37</v>
+      </c>
+      <c r="D11" s="20" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="24" t="s">
+        <v>173</v>
+      </c>
+      <c r="B12" s="24" t="str">
+        <f aca="false">AMS!A43</f>
+        <v>Pisos</v>
+      </c>
+      <c r="C12" s="25" t="n">
+        <f aca="false">AMS!B43</f>
+        <v>100000</v>
+      </c>
+      <c r="D12" s="20" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="26" t="s">
+        <v>176</v>
+      </c>
+      <c r="B13" s="24"/>
+      <c r="C13" s="25" t="n">
+        <f aca="false">SUM(C11:C12)</f>
+        <v>211570.37</v>
+      </c>
+      <c r="D13" s="20"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="26" t="s">
+        <v>177</v>
+      </c>
+      <c r="B15" s="24"/>
+      <c r="C15" s="25" t="n">
+        <f aca="false">C8+C10+C13</f>
+        <v>1256739.02</v>
+      </c>
+      <c r="D15" s="20"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="24" t="s">
+        <v>178</v>
+      </c>
+      <c r="B16" s="24"/>
+      <c r="C16" s="25" t="n">
+        <f aca="false">C15-AMS!B45</f>
+        <v>0</v>
+      </c>
+      <c r="D16" s="20" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="21" t="s">
+        <v>180</v>
+      </c>
+      <c r="B19" s="22"/>
+      <c r="C19" s="22"/>
+      <c r="D19" s="22"/>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="23" t="s">
+        <v>163</v>
+      </c>
+      <c r="B20" s="23" t="s">
+        <v>164</v>
+      </c>
+      <c r="C20" s="23" t="s">
+        <v>27</v>
+      </c>
+      <c r="D20" s="23" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="24" t="s">
+        <v>166</v>
+      </c>
+      <c r="B21" s="24" t="str">
+        <f aca="false">AML!A43</f>
+        <v>Liquidez + Depósitos (excluido FM)</v>
+      </c>
+      <c r="C21" s="25" t="n">
+        <f aca="false">AML!B43</f>
+        <v>199375</v>
+      </c>
+      <c r="D21" s="20" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="26" t="s">
+        <v>169</v>
+      </c>
+      <c r="B22" s="24"/>
+      <c r="C22" s="25" t="n">
+        <f aca="false">C21</f>
+        <v>199375</v>
+      </c>
+      <c r="D22" s="20"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="24" t="s">
+        <v>170</v>
+      </c>
+      <c r="B23" s="24" t="str">
+        <f aca="false">AML!A39</f>
+        <v>Fondos RV</v>
+      </c>
+      <c r="C23" s="25" t="n">
+        <f aca="false">AML!B39</f>
+        <v>2183088.49</v>
+      </c>
+      <c r="D23" s="20" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="24" t="s">
+        <v>170</v>
+      </c>
+      <c r="B24" s="24" t="str">
+        <f aca="false">AML!A40</f>
+        <v>Planes de Pensiones (Papá 754.162,54 + Mamá 403.356,58)</v>
+      </c>
+      <c r="C24" s="25" t="n">
+        <f aca="false">AML!B40</f>
+        <v>1157519.11</v>
+      </c>
+      <c r="D24" s="20" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="26" t="s">
+        <v>172</v>
+      </c>
+      <c r="B25" s="24"/>
+      <c r="C25" s="25" t="n">
+        <f aca="false">SUM(C23:C24)</f>
+        <v>3340607.6</v>
+      </c>
+      <c r="D25" s="20"/>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="24" t="s">
+        <v>173</v>
+      </c>
+      <c r="B26" s="24" t="str">
+        <f aca="false">AML!A41</f>
+        <v>Acciones (Iberdrola 356.040 + BBVA 125.804,4 + TEF 56.169,35)</v>
+      </c>
+      <c r="C26" s="25" t="n">
+        <f aca="false">AML!B41</f>
+        <v>538013.75</v>
+      </c>
+      <c r="D26" s="20" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="24" t="s">
+        <v>173</v>
+      </c>
+      <c r="B27" s="24" t="str">
+        <f aca="false">AML!A42</f>
+        <v>ETF (Aristócratas)</v>
+      </c>
+      <c r="C27" s="25" t="n">
+        <f aca="false">AML!B42</f>
+        <v>139351.5</v>
+      </c>
+      <c r="D27" s="20" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="26" t="s">
+        <v>176</v>
+      </c>
+      <c r="B28" s="24"/>
+      <c r="C28" s="25" t="n">
+        <f aca="false">SUM(C26:C27)</f>
+        <v>677365.25</v>
+      </c>
+      <c r="D28" s="20"/>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="26" t="s">
+        <v>186</v>
+      </c>
+      <c r="B30" s="24"/>
+      <c r="C30" s="25" t="n">
+        <f aca="false">C22+C25+C28</f>
+        <v>4217347.85</v>
+      </c>
+      <c r="D30" s="20"/>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="24" t="s">
+        <v>187</v>
+      </c>
+      <c r="B31" s="24"/>
+      <c r="C31" s="25" t="n">
+        <f aca="false">C30-AML!B44</f>
+        <v>0</v>
+      </c>
+      <c r="D31" s="20" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="20" t="s">
+        <v>189</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:D27"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="60"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="19" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="20" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="21" t="s">
+        <v>192</v>
+      </c>
+      <c r="B4" s="22"/>
+      <c r="C4" s="22"/>
+      <c r="D4" s="22"/>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="23" t="s">
+        <v>26</v>
+      </c>
+      <c r="B5" s="23" t="s">
+        <v>27</v>
+      </c>
+      <c r="C5" s="23" t="s">
+        <v>28</v>
+      </c>
+      <c r="D5" s="23" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="24" t="s">
+        <v>193</v>
+      </c>
+      <c r="B6" s="27" t="n">
+        <v>0.07</v>
+      </c>
+      <c r="C6" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="D6" s="20" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="24" t="s">
+        <v>195</v>
+      </c>
+      <c r="B7" s="27" t="n">
+        <v>0.094</v>
+      </c>
+      <c r="C7" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="D7" s="20" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="21" t="s">
+        <v>197</v>
+      </c>
+      <c r="B9" s="22"/>
+      <c r="C9" s="22"/>
+      <c r="D9" s="22"/>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="23" t="s">
+        <v>26</v>
+      </c>
+      <c r="B10" s="23" t="s">
+        <v>27</v>
+      </c>
+      <c r="C10" s="23" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="24" t="s">
+        <v>198</v>
+      </c>
+      <c r="B11" s="25" t="n">
+        <f aca="false">Cajas!C10</f>
+        <v>872837.88</v>
+      </c>
+      <c r="C11" s="20" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="24" t="s">
+        <v>200</v>
+      </c>
+      <c r="B12" s="25" t="n">
+        <f aca="false">Cajas!C25</f>
+        <v>3340607.6</v>
+      </c>
+      <c r="C12" s="20" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="21" t="s">
+        <v>202</v>
+      </c>
+      <c r="B14" s="22"/>
+      <c r="C14" s="22"/>
+      <c r="D14" s="22"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="23" t="s">
+        <v>203</v>
+      </c>
+      <c r="B15" s="23" t="s">
+        <v>204</v>
+      </c>
+      <c r="C15" s="23" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="24" t="s">
+        <v>206</v>
+      </c>
+      <c r="B16" s="25" t="n">
+        <f aca="false">$B$11*(1+$B$6)^5</f>
+        <v>1224200.27921452</v>
+      </c>
+      <c r="C16" s="25" t="n">
+        <f aca="false">$B$11*(1+$B$7)^5</f>
+        <v>1367792.42987986</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="24" t="s">
+        <v>207</v>
+      </c>
+      <c r="B17" s="25" t="n">
+        <f aca="false">$B$11*(1+$B$6)^10</f>
+        <v>1717004.22033575</v>
+      </c>
+      <c r="C17" s="25" t="n">
+        <f aca="false">$B$11*(1+$B$7)^10</f>
+        <v>2143417.6656456</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="24" t="s">
+        <v>208</v>
+      </c>
+      <c r="B18" s="25" t="n">
+        <f aca="false">$B$11*(1+$B$6)^15</f>
+        <v>2408187.24085111</v>
+      </c>
+      <c r="C18" s="25" t="n">
+        <f aca="false">$B$11*(1+$B$7)^15</f>
+        <v>3358871.70380461</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="21" t="s">
+        <v>209</v>
+      </c>
+      <c r="B20" s="22"/>
+      <c r="C20" s="22"/>
+      <c r="D20" s="22"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="23" t="s">
+        <v>203</v>
+      </c>
+      <c r="B21" s="23" t="s">
+        <v>204</v>
+      </c>
+      <c r="C21" s="23" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="24" t="s">
+        <v>206</v>
+      </c>
+      <c r="B22" s="25" t="n">
+        <f aca="false">$B$12*(1+$B$6)^5</f>
+        <v>4685374.97096958</v>
+      </c>
+      <c r="C22" s="25" t="n">
+        <f aca="false">$B$12*(1+$B$7)^5</f>
+        <v>5234944.41657267</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="24" t="s">
+        <v>207</v>
+      </c>
+      <c r="B23" s="25" t="n">
+        <f aca="false">$B$12*(1+$B$6)^10</f>
+        <v>6571480.77451184</v>
+      </c>
+      <c r="C23" s="25" t="n">
+        <f aca="false">$B$12*(1+$B$7)^10</f>
+        <v>8203490.59991523</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="24" t="s">
+        <v>208</v>
+      </c>
+      <c r="B24" s="25" t="n">
+        <f aca="false">$B$12*(1+$B$6)^15</f>
+        <v>9216841.73355336</v>
+      </c>
+      <c r="C24" s="25" t="n">
+        <f aca="false">$B$12*(1+$B$7)^15</f>
+        <v>12855391.1307729</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="20" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="20" t="s">
+        <v>211</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Rediseño visual de pestañas Cajas y Proyecciones: colores por caja, subtotales/totales resaltados, notas sin desbordar
</commit_message>
<xml_diff>
--- a/data/raw/personal_capacity_facts.xlsx
+++ b/data/raw/personal_capacity_facts.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="417" uniqueCount="212">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="413" uniqueCount="213">
   <si>
     <t xml:space="preserve">PERSONAL CAPACITY FACTS — Notas de uso</t>
   </si>
@@ -509,7 +509,7 @@
     <t xml:space="preserve">CLASIFICACIÓN EN LAS TRES CAJAS</t>
   </si>
   <si>
-    <t xml:space="preserve">Nivel 3, CONSTITUTION.md Sección 2 — Seguridad / Motor / Rentas Pasivas</t>
+    <t xml:space="preserve">Nivel 3, CONSTITUTION.md Sección 2  ·  Seguridad · Motor · Rentas Pasivas</t>
   </si>
   <si>
     <t xml:space="preserve">AMS — patrimonio propio</t>
@@ -560,10 +560,10 @@
     <t xml:space="preserve">TOTAL AMS (3 cajas)</t>
   </si>
   <si>
-    <t xml:space="preserve">Diferencia vs. Total patrimonio AMS (control)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Debe ser 0€. Si no lo es, hay una partida nueva en AMS sección 4 sin clasificar aquí.</t>
+    <t xml:space="preserve">Diferencia vs. total patrimonio (control)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Debe ser 0€. Si no lo es, hay una partida nueva en la sección 4 sin clasificar aquí.</t>
   </si>
   <si>
     <t xml:space="preserve">AML — patrimonio de tus padres</t>
@@ -575,7 +575,13 @@
     <t xml:space="preserve">AML!B39</t>
   </si>
   <si>
-    <t xml:space="preserve">Bloqueado operativamente (ilíquido salvo jubilación/paro larga duración/enfermedad grave; destino: herencia). Clasificado en Motor por composición de activo (mayoritariamente RV), confirmado por Armando 2026-08-13.</t>
+    <t xml:space="preserve">AML!B40</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bloqueado operativamente (ilíquido salvo jubilación/paro larga duración/enfermedad grave; destino: herencia). Clasificado en Motor por composición de activo, confirmado por Armando 2026-08-13.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AML!B41</t>
   </si>
   <si>
     <t xml:space="preserve">Función declarada de renta vía dividendos, no de crecimiento (ver AML!D58). Confirmado por Armando 2026-08-13.</t>
@@ -587,13 +593,7 @@
     <t xml:space="preserve">TOTAL AML (3 cajas)</t>
   </si>
   <si>
-    <t xml:space="preserve">Diferencia vs. Total patrimonio AML (control)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Debe ser 0€. Si no lo es, hay una partida nueva en AML sección 4 sin clasificar aquí.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Clasificación fijada por Armando el 2026-08-13, sobre la tabla de cajas de CONSTITUTION.md Sección 2, Nivel 3 (Seguridad: liquidez/depósitos/monetarios · Motor: fondo indexado S&amp;P 500 y otras inversiones a largo plazo · Rentas Pasivas: JGPI, inmobiliario, oro).</t>
+    <t xml:space="preserve">Colores: Seguridad (azul) · Motor (verde) · Rentas Pasivas (naranja). Clasificación fijada por Armando el 2026-08-13 sobre la tabla de cajas de CONSTITUTION.md Sección 2, Nivel 3 — Seguridad: liquidez/depósitos/monetarios · Motor: fondo indexado S&amp;P 500 y otras inversiones a largo plazo · Rentas Pasivas: JGPI, inmobiliario, oro.</t>
   </si>
   <si>
     <t xml:space="preserve">PROYECCIÓN CAJA MOTOR — HIPÓTESIS BASE v1</t>
@@ -602,7 +602,7 @@
     <t xml:space="preserve">Ilustrativa, no un objetivo. X/Y/Z por necesidad patrimonial: CONSTITUTION.md Sección 6, Pendiente.</t>
   </si>
   <si>
-    <t xml:space="preserve">Hipótesis de rentabilidad (CONSTITUTION.md Sección 2)</t>
+    <t xml:space="preserve">Hipótesis de rentabilidad  ·  CONSTITUTION.md Sección 2</t>
   </si>
   <si>
     <t xml:space="preserve">Rentabilidad real anualizada</t>
@@ -617,31 +617,40 @@
     <t xml:space="preserve">Derivada de la rentabilidad real + inflación media histórica de la serie Shiller (~2,15%/año). Misma gobernanza que la fila anterior.</t>
   </si>
   <si>
-    <t xml:space="preserve">Base — Caja Motor (hoja 'Cajas')</t>
+    <t xml:space="preserve">Base — Caja Motor  ·  hoja 'Cajas'</t>
   </si>
   <si>
     <t xml:space="preserve">AMS — Caja Motor</t>
   </si>
   <si>
-    <t xml:space="preserve">Cajas!C10 (subtotal Motor)</t>
+    <t xml:space="preserve">Cajas!C10</t>
   </si>
   <si>
     <t xml:space="preserve">AML — Caja Motor</t>
   </si>
   <si>
-    <t xml:space="preserve">Cajas!C25 (subtotal Motor, incluye Planes de Pensiones bloqueados)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Proyección AMS — Caja Motor</t>
+    <t xml:space="preserve">Cajas!C25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Incluye Planes de Pensiones, operativamente bloqueados (ver hoja 'Cajas').</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Proyección Caja Motor a 5 / 10 / 15 años  ·  AMS vs. AML</t>
   </si>
   <si>
     <t xml:space="preserve">Horizonte</t>
   </si>
   <si>
-    <t xml:space="preserve">Real</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nominal</t>
+    <t xml:space="preserve">AMS Real</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AMS Nominal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AML Real</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AML Nominal</t>
   </si>
   <si>
     <t xml:space="preserve">5 años</t>
@@ -653,13 +662,7 @@
     <t xml:space="preserve">15 años</t>
   </si>
   <si>
-    <t xml:space="preserve">Proyección AML — Caja Motor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Proyección de puro interés compuesto sobre el saldo actual de Caja Motor. No es el objetivo X/Y/Z (todavía sin definir) — sirve para comparar, una vez fijado ese objetivo, si la trayectoria real va camino de cumplirlo.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AML incluye Planes de Pensiones, operativamente bloqueados (ver hoja 'Cajas', nota en D24).</t>
+    <t xml:space="preserve">Proyección de interés compuesto puro sobre el saldo actual de Caja Motor. No es el objetivo X/Y/Z (todavía sin definir) — sirve para comparar, una vez fijado ese objetivo, si la trayectoria real va camino de cumplirlo. AML incluye Planes de Pensiones bloqueados.</t>
   </si>
 </sst>
 </file>
@@ -672,7 +675,7 @@
     <numFmt numFmtId="166" formatCode="0.0%"/>
     <numFmt numFmtId="167" formatCode="0"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="19">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -732,8 +735,25 @@
       <charset val="1"/>
     </font>
     <font>
+      <b val="true"/>
+      <sz val="13"/>
+      <color rgb="FF1F1F1F"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <i val="true"/>
       <sz val="9"/>
-      <color rgb="FF666666"/>
+      <color rgb="FF808080"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -741,13 +761,59 @@
     <font>
       <b val="true"/>
       <sz val="10"/>
-      <color rgb="FF000000"/>
+      <color rgb="FF1F1F1F"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF1F1F1F"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="8.5"/>
+      <color rgb="FF9E9E9E"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="10.5"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <i val="true"/>
+      <sz val="8.5"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="10"/>
+      <color rgb="FF1155CC"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="10.5"/>
+      <color rgb="FF1F1F1F"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="14">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -757,28 +823,158 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFD9E1F2"/>
-        <bgColor rgb="FFF2F2F2"/>
+        <bgColor rgb="FFDDEBF7"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFF2F2F2"/>
-        <bgColor rgb="FFFFFFCC"/>
+        <bgColor rgb="FFE2EFDA"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFE699"/>
-        <bgColor rgb="FFFFCC99"/>
+        <bgColor rgb="FFFFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF2E5395"/>
+        <bgColor rgb="FF1155CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDDEBF7"/>
+        <bgColor rgb="FFD9E1F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFBDD7EE"/>
+        <bgColor rgb="FFD9D9D9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE2EFDA"/>
+        <bgColor rgb="FFDDEBF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA9D18E"/>
+        <bgColor rgb="FFBDD7EE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFCE4D6"/>
+        <bgColor rgb="FFFFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF4B183"/>
+        <bgColor rgb="FFFF8080"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF404040"/>
+        <bgColor rgb="FF595959"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF2CC"/>
+        <bgColor rgb="FFFCE4D6"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="7">
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF808080"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thin">
+        <color rgb="FFD9D9D9"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD9D9D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD9D9D9"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right style="medium">
+        <color rgb="FF595959"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF808080"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="medium">
+        <color rgb="FF595959"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF808080"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thin">
+        <color rgb="FFD9D9D9"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF595959"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD9D9D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD9D9D9"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="medium">
+        <color rgb="FF595959"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD9D9D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD9D9D9"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -807,7 +1003,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="66">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -884,40 +1080,192 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="13" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="7" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="12" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="8" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="8" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="13" fillId="8" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="8" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="8" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="9" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="9" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="12" fillId="9" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="10" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="10" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="13" fillId="10" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="10" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="10" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="11" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="11" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="12" fillId="11" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="12" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="15" fillId="12" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="12" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="8" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="10" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="17" fillId="13" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="8" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="18" fillId="8" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="3" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="3" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="13" fillId="8" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="13" fillId="8" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -932,7 +1280,7 @@
   <colors>
     <indexedColors>
       <rgbColor rgb="FF000000"/>
-      <rgbColor rgb="FFF2F2F2"/>
+      <rgbColor rgb="FFFFFFFF"/>
       <rgbColor rgb="FFFF0000"/>
       <rgbColor rgb="FF00FF00"/>
       <rgbColor rgb="FF0000FF"/>
@@ -942,19 +1290,19 @@
       <rgbColor rgb="FF800000"/>
       <rgbColor rgb="FF008000"/>
       <rgbColor rgb="FF000080"/>
-      <rgbColor rgb="FF808000"/>
+      <rgbColor rgb="FF7F7F7F"/>
       <rgbColor rgb="FF800080"/>
       <rgbColor rgb="FF008080"/>
-      <rgbColor rgb="FFC0C0C0"/>
+      <rgbColor rgb="FFA9D18E"/>
       <rgbColor rgb="FF808080"/>
       <rgbColor rgb="FF9999FF"/>
-      <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FFFFFFCC"/>
-      <rgbColor rgb="FFCCFFFF"/>
+      <rgbColor rgb="FF595959"/>
+      <rgbColor rgb="FFFFF2CC"/>
+      <rgbColor rgb="FFDDEBF7"/>
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
-      <rgbColor rgb="FF0066CC"/>
-      <rgbColor rgb="FFD9E1F2"/>
+      <rgbColor rgb="FF1155CC"/>
+      <rgbColor rgb="FFBDD7EE"/>
       <rgbColor rgb="FF000080"/>
       <rgbColor rgb="FFFF00FF"/>
       <rgbColor rgb="FFFFFF00"/>
@@ -964,13 +1312,13 @@
       <rgbColor rgb="FF008080"/>
       <rgbColor rgb="FF0000FF"/>
       <rgbColor rgb="FF00CCFF"/>
-      <rgbColor rgb="FFCCFFFF"/>
-      <rgbColor rgb="FFCCFFCC"/>
+      <rgbColor rgb="FFF2F2F2"/>
+      <rgbColor rgb="FFE2EFDA"/>
       <rgbColor rgb="FFFFE699"/>
-      <rgbColor rgb="FF99CCFF"/>
-      <rgbColor rgb="FFFF99CC"/>
-      <rgbColor rgb="FFCC99FF"/>
-      <rgbColor rgb="FFFFCC99"/>
+      <rgbColor rgb="FFD9D9D9"/>
+      <rgbColor rgb="FFFCE4D6"/>
+      <rgbColor rgb="FFD9E1F2"/>
+      <rgbColor rgb="FFF4B183"/>
       <rgbColor rgb="FF3366FF"/>
       <rgbColor rgb="FF33CCCC"/>
       <rgbColor rgb="FF99CC00"/>
@@ -978,15 +1326,15 @@
       <rgbColor rgb="FFFF9900"/>
       <rgbColor rgb="FFFF6600"/>
       <rgbColor rgb="FF666666"/>
-      <rgbColor rgb="FF969696"/>
+      <rgbColor rgb="FF9E9E9E"/>
       <rgbColor rgb="FF003366"/>
       <rgbColor rgb="FF339966"/>
       <rgbColor rgb="FF003300"/>
-      <rgbColor rgb="FF333300"/>
+      <rgbColor rgb="FF1F1F1F"/>
       <rgbColor rgb="FF993300"/>
       <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FF333399"/>
-      <rgbColor rgb="FF333333"/>
+      <rgbColor rgb="FF2E5395"/>
+      <rgbColor rgb="FF404040"/>
     </indexedColors>
   </colors>
 </styleSheet>
@@ -2892,51 +3240,64 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
+    <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:D33"/>
+  <dimension ref="A1:E35"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="46"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="60"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="52"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="19" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B1" s="19"/>
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19"/>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="20" t="s">
         <v>161</v>
       </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B2" s="20"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="21" t="s">
         <v>162</v>
       </c>
-      <c r="B4" s="22"/>
-      <c r="C4" s="22"/>
-      <c r="D4" s="22"/>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="23" t="s">
+      <c r="B4" s="21"/>
+      <c r="C4" s="21"/>
+      <c r="D4" s="21"/>
+      <c r="E4" s="21"/>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="22" t="s">
         <v>163</v>
       </c>
-      <c r="B5" s="23" t="s">
+      <c r="B5" s="22" t="s">
         <v>164</v>
       </c>
-      <c r="C5" s="23" t="s">
+      <c r="C5" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="D5" s="23" t="s">
+      <c r="D5" s="22" t="s">
         <v>165</v>
       </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="24" t="s">
+      <c r="E5" s="22" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="23" t="s">
         <v>166</v>
       </c>
       <c r="B6" s="24" t="str">
@@ -2947,14 +3308,13 @@
         <f aca="false">AMS!B41</f>
         <v>89230.77</v>
       </c>
-      <c r="D6" s="20" t="s">
+      <c r="D6" s="26" t="s">
         <v>167</v>
       </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="24" t="s">
-        <v>166</v>
-      </c>
+      <c r="E6" s="27"/>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="23"/>
       <c r="B7" s="24" t="str">
         <f aca="false">AMS!A44</f>
         <v>Liquidez (excluido FM)</v>
@@ -2963,139 +3323,148 @@
         <f aca="false">AMS!B44</f>
         <v>83100</v>
       </c>
-      <c r="D7" s="20" t="s">
+      <c r="D7" s="26" t="s">
         <v>168</v>
       </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="26" t="s">
+      <c r="E7" s="27"/>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="28"/>
+      <c r="B8" s="29" t="s">
         <v>169</v>
       </c>
-      <c r="B8" s="24"/>
-      <c r="C8" s="25" t="n">
+      <c r="C8" s="30" t="n">
         <f aca="false">SUM(C6:C7)</f>
         <v>172330.77</v>
       </c>
-      <c r="D8" s="20"/>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="24" t="s">
+      <c r="D8" s="28"/>
+      <c r="E8" s="28"/>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="31" t="s">
         <v>170</v>
       </c>
-      <c r="B9" s="24" t="str">
+      <c r="B9" s="32" t="str">
         <f aca="false">AMS!A40</f>
         <v>SP500 (fondos indexados)</v>
       </c>
-      <c r="C9" s="25" t="n">
+      <c r="C9" s="33" t="n">
         <f aca="false">AMS!B40</f>
         <v>872837.88</v>
       </c>
-      <c r="D9" s="20" t="s">
+      <c r="D9" s="34" t="s">
         <v>171</v>
       </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="26" t="s">
+      <c r="E9" s="35"/>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="36"/>
+      <c r="B10" s="37" t="s">
         <v>172</v>
       </c>
-      <c r="B10" s="24"/>
-      <c r="C10" s="25" t="n">
+      <c r="C10" s="38" t="n">
         <f aca="false">C9</f>
         <v>872837.88</v>
       </c>
-      <c r="D10" s="20"/>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="24" t="s">
+      <c r="D10" s="36"/>
+      <c r="E10" s="36"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="39" t="s">
         <v>173</v>
       </c>
-      <c r="B11" s="24" t="str">
+      <c r="B11" s="40" t="str">
         <f aca="false">AMS!A42</f>
         <v>ETF</v>
       </c>
-      <c r="C11" s="25" t="n">
+      <c r="C11" s="41" t="n">
         <f aca="false">AMS!B42</f>
         <v>111570.37</v>
       </c>
-      <c r="D11" s="20" t="s">
+      <c r="D11" s="42" t="s">
         <v>174</v>
       </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="24" t="s">
-        <v>173</v>
-      </c>
-      <c r="B12" s="24" t="str">
+      <c r="E11" s="43"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="39"/>
+      <c r="B12" s="40" t="str">
         <f aca="false">AMS!A43</f>
         <v>Pisos</v>
       </c>
-      <c r="C12" s="25" t="n">
+      <c r="C12" s="41" t="n">
         <f aca="false">AMS!B43</f>
         <v>100000</v>
       </c>
-      <c r="D12" s="20" t="s">
+      <c r="D12" s="42" t="s">
         <v>175</v>
       </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="26" t="s">
+      <c r="E12" s="43"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="44"/>
+      <c r="B13" s="45" t="s">
         <v>176</v>
       </c>
-      <c r="B13" s="24"/>
-      <c r="C13" s="25" t="n">
+      <c r="C13" s="46" t="n">
         <f aca="false">SUM(C11:C12)</f>
         <v>211570.37</v>
       </c>
-      <c r="D13" s="20"/>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="26" t="s">
+      <c r="D13" s="44"/>
+      <c r="E13" s="44"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="47" t="s">
         <v>177</v>
       </c>
-      <c r="B15" s="24"/>
-      <c r="C15" s="25" t="n">
+      <c r="B15" s="47"/>
+      <c r="C15" s="48" t="n">
         <f aca="false">C8+C10+C13</f>
         <v>1256739.02</v>
       </c>
-      <c r="D15" s="20"/>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="24" t="s">
+      <c r="D15" s="49"/>
+      <c r="E15" s="49"/>
+    </row>
+    <row r="16" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B16" s="50" t="s">
         <v>178</v>
       </c>
-      <c r="B16" s="24"/>
-      <c r="C16" s="25" t="n">
+      <c r="C16" s="51" t="n">
         <f aca="false">C15-AMS!B45</f>
         <v>0</v>
       </c>
-      <c r="D16" s="20" t="s">
+      <c r="E16" s="52" t="s">
         <v>179</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="21" t="s">
         <v>180</v>
       </c>
-      <c r="B19" s="22"/>
-      <c r="C19" s="22"/>
-      <c r="D19" s="22"/>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="23" t="s">
+      <c r="B19" s="21"/>
+      <c r="C19" s="21"/>
+      <c r="D19" s="21"/>
+      <c r="E19" s="21"/>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="22" t="s">
         <v>163</v>
       </c>
-      <c r="B20" s="23" t="s">
+      <c r="B20" s="22" t="s">
         <v>164</v>
       </c>
-      <c r="C20" s="23" t="s">
+      <c r="C20" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="D20" s="23" t="s">
+      <c r="D20" s="22" t="s">
         <v>165</v>
       </c>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="24" t="s">
+      <c r="E20" s="22" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="23" t="s">
         <v>166</v>
       </c>
       <c r="B21" s="24" t="str">
@@ -3106,140 +3475,179 @@
         <f aca="false">AML!B43</f>
         <v>199375</v>
       </c>
-      <c r="D21" s="20" t="s">
+      <c r="D21" s="26" t="s">
         <v>181</v>
       </c>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="26" t="s">
+      <c r="E21" s="27"/>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="28"/>
+      <c r="B22" s="29" t="s">
         <v>169</v>
       </c>
-      <c r="B22" s="24"/>
-      <c r="C22" s="25" t="n">
+      <c r="C22" s="30" t="n">
         <f aca="false">C21</f>
         <v>199375</v>
       </c>
-      <c r="D22" s="20"/>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="24" t="s">
+      <c r="D22" s="28"/>
+      <c r="E22" s="28"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="31" t="s">
         <v>170</v>
       </c>
-      <c r="B23" s="24" t="str">
+      <c r="B23" s="32" t="str">
         <f aca="false">AML!A39</f>
         <v>Fondos RV</v>
       </c>
-      <c r="C23" s="25" t="n">
+      <c r="C23" s="33" t="n">
         <f aca="false">AML!B39</f>
         <v>2183088.49</v>
       </c>
-      <c r="D23" s="20" t="s">
+      <c r="D23" s="34" t="s">
         <v>182</v>
       </c>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="24" t="s">
-        <v>170</v>
-      </c>
-      <c r="B24" s="24" t="str">
+      <c r="E23" s="35"/>
+    </row>
+    <row r="24" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="31"/>
+      <c r="B24" s="32" t="str">
         <f aca="false">AML!A40</f>
         <v>Planes de Pensiones (Papá 754.162,54 + Mamá 403.356,58)</v>
       </c>
-      <c r="C24" s="25" t="n">
+      <c r="C24" s="33" t="n">
         <f aca="false">AML!B40</f>
         <v>1157519.11</v>
       </c>
-      <c r="D24" s="20" t="s">
+      <c r="D24" s="34" t="s">
         <v>183</v>
       </c>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="26" t="s">
+      <c r="E24" s="53" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="36"/>
+      <c r="B25" s="37" t="s">
         <v>172</v>
       </c>
-      <c r="B25" s="24"/>
-      <c r="C25" s="25" t="n">
+      <c r="C25" s="38" t="n">
         <f aca="false">SUM(C23:C24)</f>
         <v>3340607.6</v>
       </c>
-      <c r="D25" s="20"/>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="24" t="s">
+      <c r="D25" s="36"/>
+      <c r="E25" s="36"/>
+    </row>
+    <row r="26" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="39" t="s">
         <v>173</v>
       </c>
-      <c r="B26" s="24" t="str">
+      <c r="B26" s="40" t="str">
         <f aca="false">AML!A41</f>
         <v>Acciones (Iberdrola 356.040 + BBVA 125.804,4 + TEF 56.169,35)</v>
       </c>
-      <c r="C26" s="25" t="n">
+      <c r="C26" s="41" t="n">
         <f aca="false">AML!B41</f>
         <v>538013.75</v>
       </c>
-      <c r="D26" s="20" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="24" t="s">
-        <v>173</v>
-      </c>
-      <c r="B27" s="24" t="str">
+      <c r="D26" s="42" t="s">
+        <v>185</v>
+      </c>
+      <c r="E26" s="54" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="39"/>
+      <c r="B27" s="40" t="str">
         <f aca="false">AML!A42</f>
         <v>ETF (Aristócratas)</v>
       </c>
-      <c r="C27" s="25" t="n">
+      <c r="C27" s="41" t="n">
         <f aca="false">AML!B42</f>
         <v>139351.5</v>
       </c>
-      <c r="D27" s="20" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="26" t="s">
+      <c r="D27" s="42" t="s">
+        <v>187</v>
+      </c>
+      <c r="E27" s="43"/>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="44"/>
+      <c r="B28" s="45" t="s">
         <v>176</v>
       </c>
-      <c r="B28" s="24"/>
-      <c r="C28" s="25" t="n">
+      <c r="C28" s="46" t="n">
         <f aca="false">SUM(C26:C27)</f>
         <v>677365.25</v>
       </c>
-      <c r="D28" s="20"/>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="26" t="s">
-        <v>186</v>
-      </c>
-      <c r="B30" s="24"/>
-      <c r="C30" s="25" t="n">
+      <c r="D28" s="44"/>
+      <c r="E28" s="44"/>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="47" t="s">
+        <v>188</v>
+      </c>
+      <c r="B30" s="47"/>
+      <c r="C30" s="48" t="n">
         <f aca="false">C22+C25+C28</f>
         <v>4217347.85</v>
       </c>
-      <c r="D30" s="20"/>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="24" t="s">
-        <v>187</v>
-      </c>
-      <c r="B31" s="24"/>
-      <c r="C31" s="25" t="n">
+      <c r="D30" s="49"/>
+      <c r="E30" s="49"/>
+    </row>
+    <row r="31" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B31" s="50" t="s">
+        <v>178</v>
+      </c>
+      <c r="C31" s="51" t="n">
         <f aca="false">C30-AML!B44</f>
         <v>0</v>
       </c>
-      <c r="D31" s="20" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="20" t="s">
+      <c r="E31" s="52" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="55" t="s">
         <v>189</v>
       </c>
+      <c r="B33" s="55"/>
+      <c r="C33" s="55"/>
+      <c r="D33" s="55"/>
+      <c r="E33" s="55"/>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="55"/>
+      <c r="B34" s="55"/>
+      <c r="C34" s="55"/>
+      <c r="D34" s="55"/>
+      <c r="E34" s="55"/>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="55"/>
+      <c r="B35" s="55"/>
+      <c r="C35" s="55"/>
+      <c r="D35" s="55"/>
+      <c r="E35" s="55"/>
     </row>
   </sheetData>
+  <mergeCells count="11">
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="A6:A7"/>
+    <mergeCell ref="A11:A12"/>
+    <mergeCell ref="A15:B15"/>
+    <mergeCell ref="A19:E19"/>
+    <mergeCell ref="A23:A24"/>
+    <mergeCell ref="A26:A27"/>
+    <mergeCell ref="A30:B30"/>
+    <mergeCell ref="A33:E35"/>
+  </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -3250,250 +3658,264 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
+    <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:D27"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="60"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="2" style="1" width="16"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="19" t="s">
         <v>190</v>
       </c>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B1" s="19"/>
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19"/>
+    </row>
+    <row r="2" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="20" t="s">
         <v>191</v>
       </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B2" s="20"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="21" t="s">
         <v>192</v>
       </c>
-      <c r="B4" s="22"/>
-      <c r="C4" s="22"/>
-      <c r="D4" s="22"/>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="23" t="s">
+      <c r="B4" s="21"/>
+      <c r="C4" s="21"/>
+      <c r="D4" s="21"/>
+      <c r="E4" s="21"/>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="22" t="s">
         <v>26</v>
       </c>
-      <c r="B5" s="23" t="s">
+      <c r="B5" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="C5" s="23" t="s">
+      <c r="C5" s="22" t="s">
         <v>28</v>
       </c>
-      <c r="D5" s="23" t="s">
+      <c r="D5" s="22" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="24" t="s">
+      <c r="E5" s="22"/>
+    </row>
+    <row r="6" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="56" t="s">
         <v>193</v>
       </c>
-      <c r="B6" s="27" t="n">
+      <c r="B6" s="57" t="n">
         <v>0.07</v>
       </c>
-      <c r="C6" s="20" t="s">
+      <c r="C6" s="58" t="s">
         <v>31</v>
       </c>
-      <c r="D6" s="20" t="s">
+      <c r="D6" s="59" t="s">
         <v>194</v>
       </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="24" t="s">
+      <c r="E6" s="59"/>
+    </row>
+    <row r="7" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="56" t="s">
         <v>195</v>
       </c>
-      <c r="B7" s="27" t="n">
+      <c r="B7" s="57" t="n">
         <v>0.094</v>
       </c>
-      <c r="C7" s="20" t="s">
+      <c r="C7" s="58" t="s">
         <v>31</v>
       </c>
-      <c r="D7" s="20" t="s">
+      <c r="D7" s="59" t="s">
         <v>196</v>
       </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E7" s="59"/>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="21" t="s">
         <v>197</v>
       </c>
-      <c r="B9" s="22"/>
-      <c r="C9" s="22"/>
-      <c r="D9" s="22"/>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="23" t="s">
+      <c r="B9" s="21"/>
+      <c r="C9" s="21"/>
+      <c r="D9" s="21"/>
+      <c r="E9" s="21"/>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="22" t="s">
         <v>26</v>
       </c>
-      <c r="B10" s="23" t="s">
+      <c r="B10" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="C10" s="23" t="s">
+      <c r="C10" s="22" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="24" t="s">
+      <c r="D10" s="22" t="s">
+        <v>29</v>
+      </c>
+      <c r="E10" s="22"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="60" t="s">
         <v>198</v>
       </c>
-      <c r="B11" s="25" t="n">
+      <c r="B11" s="61" t="n">
         <f aca="false">Cajas!C10</f>
         <v>872837.88</v>
       </c>
-      <c r="C11" s="20" t="s">
+      <c r="C11" s="34" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="24" t="s">
+      <c r="D11" s="35"/>
+      <c r="E11" s="35"/>
+    </row>
+    <row r="12" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="60" t="s">
         <v>200</v>
       </c>
-      <c r="B12" s="25" t="n">
+      <c r="B12" s="61" t="n">
         <f aca="false">Cajas!C25</f>
         <v>3340607.6</v>
       </c>
-      <c r="C12" s="20" t="s">
+      <c r="C12" s="34" t="s">
         <v>201</v>
       </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D12" s="53" t="s">
+        <v>202</v>
+      </c>
+      <c r="E12" s="53"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="21" t="s">
-        <v>202</v>
-      </c>
-      <c r="B14" s="22"/>
-      <c r="C14" s="22"/>
-      <c r="D14" s="22"/>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="23" t="s">
         <v>203</v>
       </c>
-      <c r="B15" s="23" t="s">
+      <c r="B14" s="21"/>
+      <c r="C14" s="21"/>
+      <c r="D14" s="21"/>
+      <c r="E14" s="21"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="22" t="s">
         <v>204</v>
       </c>
-      <c r="C15" s="23" t="s">
+      <c r="B15" s="22" t="s">
         <v>205</v>
       </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="24" t="s">
+      <c r="C15" s="62" t="s">
         <v>206</v>
       </c>
-      <c r="B16" s="25" t="n">
+      <c r="D15" s="63" t="s">
+        <v>207</v>
+      </c>
+      <c r="E15" s="22" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="60" t="s">
+        <v>209</v>
+      </c>
+      <c r="B16" s="33" t="n">
         <f aca="false">$B$11*(1+$B$6)^5</f>
         <v>1224200.27921452</v>
       </c>
-      <c r="C16" s="25" t="n">
+      <c r="C16" s="64" t="n">
         <f aca="false">$B$11*(1+$B$7)^5</f>
         <v>1367792.42987986</v>
       </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="24" t="s">
-        <v>207</v>
-      </c>
-      <c r="B17" s="25" t="n">
+      <c r="D16" s="65" t="n">
+        <f aca="false">$B$12*(1+$B$6)^5</f>
+        <v>4685374.97096958</v>
+      </c>
+      <c r="E16" s="33" t="n">
+        <f aca="false">$B$12*(1+$B$7)^5</f>
+        <v>5234944.41657267</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="60" t="s">
+        <v>210</v>
+      </c>
+      <c r="B17" s="33" t="n">
         <f aca="false">$B$11*(1+$B$6)^10</f>
         <v>1717004.22033575</v>
       </c>
-      <c r="C17" s="25" t="n">
+      <c r="C17" s="64" t="n">
         <f aca="false">$B$11*(1+$B$7)^10</f>
         <v>2143417.6656456</v>
       </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="24" t="s">
-        <v>208</v>
-      </c>
-      <c r="B18" s="25" t="n">
+      <c r="D17" s="65" t="n">
+        <f aca="false">$B$12*(1+$B$6)^10</f>
+        <v>6571480.77451184</v>
+      </c>
+      <c r="E17" s="33" t="n">
+        <f aca="false">$B$12*(1+$B$7)^10</f>
+        <v>8203490.59991523</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="60" t="s">
+        <v>211</v>
+      </c>
+      <c r="B18" s="33" t="n">
         <f aca="false">$B$11*(1+$B$6)^15</f>
         <v>2408187.24085111</v>
       </c>
-      <c r="C18" s="25" t="n">
+      <c r="C18" s="64" t="n">
         <f aca="false">$B$11*(1+$B$7)^15</f>
         <v>3358871.70380461</v>
       </c>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="21" t="s">
-        <v>209</v>
-      </c>
-      <c r="B20" s="22"/>
-      <c r="C20" s="22"/>
-      <c r="D20" s="22"/>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="23" t="s">
-        <v>203</v>
-      </c>
-      <c r="B21" s="23" t="s">
-        <v>204</v>
-      </c>
-      <c r="C21" s="23" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="24" t="s">
-        <v>206</v>
-      </c>
-      <c r="B22" s="25" t="n">
-        <f aca="false">$B$12*(1+$B$6)^5</f>
-        <v>4685374.97096958</v>
-      </c>
-      <c r="C22" s="25" t="n">
-        <f aca="false">$B$12*(1+$B$7)^5</f>
-        <v>5234944.41657267</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="24" t="s">
-        <v>207</v>
-      </c>
-      <c r="B23" s="25" t="n">
-        <f aca="false">$B$12*(1+$B$6)^10</f>
-        <v>6571480.77451184</v>
-      </c>
-      <c r="C23" s="25" t="n">
-        <f aca="false">$B$12*(1+$B$7)^10</f>
-        <v>8203490.59991523</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="24" t="s">
-        <v>208</v>
-      </c>
-      <c r="B24" s="25" t="n">
+      <c r="D18" s="65" t="n">
         <f aca="false">$B$12*(1+$B$6)^15</f>
         <v>9216841.73355336</v>
       </c>
-      <c r="C24" s="25" t="n">
+      <c r="E18" s="33" t="n">
         <f aca="false">$B$12*(1+$B$7)^15</f>
         <v>12855391.1307729</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="20" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="20" t="s">
-        <v>211</v>
-      </c>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="55" t="s">
+        <v>212</v>
+      </c>
+      <c r="B20" s="55"/>
+      <c r="C20" s="55"/>
+      <c r="D20" s="55"/>
+      <c r="E20" s="55"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="55"/>
+      <c r="B21" s="55"/>
+      <c r="C21" s="55"/>
+      <c r="D21" s="55"/>
+      <c r="E21" s="55"/>
     </row>
   </sheetData>
+  <mergeCells count="12">
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="D5:E5"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="D7:E7"/>
+    <mergeCell ref="A9:E9"/>
+    <mergeCell ref="D10:E10"/>
+    <mergeCell ref="D11:E11"/>
+    <mergeCell ref="D12:E12"/>
+    <mergeCell ref="A14:E14"/>
+    <mergeCell ref="A20:E21"/>
+  </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>

</xml_diff>

<commit_message>
Cajas: añadir % de cada caja sobre el patrimonio total (AMS/AML) + ajuste de impresión a una página
</commit_message>
<xml_diff>
--- a/data/raw/personal_capacity_facts.xlsx
+++ b/data/raw/personal_capacity_facts.xlsx
@@ -5,14 +5,14 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="Notas" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="AMS" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="AML" sheetId="3" state="visible" r:id="rId5"/>
-    <sheet name="Cajas" sheetId="4" state="visible" r:id="rId6"/>
-    <sheet name="Proyecciones" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="Proyecciones" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="Cajas" sheetId="5" state="visible" r:id="rId7"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="413" uniqueCount="213">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="415" uniqueCount="214">
   <si>
     <t xml:space="preserve">PERSONAL CAPACITY FACTS — Notas de uso</t>
   </si>
@@ -506,6 +506,75 @@
     <t xml:space="preserve">Confirmado 2026-08-10 -- la exclusión de Planes de Pensiones y la minusvalía TEF de arriba son las únicas cuestiones fiscales conocidas; ninguna de las dos es una restricción activa</t>
   </si>
   <si>
+    <t xml:space="preserve">PROYECCIÓN CAJA MOTOR — HIPÓTESIS BASE v1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ilustrativa, no un objetivo. X/Y/Z por necesidad patrimonial: CONSTITUTION.md Sección 6, Pendiente.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hipótesis de rentabilidad  ·  CONSTITUTION.md Sección 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rentabilidad real anualizada</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hipótesis base v1 — CONSTITUTION.md Sección 2. Serie total return real de Shiller (data/raw/shiller.xlsx), dividendos reinvertidos, CAGR de la serie completa. No se ajusta automáticamente por CAPE ni por el Research Engine — editar solo tras actualización explícita de la Constitución.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rentabilidad nominal anualizada (aprox.)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Derivada de la rentabilidad real + inflación media histórica de la serie Shiller (~2,15%/año). Misma gobernanza que la fila anterior.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Base — Caja Motor  ·  hoja 'Cajas'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AMS — Caja Motor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cajas!C10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AML — Caja Motor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cajas!C25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Incluye Planes de Pensiones, operativamente bloqueados (ver hoja 'Cajas').</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Proyección Caja Motor a 5 / 10 / 15 años  ·  AMS vs. AML</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Horizonte</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AMS Real</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AMS Nominal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AML Real</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AML Nominal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5 años</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10 años</t>
+  </si>
+  <si>
+    <t xml:space="preserve">15 años</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Proyección de interés compuesto puro sobre el saldo actual de Caja Motor. No es el objetivo X/Y/Z (todavía sin definir) — sirve para comparar, una vez fijado ese objetivo, si la trayectoria real va camino de cumplirlo. AML incluye Planes de Pensiones bloqueados.</t>
+  </si>
+  <si>
     <t xml:space="preserve">CLASIFICACIÓN EN LAS TRES CAJAS</t>
   </si>
   <si>
@@ -521,6 +590,9 @@
     <t xml:space="preserve">Partida</t>
   </si>
   <si>
+    <t xml:space="preserve">% Total</t>
+  </si>
+  <si>
     <t xml:space="preserve">Origen</t>
   </si>
   <si>
@@ -593,76 +665,7 @@
     <t xml:space="preserve">TOTAL AML (3 cajas)</t>
   </si>
   <si>
-    <t xml:space="preserve">Colores: Seguridad (azul) · Motor (verde) · Rentas Pasivas (naranja). Clasificación fijada por Armando el 2026-08-13 sobre la tabla de cajas de CONSTITUTION.md Sección 2, Nivel 3 — Seguridad: liquidez/depósitos/monetarios · Motor: fondo indexado S&amp;P 500 y otras inversiones a largo plazo · Rentas Pasivas: JGPI, inmobiliario, oro.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PROYECCIÓN CAJA MOTOR — HIPÓTESIS BASE v1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ilustrativa, no un objetivo. X/Y/Z por necesidad patrimonial: CONSTITUTION.md Sección 6, Pendiente.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hipótesis de rentabilidad  ·  CONSTITUTION.md Sección 2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rentabilidad real anualizada</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hipótesis base v1 — CONSTITUTION.md Sección 2. Serie total return real de Shiller (data/raw/shiller.xlsx), dividendos reinvertidos, CAGR de la serie completa. No se ajusta automáticamente por CAPE ni por el Research Engine — editar solo tras actualización explícita de la Constitución.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rentabilidad nominal anualizada (aprox.)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Derivada de la rentabilidad real + inflación media histórica de la serie Shiller (~2,15%/año). Misma gobernanza que la fila anterior.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Base — Caja Motor  ·  hoja 'Cajas'</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AMS — Caja Motor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cajas!C10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AML — Caja Motor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cajas!C25</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Incluye Planes de Pensiones, operativamente bloqueados (ver hoja 'Cajas').</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Proyección Caja Motor a 5 / 10 / 15 años  ·  AMS vs. AML</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Horizonte</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AMS Real</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AMS Nominal</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AML Real</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AML Nominal</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5 años</t>
-  </si>
-  <si>
-    <t xml:space="preserve">10 años</t>
-  </si>
-  <si>
-    <t xml:space="preserve">15 años</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Proyección de interés compuesto puro sobre el saldo actual de Caja Motor. No es el objetivo X/Y/Z (todavía sin definir) — sirve para comparar, una vez fijado ese objetivo, si la trayectoria real va camino de cumplirlo. AML incluye Planes de Pensiones bloqueados.</t>
+    <t xml:space="preserve">Colores: Seguridad (azul) · Motor (verde) · Rentas Pasivas (naranja). % Total = peso de cada caja sobre el patrimonio total de AMS o AML respectivamente. Clasificación fijada por Armando el 2026-08-13 sobre la tabla de cajas de CONSTITUTION.md Sección 2, Nivel 3 — Seguridad: liquidez/depósitos/monetarios · Motor: fondo indexado S&amp;P 500 y otras inversiones a largo plazo · Rentas Pasivas: JGPI, inmobiliario, oro.</t>
   </si>
 </sst>
 </file>
@@ -675,7 +678,7 @@
     <numFmt numFmtId="166" formatCode="0.0%"/>
     <numFmt numFmtId="167" formatCode="0"/>
   </numFmts>
-  <fonts count="19">
+  <fonts count="26">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -702,28 +705,28 @@
       <b val="true"/>
       <sz val="13"/>
       <name val="Arial"/>
-      <family val="0"/>
+      <family val="2"/>
       <charset val="1"/>
     </font>
     <font>
       <b val="true"/>
       <sz val="10"/>
       <name val="Arial"/>
-      <family val="0"/>
+      <family val="2"/>
       <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
-      <family val="0"/>
+      <family val="2"/>
       <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
       <color rgb="FF0000FF"/>
       <name val="Arial"/>
-      <family val="0"/>
+      <family val="2"/>
       <charset val="1"/>
     </font>
     <font>
@@ -731,7 +734,77 @@
       <sz val="9"/>
       <color rgb="FF666666"/>
       <name val="Arial"/>
-      <family val="0"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="13"/>
+      <color rgb="FF1F1F1F"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <i val="true"/>
+      <sz val="9"/>
+      <color rgb="FF808080"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="10"/>
+      <color rgb="FF1F1F1F"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF1F1F1F"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="10"/>
+      <color rgb="FF1155CC"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="8.5"/>
+      <color rgb="FF9E9E9E"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <i val="true"/>
+      <sz val="8.5"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="10.5"/>
+      <color rgb="FF1F1F1F"/>
+      <name val="Arial"/>
+      <family val="2"/>
       <charset val="1"/>
     </font>
     <font>
@@ -796,22 +869,6 @@
       <family val="0"/>
       <charset val="1"/>
     </font>
-    <font>
-      <b val="true"/>
-      <sz val="10"/>
-      <color rgb="FF1155CC"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="10.5"/>
-      <color rgb="FF1F1F1F"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
   </fonts>
   <fills count="14">
     <fill>
@@ -846,6 +903,18 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFFFF2CC"/>
+        <bgColor rgb="FFFCE4D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE2EFDA"/>
+        <bgColor rgb="FFDDEBF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFDDEBF7"/>
         <bgColor rgb="FFD9E1F2"/>
       </patternFill>
@@ -854,12 +923,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFBDD7EE"/>
         <bgColor rgb="FFD9D9D9"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFE2EFDA"/>
-        <bgColor rgb="FFDDEBF7"/>
       </patternFill>
     </fill>
     <fill>
@@ -884,12 +947,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="FF404040"/>
         <bgColor rgb="FF595959"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFF2CC"/>
-        <bgColor rgb="FFFCE4D6"/>
       </patternFill>
     </fill>
   </fills>
@@ -1003,15 +1060,11 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="66">
+  <cellXfs count="77">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1032,7 +1085,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1052,7 +1105,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1072,7 +1125,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1080,11 +1133,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1092,180 +1145,228 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="13" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="14" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="17" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="15" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="6" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="7" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="7" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="16" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="3" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="3" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="12" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="13" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="8" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="8" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="13" fillId="8" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="13" fillId="7" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="8" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="8" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="9" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="9" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="12" fillId="9" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="13" fillId="7" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="10" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="10" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="13" fillId="10" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="14" fillId="10" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="10" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="11" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="11" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="12" fillId="11" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="12" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="15" fillId="12" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="12" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="16" fillId="8" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="16" fillId="10" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="17" fillId="13" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="20" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="21" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="21" fillId="8" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="22" fillId="8" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="22" fillId="8" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="8" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="23" fillId="8" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="9" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="21" fillId="9" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="21" fillId="9" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="21" fillId="9" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="21" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="22" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="22" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="23" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="10" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="21" fillId="10" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="21" fillId="10" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="21" fillId="10" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="21" fillId="11" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="22" fillId="11" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="22" fillId="11" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="11" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="23" fillId="11" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="12" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="21" fillId="12" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="21" fillId="12" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="21" fillId="12" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="24" fillId="13" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="24" fillId="13" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="24" fillId="13" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="13" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="8" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="18" fillId="8" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="3" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="3" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="13" fillId="8" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="13" fillId="8" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="25" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="25" fillId="11" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -1521,141 +1622,141 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B24"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.66796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="38"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="70"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="70"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="3" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="2" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="5" t="s">
+      <c r="A6" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="3" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="4" t="s">
+      <c r="A7" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="3" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3" t="s">
+      <c r="A9" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="4" t="s">
+      <c r="A10" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="B10" s="3" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="4" t="s">
+      <c r="A11" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="B11" s="3" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="4" t="s">
+      <c r="A12" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B12" s="4" t="s">
+      <c r="B12" s="3" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="3" t="s">
+      <c r="A14" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B14" s="4" t="s">
+      <c r="B14" s="3" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="3" t="s">
+      <c r="A16" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B16" s="4" t="s">
+      <c r="B16" s="3" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="3" t="s">
+      <c r="A18" s="2" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="4" t="s">
+      <c r="A19" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B19" s="4" t="s">
+      <c r="B19" s="3" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="4" t="s">
+      <c r="A20" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B20" s="4" t="s">
+      <c r="B20" s="3" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="4" t="s">
+      <c r="A21" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B21" s="4" t="s">
+      <c r="B21" s="3" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="4" t="s">
+      <c r="A22" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B22" s="4" t="s">
+      <c r="B22" s="3" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="4" t="s">
+      <c r="A23" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B23" s="4" t="s">
+      <c r="B23" s="3" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="4" t="s">
+      <c r="A24" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B24" s="4" t="s">
+      <c r="B24" s="3" t="s">
         <v>23</v>
       </c>
     </row>
@@ -1676,707 +1777,707 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D61"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.66796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="40"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="46"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="1" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="6" t="s">
+      <c r="A3" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="B3" s="7"/>
-      <c r="C3" s="7"/>
-      <c r="D3" s="7"/>
+      <c r="B3" s="6"/>
+      <c r="C3" s="6"/>
+      <c r="D3" s="6"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="8" t="s">
+      <c r="A4" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="B4" s="8" t="s">
+      <c r="B4" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="C4" s="8" t="s">
+      <c r="C4" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="D4" s="8" t="s">
+      <c r="D4" s="7" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4" t="s">
+      <c r="A5" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="B5" s="9" t="n">
+      <c r="B5" s="8" t="n">
         <v>20000</v>
       </c>
-      <c r="C5" s="10" t="s">
+      <c r="C5" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="D5" s="10" t="s">
+      <c r="D5" s="9" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4" t="s">
+      <c r="A6" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="B6" s="9" t="n">
+      <c r="B6" s="8" t="n">
         <v>13000</v>
       </c>
-      <c r="C6" s="10" t="s">
+      <c r="C6" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="D6" s="10" t="s">
+      <c r="D6" s="9" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="4" t="s">
+      <c r="A7" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="B7" s="11" t="n">
+      <c r="B7" s="10" t="n">
         <f aca="false">B6-B5</f>
         <v>-7000</v>
       </c>
-      <c r="C7" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="D7" s="10" t="s">
+      <c r="C7" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="D7" s="9" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="4" t="s">
+      <c r="A8" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="B8" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="C8" s="10" t="s">
+      <c r="C8" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="D8" s="10" t="s">
+      <c r="D8" s="9" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="4" t="s">
+      <c r="A9" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="B9" s="9" t="n">
+      <c r="B9" s="8" t="n">
         <v>30000</v>
       </c>
-      <c r="C9" s="10" t="s">
+      <c r="C9" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="D9" s="10" t="s">
+      <c r="D9" s="9" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="4" t="s">
+      <c r="A10" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="B10" s="9" t="n">
+      <c r="B10" s="8" t="n">
         <v>70000</v>
       </c>
-      <c r="C10" s="10" t="s">
+      <c r="C10" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="D10" s="10" t="s">
+      <c r="D10" s="9" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="4" t="s">
+      <c r="A11" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="B11" s="9" t="n">
+      <c r="B11" s="8" t="n">
         <v>120000</v>
       </c>
-      <c r="C11" s="10" t="s">
+      <c r="C11" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="D11" s="10" t="s">
+      <c r="D11" s="9" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="4" t="s">
+      <c r="A12" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="B12" s="11" t="n">
+      <c r="B12" s="10" t="n">
         <f aca="false">B9+B10</f>
         <v>100000</v>
       </c>
-      <c r="C12" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="D12" s="12"/>
+      <c r="C12" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="D12" s="11"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="4" t="s">
+      <c r="A13" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="B13" s="11" t="n">
+      <c r="B13" s="10" t="n">
         <f aca="false">B9+B11</f>
         <v>150000</v>
       </c>
-      <c r="C13" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="D13" s="12"/>
+      <c r="C13" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="D13" s="11"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="4" t="s">
+      <c r="A14" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="B14" s="9" t="n">
+      <c r="B14" s="8" t="n">
         <v>83100</v>
       </c>
-      <c r="C14" s="10" t="s">
+      <c r="C14" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="D14" s="10" t="s">
+      <c r="D14" s="9" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="4" t="s">
+      <c r="A15" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="B15" s="9" t="n">
+      <c r="B15" s="8" t="n">
         <v>89230.77</v>
       </c>
-      <c r="C15" s="10" t="s">
+      <c r="C15" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="D15" s="10" t="s">
+      <c r="D15" s="9" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="4" t="s">
+      <c r="A16" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="B16" s="11" t="n">
+      <c r="B16" s="10" t="n">
         <f aca="false">SUM(B14:B15)</f>
         <v>172330.77</v>
       </c>
-      <c r="C16" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="D16" s="12"/>
+      <c r="C16" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="D16" s="11"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="4" t="s">
+      <c r="A17" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="B17" s="11" t="n">
+      <c r="B17" s="10" t="n">
         <f aca="false">B16-B9</f>
         <v>142330.77</v>
       </c>
-      <c r="C17" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="D17" s="12"/>
+      <c r="C17" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="D17" s="11"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="4" t="s">
+      <c r="A18" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="B18" s="11" t="n">
+      <c r="B18" s="10" t="n">
         <f aca="false">B16-B12</f>
         <v>72330.77</v>
       </c>
-      <c r="C18" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="D18" s="12"/>
+      <c r="C18" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="D18" s="11"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="4" t="s">
+      <c r="A19" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="B19" s="11" t="n">
+      <c r="B19" s="10" t="n">
         <f aca="false">B16-B13</f>
         <v>22330.77</v>
       </c>
-      <c r="C19" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="D19" s="10" t="s">
+      <c r="C19" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="D19" s="9" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="4" t="s">
+      <c r="A20" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="B20" s="11" t="n">
+      <c r="B20" s="10" t="n">
         <f aca="false">B17-B10</f>
         <v>72330.77</v>
       </c>
-      <c r="C20" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="D20" s="12"/>
+      <c r="C20" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="D20" s="11"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="4" t="s">
+      <c r="A21" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="B21" s="11" t="n">
+      <c r="B21" s="10" t="n">
         <f aca="false">B17-B11</f>
         <v>22330.77</v>
       </c>
-      <c r="C21" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="D21" s="12"/>
+      <c r="C21" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="D21" s="11"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="6" t="s">
+      <c r="A23" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="B23" s="7"/>
-      <c r="C23" s="7"/>
-      <c r="D23" s="7"/>
+      <c r="B23" s="6"/>
+      <c r="C23" s="6"/>
+      <c r="D23" s="6"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="8" t="s">
+      <c r="A24" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="B24" s="8" t="s">
+      <c r="B24" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="C24" s="8" t="s">
+      <c r="C24" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="D24" s="8" t="s">
+      <c r="D24" s="7" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="4" t="s">
+      <c r="A25" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="B25" s="5" t="s">
+      <c r="B25" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="C25" s="10" t="s">
+      <c r="C25" s="9" t="s">
         <v>64</v>
       </c>
-      <c r="D25" s="10" t="s">
+      <c r="D25" s="9" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="6" t="s">
+      <c r="A27" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="B27" s="7"/>
-      <c r="C27" s="7"/>
-      <c r="D27" s="7"/>
+      <c r="B27" s="6"/>
+      <c r="C27" s="6"/>
+      <c r="D27" s="6"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="8" t="s">
+      <c r="A28" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="B28" s="8" t="s">
+      <c r="B28" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="C28" s="8" t="s">
+      <c r="C28" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="D28" s="8" t="s">
+      <c r="D28" s="7" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="4" t="s">
+      <c r="A29" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="B29" s="9" t="n">
+      <c r="B29" s="8" t="n">
         <v>6000</v>
       </c>
-      <c r="C29" s="10" t="s">
+      <c r="C29" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="D29" s="12"/>
+      <c r="D29" s="11"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="4" t="s">
+      <c r="A30" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="B30" s="9" t="n">
+      <c r="B30" s="8" t="n">
         <v>5000</v>
       </c>
-      <c r="C30" s="10" t="s">
+      <c r="C30" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="D30" s="12"/>
+      <c r="D30" s="11"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="4" t="s">
+      <c r="A31" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="B31" s="9" t="n">
+      <c r="B31" s="8" t="n">
         <v>2000</v>
       </c>
-      <c r="C31" s="10" t="s">
+      <c r="C31" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="D31" s="12"/>
+      <c r="D31" s="11"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="4" t="s">
+      <c r="A32" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="B32" s="11" t="n">
+      <c r="B32" s="10" t="n">
         <f aca="false">SUM(B29:B31)</f>
         <v>13000</v>
       </c>
-      <c r="C32" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="D32" s="12"/>
+      <c r="C32" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="D32" s="11"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="4" t="s">
+      <c r="A33" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="B33" s="13" t="n">
+      <c r="B33" s="12" t="n">
         <f aca="false">B29/B32</f>
         <v>0.461538461538462</v>
       </c>
-      <c r="C33" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="D33" s="12"/>
+      <c r="C33" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="D33" s="11"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="4" t="s">
+      <c r="A34" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="B34" s="13" t="n">
+      <c r="B34" s="12" t="n">
         <f aca="false">B30/B32</f>
         <v>0.384615384615385</v>
       </c>
-      <c r="C34" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="D34" s="12"/>
+      <c r="C34" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="D34" s="11"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="4" t="s">
+      <c r="A35" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="B35" s="13" t="n">
+      <c r="B35" s="12" t="n">
         <f aca="false">B31/B32</f>
         <v>0.153846153846154</v>
       </c>
-      <c r="C35" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="D35" s="12"/>
+      <c r="C35" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="D35" s="11"/>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="4" t="s">
+      <c r="A36" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="B36" s="5" t="s">
+      <c r="B36" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="C36" s="10" t="s">
+      <c r="C36" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="D36" s="10" t="s">
+      <c r="D36" s="9" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="6" t="s">
+      <c r="A38" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="B38" s="7"/>
-      <c r="C38" s="7"/>
-      <c r="D38" s="7"/>
+      <c r="B38" s="6"/>
+      <c r="C38" s="6"/>
+      <c r="D38" s="6"/>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="8" t="s">
+      <c r="A39" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="B39" s="8" t="s">
+      <c r="B39" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="C39" s="8" t="s">
+      <c r="C39" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="D39" s="8" t="s">
+      <c r="D39" s="7" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="4" t="s">
+      <c r="A40" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="B40" s="9" t="n">
+      <c r="B40" s="8" t="n">
         <v>872837.88</v>
       </c>
-      <c r="C40" s="10" t="s">
+      <c r="C40" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="D40" s="12"/>
+      <c r="D40" s="11"/>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A41" s="4" t="s">
+      <c r="A41" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="B41" s="9" t="n">
+      <c r="B41" s="8" t="n">
         <v>89230.77</v>
       </c>
-      <c r="C41" s="10" t="s">
+      <c r="C41" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="D41" s="12"/>
+      <c r="D41" s="11"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="4" t="s">
+      <c r="A42" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="B42" s="9" t="n">
+      <c r="B42" s="8" t="n">
         <v>111570.37</v>
       </c>
-      <c r="C42" s="10" t="s">
+      <c r="C42" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="D42" s="12"/>
+      <c r="D42" s="11"/>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A43" s="4" t="s">
+      <c r="A43" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="B43" s="9" t="n">
+      <c r="B43" s="8" t="n">
         <v>100000</v>
       </c>
-      <c r="C43" s="10" t="s">
+      <c r="C43" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="D43" s="12"/>
+      <c r="D43" s="11"/>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="4" t="s">
+      <c r="A44" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="B44" s="9" t="n">
+      <c r="B44" s="8" t="n">
         <v>83100</v>
       </c>
-      <c r="C44" s="10" t="s">
+      <c r="C44" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="D44" s="10" t="s">
+      <c r="D44" s="9" t="s">
         <v>83</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A45" s="14" t="s">
+      <c r="A45" s="13" t="s">
         <v>84</v>
       </c>
-      <c r="B45" s="15" t="n">
+      <c r="B45" s="14" t="n">
         <f aca="false">SUM(B40:B44)</f>
         <v>1256739.02</v>
       </c>
-      <c r="C45" s="16" t="s">
-        <v>36</v>
-      </c>
-      <c r="D45" s="17"/>
+      <c r="C45" s="15" t="s">
+        <v>36</v>
+      </c>
+      <c r="D45" s="16"/>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A46" s="4" t="s">
+      <c r="A46" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="B46" s="13" t="n">
+      <c r="B46" s="12" t="n">
         <f aca="false">B40/B45</f>
         <v>0.694525964507731</v>
       </c>
-      <c r="C46" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="D46" s="12"/>
+      <c r="C46" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="D46" s="11"/>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A47" s="4" t="s">
+      <c r="A47" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="B47" s="13" t="n">
+      <c r="B47" s="12" t="n">
         <f aca="false">B41/B45</f>
         <v>0.0710018297991575</v>
       </c>
-      <c r="C47" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="D47" s="12"/>
+      <c r="C47" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="D47" s="11"/>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A48" s="4" t="s">
+      <c r="A48" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="B48" s="13" t="n">
+      <c r="B48" s="12" t="n">
         <f aca="false">B42/B45</f>
         <v>0.0887776763707074</v>
       </c>
-      <c r="C48" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="D48" s="12"/>
+      <c r="C48" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="D48" s="11"/>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A49" s="4" t="s">
+      <c r="A49" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="B49" s="13" t="n">
+      <c r="B49" s="12" t="n">
         <f aca="false">B43/B45</f>
         <v>0.0795710154682712</v>
       </c>
-      <c r="C49" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="D49" s="12"/>
+      <c r="C49" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="D49" s="11"/>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A50" s="4" t="s">
+      <c r="A50" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="B50" s="13" t="n">
+      <c r="B50" s="12" t="n">
         <f aca="false">B44/B45</f>
         <v>0.0661235138541334</v>
       </c>
-      <c r="C50" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="D50" s="12"/>
+      <c r="C50" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="D50" s="11"/>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A51" s="4" t="s">
+      <c r="A51" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="B51" s="5" t="s">
+      <c r="B51" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="C51" s="10" t="s">
+      <c r="C51" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="D51" s="10" t="s">
+      <c r="D51" s="9" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A53" s="6" t="s">
+      <c r="A53" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="B53" s="7"/>
-      <c r="C53" s="7"/>
-      <c r="D53" s="7"/>
+      <c r="B53" s="6"/>
+      <c r="C53" s="6"/>
+      <c r="D53" s="6"/>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A54" s="8" t="s">
+      <c r="A54" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="B54" s="8" t="s">
+      <c r="B54" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="C54" s="8" t="s">
+      <c r="C54" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="D54" s="8" t="s">
+      <c r="D54" s="7" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A55" s="4" t="s">
+      <c r="A55" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="B55" s="5" t="s">
+      <c r="B55" s="4" t="s">
         <v>94</v>
       </c>
-      <c r="C55" s="10" t="s">
+      <c r="C55" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="D55" s="10" t="s">
+      <c r="D55" s="9" t="s">
         <v>95</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A56" s="4" t="s">
+      <c r="A56" s="3" t="s">
         <v>96</v>
       </c>
-      <c r="B56" s="5" t="s">
+      <c r="B56" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="C56" s="10" t="s">
+      <c r="C56" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="D56" s="10" t="s">
+      <c r="D56" s="9" t="s">
         <v>98</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A58" s="6" t="s">
+      <c r="A58" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="B58" s="7"/>
-      <c r="C58" s="7"/>
-      <c r="D58" s="7"/>
+      <c r="B58" s="6"/>
+      <c r="C58" s="6"/>
+      <c r="D58" s="6"/>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A59" s="8" t="s">
+      <c r="A59" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="B59" s="8" t="s">
+      <c r="B59" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="C59" s="8" t="s">
+      <c r="C59" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="D59" s="8" t="s">
+      <c r="D59" s="7" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A60" s="4" t="s">
+      <c r="A60" s="3" t="s">
         <v>100</v>
       </c>
-      <c r="B60" s="9" t="n">
+      <c r="B60" s="8" t="n">
         <v>-215092</v>
       </c>
-      <c r="C60" s="10" t="s">
+      <c r="C60" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="D60" s="10" t="s">
+      <c r="D60" s="9" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A61" s="4" t="s">
+      <c r="A61" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="B61" s="5" t="s">
+      <c r="B61" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="C61" s="10" t="s">
+      <c r="C61" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="D61" s="10" t="s">
+      <c r="D61" s="9" t="s">
         <v>104</v>
       </c>
     </row>
@@ -2397,832 +2498,832 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D73"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.66796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="50"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="50"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="1" t="s">
         <v>105</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="6" t="s">
+      <c r="A3" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="B3" s="7"/>
-      <c r="C3" s="7"/>
-      <c r="D3" s="7"/>
+      <c r="B3" s="6"/>
+      <c r="C3" s="6"/>
+      <c r="D3" s="6"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="8" t="s">
+      <c r="A4" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="B4" s="8" t="s">
+      <c r="B4" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="C4" s="8" t="s">
+      <c r="C4" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="D4" s="8" t="s">
+      <c r="D4" s="7" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4" t="s">
+      <c r="A5" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="B5" s="9" t="n">
+      <c r="B5" s="8" t="n">
         <v>32500</v>
       </c>
-      <c r="C5" s="10" t="s">
+      <c r="C5" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="D5" s="10" t="s">
+      <c r="D5" s="9" t="s">
         <v>106</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4" t="s">
+      <c r="A6" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="B6" s="9" t="n">
+      <c r="B6" s="8" t="n">
         <v>80000</v>
       </c>
-      <c r="C6" s="10" t="s">
+      <c r="C6" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="D6" s="10" t="s">
+      <c r="D6" s="9" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="4" t="s">
+      <c r="A7" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="B7" s="11" t="n">
+      <c r="B7" s="10" t="n">
         <f aca="false">B6-B5</f>
         <v>47500</v>
       </c>
-      <c r="C7" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="D7" s="10" t="s">
+      <c r="C7" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="D7" s="9" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="4" t="s">
+      <c r="A8" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="B8" s="9" t="n">
+      <c r="B8" s="8" t="n">
         <v>125000</v>
       </c>
-      <c r="C8" s="10" t="s">
+      <c r="C8" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="D8" s="10" t="s">
+      <c r="D8" s="9" t="s">
         <v>110</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="4" t="s">
+      <c r="A9" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="B9" s="9" t="n">
+      <c r="B9" s="8" t="n">
         <v>125000</v>
       </c>
-      <c r="C9" s="10" t="s">
+      <c r="C9" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="D9" s="12"/>
+      <c r="D9" s="11"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="4" t="s">
+      <c r="A10" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="B10" s="9" t="n">
+      <c r="B10" s="8" t="n">
         <v>175000</v>
       </c>
-      <c r="C10" s="10" t="s">
+      <c r="C10" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="D10" s="12"/>
+      <c r="D10" s="11"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="4" t="s">
+      <c r="A11" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="B11" s="11" t="n">
+      <c r="B11" s="10" t="n">
         <f aca="false">B8+B9</f>
         <v>250000</v>
       </c>
-      <c r="C11" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="D11" s="12"/>
+      <c r="C11" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="D11" s="11"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="4" t="s">
+      <c r="A12" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="B12" s="11" t="n">
+      <c r="B12" s="10" t="n">
         <f aca="false">B8+B10</f>
         <v>300000</v>
       </c>
-      <c r="C12" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="D12" s="10" t="s">
+      <c r="C12" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="D12" s="9" t="s">
         <v>111</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="4" t="s">
+      <c r="A13" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="B13" s="9" t="n">
+      <c r="B13" s="8" t="n">
         <v>54375</v>
       </c>
-      <c r="C13" s="10" t="s">
+      <c r="C13" s="9" t="s">
         <v>112</v>
       </c>
-      <c r="D13" s="12"/>
+      <c r="D13" s="11"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="4" t="s">
+      <c r="A14" s="3" t="s">
         <v>113</v>
       </c>
-      <c r="B14" s="9" t="n">
+      <c r="B14" s="8" t="n">
         <v>60000</v>
       </c>
-      <c r="C14" s="10" t="s">
+      <c r="C14" s="9" t="s">
         <v>112</v>
       </c>
-      <c r="D14" s="10" t="s">
+      <c r="D14" s="9" t="s">
         <v>114</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="4" t="s">
+      <c r="A15" s="3" t="s">
         <v>115</v>
       </c>
-      <c r="B15" s="9" t="n">
+      <c r="B15" s="8" t="n">
         <v>85000</v>
       </c>
-      <c r="C15" s="10" t="s">
+      <c r="C15" s="9" t="s">
         <v>112</v>
       </c>
-      <c r="D15" s="10" t="s">
+      <c r="D15" s="9" t="s">
         <v>116</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="4" t="s">
+      <c r="A16" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="B16" s="9" t="n">
+      <c r="B16" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="C16" s="10" t="s">
+      <c r="C16" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="D16" s="10" t="s">
+      <c r="D16" s="9" t="s">
         <v>117</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="4" t="s">
+      <c r="A17" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="B17" s="11" t="n">
+      <c r="B17" s="10" t="n">
         <f aca="false">SUM(B13:B16)</f>
         <v>199375</v>
       </c>
-      <c r="C17" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="D17" s="12"/>
+      <c r="C17" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="D17" s="11"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="4" t="s">
+      <c r="A18" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="B18" s="11" t="n">
+      <c r="B18" s="10" t="n">
         <f aca="false">B17-B8</f>
         <v>74375</v>
       </c>
-      <c r="C18" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="D18" s="12"/>
+      <c r="C18" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="D18" s="11"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="4" t="s">
+      <c r="A19" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="B19" s="11" t="n">
+      <c r="B19" s="10" t="n">
         <f aca="false">B17-B11</f>
         <v>-50625</v>
       </c>
-      <c r="C19" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="D19" s="12"/>
+      <c r="C19" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="D19" s="11"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="4" t="s">
+      <c r="A20" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="B20" s="11" t="n">
+      <c r="B20" s="10" t="n">
         <f aca="false">B17-B12</f>
         <v>-100625</v>
       </c>
-      <c r="C20" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="D20" s="12"/>
+      <c r="C20" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="D20" s="11"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="4" t="s">
+      <c r="A21" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="B21" s="11" t="n">
+      <c r="B21" s="10" t="n">
         <f aca="false">B18-B9</f>
         <v>-50625</v>
       </c>
-      <c r="C21" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="D21" s="10" t="s">
+      <c r="C21" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="D21" s="9" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="4" t="s">
+      <c r="A22" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="B22" s="11" t="n">
+      <c r="B22" s="10" t="n">
         <f aca="false">B18-B10</f>
         <v>-100625</v>
       </c>
-      <c r="C22" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="D22" s="12"/>
+      <c r="C22" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="D22" s="11"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="6" t="s">
+      <c r="A24" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="B24" s="7"/>
-      <c r="C24" s="7"/>
-      <c r="D24" s="7"/>
+      <c r="B24" s="6"/>
+      <c r="C24" s="6"/>
+      <c r="D24" s="6"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="8" t="s">
+      <c r="A25" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="B25" s="8" t="s">
+      <c r="B25" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="C25" s="8" t="s">
+      <c r="C25" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="D25" s="8" t="s">
+      <c r="D25" s="7" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="4" t="s">
+      <c r="A26" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="B26" s="5" t="s">
+      <c r="B26" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="C26" s="10" t="s">
+      <c r="C26" s="9" t="s">
         <v>64</v>
       </c>
-      <c r="D26" s="10" t="s">
+      <c r="D26" s="9" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="6" t="s">
+      <c r="A28" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="B28" s="7"/>
-      <c r="C28" s="7"/>
-      <c r="D28" s="7"/>
+      <c r="B28" s="6"/>
+      <c r="C28" s="6"/>
+      <c r="D28" s="6"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="8" t="s">
+      <c r="A29" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="B29" s="8" t="s">
+      <c r="B29" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="C29" s="8" t="s">
+      <c r="C29" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="D29" s="8" t="s">
+      <c r="D29" s="7" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="4" t="s">
+      <c r="A30" s="3" t="s">
         <v>119</v>
       </c>
-      <c r="B30" s="9" t="n">
+      <c r="B30" s="8" t="n">
         <v>60000</v>
       </c>
-      <c r="C30" s="10" t="s">
+      <c r="C30" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="D30" s="10" t="s">
+      <c r="D30" s="9" t="s">
         <v>120</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="4" t="s">
+      <c r="A31" s="3" t="s">
         <v>121</v>
       </c>
-      <c r="B31" s="9" t="n">
+      <c r="B31" s="8" t="n">
         <v>20000</v>
       </c>
-      <c r="C31" s="10" t="s">
+      <c r="C31" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="D31" s="12"/>
+      <c r="D31" s="11"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="4" t="s">
+      <c r="A32" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="B32" s="11" t="n">
+      <c r="B32" s="10" t="n">
         <f aca="false">SUM(B30:B31)</f>
         <v>80000</v>
       </c>
-      <c r="C32" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="D32" s="12"/>
+      <c r="C32" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="D32" s="11"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="4" t="s">
+      <c r="A33" s="3" t="s">
         <v>122</v>
       </c>
-      <c r="B33" s="13" t="n">
+      <c r="B33" s="12" t="n">
         <f aca="false">B30/B32</f>
         <v>0.75</v>
       </c>
-      <c r="C33" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="D33" s="12"/>
+      <c r="C33" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="D33" s="11"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="4" t="s">
+      <c r="A34" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="B34" s="13" t="n">
+      <c r="B34" s="12" t="n">
         <f aca="false">B31/B32</f>
         <v>0.25</v>
       </c>
-      <c r="C34" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="D34" s="12"/>
+      <c r="C34" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="D34" s="11"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="4" t="s">
+      <c r="A35" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="B35" s="5" t="s">
+      <c r="B35" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="C35" s="10" t="s">
+      <c r="C35" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="D35" s="10" t="s">
+      <c r="D35" s="9" t="s">
         <v>124</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="6" t="s">
+      <c r="A37" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="B37" s="7"/>
-      <c r="C37" s="7"/>
-      <c r="D37" s="7"/>
+      <c r="B37" s="6"/>
+      <c r="C37" s="6"/>
+      <c r="D37" s="6"/>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="8" t="s">
+      <c r="A38" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="B38" s="8" t="s">
+      <c r="B38" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="C38" s="8" t="s">
+      <c r="C38" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="D38" s="8" t="s">
+      <c r="D38" s="7" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="4" t="s">
+      <c r="A39" s="3" t="s">
         <v>125</v>
       </c>
-      <c r="B39" s="9" t="n">
+      <c r="B39" s="8" t="n">
         <v>2183088.49</v>
       </c>
-      <c r="C39" s="10" t="s">
+      <c r="C39" s="9" t="s">
         <v>112</v>
       </c>
-      <c r="D39" s="12"/>
+      <c r="D39" s="11"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="4" t="s">
+      <c r="A40" s="3" t="s">
         <v>126</v>
       </c>
-      <c r="B40" s="9" t="n">
+      <c r="B40" s="8" t="n">
         <v>1157519.11</v>
       </c>
-      <c r="C40" s="10" t="s">
+      <c r="C40" s="9" t="s">
         <v>112</v>
       </c>
-      <c r="D40" s="10" t="s">
+      <c r="D40" s="9" t="s">
         <v>127</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A41" s="4" t="s">
+      <c r="A41" s="3" t="s">
         <v>128</v>
       </c>
-      <c r="B41" s="9" t="n">
+      <c r="B41" s="8" t="n">
         <v>538013.75</v>
       </c>
-      <c r="C41" s="10" t="s">
+      <c r="C41" s="9" t="s">
         <v>112</v>
       </c>
-      <c r="D41" s="12"/>
+      <c r="D41" s="11"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="4" t="s">
+      <c r="A42" s="3" t="s">
         <v>129</v>
       </c>
-      <c r="B42" s="9" t="n">
+      <c r="B42" s="8" t="n">
         <v>139351.5</v>
       </c>
-      <c r="C42" s="10" t="s">
+      <c r="C42" s="9" t="s">
         <v>112</v>
       </c>
-      <c r="D42" s="12"/>
+      <c r="D42" s="11"/>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A43" s="4" t="s">
+      <c r="A43" s="3" t="s">
         <v>130</v>
       </c>
-      <c r="B43" s="9" t="n">
+      <c r="B43" s="8" t="n">
         <v>199375</v>
       </c>
-      <c r="C43" s="10" t="s">
+      <c r="C43" s="9" t="s">
         <v>112</v>
       </c>
-      <c r="D43" s="10" t="s">
+      <c r="D43" s="9" t="s">
         <v>131</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="14" t="s">
+      <c r="A44" s="13" t="s">
         <v>84</v>
       </c>
-      <c r="B44" s="15" t="n">
+      <c r="B44" s="14" t="n">
         <f aca="false">SUM(B39:B43)</f>
         <v>4217347.85</v>
       </c>
-      <c r="C44" s="16" t="s">
-        <v>36</v>
-      </c>
-      <c r="D44" s="17"/>
+      <c r="C44" s="15" t="s">
+        <v>36</v>
+      </c>
+      <c r="D44" s="16"/>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A45" s="4" t="s">
+      <c r="A45" s="3" t="s">
         <v>132</v>
       </c>
-      <c r="B45" s="13" t="n">
+      <c r="B45" s="12" t="n">
         <f aca="false">B39/B44</f>
         <v>0.517644872475957</v>
       </c>
-      <c r="C45" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="D45" s="12"/>
+      <c r="C45" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="D45" s="11"/>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A46" s="4" t="s">
+      <c r="A46" s="3" t="s">
         <v>133</v>
       </c>
-      <c r="B46" s="13" t="n">
+      <c r="B46" s="12" t="n">
         <f aca="false">B40/B44</f>
         <v>0.274466122115111</v>
       </c>
-      <c r="C46" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="D46" s="12"/>
+      <c r="C46" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="D46" s="11"/>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A47" s="4" t="s">
+      <c r="A47" s="3" t="s">
         <v>134</v>
       </c>
-      <c r="B47" s="13" t="n">
+      <c r="B47" s="12" t="n">
         <f aca="false">B41/B44</f>
         <v>0.127571585066193</v>
       </c>
-      <c r="C47" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="D47" s="12"/>
+      <c r="C47" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="D47" s="11"/>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A48" s="4" t="s">
+      <c r="A48" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="B48" s="13" t="n">
+      <c r="B48" s="12" t="n">
         <f aca="false">B42/B44</f>
         <v>0.0330424487038697</v>
       </c>
-      <c r="C48" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="D48" s="12"/>
+      <c r="C48" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="D48" s="11"/>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A49" s="4" t="s">
+      <c r="A49" s="3" t="s">
         <v>135</v>
       </c>
-      <c r="B49" s="13" t="n">
+      <c r="B49" s="12" t="n">
         <f aca="false">B43/B44</f>
         <v>0.0472749716388701</v>
       </c>
-      <c r="C49" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="D49" s="12"/>
+      <c r="C49" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="D49" s="11"/>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A51" s="3" t="s">
+      <c r="A51" s="2" t="s">
         <v>136</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A52" s="4" t="s">
+      <c r="A52" s="3" t="s">
         <v>137</v>
       </c>
-      <c r="B52" s="9" t="n">
+      <c r="B52" s="8" t="n">
         <v>356040</v>
       </c>
-      <c r="C52" s="10" t="s">
+      <c r="C52" s="9" t="s">
         <v>138</v>
       </c>
-      <c r="D52" s="12"/>
+      <c r="D52" s="11"/>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A53" s="4" t="s">
+      <c r="A53" s="3" t="s">
         <v>139</v>
       </c>
-      <c r="B53" s="9" t="n">
+      <c r="B53" s="8" t="n">
         <v>125804.4</v>
       </c>
-      <c r="C53" s="10" t="s">
+      <c r="C53" s="9" t="s">
         <v>138</v>
       </c>
-      <c r="D53" s="12"/>
+      <c r="D53" s="11"/>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A54" s="4" t="s">
+      <c r="A54" s="3" t="s">
         <v>140</v>
       </c>
-      <c r="B54" s="9" t="n">
+      <c r="B54" s="8" t="n">
         <v>56169.35</v>
       </c>
-      <c r="C54" s="10" t="s">
+      <c r="C54" s="9" t="s">
         <v>138</v>
       </c>
-      <c r="D54" s="12"/>
+      <c r="D54" s="11"/>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A55" s="4" t="s">
+      <c r="A55" s="3" t="s">
         <v>141</v>
       </c>
-      <c r="B55" s="13" t="n">
+      <c r="B55" s="12" t="n">
         <f aca="false">B52/B41</f>
         <v>0.661767473414945</v>
       </c>
-      <c r="C55" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="D55" s="12"/>
+      <c r="C55" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="D55" s="11"/>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A56" s="4" t="s">
+      <c r="A56" s="3" t="s">
         <v>142</v>
       </c>
-      <c r="B56" s="13" t="n">
+      <c r="B56" s="12" t="n">
         <f aca="false">B53/B41</f>
         <v>0.233831198552082</v>
       </c>
-      <c r="C56" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="D56" s="12"/>
+      <c r="C56" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="D56" s="11"/>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A57" s="4" t="s">
+      <c r="A57" s="3" t="s">
         <v>143</v>
       </c>
-      <c r="B57" s="13" t="n">
+      <c r="B57" s="12" t="n">
         <f aca="false">B54/B41</f>
         <v>0.104401328032973</v>
       </c>
-      <c r="C57" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="D57" s="12"/>
+      <c r="C57" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="D57" s="11"/>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A58" s="4" t="s">
+      <c r="A58" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="B58" s="5" t="s">
+      <c r="B58" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="C58" s="10" t="s">
+      <c r="C58" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="D58" s="10" t="s">
+      <c r="D58" s="9" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A60" s="6" t="s">
+      <c r="A60" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="B60" s="7"/>
-      <c r="C60" s="7"/>
-      <c r="D60" s="7"/>
+      <c r="B60" s="6"/>
+      <c r="C60" s="6"/>
+      <c r="D60" s="6"/>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A61" s="8" t="s">
+      <c r="A61" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="B61" s="8" t="s">
+      <c r="B61" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="C61" s="8" t="s">
+      <c r="C61" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="D61" s="8" t="s">
+      <c r="D61" s="7" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A62" s="4" t="s">
+      <c r="A62" s="3" t="s">
         <v>145</v>
       </c>
-      <c r="B62" s="5" t="s">
+      <c r="B62" s="4" t="s">
         <v>146</v>
       </c>
-      <c r="C62" s="10" t="s">
+      <c r="C62" s="9" t="s">
         <v>147</v>
       </c>
-      <c r="D62" s="10" t="s">
+      <c r="D62" s="9" t="s">
         <v>148</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A63" s="4" t="s">
+      <c r="A63" s="3" t="s">
         <v>149</v>
       </c>
-      <c r="B63" s="18" t="n">
+      <c r="B63" s="17" t="n">
         <f aca="true">DATE(2026,9,29)-TODAY()</f>
         <v>47</v>
       </c>
-      <c r="C63" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="D63" s="12"/>
+      <c r="C63" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="D63" s="11"/>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A64" s="4" t="s">
+      <c r="A64" s="3" t="s">
         <v>150</v>
       </c>
-      <c r="B64" s="5" t="s">
+      <c r="B64" s="4" t="s">
         <v>151</v>
       </c>
-      <c r="C64" s="10" t="s">
+      <c r="C64" s="9" t="s">
         <v>147</v>
       </c>
-      <c r="D64" s="10" t="s">
+      <c r="D64" s="9" t="s">
         <v>152</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A65" s="4" t="s">
+      <c r="A65" s="3" t="s">
         <v>149</v>
       </c>
-      <c r="B65" s="18" t="n">
+      <c r="B65" s="17" t="n">
         <f aca="true">DATE(2026,8,26)-TODAY()</f>
         <v>13</v>
       </c>
-      <c r="C65" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="D65" s="10" t="s">
+      <c r="C65" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="D65" s="9" t="s">
         <v>153</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A67" s="4" t="s">
+      <c r="A67" s="3" t="s">
         <v>96</v>
       </c>
-      <c r="B67" s="5" t="s">
+      <c r="B67" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="C67" s="10" t="s">
+      <c r="C67" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="D67" s="10" t="s">
+      <c r="D67" s="9" t="s">
         <v>154</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A69" s="6" t="s">
+      <c r="A69" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="B69" s="7"/>
-      <c r="C69" s="7"/>
-      <c r="D69" s="7"/>
+      <c r="B69" s="6"/>
+      <c r="C69" s="6"/>
+      <c r="D69" s="6"/>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A70" s="8" t="s">
+      <c r="A70" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="B70" s="8" t="s">
+      <c r="B70" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="C70" s="8" t="s">
+      <c r="C70" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="D70" s="8" t="s">
+      <c r="D70" s="7" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A71" s="4" t="s">
+      <c r="A71" s="3" t="s">
         <v>155</v>
       </c>
-      <c r="B71" s="9" t="n">
+      <c r="B71" s="8" t="n">
         <v>1157519.11</v>
       </c>
-      <c r="C71" s="10" t="s">
+      <c r="C71" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="D71" s="10" t="s">
+      <c r="D71" s="9" t="s">
         <v>156</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A72" s="4" t="s">
+      <c r="A72" s="3" t="s">
         <v>100</v>
       </c>
-      <c r="B72" s="9" t="n">
+      <c r="B72" s="8" t="n">
         <v>-162000</v>
       </c>
-      <c r="C72" s="10" t="s">
+      <c r="C72" s="9" t="s">
         <v>157</v>
       </c>
-      <c r="D72" s="10" t="s">
+      <c r="D72" s="9" t="s">
         <v>158</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A73" s="4" t="s">
+      <c r="A73" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="B73" s="5" t="s">
+      <c r="B73" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="C73" s="10" t="s">
+      <c r="C73" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="D73" s="10" t="s">
+      <c r="D73" s="9" t="s">
         <v>159</v>
       </c>
     </row>
@@ -3242,596 +3343,178 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:E35"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:E21"/>
+  <sheetFormatPr defaultColWidth="8.66796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="2" style="0" width="16"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="19" t="s">
+      <c r="A1" s="18" t="s">
         <v>160</v>
       </c>
-      <c r="B1" s="19"/>
-      <c r="C1" s="19"/>
-      <c r="D1" s="19"/>
-      <c r="E1" s="19"/>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="20" t="s">
+      <c r="B1" s="18"/>
+      <c r="C1" s="18"/>
+      <c r="D1" s="18"/>
+      <c r="E1" s="18"/>
+    </row>
+    <row r="2" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="19" t="s">
         <v>161</v>
       </c>
-      <c r="B2" s="20"/>
-      <c r="C2" s="20"/>
-      <c r="D2" s="20"/>
-      <c r="E2" s="20"/>
+      <c r="B2" s="19"/>
+      <c r="C2" s="19"/>
+      <c r="D2" s="19"/>
+      <c r="E2" s="19"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="21" t="s">
+      <c r="A4" s="20" t="s">
         <v>162</v>
       </c>
-      <c r="B4" s="21"/>
-      <c r="C4" s="21"/>
-      <c r="D4" s="21"/>
-      <c r="E4" s="21"/>
+      <c r="B4" s="20"/>
+      <c r="C4" s="20"/>
+      <c r="D4" s="20"/>
+      <c r="E4" s="20"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="22" t="s">
+      <c r="A5" s="21" t="s">
+        <v>26</v>
+      </c>
+      <c r="B5" s="21" t="s">
+        <v>27</v>
+      </c>
+      <c r="C5" s="21" t="s">
+        <v>28</v>
+      </c>
+      <c r="D5" s="21" t="s">
+        <v>29</v>
+      </c>
+      <c r="E5" s="21"/>
+    </row>
+    <row r="6" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="22" t="s">
         <v>163</v>
       </c>
-      <c r="B5" s="22" t="s">
+      <c r="B6" s="23" t="n">
+        <v>0.07</v>
+      </c>
+      <c r="C6" s="24" t="s">
+        <v>31</v>
+      </c>
+      <c r="D6" s="25" t="s">
         <v>164</v>
       </c>
-      <c r="C5" s="22" t="s">
+      <c r="E6" s="25"/>
+    </row>
+    <row r="7" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="22" t="s">
+        <v>165</v>
+      </c>
+      <c r="B7" s="23" t="n">
+        <v>0.094</v>
+      </c>
+      <c r="C7" s="24" t="s">
+        <v>31</v>
+      </c>
+      <c r="D7" s="25" t="s">
+        <v>166</v>
+      </c>
+      <c r="E7" s="25"/>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="20" t="s">
+        <v>167</v>
+      </c>
+      <c r="B9" s="20"/>
+      <c r="C9" s="20"/>
+      <c r="D9" s="20"/>
+      <c r="E9" s="20"/>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="21" t="s">
+        <v>26</v>
+      </c>
+      <c r="B10" s="21" t="s">
         <v>27</v>
       </c>
-      <c r="D5" s="22" t="s">
-        <v>165</v>
-      </c>
-      <c r="E5" s="22" t="s">
+      <c r="C10" s="21" t="s">
+        <v>28</v>
+      </c>
+      <c r="D10" s="21" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="23" t="s">
-        <v>166</v>
-      </c>
-      <c r="B6" s="24" t="str">
-        <f aca="false">AMS!A41</f>
-        <v>Fondo Monetario</v>
-      </c>
-      <c r="C6" s="25" t="n">
-        <f aca="false">AMS!B41</f>
-        <v>89230.77</v>
-      </c>
-      <c r="D6" s="26" t="s">
-        <v>167</v>
-      </c>
-      <c r="E6" s="27"/>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="23"/>
-      <c r="B7" s="24" t="str">
-        <f aca="false">AMS!A44</f>
-        <v>Liquidez (excluido FM)</v>
-      </c>
-      <c r="C7" s="25" t="n">
-        <f aca="false">AMS!B44</f>
-        <v>83100</v>
-      </c>
-      <c r="D7" s="26" t="s">
+      <c r="E10" s="21"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="26" t="s">
         <v>168</v>
       </c>
-      <c r="E7" s="27"/>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="28"/>
-      <c r="B8" s="29" t="s">
-        <v>169</v>
-      </c>
-      <c r="C8" s="30" t="n">
-        <f aca="false">SUM(C6:C7)</f>
-        <v>172330.77</v>
-      </c>
-      <c r="D8" s="28"/>
-      <c r="E8" s="28"/>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="31" t="s">
-        <v>170</v>
-      </c>
-      <c r="B9" s="32" t="str">
-        <f aca="false">AMS!A40</f>
-        <v>SP500 (fondos indexados)</v>
-      </c>
-      <c r="C9" s="33" t="n">
-        <f aca="false">AMS!B40</f>
-        <v>872837.88</v>
-      </c>
-      <c r="D9" s="34" t="s">
-        <v>171</v>
-      </c>
-      <c r="E9" s="35"/>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="36"/>
-      <c r="B10" s="37" t="s">
-        <v>172</v>
-      </c>
-      <c r="C10" s="38" t="n">
-        <f aca="false">C9</f>
-        <v>872837.88</v>
-      </c>
-      <c r="D10" s="36"/>
-      <c r="E10" s="36"/>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="39" t="s">
-        <v>173</v>
-      </c>
-      <c r="B11" s="40" t="str">
-        <f aca="false">AMS!A42</f>
-        <v>ETF</v>
-      </c>
-      <c r="C11" s="41" t="n">
-        <f aca="false">AMS!B42</f>
-        <v>111570.37</v>
-      </c>
-      <c r="D11" s="42" t="s">
-        <v>174</v>
-      </c>
-      <c r="E11" s="43"/>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="39"/>
-      <c r="B12" s="40" t="str">
-        <f aca="false">AMS!A43</f>
-        <v>Pisos</v>
-      </c>
-      <c r="C12" s="41" t="n">
-        <f aca="false">AMS!B43</f>
-        <v>100000</v>
-      </c>
-      <c r="D12" s="42" t="s">
-        <v>175</v>
-      </c>
-      <c r="E12" s="43"/>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="44"/>
-      <c r="B13" s="45" t="s">
-        <v>176</v>
-      </c>
-      <c r="C13" s="46" t="n">
-        <f aca="false">SUM(C11:C12)</f>
-        <v>211570.37</v>
-      </c>
-      <c r="D13" s="44"/>
-      <c r="E13" s="44"/>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="47" t="s">
-        <v>177</v>
-      </c>
-      <c r="B15" s="47"/>
-      <c r="C15" s="48" t="n">
-        <f aca="false">C8+C10+C13</f>
-        <v>1256739.02</v>
-      </c>
-      <c r="D15" s="49"/>
-      <c r="E15" s="49"/>
-    </row>
-    <row r="16" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B16" s="50" t="s">
-        <v>178</v>
-      </c>
-      <c r="C16" s="51" t="n">
-        <f aca="false">C15-AMS!B45</f>
-        <v>0</v>
-      </c>
-      <c r="E16" s="52" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="21" t="s">
-        <v>180</v>
-      </c>
-      <c r="B19" s="21"/>
-      <c r="C19" s="21"/>
-      <c r="D19" s="21"/>
-      <c r="E19" s="21"/>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="22" t="s">
-        <v>163</v>
-      </c>
-      <c r="B20" s="22" t="s">
-        <v>164</v>
-      </c>
-      <c r="C20" s="22" t="s">
-        <v>27</v>
-      </c>
-      <c r="D20" s="22" t="s">
-        <v>165</v>
-      </c>
-      <c r="E20" s="22" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="23" t="s">
-        <v>166</v>
-      </c>
-      <c r="B21" s="24" t="str">
-        <f aca="false">AML!A43</f>
-        <v>Liquidez + Depósitos (excluido FM)</v>
-      </c>
-      <c r="C21" s="25" t="n">
-        <f aca="false">AML!B43</f>
-        <v>199375</v>
-      </c>
-      <c r="D21" s="26" t="s">
-        <v>181</v>
-      </c>
-      <c r="E21" s="27"/>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="28"/>
-      <c r="B22" s="29" t="s">
-        <v>169</v>
-      </c>
-      <c r="C22" s="30" t="n">
-        <f aca="false">C21</f>
-        <v>199375</v>
-      </c>
-      <c r="D22" s="28"/>
-      <c r="E22" s="28"/>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="31" t="s">
-        <v>170</v>
-      </c>
-      <c r="B23" s="32" t="str">
-        <f aca="false">AML!A39</f>
-        <v>Fondos RV</v>
-      </c>
-      <c r="C23" s="33" t="n">
-        <f aca="false">AML!B39</f>
-        <v>2183088.49</v>
-      </c>
-      <c r="D23" s="34" t="s">
-        <v>182</v>
-      </c>
-      <c r="E23" s="35"/>
-    </row>
-    <row r="24" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="31"/>
-      <c r="B24" s="32" t="str">
-        <f aca="false">AML!A40</f>
-        <v>Planes de Pensiones (Papá 754.162,54 + Mamá 403.356,58)</v>
-      </c>
-      <c r="C24" s="33" t="n">
-        <f aca="false">AML!B40</f>
-        <v>1157519.11</v>
-      </c>
-      <c r="D24" s="34" t="s">
-        <v>183</v>
-      </c>
-      <c r="E24" s="53" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="36"/>
-      <c r="B25" s="37" t="s">
-        <v>172</v>
-      </c>
-      <c r="C25" s="38" t="n">
-        <f aca="false">SUM(C23:C24)</f>
-        <v>3340607.6</v>
-      </c>
-      <c r="D25" s="36"/>
-      <c r="E25" s="36"/>
-    </row>
-    <row r="26" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="39" t="s">
-        <v>173</v>
-      </c>
-      <c r="B26" s="40" t="str">
-        <f aca="false">AML!A41</f>
-        <v>Acciones (Iberdrola 356.040 + BBVA 125.804,4 + TEF 56.169,35)</v>
-      </c>
-      <c r="C26" s="41" t="n">
-        <f aca="false">AML!B41</f>
-        <v>538013.75</v>
-      </c>
-      <c r="D26" s="42" t="s">
-        <v>185</v>
-      </c>
-      <c r="E26" s="54" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="39"/>
-      <c r="B27" s="40" t="str">
-        <f aca="false">AML!A42</f>
-        <v>ETF (Aristócratas)</v>
-      </c>
-      <c r="C27" s="41" t="n">
-        <f aca="false">AML!B42</f>
-        <v>139351.5</v>
-      </c>
-      <c r="D27" s="42" t="s">
-        <v>187</v>
-      </c>
-      <c r="E27" s="43"/>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="44"/>
-      <c r="B28" s="45" t="s">
-        <v>176</v>
-      </c>
-      <c r="C28" s="46" t="n">
-        <f aca="false">SUM(C26:C27)</f>
-        <v>677365.25</v>
-      </c>
-      <c r="D28" s="44"/>
-      <c r="E28" s="44"/>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="47" t="s">
-        <v>188</v>
-      </c>
-      <c r="B30" s="47"/>
-      <c r="C30" s="48" t="n">
-        <f aca="false">C22+C25+C28</f>
-        <v>4217347.85</v>
-      </c>
-      <c r="D30" s="49"/>
-      <c r="E30" s="49"/>
-    </row>
-    <row r="31" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B31" s="50" t="s">
-        <v>178</v>
-      </c>
-      <c r="C31" s="51" t="n">
-        <f aca="false">C30-AML!B44</f>
-        <v>0</v>
-      </c>
-      <c r="E31" s="52" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="55" t="s">
-        <v>189</v>
-      </c>
-      <c r="B33" s="55"/>
-      <c r="C33" s="55"/>
-      <c r="D33" s="55"/>
-      <c r="E33" s="55"/>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="55"/>
-      <c r="B34" s="55"/>
-      <c r="C34" s="55"/>
-      <c r="D34" s="55"/>
-      <c r="E34" s="55"/>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="55"/>
-      <c r="B35" s="55"/>
-      <c r="C35" s="55"/>
-      <c r="D35" s="55"/>
-      <c r="E35" s="55"/>
-    </row>
-  </sheetData>
-  <mergeCells count="11">
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="A6:A7"/>
-    <mergeCell ref="A11:A12"/>
-    <mergeCell ref="A15:B15"/>
-    <mergeCell ref="A19:E19"/>
-    <mergeCell ref="A23:A24"/>
-    <mergeCell ref="A26:A27"/>
-    <mergeCell ref="A30:B30"/>
-    <mergeCell ref="A33:E35"/>
-  </mergeCells>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="true"/>
-  </sheetPr>
-  <dimension ref="A1:E21"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
-  <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="2" style="1" width="16"/>
-  </cols>
-  <sheetData>
-    <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="19" t="s">
-        <v>190</v>
-      </c>
-      <c r="B1" s="19"/>
-      <c r="C1" s="19"/>
-      <c r="D1" s="19"/>
-      <c r="E1" s="19"/>
-    </row>
-    <row r="2" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="20" t="s">
-        <v>191</v>
-      </c>
-      <c r="B2" s="20"/>
-      <c r="C2" s="20"/>
-      <c r="D2" s="20"/>
-      <c r="E2" s="20"/>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="21" t="s">
-        <v>192</v>
-      </c>
-      <c r="B4" s="21"/>
-      <c r="C4" s="21"/>
-      <c r="D4" s="21"/>
-      <c r="E4" s="21"/>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="22" t="s">
-        <v>26</v>
-      </c>
-      <c r="B5" s="22" t="s">
-        <v>27</v>
-      </c>
-      <c r="C5" s="22" t="s">
-        <v>28</v>
-      </c>
-      <c r="D5" s="22" t="s">
-        <v>29</v>
-      </c>
-      <c r="E5" s="22"/>
-    </row>
-    <row r="6" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="56" t="s">
-        <v>193</v>
-      </c>
-      <c r="B6" s="57" t="n">
-        <v>0.07</v>
-      </c>
-      <c r="C6" s="58" t="s">
-        <v>31</v>
-      </c>
-      <c r="D6" s="59" t="s">
-        <v>194</v>
-      </c>
-      <c r="E6" s="59"/>
-    </row>
-    <row r="7" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="56" t="s">
-        <v>195</v>
-      </c>
-      <c r="B7" s="57" t="n">
-        <v>0.094</v>
-      </c>
-      <c r="C7" s="58" t="s">
-        <v>31</v>
-      </c>
-      <c r="D7" s="59" t="s">
-        <v>196</v>
-      </c>
-      <c r="E7" s="59"/>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="21" t="s">
-        <v>197</v>
-      </c>
-      <c r="B9" s="21"/>
-      <c r="C9" s="21"/>
-      <c r="D9" s="21"/>
-      <c r="E9" s="21"/>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="22" t="s">
-        <v>26</v>
-      </c>
-      <c r="B10" s="22" t="s">
-        <v>27</v>
-      </c>
-      <c r="C10" s="22" t="s">
-        <v>28</v>
-      </c>
-      <c r="D10" s="22" t="s">
-        <v>29</v>
-      </c>
-      <c r="E10" s="22"/>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="60" t="s">
-        <v>198</v>
-      </c>
-      <c r="B11" s="61" t="n">
+      <c r="B11" s="27" t="n">
         <f aca="false">Cajas!C10</f>
         <v>872837.88</v>
       </c>
-      <c r="C11" s="34" t="s">
-        <v>199</v>
-      </c>
-      <c r="D11" s="35"/>
-      <c r="E11" s="35"/>
+      <c r="C11" s="28" t="s">
+        <v>169</v>
+      </c>
+      <c r="D11" s="29"/>
+      <c r="E11" s="29"/>
     </row>
     <row r="12" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="60" t="s">
-        <v>200</v>
-      </c>
-      <c r="B12" s="61" t="n">
+      <c r="A12" s="26" t="s">
+        <v>170</v>
+      </c>
+      <c r="B12" s="27" t="n">
         <f aca="false">Cajas!C25</f>
         <v>3340607.6</v>
       </c>
-      <c r="C12" s="34" t="s">
-        <v>201</v>
-      </c>
-      <c r="D12" s="53" t="s">
-        <v>202</v>
-      </c>
-      <c r="E12" s="53"/>
+      <c r="C12" s="28" t="s">
+        <v>171</v>
+      </c>
+      <c r="D12" s="30" t="s">
+        <v>172</v>
+      </c>
+      <c r="E12" s="30"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="21" t="s">
-        <v>203</v>
-      </c>
-      <c r="B14" s="21"/>
-      <c r="C14" s="21"/>
-      <c r="D14" s="21"/>
-      <c r="E14" s="21"/>
+      <c r="A14" s="20" t="s">
+        <v>173</v>
+      </c>
+      <c r="B14" s="20"/>
+      <c r="C14" s="20"/>
+      <c r="D14" s="20"/>
+      <c r="E14" s="20"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="22" t="s">
-        <v>204</v>
-      </c>
-      <c r="B15" s="22" t="s">
-        <v>205</v>
-      </c>
-      <c r="C15" s="62" t="s">
-        <v>206</v>
-      </c>
-      <c r="D15" s="63" t="s">
-        <v>207</v>
-      </c>
-      <c r="E15" s="22" t="s">
-        <v>208</v>
+      <c r="A15" s="21" t="s">
+        <v>174</v>
+      </c>
+      <c r="B15" s="21" t="s">
+        <v>175</v>
+      </c>
+      <c r="C15" s="31" t="s">
+        <v>176</v>
+      </c>
+      <c r="D15" s="32" t="s">
+        <v>177</v>
+      </c>
+      <c r="E15" s="21" t="s">
+        <v>178</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="60" t="s">
-        <v>209</v>
+      <c r="A16" s="26" t="s">
+        <v>179</v>
       </c>
       <c r="B16" s="33" t="n">
         <f aca="false">$B$11*(1+$B$6)^5</f>
         <v>1224200.27921452</v>
       </c>
-      <c r="C16" s="64" t="n">
+      <c r="C16" s="34" t="n">
         <f aca="false">$B$11*(1+$B$7)^5</f>
         <v>1367792.42987986</v>
       </c>
-      <c r="D16" s="65" t="n">
+      <c r="D16" s="35" t="n">
         <f aca="false">$B$12*(1+$B$6)^5</f>
         <v>4685374.97096958</v>
       </c>
@@ -3841,18 +3524,18 @@
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="60" t="s">
-        <v>210</v>
+      <c r="A17" s="26" t="s">
+        <v>180</v>
       </c>
       <c r="B17" s="33" t="n">
         <f aca="false">$B$11*(1+$B$6)^10</f>
         <v>1717004.22033575</v>
       </c>
-      <c r="C17" s="64" t="n">
+      <c r="C17" s="34" t="n">
         <f aca="false">$B$11*(1+$B$7)^10</f>
         <v>2143417.6656456</v>
       </c>
-      <c r="D17" s="65" t="n">
+      <c r="D17" s="35" t="n">
         <f aca="false">$B$12*(1+$B$6)^10</f>
         <v>6571480.77451184</v>
       </c>
@@ -3862,18 +3545,18 @@
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="60" t="s">
-        <v>211</v>
+      <c r="A18" s="26" t="s">
+        <v>181</v>
       </c>
       <c r="B18" s="33" t="n">
         <f aca="false">$B$11*(1+$B$6)^15</f>
         <v>2408187.24085111</v>
       </c>
-      <c r="C18" s="64" t="n">
+      <c r="C18" s="34" t="n">
         <f aca="false">$B$11*(1+$B$7)^15</f>
         <v>3358871.70380461</v>
       </c>
-      <c r="D18" s="65" t="n">
+      <c r="D18" s="35" t="n">
         <f aca="false">$B$12*(1+$B$6)^15</f>
         <v>9216841.73355336</v>
       </c>
@@ -3883,20 +3566,20 @@
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="55" t="s">
-        <v>212</v>
-      </c>
-      <c r="B20" s="55"/>
-      <c r="C20" s="55"/>
-      <c r="D20" s="55"/>
-      <c r="E20" s="55"/>
+      <c r="A20" s="36" t="s">
+        <v>182</v>
+      </c>
+      <c r="B20" s="36"/>
+      <c r="C20" s="36"/>
+      <c r="D20" s="36"/>
+      <c r="E20" s="36"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="55"/>
-      <c r="B21" s="55"/>
-      <c r="C21" s="55"/>
-      <c r="D21" s="55"/>
-      <c r="E21" s="55"/>
+      <c r="A21" s="36"/>
+      <c r="B21" s="36"/>
+      <c r="C21" s="36"/>
+      <c r="D21" s="36"/>
+      <c r="E21" s="36"/>
     </row>
   </sheetData>
   <mergeCells count="12">
@@ -3921,4 +3604,477 @@
     <oddFooter/>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="true"/>
+  </sheetPr>
+  <dimension ref="A1:F35"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="50"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="37" t="s">
+        <v>183</v>
+      </c>
+      <c r="B1" s="37"/>
+      <c r="C1" s="37"/>
+      <c r="D1" s="37"/>
+      <c r="E1" s="37"/>
+      <c r="F1" s="37"/>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="38" t="s">
+        <v>184</v>
+      </c>
+      <c r="B2" s="38"/>
+      <c r="C2" s="38"/>
+      <c r="D2" s="38"/>
+      <c r="E2" s="38"/>
+      <c r="F2" s="38"/>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="39" t="s">
+        <v>185</v>
+      </c>
+      <c r="B4" s="39"/>
+      <c r="C4" s="39"/>
+      <c r="D4" s="39"/>
+      <c r="E4" s="39"/>
+      <c r="F4" s="39"/>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="40" t="s">
+        <v>186</v>
+      </c>
+      <c r="B5" s="40" t="s">
+        <v>187</v>
+      </c>
+      <c r="C5" s="40" t="s">
+        <v>27</v>
+      </c>
+      <c r="D5" s="40" t="s">
+        <v>188</v>
+      </c>
+      <c r="E5" s="40" t="s">
+        <v>189</v>
+      </c>
+      <c r="F5" s="40" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="41" t="s">
+        <v>190</v>
+      </c>
+      <c r="B6" s="42" t="str">
+        <f aca="false">AMS!A41</f>
+        <v>Fondo Monetario</v>
+      </c>
+      <c r="C6" s="43" t="n">
+        <f aca="false">AMS!B41</f>
+        <v>89230.77</v>
+      </c>
+      <c r="D6" s="44"/>
+      <c r="E6" s="45" t="s">
+        <v>191</v>
+      </c>
+      <c r="F6" s="44"/>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="41"/>
+      <c r="B7" s="42" t="str">
+        <f aca="false">AMS!A44</f>
+        <v>Liquidez (excluido FM)</v>
+      </c>
+      <c r="C7" s="43" t="n">
+        <f aca="false">AMS!B44</f>
+        <v>83100</v>
+      </c>
+      <c r="D7" s="44"/>
+      <c r="E7" s="45" t="s">
+        <v>192</v>
+      </c>
+      <c r="F7" s="44"/>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="46"/>
+      <c r="B8" s="47" t="s">
+        <v>193</v>
+      </c>
+      <c r="C8" s="48" t="n">
+        <f aca="false">SUM(C6:C7)</f>
+        <v>172330.77</v>
+      </c>
+      <c r="D8" s="49" t="n">
+        <f aca="false">C8/C$15</f>
+        <v>0.137125343653291</v>
+      </c>
+      <c r="E8" s="46"/>
+      <c r="F8" s="46"/>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="50" t="s">
+        <v>194</v>
+      </c>
+      <c r="B9" s="51" t="str">
+        <f aca="false">AMS!A40</f>
+        <v>SP500 (fondos indexados)</v>
+      </c>
+      <c r="C9" s="52" t="n">
+        <f aca="false">AMS!B40</f>
+        <v>872837.88</v>
+      </c>
+      <c r="D9" s="29"/>
+      <c r="E9" s="53" t="s">
+        <v>195</v>
+      </c>
+      <c r="F9" s="29"/>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="54"/>
+      <c r="B10" s="55" t="s">
+        <v>196</v>
+      </c>
+      <c r="C10" s="56" t="n">
+        <f aca="false">C9</f>
+        <v>872837.88</v>
+      </c>
+      <c r="D10" s="57" t="n">
+        <f aca="false">C10/C$15</f>
+        <v>0.694525964507731</v>
+      </c>
+      <c r="E10" s="54"/>
+      <c r="F10" s="54"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="58" t="s">
+        <v>197</v>
+      </c>
+      <c r="B11" s="59" t="str">
+        <f aca="false">AMS!A42</f>
+        <v>ETF</v>
+      </c>
+      <c r="C11" s="60" t="n">
+        <f aca="false">AMS!B42</f>
+        <v>111570.37</v>
+      </c>
+      <c r="D11" s="61"/>
+      <c r="E11" s="62" t="s">
+        <v>198</v>
+      </c>
+      <c r="F11" s="61"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="58"/>
+      <c r="B12" s="59" t="str">
+        <f aca="false">AMS!A43</f>
+        <v>Pisos</v>
+      </c>
+      <c r="C12" s="60" t="n">
+        <f aca="false">AMS!B43</f>
+        <v>100000</v>
+      </c>
+      <c r="D12" s="61"/>
+      <c r="E12" s="62" t="s">
+        <v>199</v>
+      </c>
+      <c r="F12" s="61"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="63"/>
+      <c r="B13" s="64" t="s">
+        <v>200</v>
+      </c>
+      <c r="C13" s="65" t="n">
+        <f aca="false">SUM(C11:C12)</f>
+        <v>211570.37</v>
+      </c>
+      <c r="D13" s="66" t="n">
+        <f aca="false">C13/C$15</f>
+        <v>0.168348691838979</v>
+      </c>
+      <c r="E13" s="63"/>
+      <c r="F13" s="63"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="67" t="s">
+        <v>201</v>
+      </c>
+      <c r="B15" s="67"/>
+      <c r="C15" s="68" t="n">
+        <f aca="false">C8+C10+C13</f>
+        <v>1256739.02</v>
+      </c>
+      <c r="D15" s="69" t="n">
+        <f aca="false">C15/C15</f>
+        <v>1</v>
+      </c>
+      <c r="E15" s="70"/>
+      <c r="F15" s="70"/>
+    </row>
+    <row r="16" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B16" s="71" t="s">
+        <v>202</v>
+      </c>
+      <c r="C16" s="72" t="n">
+        <f aca="false">C15-AMS!B45</f>
+        <v>0</v>
+      </c>
+      <c r="F16" s="73" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="39" t="s">
+        <v>204</v>
+      </c>
+      <c r="B19" s="39"/>
+      <c r="C19" s="39"/>
+      <c r="D19" s="39"/>
+      <c r="E19" s="39"/>
+      <c r="F19" s="39"/>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="40" t="s">
+        <v>186</v>
+      </c>
+      <c r="B20" s="40" t="s">
+        <v>187</v>
+      </c>
+      <c r="C20" s="40" t="s">
+        <v>27</v>
+      </c>
+      <c r="D20" s="40" t="s">
+        <v>188</v>
+      </c>
+      <c r="E20" s="40" t="s">
+        <v>189</v>
+      </c>
+      <c r="F20" s="40" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="41" t="s">
+        <v>190</v>
+      </c>
+      <c r="B21" s="42" t="str">
+        <f aca="false">AML!A43</f>
+        <v>Liquidez + Depósitos (excluido FM)</v>
+      </c>
+      <c r="C21" s="43" t="n">
+        <f aca="false">AML!B43</f>
+        <v>199375</v>
+      </c>
+      <c r="D21" s="44"/>
+      <c r="E21" s="45" t="s">
+        <v>205</v>
+      </c>
+      <c r="F21" s="44"/>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="46"/>
+      <c r="B22" s="47" t="s">
+        <v>193</v>
+      </c>
+      <c r="C22" s="48" t="n">
+        <f aca="false">C21</f>
+        <v>199375</v>
+      </c>
+      <c r="D22" s="49" t="n">
+        <f aca="false">C22/C$30</f>
+        <v>0.0472749716388701</v>
+      </c>
+      <c r="E22" s="46"/>
+      <c r="F22" s="46"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="50" t="s">
+        <v>194</v>
+      </c>
+      <c r="B23" s="51" t="str">
+        <f aca="false">AML!A39</f>
+        <v>Fondos RV</v>
+      </c>
+      <c r="C23" s="52" t="n">
+        <f aca="false">AML!B39</f>
+        <v>2183088.49</v>
+      </c>
+      <c r="D23" s="29"/>
+      <c r="E23" s="53" t="s">
+        <v>206</v>
+      </c>
+      <c r="F23" s="29"/>
+    </row>
+    <row r="24" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="50"/>
+      <c r="B24" s="51" t="str">
+        <f aca="false">AML!A40</f>
+        <v>Planes de Pensiones (Papá 754.162,54 + Mamá 403.356,58)</v>
+      </c>
+      <c r="C24" s="52" t="n">
+        <f aca="false">AML!B40</f>
+        <v>1157519.11</v>
+      </c>
+      <c r="D24" s="29"/>
+      <c r="E24" s="53" t="s">
+        <v>207</v>
+      </c>
+      <c r="F24" s="74" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="54"/>
+      <c r="B25" s="55" t="s">
+        <v>196</v>
+      </c>
+      <c r="C25" s="56" t="n">
+        <f aca="false">SUM(C23:C24)</f>
+        <v>3340607.6</v>
+      </c>
+      <c r="D25" s="57" t="n">
+        <f aca="false">C25/C$30</f>
+        <v>0.792110994591068</v>
+      </c>
+      <c r="E25" s="54"/>
+      <c r="F25" s="54"/>
+    </row>
+    <row r="26" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="58" t="s">
+        <v>197</v>
+      </c>
+      <c r="B26" s="59" t="str">
+        <f aca="false">AML!A41</f>
+        <v>Acciones (Iberdrola 356.040 + BBVA 125.804,4 + TEF 56.169,35)</v>
+      </c>
+      <c r="C26" s="60" t="n">
+        <f aca="false">AML!B41</f>
+        <v>538013.75</v>
+      </c>
+      <c r="D26" s="61"/>
+      <c r="E26" s="62" t="s">
+        <v>209</v>
+      </c>
+      <c r="F26" s="75" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="58"/>
+      <c r="B27" s="59" t="str">
+        <f aca="false">AML!A42</f>
+        <v>ETF (Aristócratas)</v>
+      </c>
+      <c r="C27" s="60" t="n">
+        <f aca="false">AML!B42</f>
+        <v>139351.5</v>
+      </c>
+      <c r="D27" s="61"/>
+      <c r="E27" s="62" t="s">
+        <v>211</v>
+      </c>
+      <c r="F27" s="61"/>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="63"/>
+      <c r="B28" s="64" t="s">
+        <v>200</v>
+      </c>
+      <c r="C28" s="65" t="n">
+        <f aca="false">SUM(C26:C27)</f>
+        <v>677365.25</v>
+      </c>
+      <c r="D28" s="66" t="n">
+        <f aca="false">C28/C$30</f>
+        <v>0.160614033770062</v>
+      </c>
+      <c r="E28" s="63"/>
+      <c r="F28" s="63"/>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="67" t="s">
+        <v>212</v>
+      </c>
+      <c r="B30" s="67"/>
+      <c r="C30" s="68" t="n">
+        <f aca="false">C22+C25+C28</f>
+        <v>4217347.85</v>
+      </c>
+      <c r="D30" s="69" t="n">
+        <f aca="false">C30/C30</f>
+        <v>1</v>
+      </c>
+      <c r="E30" s="70"/>
+      <c r="F30" s="70"/>
+    </row>
+    <row r="31" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B31" s="71" t="s">
+        <v>202</v>
+      </c>
+      <c r="C31" s="72" t="n">
+        <f aca="false">C30-AML!B44</f>
+        <v>0</v>
+      </c>
+      <c r="F31" s="73" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="76" t="s">
+        <v>213</v>
+      </c>
+      <c r="B33" s="76"/>
+      <c r="C33" s="76"/>
+      <c r="D33" s="76"/>
+      <c r="E33" s="76"/>
+      <c r="F33" s="76"/>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="76"/>
+      <c r="B34" s="76"/>
+      <c r="C34" s="76"/>
+      <c r="D34" s="76"/>
+      <c r="E34" s="76"/>
+      <c r="F34" s="76"/>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="76"/>
+      <c r="B35" s="76"/>
+      <c r="C35" s="76"/>
+      <c r="D35" s="76"/>
+      <c r="E35" s="76"/>
+      <c r="F35" s="76"/>
+    </row>
+  </sheetData>
+  <mergeCells count="11">
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A4:F4"/>
+    <mergeCell ref="A6:A7"/>
+    <mergeCell ref="A11:A12"/>
+    <mergeCell ref="A15:B15"/>
+    <mergeCell ref="A19:F19"/>
+    <mergeCell ref="A23:A24"/>
+    <mergeCell ref="A26:A27"/>
+    <mergeCell ref="A30:B30"/>
+    <mergeCell ref="A33:F35"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Proyecciones: congelar fecha+importe de referencia, trayectoria fija, tabla de seguimiento. Actualizar cifras AMS/AML a hoy. CONSTITUTION v1.5
</commit_message>
<xml_diff>
--- a/data/raw/personal_capacity_facts.xlsx
+++ b/data/raw/personal_capacity_facts.xlsx
@@ -5,14 +5,14 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Notas" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="AMS" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="AML" sheetId="3" state="visible" r:id="rId5"/>
-    <sheet name="Proyecciones" sheetId="4" state="visible" r:id="rId6"/>
-    <sheet name="Cajas" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="Cajas" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="Proyecciones" sheetId="5" state="visible" r:id="rId7"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="415" uniqueCount="214">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="435" uniqueCount="229">
   <si>
     <t xml:space="preserve">PERSONAL CAPACITY FACTS — Notas de uso</t>
   </si>
@@ -506,12 +506,138 @@
     <t xml:space="preserve">Confirmado 2026-08-10 -- la exclusión de Planes de Pensiones y la minusvalía TEF de arriba son las únicas cuestiones fiscales conocidas; ninguna de las dos es una restricción activa</t>
   </si>
   <si>
+    <t xml:space="preserve">CLASIFICACIÓN EN LAS TRES CAJAS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nivel 3, CONSTITUTION.md Sección 2  ·  Seguridad · Motor · Rentas Pasivas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AMS — patrimonio propio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Caja</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Partida</t>
+  </si>
+  <si>
+    <t xml:space="preserve">% Total</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Origen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Seguridad</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AMS!B41</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AMS!B44</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Subtotal Seguridad</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Motor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AMS!B40</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Subtotal Motor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rentas Pasivas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AMS!B42</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AMS!B43</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Subtotal Rentas Pasivas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOTAL AMS (3 cajas)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Diferencia vs. total patrimonio (control)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Debe ser 0€. Si no lo es, hay una partida nueva en la sección 4 sin clasificar aquí.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AML — patrimonio de tus padres</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AML!B43</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AML!B39</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AML!B40</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bloqueado operativamente (ilíquido salvo jubilación/paro larga duración/enfermedad grave; destino: herencia). Clasificado en Motor por composición de activo, confirmado por Armando 2026-08-13.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AML!B41</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Función declarada de renta vía dividendos, no de crecimiento (ver AML!D58). Confirmado por Armando 2026-08-13.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AML!B42</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOTAL AML (3 cajas)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Colores: Seguridad (azul) · Motor (verde) · Rentas Pasivas (naranja). % Total = peso de cada caja sobre el patrimonio total de AMS o AML respectivamente. Clasificación fijada por Armando el 2026-08-13 sobre la tabla de cajas de CONSTITUTION.md Sección 2, Nivel 3 — Seguridad: liquidez/depósitos/monetarios · Motor: fondo indexado S&amp;P 500 y otras inversiones a largo plazo · Rentas Pasivas: JGPI, inmobiliario, oro.</t>
+  </si>
+  <si>
     <t xml:space="preserve">PROYECCIÓN CAJA MOTOR — HIPÓTESIS BASE v1</t>
   </si>
   <si>
     <t xml:space="preserve">Ilustrativa, no un objetivo. X/Y/Z por necesidad patrimonial: CONSTITUTION.md Sección 6, Pendiente.</t>
   </si>
   <si>
+    <t xml:space="preserve">Fecha y saldo de referencia  ·  CONGELADOS — no enlazados por fórmula</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fecha de referencia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Provisional. Se sustituirá por el cierre a 31/12/2026 para anclar la trayectoria en año natural — al cambiar esta fecha (y los importes de abajo) toda la trayectoria esperada y el seguimiento se recalculan solos.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AMS — Caja Motor (congelado)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cifra dada por Armando a la fecha de referencia (2026-08-13). No enlazada a la hoja Cajas — solo cambia con actualización explícita de este congelado.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AML — Fondos RV (congelado)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cifra dada por Armando a la fecha de referencia (2026-08-13).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AML — Planes de Pensiones (congelado)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bloqueados operativamente (ver hoja Cajas, fila 24). Incluidos en Motor por composición de activo, confirmado por Armando 2026-08-13.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AML — Caja Motor (congelado, total)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Suma de las dos filas anteriores. Sigue siendo un congelado: solo se mueve si cambian esas dos celdas manualmente.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Hipótesis de rentabilidad  ·  CONSTITUTION.md Sección 2</t>
   </si>
   <si>
@@ -527,30 +653,15 @@
     <t xml:space="preserve">Derivada de la rentabilidad real + inflación media histórica de la serie Shiller (~2,15%/año). Misma gobernanza que la fila anterior.</t>
   </si>
   <si>
-    <t xml:space="preserve">Base — Caja Motor  ·  hoja 'Cajas'</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AMS — Caja Motor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cajas!C10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AML — Caja Motor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cajas!C25</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Incluye Planes de Pensiones, operativamente bloqueados (ver hoja 'Cajas').</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Proyección Caja Motor a 5 / 10 / 15 años  ·  AMS vs. AML</t>
+    <t xml:space="preserve">Trayectoria esperada — Caja Motor, desde el congelado</t>
   </si>
   <si>
     <t xml:space="preserve">Horizonte</t>
   </si>
   <si>
+    <t xml:space="preserve">Fecha objetivo</t>
+  </si>
+  <si>
     <t xml:space="preserve">AMS Real</t>
   </si>
   <si>
@@ -572,111 +683,47 @@
     <t xml:space="preserve">15 años</t>
   </si>
   <si>
-    <t xml:space="preserve">Proyección de interés compuesto puro sobre el saldo actual de Caja Motor. No es el objetivo X/Y/Z (todavía sin definir) — sirve para comparar, una vez fijado ese objetivo, si la trayectoria real va camino de cumplirlo. AML incluye Planes de Pensiones bloqueados.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CLASIFICACIÓN EN LAS TRES CAJAS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nivel 3, CONSTITUTION.md Sección 2  ·  Seguridad · Motor · Rentas Pasivas</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AMS — patrimonio propio</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Caja</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Partida</t>
-  </si>
-  <si>
-    <t xml:space="preserve">% Total</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Origen</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Seguridad</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AMS!B41</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AMS!B44</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Subtotal Seguridad</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Motor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AMS!B40</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Subtotal Motor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rentas Pasivas</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AMS!B42</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AMS!B43</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Subtotal Rentas Pasivas</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TOTAL AMS (3 cajas)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Diferencia vs. total patrimonio (control)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Debe ser 0€. Si no lo es, hay una partida nueva en la sección 4 sin clasificar aquí.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AML — patrimonio de tus padres</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AML!B43</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AML!B39</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AML!B40</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bloqueado operativamente (ilíquido salvo jubilación/paro larga duración/enfermedad grave; destino: herencia). Clasificado en Motor por composición de activo, confirmado por Armando 2026-08-13.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AML!B41</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Función declarada de renta vía dividendos, no de crecimiento (ver AML!D58). Confirmado por Armando 2026-08-13.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AML!B42</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TOTAL AML (3 cajas)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Colores: Seguridad (azul) · Motor (verde) · Rentas Pasivas (naranja). % Total = peso de cada caja sobre el patrimonio total de AMS o AML respectivamente. Clasificación fijada por Armando el 2026-08-13 sobre la tabla de cajas de CONSTITUTION.md Sección 2, Nivel 3 — Seguridad: liquidez/depósitos/monetarios · Motor: fondo indexado S&amp;P 500 y otras inversiones a largo plazo · Rentas Pasivas: JGPI, inmobiliario, oro.</t>
+    <t xml:space="preserve">Seguimiento — saldo real vs. trayectoria esperada (nominal)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fecha de control</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Años</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AMS Actual</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AMS Esperado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AMS Δ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AML Actual</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AML Esperado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AML Δ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Celdas azules/amarillas = escribe tú (Fecha de control, AMS Actual, AML Actual). El resto son fórmulas. 'Esperado' compara contra la trayectoria nominal (euros corrientes), igual que el saldo observado — no está ajustado por inflación. Δ positivo = vas por delante de la trayectoria; negativo = por detrás. Esto compara contra la hipótesis base, no contra un objetivo X/Y/Z (todavía sin definir).</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="6">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="#,##0\€;\(#,##0&quot;€)&quot;"/>
     <numFmt numFmtId="166" formatCode="0.0%"/>
     <numFmt numFmtId="167" formatCode="0"/>
+    <numFmt numFmtId="168" formatCode="dd/mm/yyyy"/>
+    <numFmt numFmtId="169" formatCode="0.00"/>
   </numFmts>
   <fonts count="26">
     <font>
@@ -777,16 +824,16 @@
       <charset val="1"/>
     </font>
     <font>
-      <b val="true"/>
-      <sz val="10"/>
-      <color rgb="FF1155CC"/>
+      <sz val="8.5"/>
+      <color rgb="FF9E9E9E"/>
       <name val="Arial"/>
       <family val="2"/>
       <charset val="1"/>
     </font>
     <font>
-      <sz val="8.5"/>
-      <color rgb="FF9E9E9E"/>
+      <b val="true"/>
+      <sz val="10.5"/>
+      <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
       <family val="2"/>
       <charset val="1"/>
@@ -795,14 +842,6 @@
       <i val="true"/>
       <sz val="8.5"/>
       <color rgb="FF7F7F7F"/>
-      <name val="Arial"/>
-      <family val="2"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="10.5"/>
-      <color rgb="FF1F1F1F"/>
       <name val="Arial"/>
       <family val="2"/>
       <charset val="1"/>
@@ -847,16 +886,16 @@
       <charset val="1"/>
     </font>
     <font>
-      <sz val="8.5"/>
-      <color rgb="FF9E9E9E"/>
+      <b val="true"/>
+      <sz val="10"/>
+      <color rgb="FF1155CC"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
-      <b val="true"/>
-      <sz val="10.5"/>
-      <color rgb="FFFFFFFF"/>
+      <sz val="8.5"/>
+      <color rgb="FF9E9E9E"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -865,6 +904,14 @@
       <i val="true"/>
       <sz val="8.5"/>
       <color rgb="FF7F7F7F"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="10.5"/>
+      <color rgb="FF1F1F1F"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -903,18 +950,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFF2CC"/>
-        <bgColor rgb="FFFCE4D6"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFE2EFDA"/>
-        <bgColor rgb="FFDDEBF7"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFDDEBF7"/>
         <bgColor rgb="FFD9E1F2"/>
       </patternFill>
@@ -923,6 +958,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFBDD7EE"/>
         <bgColor rgb="FFD9D9D9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE2EFDA"/>
+        <bgColor rgb="FFDDEBF7"/>
       </patternFill>
     </fill>
     <fill>
@@ -947,6 +988,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FF404040"/>
         <bgColor rgb="FF595959"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF2CC"/>
+        <bgColor rgb="FFFCE4D6"/>
       </patternFill>
     </fill>
   </fills>
@@ -1060,11 +1107,15 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="77">
+  <cellXfs count="86">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1085,7 +1136,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1105,7 +1156,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1125,7 +1176,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1133,11 +1184,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1145,227 +1196,259 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="14" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="13" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="7" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="12" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="12" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="8" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="8" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="13" fillId="8" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="8" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="8" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="9" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="9" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="12" fillId="9" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="12" fillId="9" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="10" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="10" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="13" fillId="10" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="10" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="10" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="11" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="11" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="12" fillId="11" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="12" fillId="11" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="12" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="15" fillId="12" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="15" fillId="12" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="12" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="17" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="7" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="16" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="16" fillId="8" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="3" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="3" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="13" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="13" fillId="7" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="13" fillId="7" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="16" fillId="10" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="20" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="21" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="20" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="21" fillId="8" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="22" fillId="8" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="21" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="22" fillId="8" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="22" fillId="13" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="8" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="23" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="23" fillId="8" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="24" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="22" fillId="13" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="20" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="9" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="25" fillId="8" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="22" fillId="13" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="20" fillId="3" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="21" fillId="9" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="20" fillId="3" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="21" fillId="9" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="20" fillId="8" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="8" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="21" fillId="9" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="21" fillId="8" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="21" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="22" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="21" fillId="8" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="21" fillId="8" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="22" fillId="13" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="22" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="169" fontId="21" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="21" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="23" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="10" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="21" fillId="10" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="21" fillId="10" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="25" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="21" fillId="10" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="22" fillId="13" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="21" fillId="11" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="22" fillId="11" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="22" fillId="11" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="25" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="11" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="23" fillId="11" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="12" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="21" fillId="12" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="21" fillId="12" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="21" fillId="12" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="24" fillId="13" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="24" fillId="13" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="24" fillId="13" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="13" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="25" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="25" fillId="11" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1624,139 +1707,139 @@
   <dimension ref="A1:B24"/>
   <sheetFormatPr defaultColWidth="8.66796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="38"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="70"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="70"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="4" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="2" t="s">
+      <c r="A5" s="3" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4" t="s">
+      <c r="A6" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="4" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="3" t="s">
+      <c r="A7" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="4" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="2" t="s">
+      <c r="A9" s="3" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="3" t="s">
+      <c r="A10" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="B10" s="4" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="3" t="s">
+      <c r="A11" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="B11" s="3" t="s">
+      <c r="B11" s="4" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="3" t="s">
+      <c r="A12" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="B12" s="3" t="s">
+      <c r="B12" s="4" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="2" t="s">
+      <c r="A14" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="B14" s="3" t="s">
+      <c r="B14" s="4" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="2" t="s">
+      <c r="A16" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="B16" s="3" t="s">
+      <c r="B16" s="4" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="2" t="s">
+      <c r="A18" s="3" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="3" t="s">
+      <c r="A19" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="B19" s="3" t="s">
+      <c r="B19" s="4" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="3" t="s">
+      <c r="A20" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="B20" s="3" t="s">
+      <c r="B20" s="4" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="3" t="s">
+      <c r="A21" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="B21" s="3" t="s">
+      <c r="B21" s="4" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="3" t="s">
+      <c r="A22" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="B22" s="3" t="s">
+      <c r="B22" s="4" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="3" t="s">
+      <c r="A23" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="B23" s="3" t="s">
+      <c r="B23" s="4" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="3" t="s">
+      <c r="A24" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="B24" s="3" t="s">
+      <c r="B24" s="4" t="s">
         <v>23</v>
       </c>
     </row>
@@ -1779,705 +1862,705 @@
   <dimension ref="A1:D61"/>
   <sheetFormatPr defaultColWidth="8.66796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="46"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="5" t="s">
+      <c r="A3" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="B3" s="6"/>
-      <c r="C3" s="6"/>
-      <c r="D3" s="6"/>
+      <c r="B3" s="7"/>
+      <c r="C3" s="7"/>
+      <c r="D3" s="7"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="7" t="s">
+      <c r="A4" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="B4" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="C4" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="D4" s="7" t="s">
+      <c r="D4" s="8" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="B5" s="8" t="n">
+      <c r="B5" s="9" t="n">
         <v>20000</v>
       </c>
-      <c r="C5" s="9" t="s">
+      <c r="C5" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="D5" s="9" t="s">
+      <c r="D5" s="10" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="B6" s="8" t="n">
+      <c r="B6" s="9" t="n">
         <v>13000</v>
       </c>
-      <c r="C6" s="9" t="s">
+      <c r="C6" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="D6" s="9" t="s">
+      <c r="D6" s="10" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="3" t="s">
+      <c r="A7" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="B7" s="10" t="n">
+      <c r="B7" s="11" t="n">
         <f aca="false">B6-B5</f>
         <v>-7000</v>
       </c>
-      <c r="C7" s="9" t="s">
+      <c r="C7" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="D7" s="9" t="s">
+      <c r="D7" s="10" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="3" t="s">
+      <c r="A8" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="C8" s="9" t="s">
+      <c r="C8" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="D8" s="9" t="s">
+      <c r="D8" s="10" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3" t="s">
+      <c r="A9" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="B9" s="8" t="n">
+      <c r="B9" s="9" t="n">
         <v>30000</v>
       </c>
-      <c r="C9" s="9" t="s">
+      <c r="C9" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="D9" s="9" t="s">
+      <c r="D9" s="10" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="3" t="s">
+      <c r="A10" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="B10" s="8" t="n">
+      <c r="B10" s="9" t="n">
         <v>70000</v>
       </c>
-      <c r="C10" s="9" t="s">
+      <c r="C10" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="D10" s="9" t="s">
+      <c r="D10" s="10" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="3" t="s">
+      <c r="A11" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="B11" s="8" t="n">
+      <c r="B11" s="9" t="n">
         <v>120000</v>
       </c>
-      <c r="C11" s="9" t="s">
+      <c r="C11" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="D11" s="9" t="s">
+      <c r="D11" s="10" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="3" t="s">
+      <c r="A12" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="B12" s="10" t="n">
+      <c r="B12" s="11" t="n">
         <f aca="false">B9+B10</f>
         <v>100000</v>
       </c>
-      <c r="C12" s="9" t="s">
+      <c r="C12" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="D12" s="11"/>
+      <c r="D12" s="12"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="3" t="s">
+      <c r="A13" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="B13" s="10" t="n">
+      <c r="B13" s="11" t="n">
         <f aca="false">B9+B11</f>
         <v>150000</v>
       </c>
-      <c r="C13" s="9" t="s">
+      <c r="C13" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="D13" s="11"/>
+      <c r="D13" s="12"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="3" t="s">
+      <c r="A14" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="B14" s="8" t="n">
+      <c r="B14" s="9" t="n">
         <v>83100</v>
       </c>
-      <c r="C14" s="9" t="s">
+      <c r="C14" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="D14" s="9" t="s">
+      <c r="D14" s="10" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="3" t="s">
+      <c r="A15" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="B15" s="8" t="n">
+      <c r="B15" s="9" t="n">
         <v>89230.77</v>
       </c>
-      <c r="C15" s="9" t="s">
+      <c r="C15" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="D15" s="9" t="s">
+      <c r="D15" s="10" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="3" t="s">
+      <c r="A16" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="B16" s="10" t="n">
+      <c r="B16" s="11" t="n">
         <f aca="false">SUM(B14:B15)</f>
         <v>172330.77</v>
       </c>
-      <c r="C16" s="9" t="s">
+      <c r="C16" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="D16" s="11"/>
+      <c r="D16" s="12"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="3" t="s">
+      <c r="A17" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="B17" s="10" t="n">
+      <c r="B17" s="11" t="n">
         <f aca="false">B16-B9</f>
         <v>142330.77</v>
       </c>
-      <c r="C17" s="9" t="s">
+      <c r="C17" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="D17" s="11"/>
+      <c r="D17" s="12"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="3" t="s">
+      <c r="A18" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="B18" s="10" t="n">
+      <c r="B18" s="11" t="n">
         <f aca="false">B16-B12</f>
         <v>72330.77</v>
       </c>
-      <c r="C18" s="9" t="s">
+      <c r="C18" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="D18" s="11"/>
+      <c r="D18" s="12"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="3" t="s">
+      <c r="A19" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="B19" s="10" t="n">
+      <c r="B19" s="11" t="n">
         <f aca="false">B16-B13</f>
         <v>22330.77</v>
       </c>
-      <c r="C19" s="9" t="s">
+      <c r="C19" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="D19" s="9" t="s">
+      <c r="D19" s="10" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="3" t="s">
+      <c r="A20" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="B20" s="10" t="n">
+      <c r="B20" s="11" t="n">
         <f aca="false">B17-B10</f>
         <v>72330.77</v>
       </c>
-      <c r="C20" s="9" t="s">
+      <c r="C20" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="D20" s="11"/>
+      <c r="D20" s="12"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="3" t="s">
+      <c r="A21" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="B21" s="10" t="n">
+      <c r="B21" s="11" t="n">
         <f aca="false">B17-B11</f>
         <v>22330.77</v>
       </c>
-      <c r="C21" s="9" t="s">
+      <c r="C21" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="D21" s="11"/>
+      <c r="D21" s="12"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="5" t="s">
+      <c r="A23" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="B23" s="6"/>
-      <c r="C23" s="6"/>
-      <c r="D23" s="6"/>
+      <c r="B23" s="7"/>
+      <c r="C23" s="7"/>
+      <c r="D23" s="7"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="7" t="s">
+      <c r="A24" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="B24" s="7" t="s">
+      <c r="B24" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="C24" s="7" t="s">
+      <c r="C24" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="D24" s="7" t="s">
+      <c r="D24" s="8" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="3" t="s">
+      <c r="A25" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="B25" s="4" t="s">
+      <c r="B25" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="C25" s="9" t="s">
+      <c r="C25" s="10" t="s">
         <v>64</v>
       </c>
-      <c r="D25" s="9" t="s">
+      <c r="D25" s="10" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="5" t="s">
+      <c r="A27" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="B27" s="6"/>
-      <c r="C27" s="6"/>
-      <c r="D27" s="6"/>
+      <c r="B27" s="7"/>
+      <c r="C27" s="7"/>
+      <c r="D27" s="7"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="7" t="s">
+      <c r="A28" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="B28" s="7" t="s">
+      <c r="B28" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="C28" s="7" t="s">
+      <c r="C28" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="D28" s="7" t="s">
+      <c r="D28" s="8" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="3" t="s">
+      <c r="A29" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="B29" s="8" t="n">
+      <c r="B29" s="9" t="n">
         <v>6000</v>
       </c>
-      <c r="C29" s="9" t="s">
+      <c r="C29" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="D29" s="11"/>
+      <c r="D29" s="12"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="3" t="s">
+      <c r="A30" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="B30" s="8" t="n">
+      <c r="B30" s="9" t="n">
         <v>5000</v>
       </c>
-      <c r="C30" s="9" t="s">
+      <c r="C30" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="D30" s="11"/>
+      <c r="D30" s="12"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="3" t="s">
+      <c r="A31" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="B31" s="8" t="n">
+      <c r="B31" s="9" t="n">
         <v>2000</v>
       </c>
-      <c r="C31" s="9" t="s">
+      <c r="C31" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="D31" s="11"/>
+      <c r="D31" s="12"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="3" t="s">
+      <c r="A32" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="B32" s="10" t="n">
+      <c r="B32" s="11" t="n">
         <f aca="false">SUM(B29:B31)</f>
         <v>13000</v>
       </c>
-      <c r="C32" s="9" t="s">
+      <c r="C32" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="D32" s="11"/>
+      <c r="D32" s="12"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="3" t="s">
+      <c r="A33" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="B33" s="12" t="n">
+      <c r="B33" s="13" t="n">
         <f aca="false">B29/B32</f>
         <v>0.461538461538462</v>
       </c>
-      <c r="C33" s="9" t="s">
+      <c r="C33" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="D33" s="11"/>
+      <c r="D33" s="12"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="3" t="s">
+      <c r="A34" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="B34" s="12" t="n">
+      <c r="B34" s="13" t="n">
         <f aca="false">B30/B32</f>
         <v>0.384615384615385</v>
       </c>
-      <c r="C34" s="9" t="s">
+      <c r="C34" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="D34" s="11"/>
+      <c r="D34" s="12"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="3" t="s">
+      <c r="A35" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="B35" s="12" t="n">
+      <c r="B35" s="13" t="n">
         <f aca="false">B31/B32</f>
         <v>0.153846153846154</v>
       </c>
-      <c r="C35" s="9" t="s">
+      <c r="C35" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="D35" s="11"/>
+      <c r="D35" s="12"/>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="3" t="s">
+      <c r="A36" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="B36" s="4" t="s">
+      <c r="B36" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="C36" s="9" t="s">
+      <c r="C36" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="D36" s="9" t="s">
+      <c r="D36" s="10" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="5" t="s">
+      <c r="A38" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="B38" s="6"/>
-      <c r="C38" s="6"/>
-      <c r="D38" s="6"/>
+      <c r="B38" s="7"/>
+      <c r="C38" s="7"/>
+      <c r="D38" s="7"/>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="7" t="s">
+      <c r="A39" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="B39" s="7" t="s">
+      <c r="B39" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="C39" s="7" t="s">
+      <c r="C39" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="D39" s="7" t="s">
+      <c r="D39" s="8" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="3" t="s">
+      <c r="A40" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="B40" s="8" t="n">
-        <v>872837.88</v>
-      </c>
-      <c r="C40" s="9" t="s">
+      <c r="B40" s="9" t="n">
+        <v>878274</v>
+      </c>
+      <c r="C40" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="D40" s="11"/>
+      <c r="D40" s="12"/>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A41" s="3" t="s">
+      <c r="A41" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="B41" s="8" t="n">
+      <c r="B41" s="9" t="n">
         <v>89230.77</v>
       </c>
-      <c r="C41" s="9" t="s">
+      <c r="C41" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="D41" s="11"/>
+      <c r="D41" s="12"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="3" t="s">
+      <c r="A42" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="B42" s="8" t="n">
+      <c r="B42" s="9" t="n">
         <v>111570.37</v>
       </c>
-      <c r="C42" s="9" t="s">
+      <c r="C42" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="D42" s="11"/>
+      <c r="D42" s="12"/>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A43" s="3" t="s">
+      <c r="A43" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="B43" s="8" t="n">
+      <c r="B43" s="9" t="n">
         <v>100000</v>
       </c>
-      <c r="C43" s="9" t="s">
+      <c r="C43" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="D43" s="11"/>
+      <c r="D43" s="12"/>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="3" t="s">
+      <c r="A44" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="B44" s="8" t="n">
+      <c r="B44" s="9" t="n">
         <v>83100</v>
       </c>
-      <c r="C44" s="9" t="s">
+      <c r="C44" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="D44" s="9" t="s">
+      <c r="D44" s="10" t="s">
         <v>83</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A45" s="13" t="s">
+      <c r="A45" s="14" t="s">
         <v>84</v>
       </c>
-      <c r="B45" s="14" t="n">
+      <c r="B45" s="15" t="n">
         <f aca="false">SUM(B40:B44)</f>
-        <v>1256739.02</v>
-      </c>
-      <c r="C45" s="15" t="s">
+        <v>1262175.14</v>
+      </c>
+      <c r="C45" s="16" t="s">
         <v>36</v>
       </c>
-      <c r="D45" s="16"/>
+      <c r="D45" s="17"/>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A46" s="3" t="s">
+      <c r="A46" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="B46" s="12" t="n">
+      <c r="B46" s="13" t="n">
         <f aca="false">B40/B45</f>
-        <v>0.694525964507731</v>
-      </c>
-      <c r="C46" s="9" t="s">
+        <v>0.695841624641728</v>
+      </c>
+      <c r="C46" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="D46" s="11"/>
+      <c r="D46" s="12"/>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A47" s="3" t="s">
+      <c r="A47" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="B47" s="12" t="n">
+      <c r="B47" s="13" t="n">
         <f aca="false">B41/B45</f>
-        <v>0.0710018297991575</v>
-      </c>
-      <c r="C47" s="9" t="s">
+        <v>0.0706960287619038</v>
+      </c>
+      <c r="C47" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="D47" s="11"/>
+      <c r="D47" s="12"/>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A48" s="3" t="s">
+      <c r="A48" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="B48" s="12" t="n">
+      <c r="B48" s="13" t="n">
         <f aca="false">B42/B45</f>
-        <v>0.0887776763707074</v>
-      </c>
-      <c r="C48" s="9" t="s">
+        <v>0.0883953157245674</v>
+      </c>
+      <c r="C48" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="D48" s="11"/>
+      <c r="D48" s="12"/>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A49" s="3" t="s">
+      <c r="A49" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="B49" s="12" t="n">
+      <c r="B49" s="13" t="n">
         <f aca="false">B43/B45</f>
-        <v>0.0795710154682712</v>
-      </c>
-      <c r="C49" s="9" t="s">
+        <v>0.0792283074122344</v>
+      </c>
+      <c r="C49" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="D49" s="11"/>
+      <c r="D49" s="12"/>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A50" s="3" t="s">
+      <c r="A50" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="B50" s="12" t="n">
+      <c r="B50" s="13" t="n">
         <f aca="false">B44/B45</f>
-        <v>0.0661235138541334</v>
-      </c>
-      <c r="C50" s="9" t="s">
+        <v>0.0658387234595668</v>
+      </c>
+      <c r="C50" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="D50" s="11"/>
+      <c r="D50" s="12"/>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A51" s="3" t="s">
+      <c r="A51" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="B51" s="4" t="s">
+      <c r="B51" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="C51" s="9" t="s">
+      <c r="C51" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="D51" s="9" t="s">
+      <c r="D51" s="10" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A53" s="5" t="s">
+      <c r="A53" s="6" t="s">
         <v>92</v>
       </c>
-      <c r="B53" s="6"/>
-      <c r="C53" s="6"/>
-      <c r="D53" s="6"/>
+      <c r="B53" s="7"/>
+      <c r="C53" s="7"/>
+      <c r="D53" s="7"/>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A54" s="7" t="s">
+      <c r="A54" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="B54" s="7" t="s">
+      <c r="B54" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="C54" s="7" t="s">
+      <c r="C54" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="D54" s="7" t="s">
+      <c r="D54" s="8" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A55" s="3" t="s">
+      <c r="A55" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="B55" s="4" t="s">
+      <c r="B55" s="5" t="s">
         <v>94</v>
       </c>
-      <c r="C55" s="9" t="s">
+      <c r="C55" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="D55" s="9" t="s">
+      <c r="D55" s="10" t="s">
         <v>95</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A56" s="3" t="s">
+      <c r="A56" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="B56" s="4" t="s">
+      <c r="B56" s="5" t="s">
         <v>97</v>
       </c>
-      <c r="C56" s="9" t="s">
+      <c r="C56" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="D56" s="9" t="s">
+      <c r="D56" s="10" t="s">
         <v>98</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A58" s="5" t="s">
+      <c r="A58" s="6" t="s">
         <v>99</v>
       </c>
-      <c r="B58" s="6"/>
-      <c r="C58" s="6"/>
-      <c r="D58" s="6"/>
+      <c r="B58" s="7"/>
+      <c r="C58" s="7"/>
+      <c r="D58" s="7"/>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A59" s="7" t="s">
+      <c r="A59" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="B59" s="7" t="s">
+      <c r="B59" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="C59" s="7" t="s">
+      <c r="C59" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="D59" s="7" t="s">
+      <c r="D59" s="8" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A60" s="3" t="s">
+      <c r="A60" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="B60" s="8" t="n">
+      <c r="B60" s="9" t="n">
         <v>-215092</v>
       </c>
-      <c r="C60" s="9" t="s">
+      <c r="C60" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="D60" s="9" t="s">
+      <c r="D60" s="10" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A61" s="3" t="s">
+      <c r="A61" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="B61" s="4" t="s">
+      <c r="B61" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="C61" s="9" t="s">
+      <c r="C61" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="D61" s="9" t="s">
+      <c r="D61" s="10" t="s">
         <v>104</v>
       </c>
     </row>
@@ -2500,830 +2583,830 @@
   <dimension ref="A1:D73"/>
   <sheetFormatPr defaultColWidth="8.66796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="50"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="50"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>105</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="5" t="s">
+      <c r="A3" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="B3" s="6"/>
-      <c r="C3" s="6"/>
-      <c r="D3" s="6"/>
+      <c r="B3" s="7"/>
+      <c r="C3" s="7"/>
+      <c r="D3" s="7"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="7" t="s">
+      <c r="A4" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="B4" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="C4" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="D4" s="7" t="s">
+      <c r="D4" s="8" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="B5" s="8" t="n">
+      <c r="B5" s="9" t="n">
         <v>32500</v>
       </c>
-      <c r="C5" s="9" t="s">
+      <c r="C5" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="D5" s="9" t="s">
+      <c r="D5" s="10" t="s">
         <v>106</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="B6" s="8" t="n">
+      <c r="B6" s="9" t="n">
         <v>80000</v>
       </c>
-      <c r="C6" s="9" t="s">
+      <c r="C6" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="D6" s="9" t="s">
+      <c r="D6" s="10" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="3" t="s">
+      <c r="A7" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="B7" s="10" t="n">
+      <c r="B7" s="11" t="n">
         <f aca="false">B6-B5</f>
         <v>47500</v>
       </c>
-      <c r="C7" s="9" t="s">
+      <c r="C7" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="D7" s="9" t="s">
+      <c r="D7" s="10" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="3" t="s">
+      <c r="A8" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="B8" s="8" t="n">
+      <c r="B8" s="9" t="n">
         <v>125000</v>
       </c>
-      <c r="C8" s="9" t="s">
+      <c r="C8" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="D8" s="9" t="s">
+      <c r="D8" s="10" t="s">
         <v>110</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3" t="s">
+      <c r="A9" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="B9" s="8" t="n">
+      <c r="B9" s="9" t="n">
         <v>125000</v>
       </c>
-      <c r="C9" s="9" t="s">
+      <c r="C9" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="D9" s="11"/>
+      <c r="D9" s="12"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="3" t="s">
+      <c r="A10" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="B10" s="8" t="n">
+      <c r="B10" s="9" t="n">
         <v>175000</v>
       </c>
-      <c r="C10" s="9" t="s">
+      <c r="C10" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="D10" s="11"/>
+      <c r="D10" s="12"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="3" t="s">
+      <c r="A11" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="B11" s="10" t="n">
+      <c r="B11" s="11" t="n">
         <f aca="false">B8+B9</f>
         <v>250000</v>
       </c>
-      <c r="C11" s="9" t="s">
+      <c r="C11" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="D11" s="11"/>
+      <c r="D11" s="12"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="3" t="s">
+      <c r="A12" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="B12" s="10" t="n">
+      <c r="B12" s="11" t="n">
         <f aca="false">B8+B10</f>
         <v>300000</v>
       </c>
-      <c r="C12" s="9" t="s">
+      <c r="C12" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="D12" s="9" t="s">
+      <c r="D12" s="10" t="s">
         <v>111</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="3" t="s">
+      <c r="A13" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="B13" s="8" t="n">
+      <c r="B13" s="9" t="n">
         <v>54375</v>
       </c>
-      <c r="C13" s="9" t="s">
+      <c r="C13" s="10" t="s">
         <v>112</v>
       </c>
-      <c r="D13" s="11"/>
+      <c r="D13" s="12"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="3" t="s">
+      <c r="A14" s="4" t="s">
         <v>113</v>
       </c>
-      <c r="B14" s="8" t="n">
+      <c r="B14" s="9" t="n">
         <v>60000</v>
       </c>
-      <c r="C14" s="9" t="s">
+      <c r="C14" s="10" t="s">
         <v>112</v>
       </c>
-      <c r="D14" s="9" t="s">
+      <c r="D14" s="10" t="s">
         <v>114</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="3" t="s">
+      <c r="A15" s="4" t="s">
         <v>115</v>
       </c>
-      <c r="B15" s="8" t="n">
+      <c r="B15" s="9" t="n">
         <v>85000</v>
       </c>
-      <c r="C15" s="9" t="s">
+      <c r="C15" s="10" t="s">
         <v>112</v>
       </c>
-      <c r="D15" s="9" t="s">
+      <c r="D15" s="10" t="s">
         <v>116</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="3" t="s">
+      <c r="A16" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="B16" s="8" t="n">
+      <c r="B16" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="C16" s="9" t="s">
+      <c r="C16" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="D16" s="9" t="s">
+      <c r="D16" s="10" t="s">
         <v>117</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="3" t="s">
+      <c r="A17" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="B17" s="10" t="n">
+      <c r="B17" s="11" t="n">
         <f aca="false">SUM(B13:B16)</f>
         <v>199375</v>
       </c>
-      <c r="C17" s="9" t="s">
+      <c r="C17" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="D17" s="11"/>
+      <c r="D17" s="12"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="3" t="s">
+      <c r="A18" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="B18" s="10" t="n">
+      <c r="B18" s="11" t="n">
         <f aca="false">B17-B8</f>
         <v>74375</v>
       </c>
-      <c r="C18" s="9" t="s">
+      <c r="C18" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="D18" s="11"/>
+      <c r="D18" s="12"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="3" t="s">
+      <c r="A19" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="B19" s="10" t="n">
+      <c r="B19" s="11" t="n">
         <f aca="false">B17-B11</f>
         <v>-50625</v>
       </c>
-      <c r="C19" s="9" t="s">
+      <c r="C19" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="D19" s="11"/>
+      <c r="D19" s="12"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="3" t="s">
+      <c r="A20" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="B20" s="10" t="n">
+      <c r="B20" s="11" t="n">
         <f aca="false">B17-B12</f>
         <v>-100625</v>
       </c>
-      <c r="C20" s="9" t="s">
+      <c r="C20" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="D20" s="11"/>
+      <c r="D20" s="12"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="3" t="s">
+      <c r="A21" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="B21" s="10" t="n">
+      <c r="B21" s="11" t="n">
         <f aca="false">B18-B9</f>
         <v>-50625</v>
       </c>
-      <c r="C21" s="9" t="s">
+      <c r="C21" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="D21" s="9" t="s">
+      <c r="D21" s="10" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="3" t="s">
+      <c r="A22" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="B22" s="10" t="n">
+      <c r="B22" s="11" t="n">
         <f aca="false">B18-B10</f>
         <v>-100625</v>
       </c>
-      <c r="C22" s="9" t="s">
+      <c r="C22" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="D22" s="11"/>
+      <c r="D22" s="12"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="5" t="s">
+      <c r="A24" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="B24" s="6"/>
-      <c r="C24" s="6"/>
-      <c r="D24" s="6"/>
+      <c r="B24" s="7"/>
+      <c r="C24" s="7"/>
+      <c r="D24" s="7"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="7" t="s">
+      <c r="A25" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="B25" s="7" t="s">
+      <c r="B25" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="C25" s="7" t="s">
+      <c r="C25" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="D25" s="7" t="s">
+      <c r="D25" s="8" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="3" t="s">
+      <c r="A26" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="B26" s="4" t="s">
+      <c r="B26" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="C26" s="9" t="s">
+      <c r="C26" s="10" t="s">
         <v>64</v>
       </c>
-      <c r="D26" s="9" t="s">
+      <c r="D26" s="10" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="5" t="s">
+      <c r="A28" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="B28" s="6"/>
-      <c r="C28" s="6"/>
-      <c r="D28" s="6"/>
+      <c r="B28" s="7"/>
+      <c r="C28" s="7"/>
+      <c r="D28" s="7"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="7" t="s">
+      <c r="A29" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="B29" s="7" t="s">
+      <c r="B29" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="C29" s="7" t="s">
+      <c r="C29" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="D29" s="7" t="s">
+      <c r="D29" s="8" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="3" t="s">
+      <c r="A30" s="4" t="s">
         <v>119</v>
       </c>
-      <c r="B30" s="8" t="n">
+      <c r="B30" s="9" t="n">
         <v>60000</v>
       </c>
-      <c r="C30" s="9" t="s">
+      <c r="C30" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="D30" s="9" t="s">
+      <c r="D30" s="10" t="s">
         <v>120</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="3" t="s">
+      <c r="A31" s="4" t="s">
         <v>121</v>
       </c>
-      <c r="B31" s="8" t="n">
+      <c r="B31" s="9" t="n">
         <v>20000</v>
       </c>
-      <c r="C31" s="9" t="s">
+      <c r="C31" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="D31" s="11"/>
+      <c r="D31" s="12"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="3" t="s">
+      <c r="A32" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="B32" s="10" t="n">
+      <c r="B32" s="11" t="n">
         <f aca="false">SUM(B30:B31)</f>
         <v>80000</v>
       </c>
-      <c r="C32" s="9" t="s">
+      <c r="C32" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="D32" s="11"/>
+      <c r="D32" s="12"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="3" t="s">
+      <c r="A33" s="4" t="s">
         <v>122</v>
       </c>
-      <c r="B33" s="12" t="n">
+      <c r="B33" s="13" t="n">
         <f aca="false">B30/B32</f>
         <v>0.75</v>
       </c>
-      <c r="C33" s="9" t="s">
+      <c r="C33" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="D33" s="11"/>
+      <c r="D33" s="12"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="3" t="s">
+      <c r="A34" s="4" t="s">
         <v>123</v>
       </c>
-      <c r="B34" s="12" t="n">
+      <c r="B34" s="13" t="n">
         <f aca="false">B31/B32</f>
         <v>0.25</v>
       </c>
-      <c r="C34" s="9" t="s">
+      <c r="C34" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="D34" s="11"/>
+      <c r="D34" s="12"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="3" t="s">
+      <c r="A35" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="B35" s="4" t="s">
+      <c r="B35" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="C35" s="9" t="s">
+      <c r="C35" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="D35" s="9" t="s">
+      <c r="D35" s="10" t="s">
         <v>124</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="5" t="s">
+      <c r="A37" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="B37" s="6"/>
-      <c r="C37" s="6"/>
-      <c r="D37" s="6"/>
+      <c r="B37" s="7"/>
+      <c r="C37" s="7"/>
+      <c r="D37" s="7"/>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="7" t="s">
+      <c r="A38" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="B38" s="7" t="s">
+      <c r="B38" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="C38" s="7" t="s">
+      <c r="C38" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="D38" s="7" t="s">
+      <c r="D38" s="8" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="3" t="s">
+      <c r="A39" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="B39" s="8" t="n">
-        <v>2183088.49</v>
-      </c>
-      <c r="C39" s="9" t="s">
+      <c r="B39" s="9" t="n">
+        <v>2196689</v>
+      </c>
+      <c r="C39" s="10" t="s">
         <v>112</v>
       </c>
-      <c r="D39" s="11"/>
+      <c r="D39" s="12"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="3" t="s">
+      <c r="A40" s="4" t="s">
         <v>126</v>
       </c>
-      <c r="B40" s="8" t="n">
-        <v>1157519.11</v>
-      </c>
-      <c r="C40" s="9" t="s">
+      <c r="B40" s="9" t="n">
+        <v>1158833</v>
+      </c>
+      <c r="C40" s="10" t="s">
         <v>112</v>
       </c>
-      <c r="D40" s="9" t="s">
+      <c r="D40" s="10" t="s">
         <v>127</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A41" s="3" t="s">
+      <c r="A41" s="4" t="s">
         <v>128</v>
       </c>
-      <c r="B41" s="8" t="n">
+      <c r="B41" s="9" t="n">
         <v>538013.75</v>
       </c>
-      <c r="C41" s="9" t="s">
+      <c r="C41" s="10" t="s">
         <v>112</v>
       </c>
-      <c r="D41" s="11"/>
+      <c r="D41" s="12"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="3" t="s">
+      <c r="A42" s="4" t="s">
         <v>129</v>
       </c>
-      <c r="B42" s="8" t="n">
+      <c r="B42" s="9" t="n">
         <v>139351.5</v>
       </c>
-      <c r="C42" s="9" t="s">
+      <c r="C42" s="10" t="s">
         <v>112</v>
       </c>
-      <c r="D42" s="11"/>
+      <c r="D42" s="12"/>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A43" s="3" t="s">
+      <c r="A43" s="4" t="s">
         <v>130</v>
       </c>
-      <c r="B43" s="8" t="n">
+      <c r="B43" s="9" t="n">
         <v>199375</v>
       </c>
-      <c r="C43" s="9" t="s">
+      <c r="C43" s="10" t="s">
         <v>112</v>
       </c>
-      <c r="D43" s="9" t="s">
+      <c r="D43" s="10" t="s">
         <v>131</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="13" t="s">
+      <c r="A44" s="14" t="s">
         <v>84</v>
       </c>
-      <c r="B44" s="14" t="n">
+      <c r="B44" s="15" t="n">
         <f aca="false">SUM(B39:B43)</f>
-        <v>4217347.85</v>
-      </c>
-      <c r="C44" s="15" t="s">
+        <v>4232262.25</v>
+      </c>
+      <c r="C44" s="16" t="s">
         <v>36</v>
       </c>
-      <c r="D44" s="16"/>
+      <c r="D44" s="17"/>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A45" s="3" t="s">
+      <c r="A45" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="B45" s="12" t="n">
+      <c r="B45" s="13" t="n">
         <f aca="false">B39/B44</f>
-        <v>0.517644872475957</v>
-      </c>
-      <c r="C45" s="9" t="s">
+        <v>0.519034235177652</v>
+      </c>
+      <c r="C45" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="D45" s="11"/>
+      <c r="D45" s="12"/>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A46" s="3" t="s">
+      <c r="A46" s="4" t="s">
         <v>133</v>
       </c>
-      <c r="B46" s="12" t="n">
+      <c r="B46" s="13" t="n">
         <f aca="false">B40/B44</f>
-        <v>0.274466122115111</v>
-      </c>
-      <c r="C46" s="9" t="s">
+        <v>0.273809355741129</v>
+      </c>
+      <c r="C46" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="D46" s="11"/>
+      <c r="D46" s="12"/>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A47" s="3" t="s">
+      <c r="A47" s="4" t="s">
         <v>134</v>
       </c>
-      <c r="B47" s="12" t="n">
+      <c r="B47" s="13" t="n">
         <f aca="false">B41/B44</f>
-        <v>0.127571585066193</v>
-      </c>
-      <c r="C47" s="9" t="s">
+        <v>0.127122025578637</v>
+      </c>
+      <c r="C47" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="D47" s="11"/>
+      <c r="D47" s="12"/>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A48" s="3" t="s">
+      <c r="A48" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="B48" s="12" t="n">
+      <c r="B48" s="13" t="n">
         <f aca="false">B42/B44</f>
-        <v>0.0330424487038697</v>
-      </c>
-      <c r="C48" s="9" t="s">
+        <v>0.0329260078342262</v>
+      </c>
+      <c r="C48" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="D48" s="11"/>
+      <c r="D48" s="12"/>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A49" s="3" t="s">
+      <c r="A49" s="4" t="s">
         <v>135</v>
       </c>
-      <c r="B49" s="12" t="n">
+      <c r="B49" s="13" t="n">
         <f aca="false">B43/B44</f>
-        <v>0.0472749716388701</v>
-      </c>
-      <c r="C49" s="9" t="s">
+        <v>0.0471083756683556</v>
+      </c>
+      <c r="C49" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="D49" s="11"/>
+      <c r="D49" s="12"/>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A51" s="2" t="s">
+      <c r="A51" s="3" t="s">
         <v>136</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A52" s="3" t="s">
+      <c r="A52" s="4" t="s">
         <v>137</v>
       </c>
-      <c r="B52" s="8" t="n">
+      <c r="B52" s="9" t="n">
         <v>356040</v>
       </c>
-      <c r="C52" s="9" t="s">
+      <c r="C52" s="10" t="s">
         <v>138</v>
       </c>
-      <c r="D52" s="11"/>
+      <c r="D52" s="12"/>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A53" s="3" t="s">
+      <c r="A53" s="4" t="s">
         <v>139</v>
       </c>
-      <c r="B53" s="8" t="n">
+      <c r="B53" s="9" t="n">
         <v>125804.4</v>
       </c>
-      <c r="C53" s="9" t="s">
+      <c r="C53" s="10" t="s">
         <v>138</v>
       </c>
-      <c r="D53" s="11"/>
+      <c r="D53" s="12"/>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A54" s="3" t="s">
+      <c r="A54" s="4" t="s">
         <v>140</v>
       </c>
-      <c r="B54" s="8" t="n">
+      <c r="B54" s="9" t="n">
         <v>56169.35</v>
       </c>
-      <c r="C54" s="9" t="s">
+      <c r="C54" s="10" t="s">
         <v>138</v>
       </c>
-      <c r="D54" s="11"/>
+      <c r="D54" s="12"/>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A55" s="3" t="s">
+      <c r="A55" s="4" t="s">
         <v>141</v>
       </c>
-      <c r="B55" s="12" t="n">
+      <c r="B55" s="13" t="n">
         <f aca="false">B52/B41</f>
         <v>0.661767473414945</v>
       </c>
-      <c r="C55" s="9" t="s">
+      <c r="C55" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="D55" s="11"/>
+      <c r="D55" s="12"/>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A56" s="3" t="s">
+      <c r="A56" s="4" t="s">
         <v>142</v>
       </c>
-      <c r="B56" s="12" t="n">
+      <c r="B56" s="13" t="n">
         <f aca="false">B53/B41</f>
         <v>0.233831198552082</v>
       </c>
-      <c r="C56" s="9" t="s">
+      <c r="C56" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="D56" s="11"/>
+      <c r="D56" s="12"/>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A57" s="3" t="s">
+      <c r="A57" s="4" t="s">
         <v>143</v>
       </c>
-      <c r="B57" s="12" t="n">
+      <c r="B57" s="13" t="n">
         <f aca="false">B54/B41</f>
         <v>0.104401328032973</v>
       </c>
-      <c r="C57" s="9" t="s">
+      <c r="C57" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="D57" s="11"/>
+      <c r="D57" s="12"/>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A58" s="3" t="s">
+      <c r="A58" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="B58" s="4" t="s">
+      <c r="B58" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="C58" s="9" t="s">
+      <c r="C58" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="D58" s="9" t="s">
+      <c r="D58" s="10" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A60" s="5" t="s">
+      <c r="A60" s="6" t="s">
         <v>92</v>
       </c>
-      <c r="B60" s="6"/>
-      <c r="C60" s="6"/>
-      <c r="D60" s="6"/>
+      <c r="B60" s="7"/>
+      <c r="C60" s="7"/>
+      <c r="D60" s="7"/>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A61" s="7" t="s">
+      <c r="A61" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="B61" s="7" t="s">
+      <c r="B61" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="C61" s="7" t="s">
+      <c r="C61" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="D61" s="7" t="s">
+      <c r="D61" s="8" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A62" s="3" t="s">
+      <c r="A62" s="4" t="s">
         <v>145</v>
       </c>
-      <c r="B62" s="4" t="s">
+      <c r="B62" s="5" t="s">
         <v>146</v>
       </c>
-      <c r="C62" s="9" t="s">
+      <c r="C62" s="10" t="s">
         <v>147</v>
       </c>
-      <c r="D62" s="9" t="s">
+      <c r="D62" s="10" t="s">
         <v>148</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A63" s="3" t="s">
+      <c r="A63" s="4" t="s">
         <v>149</v>
       </c>
-      <c r="B63" s="17" t="n">
+      <c r="B63" s="18" t="n">
         <f aca="true">DATE(2026,9,29)-TODAY()</f>
-        <v>47</v>
-      </c>
-      <c r="C63" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="C63" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="D63" s="11"/>
+      <c r="D63" s="12"/>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A64" s="3" t="s">
+      <c r="A64" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="B64" s="4" t="s">
+      <c r="B64" s="5" t="s">
         <v>151</v>
       </c>
-      <c r="C64" s="9" t="s">
+      <c r="C64" s="10" t="s">
         <v>147</v>
       </c>
-      <c r="D64" s="9" t="s">
+      <c r="D64" s="10" t="s">
         <v>152</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A65" s="3" t="s">
+      <c r="A65" s="4" t="s">
         <v>149</v>
       </c>
-      <c r="B65" s="17" t="n">
+      <c r="B65" s="18" t="n">
         <f aca="true">DATE(2026,8,26)-TODAY()</f>
-        <v>13</v>
-      </c>
-      <c r="C65" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="C65" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="D65" s="9" t="s">
+      <c r="D65" s="10" t="s">
         <v>153</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A67" s="3" t="s">
+      <c r="A67" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="B67" s="4" t="s">
+      <c r="B67" s="5" t="s">
         <v>97</v>
       </c>
-      <c r="C67" s="9" t="s">
+      <c r="C67" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="D67" s="9" t="s">
+      <c r="D67" s="10" t="s">
         <v>154</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A69" s="5" t="s">
+      <c r="A69" s="6" t="s">
         <v>99</v>
       </c>
-      <c r="B69" s="6"/>
-      <c r="C69" s="6"/>
-      <c r="D69" s="6"/>
+      <c r="B69" s="7"/>
+      <c r="C69" s="7"/>
+      <c r="D69" s="7"/>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A70" s="7" t="s">
+      <c r="A70" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="B70" s="7" t="s">
+      <c r="B70" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="C70" s="7" t="s">
+      <c r="C70" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="D70" s="7" t="s">
+      <c r="D70" s="8" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A71" s="3" t="s">
+      <c r="A71" s="4" t="s">
         <v>155</v>
       </c>
-      <c r="B71" s="8" t="n">
+      <c r="B71" s="9" t="n">
         <v>1157519.11</v>
       </c>
-      <c r="C71" s="9" t="s">
+      <c r="C71" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="D71" s="9" t="s">
+      <c r="D71" s="10" t="s">
         <v>156</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A72" s="3" t="s">
+      <c r="A72" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="B72" s="8" t="n">
+      <c r="B72" s="9" t="n">
         <v>-162000</v>
       </c>
-      <c r="C72" s="9" t="s">
+      <c r="C72" s="10" t="s">
         <v>157</v>
       </c>
-      <c r="D72" s="9" t="s">
+      <c r="D72" s="10" t="s">
         <v>158</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A73" s="3" t="s">
+      <c r="A73" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="B73" s="4" t="s">
+      <c r="B73" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="C73" s="9" t="s">
+      <c r="C73" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="D73" s="9" t="s">
+      <c r="D73" s="10" t="s">
         <v>159</v>
       </c>
     </row>
@@ -3343,717 +3426,449 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:F35"/>
   <sheetFormatPr defaultColWidth="8.66796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="2" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="1" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="50"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="18" t="s">
+    <row r="1" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="19" t="s">
         <v>160</v>
       </c>
-      <c r="B1" s="18"/>
-      <c r="C1" s="18"/>
-      <c r="D1" s="18"/>
-      <c r="E1" s="18"/>
-    </row>
-    <row r="2" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="19" t="s">
+      <c r="B1" s="19"/>
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19"/>
+      <c r="F1" s="19"/>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="20" t="s">
         <v>161</v>
       </c>
-      <c r="B2" s="19"/>
-      <c r="C2" s="19"/>
-      <c r="D2" s="19"/>
-      <c r="E2" s="19"/>
+      <c r="B2" s="20"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
+      <c r="F2" s="20"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="20" t="s">
+      <c r="A4" s="21" t="s">
         <v>162</v>
       </c>
-      <c r="B4" s="20"/>
-      <c r="C4" s="20"/>
-      <c r="D4" s="20"/>
-      <c r="E4" s="20"/>
+      <c r="B4" s="21"/>
+      <c r="C4" s="21"/>
+      <c r="D4" s="21"/>
+      <c r="E4" s="21"/>
+      <c r="F4" s="21"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="21" t="s">
-        <v>26</v>
-      </c>
-      <c r="B5" s="21" t="s">
+      <c r="A5" s="22" t="s">
+        <v>163</v>
+      </c>
+      <c r="B5" s="22" t="s">
+        <v>164</v>
+      </c>
+      <c r="C5" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="C5" s="21" t="s">
-        <v>28</v>
-      </c>
-      <c r="D5" s="21" t="s">
+      <c r="D5" s="22" t="s">
+        <v>165</v>
+      </c>
+      <c r="E5" s="22" t="s">
+        <v>166</v>
+      </c>
+      <c r="F5" s="22" t="s">
         <v>29</v>
       </c>
-      <c r="E5" s="21"/>
-    </row>
-    <row r="6" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="22" t="s">
-        <v>163</v>
-      </c>
-      <c r="B6" s="23" t="n">
-        <v>0.07</v>
-      </c>
-      <c r="C6" s="24" t="s">
-        <v>31</v>
-      </c>
-      <c r="D6" s="25" t="s">
-        <v>164</v>
-      </c>
-      <c r="E6" s="25"/>
-    </row>
-    <row r="7" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="22" t="s">
-        <v>165</v>
-      </c>
-      <c r="B7" s="23" t="n">
-        <v>0.094</v>
-      </c>
-      <c r="C7" s="24" t="s">
-        <v>31</v>
-      </c>
-      <c r="D7" s="25" t="s">
-        <v>166</v>
-      </c>
-      <c r="E7" s="25"/>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="20" t="s">
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="23" t="s">
         <v>167</v>
       </c>
-      <c r="B9" s="20"/>
-      <c r="C9" s="20"/>
-      <c r="D9" s="20"/>
-      <c r="E9" s="20"/>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="21" t="s">
-        <v>26</v>
-      </c>
-      <c r="B10" s="21" t="s">
-        <v>27</v>
-      </c>
-      <c r="C10" s="21" t="s">
-        <v>28</v>
-      </c>
-      <c r="D10" s="21" t="s">
-        <v>29</v>
-      </c>
-      <c r="E10" s="21"/>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="26" t="s">
-        <v>168</v>
-      </c>
-      <c r="B11" s="27" t="n">
-        <f aca="false">Cajas!C10</f>
-        <v>872837.88</v>
-      </c>
-      <c r="C11" s="28" t="s">
-        <v>169</v>
-      </c>
-      <c r="D11" s="29"/>
-      <c r="E11" s="29"/>
-    </row>
-    <row r="12" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="26" t="s">
-        <v>170</v>
-      </c>
-      <c r="B12" s="27" t="n">
-        <f aca="false">Cajas!C25</f>
-        <v>3340607.6</v>
-      </c>
-      <c r="C12" s="28" t="s">
-        <v>171</v>
-      </c>
-      <c r="D12" s="30" t="s">
-        <v>172</v>
-      </c>
-      <c r="E12" s="30"/>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="20" t="s">
-        <v>173</v>
-      </c>
-      <c r="B14" s="20"/>
-      <c r="C14" s="20"/>
-      <c r="D14" s="20"/>
-      <c r="E14" s="20"/>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="21" t="s">
-        <v>174</v>
-      </c>
-      <c r="B15" s="21" t="s">
-        <v>175</v>
-      </c>
-      <c r="C15" s="31" t="s">
-        <v>176</v>
-      </c>
-      <c r="D15" s="32" t="s">
-        <v>177</v>
-      </c>
-      <c r="E15" s="21" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="26" t="s">
-        <v>179</v>
-      </c>
-      <c r="B16" s="33" t="n">
-        <f aca="false">$B$11*(1+$B$6)^5</f>
-        <v>1224200.27921452</v>
-      </c>
-      <c r="C16" s="34" t="n">
-        <f aca="false">$B$11*(1+$B$7)^5</f>
-        <v>1367792.42987986</v>
-      </c>
-      <c r="D16" s="35" t="n">
-        <f aca="false">$B$12*(1+$B$6)^5</f>
-        <v>4685374.97096958</v>
-      </c>
-      <c r="E16" s="33" t="n">
-        <f aca="false">$B$12*(1+$B$7)^5</f>
-        <v>5234944.41657267</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="26" t="s">
-        <v>180</v>
-      </c>
-      <c r="B17" s="33" t="n">
-        <f aca="false">$B$11*(1+$B$6)^10</f>
-        <v>1717004.22033575</v>
-      </c>
-      <c r="C17" s="34" t="n">
-        <f aca="false">$B$11*(1+$B$7)^10</f>
-        <v>2143417.6656456</v>
-      </c>
-      <c r="D17" s="35" t="n">
-        <f aca="false">$B$12*(1+$B$6)^10</f>
-        <v>6571480.77451184</v>
-      </c>
-      <c r="E17" s="33" t="n">
-        <f aca="false">$B$12*(1+$B$7)^10</f>
-        <v>8203490.59991523</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="26" t="s">
-        <v>181</v>
-      </c>
-      <c r="B18" s="33" t="n">
-        <f aca="false">$B$11*(1+$B$6)^15</f>
-        <v>2408187.24085111</v>
-      </c>
-      <c r="C18" s="34" t="n">
-        <f aca="false">$B$11*(1+$B$7)^15</f>
-        <v>3358871.70380461</v>
-      </c>
-      <c r="D18" s="35" t="n">
-        <f aca="false">$B$12*(1+$B$6)^15</f>
-        <v>9216841.73355336</v>
-      </c>
-      <c r="E18" s="33" t="n">
-        <f aca="false">$B$12*(1+$B$7)^15</f>
-        <v>12855391.1307729</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="36" t="s">
-        <v>182</v>
-      </c>
-      <c r="B20" s="36"/>
-      <c r="C20" s="36"/>
-      <c r="D20" s="36"/>
-      <c r="E20" s="36"/>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="36"/>
-      <c r="B21" s="36"/>
-      <c r="C21" s="36"/>
-      <c r="D21" s="36"/>
-      <c r="E21" s="36"/>
-    </row>
-  </sheetData>
-  <mergeCells count="12">
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="D5:E5"/>
-    <mergeCell ref="D6:E6"/>
-    <mergeCell ref="D7:E7"/>
-    <mergeCell ref="A9:E9"/>
-    <mergeCell ref="D10:E10"/>
-    <mergeCell ref="D11:E11"/>
-    <mergeCell ref="D12:E12"/>
-    <mergeCell ref="A14:E14"/>
-    <mergeCell ref="A20:E21"/>
-  </mergeCells>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="true"/>
-  </sheetPr>
-  <dimension ref="A1:F35"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
-  <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="50"/>
-  </cols>
-  <sheetData>
-    <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="37" t="s">
-        <v>183</v>
-      </c>
-      <c r="B1" s="37"/>
-      <c r="C1" s="37"/>
-      <c r="D1" s="37"/>
-      <c r="E1" s="37"/>
-      <c r="F1" s="37"/>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="38" t="s">
-        <v>184</v>
-      </c>
-      <c r="B2" s="38"/>
-      <c r="C2" s="38"/>
-      <c r="D2" s="38"/>
-      <c r="E2" s="38"/>
-      <c r="F2" s="38"/>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="39" t="s">
-        <v>185</v>
-      </c>
-      <c r="B4" s="39"/>
-      <c r="C4" s="39"/>
-      <c r="D4" s="39"/>
-      <c r="E4" s="39"/>
-      <c r="F4" s="39"/>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="40" t="s">
-        <v>186</v>
-      </c>
-      <c r="B5" s="40" t="s">
-        <v>187</v>
-      </c>
-      <c r="C5" s="40" t="s">
-        <v>27</v>
-      </c>
-      <c r="D5" s="40" t="s">
-        <v>188</v>
-      </c>
-      <c r="E5" s="40" t="s">
-        <v>189</v>
-      </c>
-      <c r="F5" s="40" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="41" t="s">
-        <v>190</v>
-      </c>
-      <c r="B6" s="42" t="str">
+      <c r="B6" s="24" t="str">
         <f aca="false">AMS!A41</f>
         <v>Fondo Monetario</v>
       </c>
-      <c r="C6" s="43" t="n">
+      <c r="C6" s="25" t="n">
         <f aca="false">AMS!B41</f>
         <v>89230.77</v>
       </c>
-      <c r="D6" s="44"/>
-      <c r="E6" s="45" t="s">
-        <v>191</v>
-      </c>
-      <c r="F6" s="44"/>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="41"/>
-      <c r="B7" s="42" t="str">
+      <c r="D6" s="26"/>
+      <c r="E6" s="27" t="s">
+        <v>168</v>
+      </c>
+      <c r="F6" s="26"/>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="23"/>
+      <c r="B7" s="24" t="str">
         <f aca="false">AMS!A44</f>
         <v>Liquidez (excluido FM)</v>
       </c>
-      <c r="C7" s="43" t="n">
+      <c r="C7" s="25" t="n">
         <f aca="false">AMS!B44</f>
         <v>83100</v>
       </c>
-      <c r="D7" s="44"/>
-      <c r="E7" s="45" t="s">
-        <v>192</v>
-      </c>
-      <c r="F7" s="44"/>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="46"/>
-      <c r="B8" s="47" t="s">
-        <v>193</v>
-      </c>
-      <c r="C8" s="48" t="n">
+      <c r="D7" s="26"/>
+      <c r="E7" s="27" t="s">
+        <v>169</v>
+      </c>
+      <c r="F7" s="26"/>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="28"/>
+      <c r="B8" s="29" t="s">
+        <v>170</v>
+      </c>
+      <c r="C8" s="30" t="n">
         <f aca="false">SUM(C6:C7)</f>
         <v>172330.77</v>
       </c>
-      <c r="D8" s="49" t="n">
+      <c r="D8" s="31" t="n">
         <f aca="false">C8/C$15</f>
-        <v>0.137125343653291</v>
-      </c>
-      <c r="E8" s="46"/>
-      <c r="F8" s="46"/>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="50" t="s">
-        <v>194</v>
-      </c>
-      <c r="B9" s="51" t="str">
+        <v>0.136534752221471</v>
+      </c>
+      <c r="E8" s="28"/>
+      <c r="F8" s="28"/>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="32" t="s">
+        <v>171</v>
+      </c>
+      <c r="B9" s="33" t="str">
         <f aca="false">AMS!A40</f>
         <v>SP500 (fondos indexados)</v>
       </c>
-      <c r="C9" s="52" t="n">
+      <c r="C9" s="34" t="n">
         <f aca="false">AMS!B40</f>
-        <v>872837.88</v>
-      </c>
-      <c r="D9" s="29"/>
-      <c r="E9" s="53" t="s">
-        <v>195</v>
-      </c>
-      <c r="F9" s="29"/>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="54"/>
-      <c r="B10" s="55" t="s">
-        <v>196</v>
-      </c>
-      <c r="C10" s="56" t="n">
+        <v>878274</v>
+      </c>
+      <c r="D9" s="35"/>
+      <c r="E9" s="36" t="s">
+        <v>172</v>
+      </c>
+      <c r="F9" s="35"/>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="37"/>
+      <c r="B10" s="38" t="s">
+        <v>173</v>
+      </c>
+      <c r="C10" s="39" t="n">
         <f aca="false">C9</f>
-        <v>872837.88</v>
-      </c>
-      <c r="D10" s="57" t="n">
+        <v>878274</v>
+      </c>
+      <c r="D10" s="40" t="n">
         <f aca="false">C10/C$15</f>
-        <v>0.694525964507731</v>
-      </c>
-      <c r="E10" s="54"/>
-      <c r="F10" s="54"/>
+        <v>0.695841624641728</v>
+      </c>
+      <c r="E10" s="37"/>
+      <c r="F10" s="37"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="58" t="s">
-        <v>197</v>
-      </c>
-      <c r="B11" s="59" t="str">
+      <c r="A11" s="41" t="s">
+        <v>174</v>
+      </c>
+      <c r="B11" s="42" t="str">
         <f aca="false">AMS!A42</f>
         <v>ETF</v>
       </c>
-      <c r="C11" s="60" t="n">
+      <c r="C11" s="43" t="n">
         <f aca="false">AMS!B42</f>
         <v>111570.37</v>
       </c>
-      <c r="D11" s="61"/>
-      <c r="E11" s="62" t="s">
-        <v>198</v>
-      </c>
-      <c r="F11" s="61"/>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="58"/>
-      <c r="B12" s="59" t="str">
+      <c r="D11" s="44"/>
+      <c r="E11" s="45" t="s">
+        <v>175</v>
+      </c>
+      <c r="F11" s="44"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="41"/>
+      <c r="B12" s="42" t="str">
         <f aca="false">AMS!A43</f>
         <v>Pisos</v>
       </c>
-      <c r="C12" s="60" t="n">
+      <c r="C12" s="43" t="n">
         <f aca="false">AMS!B43</f>
         <v>100000</v>
       </c>
-      <c r="D12" s="61"/>
-      <c r="E12" s="62" t="s">
-        <v>199</v>
-      </c>
-      <c r="F12" s="61"/>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="63"/>
-      <c r="B13" s="64" t="s">
-        <v>200</v>
-      </c>
-      <c r="C13" s="65" t="n">
+      <c r="D12" s="44"/>
+      <c r="E12" s="45" t="s">
+        <v>176</v>
+      </c>
+      <c r="F12" s="44"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="46"/>
+      <c r="B13" s="47" t="s">
+        <v>177</v>
+      </c>
+      <c r="C13" s="48" t="n">
         <f aca="false">SUM(C11:C12)</f>
         <v>211570.37</v>
       </c>
-      <c r="D13" s="66" t="n">
+      <c r="D13" s="49" t="n">
         <f aca="false">C13/C$15</f>
-        <v>0.168348691838979</v>
-      </c>
-      <c r="E13" s="63"/>
-      <c r="F13" s="63"/>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="67" t="s">
-        <v>201</v>
-      </c>
-      <c r="B15" s="67"/>
-      <c r="C15" s="68" t="n">
+        <v>0.167623623136802</v>
+      </c>
+      <c r="E13" s="46"/>
+      <c r="F13" s="46"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="50" t="s">
+        <v>178</v>
+      </c>
+      <c r="B15" s="50"/>
+      <c r="C15" s="51" t="n">
         <f aca="false">C8+C10+C13</f>
-        <v>1256739.02</v>
-      </c>
-      <c r="D15" s="69" t="n">
+        <v>1262175.14</v>
+      </c>
+      <c r="D15" s="52" t="n">
         <f aca="false">C15/C15</f>
         <v>1</v>
       </c>
-      <c r="E15" s="70"/>
-      <c r="F15" s="70"/>
-    </row>
-    <row r="16" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B16" s="71" t="s">
-        <v>202</v>
-      </c>
-      <c r="C16" s="72" t="n">
+      <c r="E15" s="53"/>
+      <c r="F15" s="53"/>
+    </row>
+    <row r="16" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B16" s="54" t="s">
+        <v>179</v>
+      </c>
+      <c r="C16" s="55" t="n">
         <f aca="false">C15-AMS!B45</f>
         <v>0</v>
       </c>
-      <c r="F16" s="73" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="39" t="s">
-        <v>204</v>
-      </c>
-      <c r="B19" s="39"/>
-      <c r="C19" s="39"/>
-      <c r="D19" s="39"/>
-      <c r="E19" s="39"/>
-      <c r="F19" s="39"/>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="40" t="s">
-        <v>186</v>
-      </c>
-      <c r="B20" s="40" t="s">
-        <v>187</v>
-      </c>
-      <c r="C20" s="40" t="s">
+      <c r="F16" s="56" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="21" t="s">
+        <v>181</v>
+      </c>
+      <c r="B19" s="21"/>
+      <c r="C19" s="21"/>
+      <c r="D19" s="21"/>
+      <c r="E19" s="21"/>
+      <c r="F19" s="21"/>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="22" t="s">
+        <v>163</v>
+      </c>
+      <c r="B20" s="22" t="s">
+        <v>164</v>
+      </c>
+      <c r="C20" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="D20" s="40" t="s">
-        <v>188</v>
-      </c>
-      <c r="E20" s="40" t="s">
-        <v>189</v>
-      </c>
-      <c r="F20" s="40" t="s">
+      <c r="D20" s="22" t="s">
+        <v>165</v>
+      </c>
+      <c r="E20" s="22" t="s">
+        <v>166</v>
+      </c>
+      <c r="F20" s="22" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="41" t="s">
-        <v>190</v>
-      </c>
-      <c r="B21" s="42" t="str">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="23" t="s">
+        <v>167</v>
+      </c>
+      <c r="B21" s="24" t="str">
         <f aca="false">AML!A43</f>
         <v>Liquidez + Depósitos (excluido FM)</v>
       </c>
-      <c r="C21" s="43" t="n">
+      <c r="C21" s="25" t="n">
         <f aca="false">AML!B43</f>
         <v>199375</v>
       </c>
-      <c r="D21" s="44"/>
-      <c r="E21" s="45" t="s">
-        <v>205</v>
-      </c>
-      <c r="F21" s="44"/>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="46"/>
-      <c r="B22" s="47" t="s">
-        <v>193</v>
-      </c>
-      <c r="C22" s="48" t="n">
+      <c r="D21" s="26"/>
+      <c r="E21" s="27" t="s">
+        <v>182</v>
+      </c>
+      <c r="F21" s="26"/>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="28"/>
+      <c r="B22" s="29" t="s">
+        <v>170</v>
+      </c>
+      <c r="C22" s="30" t="n">
         <f aca="false">C21</f>
         <v>199375</v>
       </c>
-      <c r="D22" s="49" t="n">
+      <c r="D22" s="31" t="n">
         <f aca="false">C22/C$30</f>
-        <v>0.0472749716388701</v>
-      </c>
-      <c r="E22" s="46"/>
-      <c r="F22" s="46"/>
+        <v>0.0471083756683556</v>
+      </c>
+      <c r="E22" s="28"/>
+      <c r="F22" s="28"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="50" t="s">
-        <v>194</v>
-      </c>
-      <c r="B23" s="51" t="str">
+      <c r="A23" s="32" t="s">
+        <v>171</v>
+      </c>
+      <c r="B23" s="33" t="str">
         <f aca="false">AML!A39</f>
         <v>Fondos RV</v>
       </c>
-      <c r="C23" s="52" t="n">
+      <c r="C23" s="34" t="n">
         <f aca="false">AML!B39</f>
-        <v>2183088.49</v>
-      </c>
-      <c r="D23" s="29"/>
-      <c r="E23" s="53" t="s">
-        <v>206</v>
-      </c>
-      <c r="F23" s="29"/>
+        <v>2196689</v>
+      </c>
+      <c r="D23" s="35"/>
+      <c r="E23" s="36" t="s">
+        <v>183</v>
+      </c>
+      <c r="F23" s="35"/>
     </row>
     <row r="24" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="50"/>
-      <c r="B24" s="51" t="str">
+      <c r="A24" s="32"/>
+      <c r="B24" s="33" t="str">
         <f aca="false">AML!A40</f>
         <v>Planes de Pensiones (Papá 754.162,54 + Mamá 403.356,58)</v>
       </c>
-      <c r="C24" s="52" t="n">
+      <c r="C24" s="34" t="n">
         <f aca="false">AML!B40</f>
-        <v>1157519.11</v>
-      </c>
-      <c r="D24" s="29"/>
-      <c r="E24" s="53" t="s">
-        <v>207</v>
-      </c>
-      <c r="F24" s="74" t="s">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="54"/>
-      <c r="B25" s="55" t="s">
-        <v>196</v>
-      </c>
-      <c r="C25" s="56" t="n">
+        <v>1158833</v>
+      </c>
+      <c r="D24" s="35"/>
+      <c r="E24" s="36" t="s">
+        <v>184</v>
+      </c>
+      <c r="F24" s="57" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="37"/>
+      <c r="B25" s="38" t="s">
+        <v>173</v>
+      </c>
+      <c r="C25" s="39" t="n">
         <f aca="false">SUM(C23:C24)</f>
-        <v>3340607.6</v>
-      </c>
-      <c r="D25" s="57" t="n">
+        <v>3355522</v>
+      </c>
+      <c r="D25" s="40" t="n">
         <f aca="false">C25/C$30</f>
-        <v>0.792110994591068</v>
-      </c>
-      <c r="E25" s="54"/>
-      <c r="F25" s="54"/>
+        <v>0.792843590918781</v>
+      </c>
+      <c r="E25" s="37"/>
+      <c r="F25" s="37"/>
     </row>
     <row r="26" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="58" t="s">
-        <v>197</v>
-      </c>
-      <c r="B26" s="59" t="str">
+      <c r="A26" s="41" t="s">
+        <v>174</v>
+      </c>
+      <c r="B26" s="42" t="str">
         <f aca="false">AML!A41</f>
         <v>Acciones (Iberdrola 356.040 + BBVA 125.804,4 + TEF 56.169,35)</v>
       </c>
-      <c r="C26" s="60" t="n">
+      <c r="C26" s="43" t="n">
         <f aca="false">AML!B41</f>
         <v>538013.75</v>
       </c>
-      <c r="D26" s="61"/>
-      <c r="E26" s="62" t="s">
-        <v>209</v>
-      </c>
-      <c r="F26" s="75" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="58"/>
-      <c r="B27" s="59" t="str">
+      <c r="D26" s="44"/>
+      <c r="E26" s="45" t="s">
+        <v>186</v>
+      </c>
+      <c r="F26" s="58" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="41"/>
+      <c r="B27" s="42" t="str">
         <f aca="false">AML!A42</f>
         <v>ETF (Aristócratas)</v>
       </c>
-      <c r="C27" s="60" t="n">
+      <c r="C27" s="43" t="n">
         <f aca="false">AML!B42</f>
         <v>139351.5</v>
       </c>
-      <c r="D27" s="61"/>
-      <c r="E27" s="62" t="s">
-        <v>211</v>
-      </c>
-      <c r="F27" s="61"/>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="63"/>
-      <c r="B28" s="64" t="s">
-        <v>200</v>
-      </c>
-      <c r="C28" s="65" t="n">
+      <c r="D27" s="44"/>
+      <c r="E27" s="45" t="s">
+        <v>188</v>
+      </c>
+      <c r="F27" s="44"/>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="46"/>
+      <c r="B28" s="47" t="s">
+        <v>177</v>
+      </c>
+      <c r="C28" s="48" t="n">
         <f aca="false">SUM(C26:C27)</f>
         <v>677365.25</v>
       </c>
-      <c r="D28" s="66" t="n">
+      <c r="D28" s="49" t="n">
         <f aca="false">C28/C$30</f>
-        <v>0.160614033770062</v>
-      </c>
-      <c r="E28" s="63"/>
-      <c r="F28" s="63"/>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="67" t="s">
-        <v>212</v>
-      </c>
-      <c r="B30" s="67"/>
-      <c r="C30" s="68" t="n">
+        <v>0.160048033412863</v>
+      </c>
+      <c r="E28" s="46"/>
+      <c r="F28" s="46"/>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="50" t="s">
+        <v>189</v>
+      </c>
+      <c r="B30" s="50"/>
+      <c r="C30" s="51" t="n">
         <f aca="false">C22+C25+C28</f>
-        <v>4217347.85</v>
-      </c>
-      <c r="D30" s="69" t="n">
+        <v>4232262.25</v>
+      </c>
+      <c r="D30" s="52" t="n">
         <f aca="false">C30/C30</f>
         <v>1</v>
       </c>
-      <c r="E30" s="70"/>
-      <c r="F30" s="70"/>
-    </row>
-    <row r="31" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B31" s="71" t="s">
-        <v>202</v>
-      </c>
-      <c r="C31" s="72" t="n">
+      <c r="E30" s="53"/>
+      <c r="F30" s="53"/>
+    </row>
+    <row r="31" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B31" s="54" t="s">
+        <v>179</v>
+      </c>
+      <c r="C31" s="55" t="n">
         <f aca="false">C30-AML!B44</f>
         <v>0</v>
       </c>
-      <c r="F31" s="73" t="s">
-        <v>203</v>
+      <c r="F31" s="56" t="s">
+        <v>180</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="76" t="s">
-        <v>213</v>
-      </c>
-      <c r="B33" s="76"/>
-      <c r="C33" s="76"/>
-      <c r="D33" s="76"/>
-      <c r="E33" s="76"/>
-      <c r="F33" s="76"/>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="76"/>
-      <c r="B34" s="76"/>
-      <c r="C34" s="76"/>
-      <c r="D34" s="76"/>
-      <c r="E34" s="76"/>
-      <c r="F34" s="76"/>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="76"/>
-      <c r="B35" s="76"/>
-      <c r="C35" s="76"/>
-      <c r="D35" s="76"/>
-      <c r="E35" s="76"/>
-      <c r="F35" s="76"/>
+      <c r="A33" s="59" t="s">
+        <v>190</v>
+      </c>
+      <c r="B33" s="59"/>
+      <c r="C33" s="59"/>
+      <c r="D33" s="59"/>
+      <c r="E33" s="59"/>
+      <c r="F33" s="59"/>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="59"/>
+      <c r="B34" s="59"/>
+      <c r="C34" s="59"/>
+      <c r="D34" s="59"/>
+      <c r="E34" s="59"/>
+      <c r="F34" s="59"/>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="59"/>
+      <c r="B35" s="59"/>
+      <c r="C35" s="59"/>
+      <c r="D35" s="59"/>
+      <c r="E35" s="59"/>
+      <c r="F35" s="59"/>
     </row>
   </sheetData>
   <mergeCells count="11">
@@ -4077,4 +3892,585 @@
     <oddFooter/>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="true"/>
+  </sheetPr>
+  <dimension ref="A1:H34"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="2" style="1" width="16"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="60" t="s">
+        <v>191</v>
+      </c>
+      <c r="B1" s="60"/>
+      <c r="C1" s="60"/>
+      <c r="D1" s="60"/>
+      <c r="E1" s="60"/>
+      <c r="F1" s="60"/>
+      <c r="G1" s="60"/>
+      <c r="H1" s="60"/>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="61" t="s">
+        <v>192</v>
+      </c>
+      <c r="B2" s="61"/>
+      <c r="C2" s="61"/>
+      <c r="D2" s="61"/>
+      <c r="E2" s="61"/>
+      <c r="F2" s="61"/>
+      <c r="G2" s="61"/>
+      <c r="H2" s="61"/>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="62" t="s">
+        <v>193</v>
+      </c>
+      <c r="B4" s="62"/>
+      <c r="C4" s="62"/>
+      <c r="D4" s="62"/>
+      <c r="E4" s="62"/>
+      <c r="F4" s="62"/>
+      <c r="G4" s="62"/>
+      <c r="H4" s="62"/>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="63" t="s">
+        <v>26</v>
+      </c>
+      <c r="B5" s="63" t="s">
+        <v>27</v>
+      </c>
+      <c r="C5" s="63" t="s">
+        <v>28</v>
+      </c>
+      <c r="D5" s="63" t="s">
+        <v>29</v>
+      </c>
+      <c r="E5" s="63"/>
+      <c r="F5" s="63"/>
+      <c r="G5" s="63"/>
+      <c r="H5" s="63"/>
+    </row>
+    <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="64" t="s">
+        <v>194</v>
+      </c>
+      <c r="B6" s="65" t="n">
+        <v>46247</v>
+      </c>
+      <c r="C6" s="66" t="s">
+        <v>31</v>
+      </c>
+      <c r="D6" s="67" t="s">
+        <v>195</v>
+      </c>
+      <c r="E6" s="67"/>
+      <c r="F6" s="67"/>
+      <c r="G6" s="67"/>
+      <c r="H6" s="67"/>
+    </row>
+    <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="64" t="s">
+        <v>196</v>
+      </c>
+      <c r="B7" s="68" t="n">
+        <v>878274</v>
+      </c>
+      <c r="C7" s="66" t="s">
+        <v>31</v>
+      </c>
+      <c r="D7" s="67" t="s">
+        <v>197</v>
+      </c>
+      <c r="E7" s="67"/>
+      <c r="F7" s="67"/>
+      <c r="G7" s="67"/>
+      <c r="H7" s="67"/>
+    </row>
+    <row r="8" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="64" t="s">
+        <v>198</v>
+      </c>
+      <c r="B8" s="68" t="n">
+        <v>2196689</v>
+      </c>
+      <c r="C8" s="66" t="s">
+        <v>31</v>
+      </c>
+      <c r="D8" s="67" t="s">
+        <v>199</v>
+      </c>
+      <c r="E8" s="67"/>
+      <c r="F8" s="67"/>
+      <c r="G8" s="67"/>
+      <c r="H8" s="67"/>
+    </row>
+    <row r="9" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="64" t="s">
+        <v>200</v>
+      </c>
+      <c r="B9" s="68" t="n">
+        <v>1158833</v>
+      </c>
+      <c r="C9" s="66" t="s">
+        <v>31</v>
+      </c>
+      <c r="D9" s="67" t="s">
+        <v>201</v>
+      </c>
+      <c r="E9" s="67"/>
+      <c r="F9" s="67"/>
+      <c r="G9" s="67"/>
+      <c r="H9" s="67"/>
+    </row>
+    <row r="10" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="69" t="s">
+        <v>202</v>
+      </c>
+      <c r="B10" s="70" t="n">
+        <f aca="false">B8+B9</f>
+        <v>3355522</v>
+      </c>
+      <c r="C10" s="66" t="s">
+        <v>36</v>
+      </c>
+      <c r="D10" s="67" t="s">
+        <v>203</v>
+      </c>
+      <c r="E10" s="67"/>
+      <c r="F10" s="67"/>
+      <c r="G10" s="67"/>
+      <c r="H10" s="67"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="62" t="s">
+        <v>204</v>
+      </c>
+      <c r="B12" s="62"/>
+      <c r="C12" s="62"/>
+      <c r="D12" s="62"/>
+      <c r="E12" s="62"/>
+      <c r="F12" s="62"/>
+      <c r="G12" s="62"/>
+      <c r="H12" s="62"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="63" t="s">
+        <v>26</v>
+      </c>
+      <c r="B13" s="63" t="s">
+        <v>27</v>
+      </c>
+      <c r="C13" s="63" t="s">
+        <v>28</v>
+      </c>
+      <c r="D13" s="63" t="s">
+        <v>29</v>
+      </c>
+      <c r="E13" s="63"/>
+      <c r="F13" s="63"/>
+      <c r="G13" s="63"/>
+      <c r="H13" s="63"/>
+    </row>
+    <row r="14" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="64" t="s">
+        <v>205</v>
+      </c>
+      <c r="B14" s="71" t="n">
+        <v>0.07</v>
+      </c>
+      <c r="C14" s="66" t="s">
+        <v>31</v>
+      </c>
+      <c r="D14" s="67" t="s">
+        <v>206</v>
+      </c>
+      <c r="E14" s="67"/>
+      <c r="F14" s="67"/>
+      <c r="G14" s="67"/>
+      <c r="H14" s="67"/>
+    </row>
+    <row r="15" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="64" t="s">
+        <v>207</v>
+      </c>
+      <c r="B15" s="71" t="n">
+        <v>0.094</v>
+      </c>
+      <c r="C15" s="66" t="s">
+        <v>31</v>
+      </c>
+      <c r="D15" s="67" t="s">
+        <v>208</v>
+      </c>
+      <c r="E15" s="67"/>
+      <c r="F15" s="67"/>
+      <c r="G15" s="67"/>
+      <c r="H15" s="67"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="62" t="s">
+        <v>209</v>
+      </c>
+      <c r="B17" s="62"/>
+      <c r="C17" s="62"/>
+      <c r="D17" s="62"/>
+      <c r="E17" s="62"/>
+      <c r="F17" s="62"/>
+      <c r="G17" s="62"/>
+      <c r="H17" s="62"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="63" t="s">
+        <v>210</v>
+      </c>
+      <c r="B18" s="63" t="s">
+        <v>211</v>
+      </c>
+      <c r="C18" s="63" t="s">
+        <v>212</v>
+      </c>
+      <c r="D18" s="72" t="s">
+        <v>213</v>
+      </c>
+      <c r="E18" s="73" t="s">
+        <v>214</v>
+      </c>
+      <c r="F18" s="63" t="s">
+        <v>215</v>
+      </c>
+      <c r="G18" s="63"/>
+      <c r="H18" s="63"/>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="74" t="s">
+        <v>216</v>
+      </c>
+      <c r="B19" s="75" t="n">
+        <f aca="false">DATE(YEAR($B$6)+5,MONTH($B$6),DAY($B$6))</f>
+        <v>48073</v>
+      </c>
+      <c r="C19" s="76" t="n">
+        <f aca="false">$B$7*(1+$B$14)^5</f>
+        <v>1231824.71872881</v>
+      </c>
+      <c r="D19" s="77" t="n">
+        <f aca="false">$B$7*(1+$B$15)^5</f>
+        <v>1376311.17540442</v>
+      </c>
+      <c r="E19" s="78" t="n">
+        <f aca="false">$B$10*(1+$B$14)^5</f>
+        <v>4706293.18850193</v>
+      </c>
+      <c r="F19" s="76" t="n">
+        <f aca="false">$B$10*(1+$B$15)^5</f>
+        <v>5258316.22923529</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="74" t="s">
+        <v>217</v>
+      </c>
+      <c r="B20" s="75" t="n">
+        <f aca="false">DATE(YEAR($B$6)+10,MONTH($B$6),DAY($B$6))</f>
+        <v>49900</v>
+      </c>
+      <c r="C20" s="76" t="n">
+        <f aca="false">$B$7*(1+$B$14)^10</f>
+        <v>1727697.89117214</v>
+      </c>
+      <c r="D20" s="77" t="n">
+        <f aca="false">$B$7*(1+$B$15)^10</f>
+        <v>2156767.08127885</v>
+      </c>
+      <c r="E20" s="78" t="n">
+        <f aca="false">$B$10*(1+$B$14)^10</f>
+        <v>6600819.656715</v>
+      </c>
+      <c r="F20" s="76" t="n">
+        <f aca="false">$B$10*(1+$B$15)^10</f>
+        <v>8240115.71571852</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="74" t="s">
+        <v>218</v>
+      </c>
+      <c r="B21" s="75" t="n">
+        <f aca="false">DATE(YEAR($B$6)+15,MONTH($B$6),DAY($B$6))</f>
+        <v>51726</v>
+      </c>
+      <c r="C21" s="76" t="n">
+        <f aca="false">$B$7*(1+$B$14)^15</f>
+        <v>2423185.66739022</v>
+      </c>
+      <c r="D21" s="77" t="n">
+        <f aca="false">$B$7*(1+$B$15)^15</f>
+        <v>3379791.08650428</v>
+      </c>
+      <c r="E21" s="78" t="n">
+        <f aca="false">$B$10*(1+$B$14)^15</f>
+        <v>9257991.03356421</v>
+      </c>
+      <c r="F21" s="76" t="n">
+        <f aca="false">$B$10*(1+$B$15)^15</f>
+        <v>12912785.0148917</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="62" t="s">
+        <v>219</v>
+      </c>
+      <c r="B23" s="62"/>
+      <c r="C23" s="62"/>
+      <c r="D23" s="62"/>
+      <c r="E23" s="62"/>
+      <c r="F23" s="62"/>
+      <c r="G23" s="62"/>
+      <c r="H23" s="62"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="63" t="s">
+        <v>220</v>
+      </c>
+      <c r="B24" s="63" t="s">
+        <v>221</v>
+      </c>
+      <c r="C24" s="63" t="s">
+        <v>222</v>
+      </c>
+      <c r="D24" s="63" t="s">
+        <v>223</v>
+      </c>
+      <c r="E24" s="72" t="s">
+        <v>224</v>
+      </c>
+      <c r="F24" s="73" t="s">
+        <v>225</v>
+      </c>
+      <c r="G24" s="63" t="s">
+        <v>226</v>
+      </c>
+      <c r="H24" s="63" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="79"/>
+      <c r="B25" s="80" t="str">
+        <f aca="false">IF($A25="","",($A25-$B$6)/365.25)</f>
+        <v/>
+      </c>
+      <c r="C25" s="68"/>
+      <c r="D25" s="81" t="str">
+        <f aca="false">IF($A25="","",$B$7*(1+$B$15)^$B25)</f>
+        <v/>
+      </c>
+      <c r="E25" s="82" t="str">
+        <f aca="false">IF(OR($A25="",$C25=""),"",$C25-$D25)</f>
+        <v/>
+      </c>
+      <c r="F25" s="83"/>
+      <c r="G25" s="81" t="str">
+        <f aca="false">IF($A25="","",$B$10*(1+$B$15)^$B25)</f>
+        <v/>
+      </c>
+      <c r="H25" s="84" t="str">
+        <f aca="false">IF(OR($A25="",$F25=""),"",$F25-$G25)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="79"/>
+      <c r="B26" s="80" t="str">
+        <f aca="false">IF($A26="","",($A26-$B$6)/365.25)</f>
+        <v/>
+      </c>
+      <c r="C26" s="68"/>
+      <c r="D26" s="81" t="str">
+        <f aca="false">IF($A26="","",$B$7*(1+$B$15)^$B26)</f>
+        <v/>
+      </c>
+      <c r="E26" s="82" t="str">
+        <f aca="false">IF(OR($A26="",$C26=""),"",$C26-$D26)</f>
+        <v/>
+      </c>
+      <c r="F26" s="83"/>
+      <c r="G26" s="81" t="str">
+        <f aca="false">IF($A26="","",$B$10*(1+$B$15)^$B26)</f>
+        <v/>
+      </c>
+      <c r="H26" s="84" t="str">
+        <f aca="false">IF(OR($A26="",$F26=""),"",$F26-$G26)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="79"/>
+      <c r="B27" s="80" t="str">
+        <f aca="false">IF($A27="","",($A27-$B$6)/365.25)</f>
+        <v/>
+      </c>
+      <c r="C27" s="68"/>
+      <c r="D27" s="81" t="str">
+        <f aca="false">IF($A27="","",$B$7*(1+$B$15)^$B27)</f>
+        <v/>
+      </c>
+      <c r="E27" s="82" t="str">
+        <f aca="false">IF(OR($A27="",$C27=""),"",$C27-$D27)</f>
+        <v/>
+      </c>
+      <c r="F27" s="83"/>
+      <c r="G27" s="81" t="str">
+        <f aca="false">IF($A27="","",$B$10*(1+$B$15)^$B27)</f>
+        <v/>
+      </c>
+      <c r="H27" s="84" t="str">
+        <f aca="false">IF(OR($A27="",$F27=""),"",$F27-$G27)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="79"/>
+      <c r="B28" s="80" t="str">
+        <f aca="false">IF($A28="","",($A28-$B$6)/365.25)</f>
+        <v/>
+      </c>
+      <c r="C28" s="68"/>
+      <c r="D28" s="81" t="str">
+        <f aca="false">IF($A28="","",$B$7*(1+$B$15)^$B28)</f>
+        <v/>
+      </c>
+      <c r="E28" s="82" t="str">
+        <f aca="false">IF(OR($A28="",$C28=""),"",$C28-$D28)</f>
+        <v/>
+      </c>
+      <c r="F28" s="83"/>
+      <c r="G28" s="81" t="str">
+        <f aca="false">IF($A28="","",$B$10*(1+$B$15)^$B28)</f>
+        <v/>
+      </c>
+      <c r="H28" s="84" t="str">
+        <f aca="false">IF(OR($A28="",$F28=""),"",$F28-$G28)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="79"/>
+      <c r="B29" s="80" t="str">
+        <f aca="false">IF($A29="","",($A29-$B$6)/365.25)</f>
+        <v/>
+      </c>
+      <c r="C29" s="68"/>
+      <c r="D29" s="81" t="str">
+        <f aca="false">IF($A29="","",$B$7*(1+$B$15)^$B29)</f>
+        <v/>
+      </c>
+      <c r="E29" s="82" t="str">
+        <f aca="false">IF(OR($A29="",$C29=""),"",$C29-$D29)</f>
+        <v/>
+      </c>
+      <c r="F29" s="83"/>
+      <c r="G29" s="81" t="str">
+        <f aca="false">IF($A29="","",$B$10*(1+$B$15)^$B29)</f>
+        <v/>
+      </c>
+      <c r="H29" s="84" t="str">
+        <f aca="false">IF(OR($A29="",$F29=""),"",$F29-$G29)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="79"/>
+      <c r="B30" s="80" t="str">
+        <f aca="false">IF($A30="","",($A30-$B$6)/365.25)</f>
+        <v/>
+      </c>
+      <c r="C30" s="68"/>
+      <c r="D30" s="81" t="str">
+        <f aca="false">IF($A30="","",$B$7*(1+$B$15)^$B30)</f>
+        <v/>
+      </c>
+      <c r="E30" s="82" t="str">
+        <f aca="false">IF(OR($A30="",$C30=""),"",$C30-$D30)</f>
+        <v/>
+      </c>
+      <c r="F30" s="83"/>
+      <c r="G30" s="81" t="str">
+        <f aca="false">IF($A30="","",$B$10*(1+$B$15)^$B30)</f>
+        <v/>
+      </c>
+      <c r="H30" s="84" t="str">
+        <f aca="false">IF(OR($A30="",$F30=""),"",$F30-$G30)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="85" t="s">
+        <v>228</v>
+      </c>
+      <c r="B32" s="85"/>
+      <c r="C32" s="85"/>
+      <c r="D32" s="85"/>
+      <c r="E32" s="85"/>
+      <c r="F32" s="85"/>
+      <c r="G32" s="85"/>
+      <c r="H32" s="85"/>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="85"/>
+      <c r="B33" s="85"/>
+      <c r="C33" s="85"/>
+      <c r="D33" s="85"/>
+      <c r="E33" s="85"/>
+      <c r="F33" s="85"/>
+      <c r="G33" s="85"/>
+      <c r="H33" s="85"/>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="85"/>
+      <c r="B34" s="85"/>
+      <c r="C34" s="85"/>
+      <c r="D34" s="85"/>
+      <c r="E34" s="85"/>
+      <c r="F34" s="85"/>
+      <c r="G34" s="85"/>
+      <c r="H34" s="85"/>
+    </row>
+  </sheetData>
+  <mergeCells count="16">
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A4:H4"/>
+    <mergeCell ref="D5:H5"/>
+    <mergeCell ref="D6:H6"/>
+    <mergeCell ref="D7:H7"/>
+    <mergeCell ref="D8:H8"/>
+    <mergeCell ref="D9:H9"/>
+    <mergeCell ref="D10:H10"/>
+    <mergeCell ref="A12:H12"/>
+    <mergeCell ref="D13:H13"/>
+    <mergeCell ref="D14:H14"/>
+    <mergeCell ref="D15:H15"/>
+    <mergeCell ref="A17:H17"/>
+    <mergeCell ref="A23:H23"/>
+    <mergeCell ref="A32:H34"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
AML: desglose real Papá/Mamá en Planes de Pensiones, total por fórmula; corregir duplicado stale en restricciones fiscales; total Acciones por fórmula
</commit_message>
<xml_diff>
--- a/data/raw/personal_capacity_facts.xlsx
+++ b/data/raw/personal_capacity_facts.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="Notas" sheetId="1" state="visible" r:id="rId3"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="435" uniqueCount="229">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="440" uniqueCount="234">
   <si>
     <t xml:space="preserve">PERSONAL CAPACITY FACTS — Notas de uso</t>
   </si>
@@ -404,13 +404,13 @@
     <t xml:space="preserve">Fondos RV</t>
   </si>
   <si>
-    <t xml:space="preserve">Planes de Pensiones (Papá 754.162,54 + Mamá 403.356,58)</t>
+    <t xml:space="preserve">Planes de Pensiones (Papá + Mamá)</t>
   </si>
   <si>
     <t xml:space="preserve">Excluidos de liquidez/pólvora seca — ver sección 6</t>
   </si>
   <si>
-    <t xml:space="preserve">Acciones (Iberdrola 356.040 + BBVA 125.804,4 + TEF 56.169,35)</t>
+    <t xml:space="preserve">Acciones (Iberdrola + BBVA + TEF)</t>
   </si>
   <si>
     <t xml:space="preserve">ETF (Aristócratas)</t>
@@ -456,6 +456,21 @@
   </si>
   <si>
     <t xml:space="preserve">% TEF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Concentración dentro de Planes de Pensiones</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Papá</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mamá</t>
+  </si>
+  <si>
+    <t xml:space="preserve">% Papá</t>
+  </si>
+  <si>
+    <t xml:space="preserve">% Mamá</t>
   </si>
   <si>
     <t xml:space="preserve">Confirmado 2026-08-10 -- foco en USA/SP500 es la tesis de partida del SOP, no un riesgo a corregir. Verificado en '02. Fondos Myinvestor': Vanguard US500 87,2% + Fidelity S&amp;P500 0,4% (mismo índice, dos proveedores) + iShares Developed World 4,0%. Iberdrola 66% de la sub-cartera de Acciones mas solo 8,4% del patrimonio total, con función de renta vía dividendos, no de crecimiento</t>
@@ -725,7 +740,7 @@
     <numFmt numFmtId="168" formatCode="dd/mm/yyyy"/>
     <numFmt numFmtId="169" formatCode="0.00"/>
   </numFmts>
-  <fonts count="26">
+  <fonts count="20">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -780,6 +795,12 @@
       <i val="true"/>
       <sz val="9"/>
       <color rgb="FF666666"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
       <charset val="1"/>
@@ -848,64 +869,10 @@
     </font>
     <font>
       <b val="true"/>
-      <sz val="13"/>
-      <color rgb="FF1F1F1F"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <i val="true"/>
-      <sz val="9"/>
-      <color rgb="FF808080"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="10"/>
-      <color rgb="FF1F1F1F"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF1F1F1F"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <b val="true"/>
       <sz val="10"/>
       <color rgb="FF1155CC"/>
       <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="8.5"/>
-      <color rgb="FF9E9E9E"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <i val="true"/>
-      <sz val="8.5"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="Arial"/>
-      <family val="0"/>
+      <family val="2"/>
       <charset val="1"/>
     </font>
     <font>
@@ -913,7 +880,7 @@
       <sz val="10.5"/>
       <color rgb="FF1F1F1F"/>
       <name val="Arial"/>
-      <family val="0"/>
+      <family val="2"/>
       <charset val="1"/>
     </font>
   </fonts>
@@ -1107,7 +1074,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="86">
+  <cellXfs count="82">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1180,276 +1147,260 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="165" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="167" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="13" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="14" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="6" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="14" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="7" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="12" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="13" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="12" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="13" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="8" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="8" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="14" fillId="8" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="14" fillId="8" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="8" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="8" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="9" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="9" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="13" fillId="9" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="13" fillId="9" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="10" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="10" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="14" fillId="10" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="10" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="10" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="11" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="11" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="13" fillId="11" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="13" fillId="11" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="12" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="16" fillId="12" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="16" fillId="12" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="12" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="8" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="10" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="18" fillId="13" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="18" fillId="13" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="19" fillId="8" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="18" fillId="13" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="3" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="3" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="13" fillId="8" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="13" fillId="8" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="8" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="14" fillId="8" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="9" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="9" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="12" fillId="9" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="12" fillId="9" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="10" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="10" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="13" fillId="10" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="10" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="14" fillId="10" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="11" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="11" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="12" fillId="11" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="12" fillId="11" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="12" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="15" fillId="12" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="15" fillId="12" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="12" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="16" fillId="8" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="16" fillId="10" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="20" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="21" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="22" fillId="13" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="23" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="24" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="22" fillId="13" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="20" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="25" fillId="8" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="22" fillId="13" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="20" fillId="3" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="20" fillId="3" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="20" fillId="8" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="168" fontId="0" fillId="8" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="21" fillId="8" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="14" fillId="8" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="21" fillId="8" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="14" fillId="8" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="21" fillId="8" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="18" fillId="13" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="14" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="14" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="22" fillId="13" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="169" fontId="21" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="21" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="19" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="25" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="18" fillId="13" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="22" fillId="13" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="19" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="25" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -2580,10 +2531,10 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D73"/>
+  <dimension ref="A1:D79"/>
   <sheetFormatPr defaultColWidth="8.66796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="57.33"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="30"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="50"/>
@@ -3034,8 +2985,9 @@
       <c r="A40" s="4" t="s">
         <v>126</v>
       </c>
-      <c r="B40" s="9" t="n">
-        <v>1158833</v>
+      <c r="B40" s="18" t="n">
+        <f aca="false">B60+B61</f>
+        <v>1158832</v>
       </c>
       <c r="C40" s="10" t="s">
         <v>112</v>
@@ -3048,8 +3000,9 @@
       <c r="A41" s="4" t="s">
         <v>128</v>
       </c>
-      <c r="B41" s="9" t="n">
-        <v>538013.75</v>
+      <c r="B41" s="18" t="n">
+        <f aca="false">SUM(B52:B54)</f>
+        <v>531793.35</v>
       </c>
       <c r="C41" s="10" t="s">
         <v>112</v>
@@ -3088,7 +3041,7 @@
       </c>
       <c r="B44" s="15" t="n">
         <f aca="false">SUM(B39:B43)</f>
-        <v>4232262.25</v>
+        <v>4226040.85</v>
       </c>
       <c r="C44" s="16" t="s">
         <v>36</v>
@@ -3101,7 +3054,7 @@
       </c>
       <c r="B45" s="13" t="n">
         <f aca="false">B39/B44</f>
-        <v>0.519034235177652</v>
+        <v>0.519798335598199</v>
       </c>
       <c r="C45" s="10" t="s">
         <v>36</v>
@@ -3114,7 +3067,7 @@
       </c>
       <c r="B46" s="13" t="n">
         <f aca="false">B40/B44</f>
-        <v>0.273809355741129</v>
+        <v>0.274212209756562</v>
       </c>
       <c r="C46" s="10" t="s">
         <v>36</v>
@@ -3127,7 +3080,7 @@
       </c>
       <c r="B47" s="13" t="n">
         <f aca="false">B41/B44</f>
-        <v>0.127122025578637</v>
+        <v>0.125837247881785</v>
       </c>
       <c r="C47" s="10" t="s">
         <v>36</v>
@@ -3140,7 +3093,7 @@
       </c>
       <c r="B48" s="13" t="n">
         <f aca="false">B42/B44</f>
-        <v>0.0329260078342262</v>
+        <v>0.03297448012127</v>
       </c>
       <c r="C48" s="10" t="s">
         <v>36</v>
@@ -3153,7 +3106,7 @@
       </c>
       <c r="B49" s="13" t="n">
         <f aca="false">B43/B44</f>
-        <v>0.0471083756683556</v>
+        <v>0.0471777266421833</v>
       </c>
       <c r="C49" s="10" t="s">
         <v>36</v>
@@ -3170,7 +3123,7 @@
         <v>137</v>
       </c>
       <c r="B52" s="9" t="n">
-        <v>356040</v>
+        <v>348644</v>
       </c>
       <c r="C52" s="10" t="s">
         <v>138</v>
@@ -3182,7 +3135,7 @@
         <v>139</v>
       </c>
       <c r="B53" s="9" t="n">
-        <v>125804.4</v>
+        <v>126980</v>
       </c>
       <c r="C53" s="10" t="s">
         <v>138</v>
@@ -3207,7 +3160,7 @@
       </c>
       <c r="B55" s="13" t="n">
         <f aca="false">B52/B41</f>
-        <v>0.661767473414945</v>
+        <v>0.655600526031399</v>
       </c>
       <c r="C55" s="10" t="s">
         <v>36</v>
@@ -3220,7 +3173,7 @@
       </c>
       <c r="B56" s="13" t="n">
         <f aca="false">B53/B41</f>
-        <v>0.233831198552082</v>
+        <v>0.238776961013145</v>
       </c>
       <c r="C56" s="10" t="s">
         <v>36</v>
@@ -3233,181 +3186,224 @@
       </c>
       <c r="B57" s="13" t="n">
         <f aca="false">B54/B41</f>
-        <v>0.104401328032973</v>
+        <v>0.105622512955455</v>
       </c>
       <c r="C57" s="10" t="s">
         <v>36</v>
       </c>
       <c r="D57" s="12"/>
     </row>
-    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A58" s="4" t="s">
-        <v>90</v>
-      </c>
-      <c r="B58" s="5" t="s">
-        <v>75</v>
-      </c>
-      <c r="C58" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="D58" s="10" t="s">
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A59" s="3" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A60" s="6" t="s">
-        <v>92</v>
-      </c>
-      <c r="B60" s="7"/>
-      <c r="C60" s="7"/>
-      <c r="D60" s="7"/>
+      <c r="A60" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="B60" s="9" t="n">
+        <v>755018</v>
+      </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A61" s="8" t="s">
-        <v>26</v>
-      </c>
-      <c r="B61" s="8" t="s">
-        <v>27</v>
-      </c>
-      <c r="C61" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="D61" s="8" t="s">
-        <v>29</v>
+      <c r="A61" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="B61" s="9" t="n">
+        <v>403814</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="4" t="s">
-        <v>145</v>
-      </c>
-      <c r="B62" s="5" t="s">
-        <v>146</v>
-      </c>
-      <c r="C62" s="10" t="s">
         <v>147</v>
       </c>
-      <c r="D62" s="10" t="s">
-        <v>148</v>
+      <c r="B62" s="13" t="n">
+        <f aca="false">B60/B40</f>
+        <v>0.651533613155315</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="B63" s="13" t="n">
+        <f aca="false">B61/B40</f>
+        <v>0.348466386844685</v>
+      </c>
+    </row>
+    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A64" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="B64" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="C64" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="D64" s="10" t="s">
         <v>149</v>
       </c>
-      <c r="B63" s="18" t="n">
+    </row>
+    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A66" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="B66" s="7"/>
+      <c r="C66" s="7"/>
+      <c r="D66" s="7"/>
+    </row>
+    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A67" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="B67" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="C67" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="D67" s="8" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A68" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="B68" s="5" t="s">
+        <v>151</v>
+      </c>
+      <c r="C68" s="10" t="s">
+        <v>152</v>
+      </c>
+      <c r="D68" s="10" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A69" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="B69" s="19" t="n">
         <f aca="true">DATE(2026,9,29)-TODAY()</f>
         <v>46</v>
       </c>
-      <c r="C63" s="10" t="s">
+      <c r="C69" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="D63" s="12"/>
-    </row>
-    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A64" s="4" t="s">
-        <v>150</v>
-      </c>
-      <c r="B64" s="5" t="s">
-        <v>151</v>
-      </c>
-      <c r="C64" s="10" t="s">
-        <v>147</v>
-      </c>
-      <c r="D64" s="10" t="s">
+      <c r="D69" s="12"/>
+    </row>
+    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A70" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="B70" s="5" t="s">
+        <v>156</v>
+      </c>
+      <c r="C70" s="10" t="s">
         <v>152</v>
       </c>
-    </row>
-    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A65" s="4" t="s">
-        <v>149</v>
-      </c>
-      <c r="B65" s="18" t="n">
+      <c r="D70" s="10" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="71" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A71" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="B71" s="19" t="n">
         <f aca="true">DATE(2026,8,26)-TODAY()</f>
         <v>12</v>
       </c>
-      <c r="C65" s="10" t="s">
+      <c r="C71" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="D65" s="10" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A67" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="B67" s="5" t="s">
-        <v>97</v>
-      </c>
-      <c r="C67" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="D67" s="10" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A69" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="B69" s="7"/>
-      <c r="C69" s="7"/>
-      <c r="D69" s="7"/>
-    </row>
-    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A70" s="8" t="s">
-        <v>26</v>
-      </c>
-      <c r="B70" s="8" t="s">
-        <v>27</v>
-      </c>
-      <c r="C70" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="D70" s="8" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="71" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A71" s="4" t="s">
-        <v>155</v>
-      </c>
-      <c r="B71" s="9" t="n">
-        <v>1157519.11</v>
-      </c>
-      <c r="C71" s="10" t="s">
-        <v>31</v>
-      </c>
       <c r="D71" s="10" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A72" s="4" t="s">
-        <v>100</v>
-      </c>
-      <c r="B72" s="9" t="n">
-        <v>-162000</v>
-      </c>
-      <c r="C72" s="10" t="s">
-        <v>157</v>
-      </c>
-      <c r="D72" s="10" t="s">
         <v>158</v>
       </c>
     </row>
+    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A73" s="4" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="B73" s="5" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="C73" s="10" t="s">
         <v>31</v>
       </c>
       <c r="D73" s="10" t="s">
         <v>159</v>
+      </c>
+    </row>
+    <row r="75" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A75" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="B75" s="7"/>
+      <c r="C75" s="7"/>
+      <c r="D75" s="7"/>
+    </row>
+    <row r="76" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A76" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="B76" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="C76" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="D76" s="8" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="77" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A77" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="B77" s="9" t="n">
+        <f aca="false">B40</f>
+        <v>1158832</v>
+      </c>
+      <c r="C77" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="D77" s="10" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="78" customFormat="false" ht="32.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A78" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="B78" s="9" t="n">
+        <v>-162000</v>
+      </c>
+      <c r="C78" s="10" t="s">
+        <v>162</v>
+      </c>
+      <c r="D78" s="10" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="79" customFormat="false" ht="32.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A79" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="B79" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="C79" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="D79" s="10" t="s">
+        <v>164</v>
       </c>
     </row>
   </sheetData>
@@ -3429,446 +3425,447 @@
   <dimension ref="A1:F35"/>
   <sheetFormatPr defaultColWidth="8.66796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="1" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="50"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="20" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="20" width="50.67"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="20" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="20" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="20" width="50"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="7" style="20" width="8.67"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="19" t="s">
-        <v>160</v>
-      </c>
-      <c r="B1" s="19"/>
-      <c r="C1" s="19"/>
-      <c r="D1" s="19"/>
-      <c r="E1" s="19"/>
-      <c r="F1" s="19"/>
+      <c r="A1" s="21" t="s">
+        <v>165</v>
+      </c>
+      <c r="B1" s="21"/>
+      <c r="C1" s="21"/>
+      <c r="D1" s="21"/>
+      <c r="E1" s="21"/>
+      <c r="F1" s="21"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="20" t="s">
-        <v>161</v>
-      </c>
-      <c r="B2" s="20"/>
-      <c r="C2" s="20"/>
-      <c r="D2" s="20"/>
-      <c r="E2" s="20"/>
-      <c r="F2" s="20"/>
+      <c r="A2" s="22" t="s">
+        <v>166</v>
+      </c>
+      <c r="B2" s="22"/>
+      <c r="C2" s="22"/>
+      <c r="D2" s="22"/>
+      <c r="E2" s="22"/>
+      <c r="F2" s="22"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="21" t="s">
-        <v>162</v>
-      </c>
-      <c r="B4" s="21"/>
-      <c r="C4" s="21"/>
-      <c r="D4" s="21"/>
-      <c r="E4" s="21"/>
-      <c r="F4" s="21"/>
+      <c r="A4" s="23" t="s">
+        <v>167</v>
+      </c>
+      <c r="B4" s="23"/>
+      <c r="C4" s="23"/>
+      <c r="D4" s="23"/>
+      <c r="E4" s="23"/>
+      <c r="F4" s="23"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="22" t="s">
-        <v>163</v>
-      </c>
-      <c r="B5" s="22" t="s">
-        <v>164</v>
-      </c>
-      <c r="C5" s="22" t="s">
+      <c r="A5" s="24" t="s">
+        <v>168</v>
+      </c>
+      <c r="B5" s="24" t="s">
+        <v>169</v>
+      </c>
+      <c r="C5" s="24" t="s">
         <v>27</v>
       </c>
-      <c r="D5" s="22" t="s">
-        <v>165</v>
-      </c>
-      <c r="E5" s="22" t="s">
-        <v>166</v>
-      </c>
-      <c r="F5" s="22" t="s">
+      <c r="D5" s="24" t="s">
+        <v>170</v>
+      </c>
+      <c r="E5" s="24" t="s">
+        <v>171</v>
+      </c>
+      <c r="F5" s="24" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="23" t="s">
-        <v>167</v>
-      </c>
-      <c r="B6" s="24" t="str">
+      <c r="A6" s="25" t="s">
+        <v>172</v>
+      </c>
+      <c r="B6" s="26" t="str">
         <f aca="false">AMS!A41</f>
         <v>Fondo Monetario</v>
       </c>
-      <c r="C6" s="25" t="n">
+      <c r="C6" s="27" t="n">
         <f aca="false">AMS!B41</f>
         <v>89230.77</v>
       </c>
-      <c r="D6" s="26"/>
-      <c r="E6" s="27" t="s">
-        <v>168</v>
-      </c>
-      <c r="F6" s="26"/>
+      <c r="D6" s="28"/>
+      <c r="E6" s="29" t="s">
+        <v>173</v>
+      </c>
+      <c r="F6" s="28"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="23"/>
-      <c r="B7" s="24" t="str">
+      <c r="A7" s="25"/>
+      <c r="B7" s="26" t="str">
         <f aca="false">AMS!A44</f>
         <v>Liquidez (excluido FM)</v>
       </c>
-      <c r="C7" s="25" t="n">
+      <c r="C7" s="27" t="n">
         <f aca="false">AMS!B44</f>
         <v>83100</v>
       </c>
-      <c r="D7" s="26"/>
-      <c r="E7" s="27" t="s">
-        <v>169</v>
-      </c>
-      <c r="F7" s="26"/>
+      <c r="D7" s="28"/>
+      <c r="E7" s="29" t="s">
+        <v>174</v>
+      </c>
+      <c r="F7" s="28"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="28"/>
-      <c r="B8" s="29" t="s">
-        <v>170</v>
-      </c>
-      <c r="C8" s="30" t="n">
+      <c r="A8" s="30"/>
+      <c r="B8" s="31" t="s">
+        <v>175</v>
+      </c>
+      <c r="C8" s="32" t="n">
         <f aca="false">SUM(C6:C7)</f>
         <v>172330.77</v>
       </c>
-      <c r="D8" s="31" t="n">
+      <c r="D8" s="33" t="n">
         <f aca="false">C8/C$15</f>
         <v>0.136534752221471</v>
       </c>
-      <c r="E8" s="28"/>
-      <c r="F8" s="28"/>
+      <c r="E8" s="30"/>
+      <c r="F8" s="30"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="32" t="s">
-        <v>171</v>
-      </c>
-      <c r="B9" s="33" t="str">
+      <c r="A9" s="34" t="s">
+        <v>176</v>
+      </c>
+      <c r="B9" s="35" t="str">
         <f aca="false">AMS!A40</f>
         <v>SP500 (fondos indexados)</v>
       </c>
-      <c r="C9" s="34" t="n">
+      <c r="C9" s="36" t="n">
         <f aca="false">AMS!B40</f>
         <v>878274</v>
       </c>
-      <c r="D9" s="35"/>
-      <c r="E9" s="36" t="s">
-        <v>172</v>
-      </c>
-      <c r="F9" s="35"/>
+      <c r="D9" s="37"/>
+      <c r="E9" s="38" t="s">
+        <v>177</v>
+      </c>
+      <c r="F9" s="37"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="37"/>
-      <c r="B10" s="38" t="s">
-        <v>173</v>
-      </c>
-      <c r="C10" s="39" t="n">
+      <c r="A10" s="39"/>
+      <c r="B10" s="40" t="s">
+        <v>178</v>
+      </c>
+      <c r="C10" s="41" t="n">
         <f aca="false">C9</f>
         <v>878274</v>
       </c>
-      <c r="D10" s="40" t="n">
+      <c r="D10" s="42" t="n">
         <f aca="false">C10/C$15</f>
         <v>0.695841624641728</v>
       </c>
-      <c r="E10" s="37"/>
-      <c r="F10" s="37"/>
+      <c r="E10" s="39"/>
+      <c r="F10" s="39"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="41" t="s">
-        <v>174</v>
-      </c>
-      <c r="B11" s="42" t="str">
+      <c r="A11" s="43" t="s">
+        <v>179</v>
+      </c>
+      <c r="B11" s="44" t="str">
         <f aca="false">AMS!A42</f>
         <v>ETF</v>
       </c>
-      <c r="C11" s="43" t="n">
+      <c r="C11" s="45" t="n">
         <f aca="false">AMS!B42</f>
         <v>111570.37</v>
       </c>
-      <c r="D11" s="44"/>
-      <c r="E11" s="45" t="s">
-        <v>175</v>
-      </c>
-      <c r="F11" s="44"/>
+      <c r="D11" s="46"/>
+      <c r="E11" s="47" t="s">
+        <v>180</v>
+      </c>
+      <c r="F11" s="46"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="41"/>
-      <c r="B12" s="42" t="str">
+      <c r="A12" s="43"/>
+      <c r="B12" s="44" t="str">
         <f aca="false">AMS!A43</f>
         <v>Pisos</v>
       </c>
-      <c r="C12" s="43" t="n">
+      <c r="C12" s="45" t="n">
         <f aca="false">AMS!B43</f>
         <v>100000</v>
       </c>
-      <c r="D12" s="44"/>
-      <c r="E12" s="45" t="s">
-        <v>176</v>
-      </c>
-      <c r="F12" s="44"/>
+      <c r="D12" s="46"/>
+      <c r="E12" s="47" t="s">
+        <v>181</v>
+      </c>
+      <c r="F12" s="46"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="46"/>
-      <c r="B13" s="47" t="s">
-        <v>177</v>
-      </c>
-      <c r="C13" s="48" t="n">
+      <c r="A13" s="48"/>
+      <c r="B13" s="49" t="s">
+        <v>182</v>
+      </c>
+      <c r="C13" s="50" t="n">
         <f aca="false">SUM(C11:C12)</f>
         <v>211570.37</v>
       </c>
-      <c r="D13" s="49" t="n">
+      <c r="D13" s="51" t="n">
         <f aca="false">C13/C$15</f>
         <v>0.167623623136802</v>
       </c>
-      <c r="E13" s="46"/>
-      <c r="F13" s="46"/>
+      <c r="E13" s="48"/>
+      <c r="F13" s="48"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="50" t="s">
-        <v>178</v>
-      </c>
-      <c r="B15" s="50"/>
-      <c r="C15" s="51" t="n">
+      <c r="A15" s="52" t="s">
+        <v>183</v>
+      </c>
+      <c r="B15" s="52"/>
+      <c r="C15" s="53" t="n">
         <f aca="false">C8+C10+C13</f>
         <v>1262175.14</v>
       </c>
-      <c r="D15" s="52" t="n">
+      <c r="D15" s="54" t="n">
         <f aca="false">C15/C15</f>
         <v>1</v>
       </c>
-      <c r="E15" s="53"/>
-      <c r="F15" s="53"/>
+      <c r="E15" s="55"/>
+      <c r="F15" s="55"/>
     </row>
     <row r="16" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B16" s="54" t="s">
-        <v>179</v>
-      </c>
-      <c r="C16" s="55" t="n">
+      <c r="B16" s="56" t="s">
+        <v>184</v>
+      </c>
+      <c r="C16" s="57" t="n">
         <f aca="false">C15-AMS!B45</f>
         <v>0</v>
       </c>
-      <c r="F16" s="56" t="s">
-        <v>180</v>
+      <c r="F16" s="58" t="s">
+        <v>185</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="21" t="s">
-        <v>181</v>
-      </c>
-      <c r="B19" s="21"/>
-      <c r="C19" s="21"/>
-      <c r="D19" s="21"/>
-      <c r="E19" s="21"/>
-      <c r="F19" s="21"/>
+      <c r="A19" s="23" t="s">
+        <v>186</v>
+      </c>
+      <c r="B19" s="23"/>
+      <c r="C19" s="23"/>
+      <c r="D19" s="23"/>
+      <c r="E19" s="23"/>
+      <c r="F19" s="23"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="22" t="s">
-        <v>163</v>
-      </c>
-      <c r="B20" s="22" t="s">
-        <v>164</v>
-      </c>
-      <c r="C20" s="22" t="s">
+      <c r="A20" s="24" t="s">
+        <v>168</v>
+      </c>
+      <c r="B20" s="24" t="s">
+        <v>169</v>
+      </c>
+      <c r="C20" s="24" t="s">
         <v>27</v>
       </c>
-      <c r="D20" s="22" t="s">
-        <v>165</v>
-      </c>
-      <c r="E20" s="22" t="s">
-        <v>166</v>
-      </c>
-      <c r="F20" s="22" t="s">
+      <c r="D20" s="24" t="s">
+        <v>170</v>
+      </c>
+      <c r="E20" s="24" t="s">
+        <v>171</v>
+      </c>
+      <c r="F20" s="24" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="23" t="s">
-        <v>167</v>
-      </c>
-      <c r="B21" s="24" t="str">
+      <c r="A21" s="25" t="s">
+        <v>172</v>
+      </c>
+      <c r="B21" s="26" t="str">
         <f aca="false">AML!A43</f>
         <v>Liquidez + Depósitos (excluido FM)</v>
       </c>
-      <c r="C21" s="25" t="n">
+      <c r="C21" s="27" t="n">
         <f aca="false">AML!B43</f>
         <v>199375</v>
       </c>
-      <c r="D21" s="26"/>
-      <c r="E21" s="27" t="s">
-        <v>182</v>
-      </c>
-      <c r="F21" s="26"/>
+      <c r="D21" s="28"/>
+      <c r="E21" s="29" t="s">
+        <v>187</v>
+      </c>
+      <c r="F21" s="28"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="28"/>
-      <c r="B22" s="29" t="s">
-        <v>170</v>
-      </c>
-      <c r="C22" s="30" t="n">
+      <c r="A22" s="30"/>
+      <c r="B22" s="31" t="s">
+        <v>175</v>
+      </c>
+      <c r="C22" s="32" t="n">
         <f aca="false">C21</f>
         <v>199375</v>
       </c>
-      <c r="D22" s="31" t="n">
+      <c r="D22" s="33" t="n">
         <f aca="false">C22/C$30</f>
-        <v>0.0471083756683556</v>
-      </c>
-      <c r="E22" s="28"/>
-      <c r="F22" s="28"/>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="32" t="s">
-        <v>171</v>
-      </c>
-      <c r="B23" s="33" t="str">
+        <v>0.0471777266421833</v>
+      </c>
+      <c r="E22" s="30"/>
+      <c r="F22" s="30"/>
+    </row>
+    <row r="23" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="34" t="s">
+        <v>176</v>
+      </c>
+      <c r="B23" s="35" t="str">
         <f aca="false">AML!A39</f>
         <v>Fondos RV</v>
       </c>
-      <c r="C23" s="34" t="n">
+      <c r="C23" s="36" t="n">
         <f aca="false">AML!B39</f>
         <v>2196689</v>
       </c>
-      <c r="D23" s="35"/>
-      <c r="E23" s="36" t="s">
-        <v>183</v>
-      </c>
-      <c r="F23" s="35"/>
-    </row>
-    <row r="24" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="32"/>
-      <c r="B24" s="33" t="str">
+      <c r="D23" s="37"/>
+      <c r="E23" s="38" t="s">
+        <v>188</v>
+      </c>
+      <c r="F23" s="37"/>
+    </row>
+    <row r="24" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="34"/>
+      <c r="B24" s="35" t="str">
         <f aca="false">AML!A40</f>
-        <v>Planes de Pensiones (Papá 754.162,54 + Mamá 403.356,58)</v>
-      </c>
-      <c r="C24" s="34" t="n">
+        <v>Planes de Pensiones (Papá + Mamá)</v>
+      </c>
+      <c r="C24" s="36" t="n">
         <f aca="false">AML!B40</f>
-        <v>1158833</v>
-      </c>
-      <c r="D24" s="35"/>
-      <c r="E24" s="36" t="s">
-        <v>184</v>
-      </c>
-      <c r="F24" s="57" t="s">
-        <v>185</v>
+        <v>1158832</v>
+      </c>
+      <c r="D24" s="37"/>
+      <c r="E24" s="38" t="s">
+        <v>189</v>
+      </c>
+      <c r="F24" s="59" t="s">
+        <v>190</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="37"/>
-      <c r="B25" s="38" t="s">
-        <v>173</v>
-      </c>
-      <c r="C25" s="39" t="n">
+      <c r="A25" s="39"/>
+      <c r="B25" s="40" t="s">
+        <v>178</v>
+      </c>
+      <c r="C25" s="41" t="n">
         <f aca="false">SUM(C23:C24)</f>
-        <v>3355522</v>
-      </c>
-      <c r="D25" s="40" t="n">
+        <v>3355521</v>
+      </c>
+      <c r="D25" s="42" t="n">
         <f aca="false">C25/C$30</f>
-        <v>0.792843590918781</v>
-      </c>
-      <c r="E25" s="37"/>
-      <c r="F25" s="37"/>
+        <v>0.794010545354762</v>
+      </c>
+      <c r="E25" s="39"/>
+      <c r="F25" s="39"/>
     </row>
     <row r="26" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="41" t="s">
-        <v>174</v>
-      </c>
-      <c r="B26" s="42" t="str">
+      <c r="A26" s="43" t="s">
+        <v>179</v>
+      </c>
+      <c r="B26" s="44" t="str">
         <f aca="false">AML!A41</f>
-        <v>Acciones (Iberdrola 356.040 + BBVA 125.804,4 + TEF 56.169,35)</v>
-      </c>
-      <c r="C26" s="43" t="n">
+        <v>Acciones (Iberdrola + BBVA + TEF)</v>
+      </c>
+      <c r="C26" s="45" t="n">
         <f aca="false">AML!B41</f>
-        <v>538013.75</v>
-      </c>
-      <c r="D26" s="44"/>
-      <c r="E26" s="45" t="s">
-        <v>186</v>
-      </c>
-      <c r="F26" s="58" t="s">
-        <v>187</v>
+        <v>531793.35</v>
+      </c>
+      <c r="D26" s="46"/>
+      <c r="E26" s="47" t="s">
+        <v>191</v>
+      </c>
+      <c r="F26" s="60" t="s">
+        <v>192</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="41"/>
-      <c r="B27" s="42" t="str">
+      <c r="A27" s="43"/>
+      <c r="B27" s="44" t="str">
         <f aca="false">AML!A42</f>
         <v>ETF (Aristócratas)</v>
       </c>
-      <c r="C27" s="43" t="n">
+      <c r="C27" s="45" t="n">
         <f aca="false">AML!B42</f>
         <v>139351.5</v>
       </c>
-      <c r="D27" s="44"/>
-      <c r="E27" s="45" t="s">
-        <v>188</v>
-      </c>
-      <c r="F27" s="44"/>
+      <c r="D27" s="46"/>
+      <c r="E27" s="47" t="s">
+        <v>193</v>
+      </c>
+      <c r="F27" s="46"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="46"/>
-      <c r="B28" s="47" t="s">
-        <v>177</v>
-      </c>
-      <c r="C28" s="48" t="n">
+      <c r="A28" s="48"/>
+      <c r="B28" s="49" t="s">
+        <v>182</v>
+      </c>
+      <c r="C28" s="50" t="n">
         <f aca="false">SUM(C26:C27)</f>
-        <v>677365.25</v>
-      </c>
-      <c r="D28" s="49" t="n">
+        <v>671144.85</v>
+      </c>
+      <c r="D28" s="51" t="n">
         <f aca="false">C28/C$30</f>
-        <v>0.160048033412863</v>
-      </c>
-      <c r="E28" s="46"/>
-      <c r="F28" s="46"/>
+        <v>0.158811728003055</v>
+      </c>
+      <c r="E28" s="48"/>
+      <c r="F28" s="48"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="50" t="s">
-        <v>189</v>
-      </c>
-      <c r="B30" s="50"/>
-      <c r="C30" s="51" t="n">
+      <c r="A30" s="52" t="s">
+        <v>194</v>
+      </c>
+      <c r="B30" s="52"/>
+      <c r="C30" s="53" t="n">
         <f aca="false">C22+C25+C28</f>
-        <v>4232262.25</v>
-      </c>
-      <c r="D30" s="52" t="n">
+        <v>4226040.85</v>
+      </c>
+      <c r="D30" s="54" t="n">
         <f aca="false">C30/C30</f>
         <v>1</v>
       </c>
-      <c r="E30" s="53"/>
-      <c r="F30" s="53"/>
+      <c r="E30" s="55"/>
+      <c r="F30" s="55"/>
     </row>
     <row r="31" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B31" s="54" t="s">
-        <v>179</v>
-      </c>
-      <c r="C31" s="55" t="n">
+      <c r="B31" s="56" t="s">
+        <v>184</v>
+      </c>
+      <c r="C31" s="57" t="n">
         <f aca="false">C30-AML!B44</f>
         <v>0</v>
       </c>
-      <c r="F31" s="56" t="s">
-        <v>180</v>
+      <c r="F31" s="58" t="s">
+        <v>185</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="59" t="s">
-        <v>190</v>
-      </c>
-      <c r="B33" s="59"/>
-      <c r="C33" s="59"/>
-      <c r="D33" s="59"/>
-      <c r="E33" s="59"/>
-      <c r="F33" s="59"/>
+      <c r="A33" s="61" t="s">
+        <v>195</v>
+      </c>
+      <c r="B33" s="61"/>
+      <c r="C33" s="61"/>
+      <c r="D33" s="61"/>
+      <c r="E33" s="61"/>
+      <c r="F33" s="61"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="59"/>
-      <c r="B34" s="59"/>
-      <c r="C34" s="59"/>
-      <c r="D34" s="59"/>
-      <c r="E34" s="59"/>
-      <c r="F34" s="59"/>
+      <c r="A34" s="61"/>
+      <c r="B34" s="61"/>
+      <c r="C34" s="61"/>
+      <c r="D34" s="61"/>
+      <c r="E34" s="61"/>
+      <c r="F34" s="61"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="59"/>
-      <c r="B35" s="59"/>
-      <c r="C35" s="59"/>
-      <c r="D35" s="59"/>
-      <c r="E35" s="59"/>
-      <c r="F35" s="59"/>
+      <c r="A35" s="61"/>
+      <c r="B35" s="61"/>
+      <c r="C35" s="61"/>
+      <c r="D35" s="61"/>
+      <c r="E35" s="61"/>
+      <c r="F35" s="61"/>
     </row>
   </sheetData>
   <mergeCells count="11">
@@ -3900,551 +3897,552 @@
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:H34"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.66796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="2" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="20" width="42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="2" style="20" width="16"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="9" style="20" width="8.67"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="60" t="s">
-        <v>191</v>
-      </c>
-      <c r="B1" s="60"/>
-      <c r="C1" s="60"/>
-      <c r="D1" s="60"/>
-      <c r="E1" s="60"/>
-      <c r="F1" s="60"/>
-      <c r="G1" s="60"/>
-      <c r="H1" s="60"/>
+      <c r="A1" s="21" t="s">
+        <v>196</v>
+      </c>
+      <c r="B1" s="21"/>
+      <c r="C1" s="21"/>
+      <c r="D1" s="21"/>
+      <c r="E1" s="21"/>
+      <c r="F1" s="21"/>
+      <c r="G1" s="21"/>
+      <c r="H1" s="21"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="61" t="s">
-        <v>192</v>
-      </c>
-      <c r="B2" s="61"/>
-      <c r="C2" s="61"/>
-      <c r="D2" s="61"/>
-      <c r="E2" s="61"/>
-      <c r="F2" s="61"/>
-      <c r="G2" s="61"/>
-      <c r="H2" s="61"/>
+      <c r="A2" s="22" t="s">
+        <v>197</v>
+      </c>
+      <c r="B2" s="22"/>
+      <c r="C2" s="22"/>
+      <c r="D2" s="22"/>
+      <c r="E2" s="22"/>
+      <c r="F2" s="22"/>
+      <c r="G2" s="22"/>
+      <c r="H2" s="22"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="62" t="s">
-        <v>193</v>
-      </c>
-      <c r="B4" s="62"/>
-      <c r="C4" s="62"/>
-      <c r="D4" s="62"/>
-      <c r="E4" s="62"/>
-      <c r="F4" s="62"/>
-      <c r="G4" s="62"/>
-      <c r="H4" s="62"/>
+      <c r="A4" s="23" t="s">
+        <v>198</v>
+      </c>
+      <c r="B4" s="23"/>
+      <c r="C4" s="23"/>
+      <c r="D4" s="23"/>
+      <c r="E4" s="23"/>
+      <c r="F4" s="23"/>
+      <c r="G4" s="23"/>
+      <c r="H4" s="23"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="63" t="s">
+      <c r="A5" s="24" t="s">
         <v>26</v>
       </c>
-      <c r="B5" s="63" t="s">
+      <c r="B5" s="24" t="s">
         <v>27</v>
       </c>
-      <c r="C5" s="63" t="s">
+      <c r="C5" s="24" t="s">
         <v>28</v>
       </c>
-      <c r="D5" s="63" t="s">
+      <c r="D5" s="24" t="s">
         <v>29</v>
       </c>
-      <c r="E5" s="63"/>
-      <c r="F5" s="63"/>
-      <c r="G5" s="63"/>
-      <c r="H5" s="63"/>
+      <c r="E5" s="24"/>
+      <c r="F5" s="24"/>
+      <c r="G5" s="24"/>
+      <c r="H5" s="24"/>
     </row>
     <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="64" t="s">
-        <v>194</v>
-      </c>
-      <c r="B6" s="65" t="n">
+      <c r="A6" s="62" t="s">
+        <v>199</v>
+      </c>
+      <c r="B6" s="63" t="n">
         <v>46247</v>
       </c>
-      <c r="C6" s="66" t="s">
+      <c r="C6" s="64" t="s">
         <v>31</v>
       </c>
-      <c r="D6" s="67" t="s">
-        <v>195</v>
-      </c>
-      <c r="E6" s="67"/>
-      <c r="F6" s="67"/>
-      <c r="G6" s="67"/>
-      <c r="H6" s="67"/>
+      <c r="D6" s="65" t="s">
+        <v>200</v>
+      </c>
+      <c r="E6" s="65"/>
+      <c r="F6" s="65"/>
+      <c r="G6" s="65"/>
+      <c r="H6" s="65"/>
     </row>
     <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="64" t="s">
-        <v>196</v>
-      </c>
-      <c r="B7" s="68" t="n">
+      <c r="A7" s="62" t="s">
+        <v>201</v>
+      </c>
+      <c r="B7" s="66" t="n">
         <v>878274</v>
       </c>
-      <c r="C7" s="66" t="s">
+      <c r="C7" s="64" t="s">
         <v>31</v>
       </c>
-      <c r="D7" s="67" t="s">
-        <v>197</v>
-      </c>
-      <c r="E7" s="67"/>
-      <c r="F7" s="67"/>
-      <c r="G7" s="67"/>
-      <c r="H7" s="67"/>
+      <c r="D7" s="65" t="s">
+        <v>202</v>
+      </c>
+      <c r="E7" s="65"/>
+      <c r="F7" s="65"/>
+      <c r="G7" s="65"/>
+      <c r="H7" s="65"/>
     </row>
     <row r="8" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="64" t="s">
-        <v>198</v>
-      </c>
-      <c r="B8" s="68" t="n">
+      <c r="A8" s="62" t="s">
+        <v>203</v>
+      </c>
+      <c r="B8" s="66" t="n">
         <v>2196689</v>
       </c>
-      <c r="C8" s="66" t="s">
+      <c r="C8" s="64" t="s">
         <v>31</v>
       </c>
-      <c r="D8" s="67" t="s">
-        <v>199</v>
-      </c>
-      <c r="E8" s="67"/>
-      <c r="F8" s="67"/>
-      <c r="G8" s="67"/>
-      <c r="H8" s="67"/>
+      <c r="D8" s="65" t="s">
+        <v>204</v>
+      </c>
+      <c r="E8" s="65"/>
+      <c r="F8" s="65"/>
+      <c r="G8" s="65"/>
+      <c r="H8" s="65"/>
     </row>
     <row r="9" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="64" t="s">
-        <v>200</v>
-      </c>
-      <c r="B9" s="68" t="n">
+      <c r="A9" s="62" t="s">
+        <v>205</v>
+      </c>
+      <c r="B9" s="66" t="n">
         <v>1158833</v>
       </c>
-      <c r="C9" s="66" t="s">
+      <c r="C9" s="64" t="s">
         <v>31</v>
       </c>
-      <c r="D9" s="67" t="s">
-        <v>201</v>
-      </c>
-      <c r="E9" s="67"/>
-      <c r="F9" s="67"/>
-      <c r="G9" s="67"/>
-      <c r="H9" s="67"/>
+      <c r="D9" s="65" t="s">
+        <v>206</v>
+      </c>
+      <c r="E9" s="65"/>
+      <c r="F9" s="65"/>
+      <c r="G9" s="65"/>
+      <c r="H9" s="65"/>
     </row>
     <row r="10" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="69" t="s">
-        <v>202</v>
-      </c>
-      <c r="B10" s="70" t="n">
+      <c r="A10" s="67" t="s">
+        <v>207</v>
+      </c>
+      <c r="B10" s="68" t="n">
         <f aca="false">B8+B9</f>
         <v>3355522</v>
       </c>
-      <c r="C10" s="66" t="s">
+      <c r="C10" s="64" t="s">
         <v>36</v>
       </c>
-      <c r="D10" s="67" t="s">
-        <v>203</v>
-      </c>
-      <c r="E10" s="67"/>
-      <c r="F10" s="67"/>
-      <c r="G10" s="67"/>
-      <c r="H10" s="67"/>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="62" t="s">
-        <v>204</v>
-      </c>
-      <c r="B12" s="62"/>
-      <c r="C12" s="62"/>
-      <c r="D12" s="62"/>
-      <c r="E12" s="62"/>
-      <c r="F12" s="62"/>
-      <c r="G12" s="62"/>
-      <c r="H12" s="62"/>
+      <c r="D10" s="65" t="s">
+        <v>208</v>
+      </c>
+      <c r="E10" s="65"/>
+      <c r="F10" s="65"/>
+      <c r="G10" s="65"/>
+      <c r="H10" s="65"/>
+    </row>
+    <row r="12" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="23" t="s">
+        <v>209</v>
+      </c>
+      <c r="B12" s="23"/>
+      <c r="C12" s="23"/>
+      <c r="D12" s="23"/>
+      <c r="E12" s="23"/>
+      <c r="F12" s="23"/>
+      <c r="G12" s="23"/>
+      <c r="H12" s="23"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="63" t="s">
+      <c r="A13" s="24" t="s">
         <v>26</v>
       </c>
-      <c r="B13" s="63" t="s">
+      <c r="B13" s="24" t="s">
         <v>27</v>
       </c>
-      <c r="C13" s="63" t="s">
+      <c r="C13" s="24" t="s">
         <v>28</v>
       </c>
-      <c r="D13" s="63" t="s">
+      <c r="D13" s="24" t="s">
         <v>29</v>
       </c>
-      <c r="E13" s="63"/>
-      <c r="F13" s="63"/>
-      <c r="G13" s="63"/>
-      <c r="H13" s="63"/>
+      <c r="E13" s="24"/>
+      <c r="F13" s="24"/>
+      <c r="G13" s="24"/>
+      <c r="H13" s="24"/>
     </row>
     <row r="14" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="64" t="s">
-        <v>205</v>
-      </c>
-      <c r="B14" s="71" t="n">
+      <c r="A14" s="62" t="s">
+        <v>210</v>
+      </c>
+      <c r="B14" s="69" t="n">
         <v>0.07</v>
       </c>
-      <c r="C14" s="66" t="s">
+      <c r="C14" s="64" t="s">
         <v>31</v>
       </c>
-      <c r="D14" s="67" t="s">
-        <v>206</v>
-      </c>
-      <c r="E14" s="67"/>
-      <c r="F14" s="67"/>
-      <c r="G14" s="67"/>
-      <c r="H14" s="67"/>
+      <c r="D14" s="65" t="s">
+        <v>211</v>
+      </c>
+      <c r="E14" s="65"/>
+      <c r="F14" s="65"/>
+      <c r="G14" s="65"/>
+      <c r="H14" s="65"/>
     </row>
     <row r="15" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="64" t="s">
-        <v>207</v>
-      </c>
-      <c r="B15" s="71" t="n">
+      <c r="A15" s="62" t="s">
+        <v>212</v>
+      </c>
+      <c r="B15" s="69" t="n">
         <v>0.094</v>
       </c>
-      <c r="C15" s="66" t="s">
+      <c r="C15" s="64" t="s">
         <v>31</v>
       </c>
-      <c r="D15" s="67" t="s">
-        <v>208</v>
-      </c>
-      <c r="E15" s="67"/>
-      <c r="F15" s="67"/>
-      <c r="G15" s="67"/>
-      <c r="H15" s="67"/>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="62" t="s">
-        <v>209</v>
-      </c>
-      <c r="B17" s="62"/>
-      <c r="C17" s="62"/>
-      <c r="D17" s="62"/>
-      <c r="E17" s="62"/>
-      <c r="F17" s="62"/>
-      <c r="G17" s="62"/>
-      <c r="H17" s="62"/>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="63" t="s">
-        <v>210</v>
-      </c>
-      <c r="B18" s="63" t="s">
-        <v>211</v>
-      </c>
-      <c r="C18" s="63" t="s">
-        <v>212</v>
-      </c>
-      <c r="D18" s="72" t="s">
+      <c r="D15" s="65" t="s">
         <v>213</v>
       </c>
-      <c r="E18" s="73" t="s">
+      <c r="E15" s="65"/>
+      <c r="F15" s="65"/>
+      <c r="G15" s="65"/>
+      <c r="H15" s="65"/>
+    </row>
+    <row r="17" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="23" t="s">
         <v>214</v>
       </c>
-      <c r="F18" s="63" t="s">
+      <c r="B17" s="23"/>
+      <c r="C17" s="23"/>
+      <c r="D17" s="23"/>
+      <c r="E17" s="23"/>
+      <c r="F17" s="23"/>
+      <c r="G17" s="23"/>
+      <c r="H17" s="23"/>
+    </row>
+    <row r="18" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="24" t="s">
         <v>215</v>
       </c>
-      <c r="G18" s="63"/>
-      <c r="H18" s="63"/>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="74" t="s">
+      <c r="B18" s="24" t="s">
         <v>216</v>
       </c>
-      <c r="B19" s="75" t="n">
+      <c r="C18" s="24" t="s">
+        <v>217</v>
+      </c>
+      <c r="D18" s="70" t="s">
+        <v>218</v>
+      </c>
+      <c r="E18" s="71" t="s">
+        <v>219</v>
+      </c>
+      <c r="F18" s="24" t="s">
+        <v>220</v>
+      </c>
+      <c r="G18" s="24"/>
+      <c r="H18" s="24"/>
+    </row>
+    <row r="19" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="72" t="s">
+        <v>221</v>
+      </c>
+      <c r="B19" s="73" t="n">
         <f aca="false">DATE(YEAR($B$6)+5,MONTH($B$6),DAY($B$6))</f>
         <v>48073</v>
       </c>
-      <c r="C19" s="76" t="n">
+      <c r="C19" s="36" t="n">
         <f aca="false">$B$7*(1+$B$14)^5</f>
         <v>1231824.71872881</v>
       </c>
-      <c r="D19" s="77" t="n">
+      <c r="D19" s="74" t="n">
         <f aca="false">$B$7*(1+$B$15)^5</f>
         <v>1376311.17540442</v>
       </c>
-      <c r="E19" s="78" t="n">
+      <c r="E19" s="75" t="n">
         <f aca="false">$B$10*(1+$B$14)^5</f>
         <v>4706293.18850193</v>
       </c>
-      <c r="F19" s="76" t="n">
+      <c r="F19" s="36" t="n">
         <f aca="false">$B$10*(1+$B$15)^5</f>
         <v>5258316.22923529</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="74" t="s">
-        <v>217</v>
-      </c>
-      <c r="B20" s="75" t="n">
+    <row r="20" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="72" t="s">
+        <v>222</v>
+      </c>
+      <c r="B20" s="73" t="n">
         <f aca="false">DATE(YEAR($B$6)+10,MONTH($B$6),DAY($B$6))</f>
         <v>49900</v>
       </c>
-      <c r="C20" s="76" t="n">
+      <c r="C20" s="36" t="n">
         <f aca="false">$B$7*(1+$B$14)^10</f>
         <v>1727697.89117214</v>
       </c>
-      <c r="D20" s="77" t="n">
+      <c r="D20" s="74" t="n">
         <f aca="false">$B$7*(1+$B$15)^10</f>
         <v>2156767.08127885</v>
       </c>
-      <c r="E20" s="78" t="n">
+      <c r="E20" s="75" t="n">
         <f aca="false">$B$10*(1+$B$14)^10</f>
         <v>6600819.656715</v>
       </c>
-      <c r="F20" s="76" t="n">
+      <c r="F20" s="36" t="n">
         <f aca="false">$B$10*(1+$B$15)^10</f>
         <v>8240115.71571852</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="74" t="s">
-        <v>218</v>
-      </c>
-      <c r="B21" s="75" t="n">
+    <row r="21" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="72" t="s">
+        <v>223</v>
+      </c>
+      <c r="B21" s="73" t="n">
         <f aca="false">DATE(YEAR($B$6)+15,MONTH($B$6),DAY($B$6))</f>
         <v>51726</v>
       </c>
-      <c r="C21" s="76" t="n">
+      <c r="C21" s="36" t="n">
         <f aca="false">$B$7*(1+$B$14)^15</f>
         <v>2423185.66739022</v>
       </c>
-      <c r="D21" s="77" t="n">
+      <c r="D21" s="74" t="n">
         <f aca="false">$B$7*(1+$B$15)^15</f>
         <v>3379791.08650428</v>
       </c>
-      <c r="E21" s="78" t="n">
+      <c r="E21" s="75" t="n">
         <f aca="false">$B$10*(1+$B$14)^15</f>
         <v>9257991.03356421</v>
       </c>
-      <c r="F21" s="76" t="n">
+      <c r="F21" s="36" t="n">
         <f aca="false">$B$10*(1+$B$15)^15</f>
         <v>12912785.0148917</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="62" t="s">
-        <v>219</v>
-      </c>
-      <c r="B23" s="62"/>
-      <c r="C23" s="62"/>
-      <c r="D23" s="62"/>
-      <c r="E23" s="62"/>
-      <c r="F23" s="62"/>
-      <c r="G23" s="62"/>
-      <c r="H23" s="62"/>
+    <row r="23" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="23" t="s">
+        <v>224</v>
+      </c>
+      <c r="B23" s="23"/>
+      <c r="C23" s="23"/>
+      <c r="D23" s="23"/>
+      <c r="E23" s="23"/>
+      <c r="F23" s="23"/>
+      <c r="G23" s="23"/>
+      <c r="H23" s="23"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="63" t="s">
-        <v>220</v>
-      </c>
-      <c r="B24" s="63" t="s">
-        <v>221</v>
-      </c>
-      <c r="C24" s="63" t="s">
-        <v>222</v>
-      </c>
-      <c r="D24" s="63" t="s">
-        <v>223</v>
-      </c>
-      <c r="E24" s="72" t="s">
-        <v>224</v>
-      </c>
-      <c r="F24" s="73" t="s">
+      <c r="A24" s="24" t="s">
         <v>225</v>
       </c>
-      <c r="G24" s="63" t="s">
+      <c r="B24" s="24" t="s">
         <v>226</v>
       </c>
-      <c r="H24" s="63" t="s">
+      <c r="C24" s="24" t="s">
         <v>227</v>
       </c>
+      <c r="D24" s="24" t="s">
+        <v>228</v>
+      </c>
+      <c r="E24" s="70" t="s">
+        <v>229</v>
+      </c>
+      <c r="F24" s="71" t="s">
+        <v>230</v>
+      </c>
+      <c r="G24" s="24" t="s">
+        <v>231</v>
+      </c>
+      <c r="H24" s="24" t="s">
+        <v>232</v>
+      </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="79"/>
-      <c r="B25" s="80" t="str">
+      <c r="A25" s="76"/>
+      <c r="B25" s="77" t="str">
         <f aca="false">IF($A25="","",($A25-$B$6)/365.25)</f>
         <v/>
       </c>
-      <c r="C25" s="68"/>
-      <c r="D25" s="81" t="str">
+      <c r="C25" s="66"/>
+      <c r="D25" s="78" t="str">
         <f aca="false">IF($A25="","",$B$7*(1+$B$15)^$B25)</f>
         <v/>
       </c>
-      <c r="E25" s="82" t="str">
+      <c r="E25" s="79" t="str">
         <f aca="false">IF(OR($A25="",$C25=""),"",$C25-$D25)</f>
         <v/>
       </c>
-      <c r="F25" s="83"/>
-      <c r="G25" s="81" t="str">
+      <c r="F25" s="80"/>
+      <c r="G25" s="78" t="str">
         <f aca="false">IF($A25="","",$B$10*(1+$B$15)^$B25)</f>
         <v/>
       </c>
-      <c r="H25" s="84" t="str">
+      <c r="H25" s="81" t="str">
         <f aca="false">IF(OR($A25="",$F25=""),"",$F25-$G25)</f>
         <v/>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="79"/>
-      <c r="B26" s="80" t="str">
+      <c r="A26" s="76"/>
+      <c r="B26" s="77" t="str">
         <f aca="false">IF($A26="","",($A26-$B$6)/365.25)</f>
         <v/>
       </c>
-      <c r="C26" s="68"/>
-      <c r="D26" s="81" t="str">
+      <c r="C26" s="66"/>
+      <c r="D26" s="78" t="str">
         <f aca="false">IF($A26="","",$B$7*(1+$B$15)^$B26)</f>
         <v/>
       </c>
-      <c r="E26" s="82" t="str">
+      <c r="E26" s="79" t="str">
         <f aca="false">IF(OR($A26="",$C26=""),"",$C26-$D26)</f>
         <v/>
       </c>
-      <c r="F26" s="83"/>
-      <c r="G26" s="81" t="str">
+      <c r="F26" s="80"/>
+      <c r="G26" s="78" t="str">
         <f aca="false">IF($A26="","",$B$10*(1+$B$15)^$B26)</f>
         <v/>
       </c>
-      <c r="H26" s="84" t="str">
+      <c r="H26" s="81" t="str">
         <f aca="false">IF(OR($A26="",$F26=""),"",$F26-$G26)</f>
         <v/>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="79"/>
-      <c r="B27" s="80" t="str">
+      <c r="A27" s="76"/>
+      <c r="B27" s="77" t="str">
         <f aca="false">IF($A27="","",($A27-$B$6)/365.25)</f>
         <v/>
       </c>
-      <c r="C27" s="68"/>
-      <c r="D27" s="81" t="str">
+      <c r="C27" s="66"/>
+      <c r="D27" s="78" t="str">
         <f aca="false">IF($A27="","",$B$7*(1+$B$15)^$B27)</f>
         <v/>
       </c>
-      <c r="E27" s="82" t="str">
+      <c r="E27" s="79" t="str">
         <f aca="false">IF(OR($A27="",$C27=""),"",$C27-$D27)</f>
         <v/>
       </c>
-      <c r="F27" s="83"/>
-      <c r="G27" s="81" t="str">
+      <c r="F27" s="80"/>
+      <c r="G27" s="78" t="str">
         <f aca="false">IF($A27="","",$B$10*(1+$B$15)^$B27)</f>
         <v/>
       </c>
-      <c r="H27" s="84" t="str">
+      <c r="H27" s="81" t="str">
         <f aca="false">IF(OR($A27="",$F27=""),"",$F27-$G27)</f>
         <v/>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="79"/>
-      <c r="B28" s="80" t="str">
+      <c r="A28" s="76"/>
+      <c r="B28" s="77" t="str">
         <f aca="false">IF($A28="","",($A28-$B$6)/365.25)</f>
         <v/>
       </c>
-      <c r="C28" s="68"/>
-      <c r="D28" s="81" t="str">
+      <c r="C28" s="66"/>
+      <c r="D28" s="78" t="str">
         <f aca="false">IF($A28="","",$B$7*(1+$B$15)^$B28)</f>
         <v/>
       </c>
-      <c r="E28" s="82" t="str">
+      <c r="E28" s="79" t="str">
         <f aca="false">IF(OR($A28="",$C28=""),"",$C28-$D28)</f>
         <v/>
       </c>
-      <c r="F28" s="83"/>
-      <c r="G28" s="81" t="str">
+      <c r="F28" s="80"/>
+      <c r="G28" s="78" t="str">
         <f aca="false">IF($A28="","",$B$10*(1+$B$15)^$B28)</f>
         <v/>
       </c>
-      <c r="H28" s="84" t="str">
+      <c r="H28" s="81" t="str">
         <f aca="false">IF(OR($A28="",$F28=""),"",$F28-$G28)</f>
         <v/>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="79"/>
-      <c r="B29" s="80" t="str">
+      <c r="A29" s="76"/>
+      <c r="B29" s="77" t="str">
         <f aca="false">IF($A29="","",($A29-$B$6)/365.25)</f>
         <v/>
       </c>
-      <c r="C29" s="68"/>
-      <c r="D29" s="81" t="str">
+      <c r="C29" s="66"/>
+      <c r="D29" s="78" t="str">
         <f aca="false">IF($A29="","",$B$7*(1+$B$15)^$B29)</f>
         <v/>
       </c>
-      <c r="E29" s="82" t="str">
+      <c r="E29" s="79" t="str">
         <f aca="false">IF(OR($A29="",$C29=""),"",$C29-$D29)</f>
         <v/>
       </c>
-      <c r="F29" s="83"/>
-      <c r="G29" s="81" t="str">
+      <c r="F29" s="80"/>
+      <c r="G29" s="78" t="str">
         <f aca="false">IF($A29="","",$B$10*(1+$B$15)^$B29)</f>
         <v/>
       </c>
-      <c r="H29" s="84" t="str">
+      <c r="H29" s="81" t="str">
         <f aca="false">IF(OR($A29="",$F29=""),"",$F29-$G29)</f>
         <v/>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="79"/>
-      <c r="B30" s="80" t="str">
+      <c r="A30" s="76"/>
+      <c r="B30" s="77" t="str">
         <f aca="false">IF($A30="","",($A30-$B$6)/365.25)</f>
         <v/>
       </c>
-      <c r="C30" s="68"/>
-      <c r="D30" s="81" t="str">
+      <c r="C30" s="66"/>
+      <c r="D30" s="78" t="str">
         <f aca="false">IF($A30="","",$B$7*(1+$B$15)^$B30)</f>
         <v/>
       </c>
-      <c r="E30" s="82" t="str">
+      <c r="E30" s="79" t="str">
         <f aca="false">IF(OR($A30="",$C30=""),"",$C30-$D30)</f>
         <v/>
       </c>
-      <c r="F30" s="83"/>
-      <c r="G30" s="81" t="str">
+      <c r="F30" s="80"/>
+      <c r="G30" s="78" t="str">
         <f aca="false">IF($A30="","",$B$10*(1+$B$15)^$B30)</f>
         <v/>
       </c>
-      <c r="H30" s="84" t="str">
+      <c r="H30" s="81" t="str">
         <f aca="false">IF(OR($A30="",$F30=""),"",$F30-$G30)</f>
         <v/>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="85" t="s">
-        <v>228</v>
-      </c>
-      <c r="B32" s="85"/>
-      <c r="C32" s="85"/>
-      <c r="D32" s="85"/>
-      <c r="E32" s="85"/>
-      <c r="F32" s="85"/>
-      <c r="G32" s="85"/>
-      <c r="H32" s="85"/>
+      <c r="A32" s="61" t="s">
+        <v>233</v>
+      </c>
+      <c r="B32" s="61"/>
+      <c r="C32" s="61"/>
+      <c r="D32" s="61"/>
+      <c r="E32" s="61"/>
+      <c r="F32" s="61"/>
+      <c r="G32" s="61"/>
+      <c r="H32" s="61"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="85"/>
-      <c r="B33" s="85"/>
-      <c r="C33" s="85"/>
-      <c r="D33" s="85"/>
-      <c r="E33" s="85"/>
-      <c r="F33" s="85"/>
-      <c r="G33" s="85"/>
-      <c r="H33" s="85"/>
+      <c r="A33" s="61"/>
+      <c r="B33" s="61"/>
+      <c r="C33" s="61"/>
+      <c r="D33" s="61"/>
+      <c r="E33" s="61"/>
+      <c r="F33" s="61"/>
+      <c r="G33" s="61"/>
+      <c r="H33" s="61"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="85"/>
-      <c r="B34" s="85"/>
-      <c r="C34" s="85"/>
-      <c r="D34" s="85"/>
-      <c r="E34" s="85"/>
-      <c r="F34" s="85"/>
-      <c r="G34" s="85"/>
-      <c r="H34" s="85"/>
+      <c r="A34" s="61"/>
+      <c r="B34" s="61"/>
+      <c r="C34" s="61"/>
+      <c r="D34" s="61"/>
+      <c r="E34" s="61"/>
+      <c r="F34" s="61"/>
+      <c r="G34" s="61"/>
+      <c r="H34" s="61"/>
     </row>
   </sheetData>
   <mergeCells count="16">

</xml_diff>

<commit_message>
Caja Motor: cerrar X/Y/Z sin cifra fija (decisión 2026-08-13) — seguimiento de trayectoria en vez de objetivo proyectado. CONSTITUTION v1.6
</commit_message>
<xml_diff>
--- a/data/raw/personal_capacity_facts.xlsx
+++ b/data/raw/personal_capacity_facts.xlsx
@@ -617,7 +617,7 @@
     <t xml:space="preserve">PROYECCIÓN CAJA MOTOR — HIPÓTESIS BASE v1</t>
   </si>
   <si>
-    <t xml:space="preserve">Ilustrativa, no un objetivo. X/Y/Z por necesidad patrimonial: CONSTITUTION.md Sección 6, Pendiente.</t>
+    <t xml:space="preserve">Caja Motor no tiene objetivo numérico fijo (CONSTITUTION.md Sección 2, decisión 2026-08-13) — seguimiento de trayectoria, no un objetivo a cumplir.</t>
   </si>
   <si>
     <t xml:space="preserve">Fecha y saldo de referencia  ·  CONGELADOS — no enlazados por fórmula</t>
@@ -1074,15 +1074,11 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="82">
+  <cellXfs count="81">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1103,7 +1099,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1123,7 +1119,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1143,7 +1139,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1658,139 +1654,139 @@
   <dimension ref="A1:B24"/>
   <sheetFormatPr defaultColWidth="8.66796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="38"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="70"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="70"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="3" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="2" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="5" t="s">
+      <c r="A6" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="3" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="4" t="s">
+      <c r="A7" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="3" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3" t="s">
+      <c r="A9" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="4" t="s">
+      <c r="A10" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="B10" s="3" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="4" t="s">
+      <c r="A11" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="B11" s="3" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="4" t="s">
+      <c r="A12" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B12" s="4" t="s">
+      <c r="B12" s="3" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="3" t="s">
+      <c r="A14" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B14" s="4" t="s">
+      <c r="B14" s="3" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="3" t="s">
+      <c r="A16" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B16" s="4" t="s">
+      <c r="B16" s="3" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="3" t="s">
+      <c r="A18" s="2" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="4" t="s">
+      <c r="A19" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B19" s="4" t="s">
+      <c r="B19" s="3" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="4" t="s">
+      <c r="A20" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B20" s="4" t="s">
+      <c r="B20" s="3" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="4" t="s">
+      <c r="A21" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B21" s="4" t="s">
+      <c r="B21" s="3" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="4" t="s">
+      <c r="A22" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B22" s="4" t="s">
+      <c r="B22" s="3" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="4" t="s">
+      <c r="A23" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B23" s="4" t="s">
+      <c r="B23" s="3" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="4" t="s">
+      <c r="A24" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B24" s="4" t="s">
+      <c r="B24" s="3" t="s">
         <v>23</v>
       </c>
     </row>
@@ -1813,705 +1809,705 @@
   <dimension ref="A1:D61"/>
   <sheetFormatPr defaultColWidth="8.66796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="40"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="46"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="1" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="6" t="s">
+      <c r="A3" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="B3" s="7"/>
-      <c r="C3" s="7"/>
-      <c r="D3" s="7"/>
+      <c r="B3" s="6"/>
+      <c r="C3" s="6"/>
+      <c r="D3" s="6"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="8" t="s">
+      <c r="A4" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="B4" s="8" t="s">
+      <c r="B4" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="C4" s="8" t="s">
+      <c r="C4" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="D4" s="8" t="s">
+      <c r="D4" s="7" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4" t="s">
+      <c r="A5" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="B5" s="9" t="n">
+      <c r="B5" s="8" t="n">
         <v>20000</v>
       </c>
-      <c r="C5" s="10" t="s">
+      <c r="C5" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="D5" s="10" t="s">
+      <c r="D5" s="9" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4" t="s">
+      <c r="A6" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="B6" s="9" t="n">
+      <c r="B6" s="8" t="n">
         <v>13000</v>
       </c>
-      <c r="C6" s="10" t="s">
+      <c r="C6" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="D6" s="10" t="s">
+      <c r="D6" s="9" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="4" t="s">
+      <c r="A7" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="B7" s="11" t="n">
+      <c r="B7" s="10" t="n">
         <f aca="false">B6-B5</f>
         <v>-7000</v>
       </c>
-      <c r="C7" s="10" t="s">
+      <c r="C7" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="D7" s="10" t="s">
+      <c r="D7" s="9" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="4" t="s">
+      <c r="A8" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="B8" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="C8" s="10" t="s">
+      <c r="C8" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="D8" s="10" t="s">
+      <c r="D8" s="9" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="4" t="s">
+      <c r="A9" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="B9" s="9" t="n">
+      <c r="B9" s="8" t="n">
         <v>30000</v>
       </c>
-      <c r="C9" s="10" t="s">
+      <c r="C9" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="D9" s="10" t="s">
+      <c r="D9" s="9" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="4" t="s">
+      <c r="A10" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="B10" s="9" t="n">
+      <c r="B10" s="8" t="n">
         <v>70000</v>
       </c>
-      <c r="C10" s="10" t="s">
+      <c r="C10" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="D10" s="10" t="s">
+      <c r="D10" s="9" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="4" t="s">
+      <c r="A11" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="B11" s="9" t="n">
+      <c r="B11" s="8" t="n">
         <v>120000</v>
       </c>
-      <c r="C11" s="10" t="s">
+      <c r="C11" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="D11" s="10" t="s">
+      <c r="D11" s="9" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="4" t="s">
+      <c r="A12" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="B12" s="11" t="n">
+      <c r="B12" s="10" t="n">
         <f aca="false">B9+B10</f>
         <v>100000</v>
       </c>
-      <c r="C12" s="10" t="s">
+      <c r="C12" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="D12" s="12"/>
+      <c r="D12" s="11"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="4" t="s">
+      <c r="A13" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="B13" s="11" t="n">
+      <c r="B13" s="10" t="n">
         <f aca="false">B9+B11</f>
         <v>150000</v>
       </c>
-      <c r="C13" s="10" t="s">
+      <c r="C13" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="D13" s="12"/>
+      <c r="D13" s="11"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="4" t="s">
+      <c r="A14" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="B14" s="9" t="n">
+      <c r="B14" s="8" t="n">
         <v>83100</v>
       </c>
-      <c r="C14" s="10" t="s">
+      <c r="C14" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="D14" s="10" t="s">
+      <c r="D14" s="9" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="4" t="s">
+      <c r="A15" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="B15" s="9" t="n">
+      <c r="B15" s="8" t="n">
         <v>89230.77</v>
       </c>
-      <c r="C15" s="10" t="s">
+      <c r="C15" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="D15" s="10" t="s">
+      <c r="D15" s="9" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="4" t="s">
+      <c r="A16" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="B16" s="11" t="n">
+      <c r="B16" s="10" t="n">
         <f aca="false">SUM(B14:B15)</f>
         <v>172330.77</v>
       </c>
-      <c r="C16" s="10" t="s">
+      <c r="C16" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="D16" s="12"/>
+      <c r="D16" s="11"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="4" t="s">
+      <c r="A17" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="B17" s="11" t="n">
+      <c r="B17" s="10" t="n">
         <f aca="false">B16-B9</f>
         <v>142330.77</v>
       </c>
-      <c r="C17" s="10" t="s">
+      <c r="C17" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="D17" s="12"/>
+      <c r="D17" s="11"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="4" t="s">
+      <c r="A18" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="B18" s="11" t="n">
+      <c r="B18" s="10" t="n">
         <f aca="false">B16-B12</f>
         <v>72330.77</v>
       </c>
-      <c r="C18" s="10" t="s">
+      <c r="C18" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="D18" s="12"/>
+      <c r="D18" s="11"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="4" t="s">
+      <c r="A19" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="B19" s="11" t="n">
+      <c r="B19" s="10" t="n">
         <f aca="false">B16-B13</f>
         <v>22330.77</v>
       </c>
-      <c r="C19" s="10" t="s">
+      <c r="C19" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="D19" s="10" t="s">
+      <c r="D19" s="9" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="4" t="s">
+      <c r="A20" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="B20" s="11" t="n">
+      <c r="B20" s="10" t="n">
         <f aca="false">B17-B10</f>
         <v>72330.77</v>
       </c>
-      <c r="C20" s="10" t="s">
+      <c r="C20" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="D20" s="12"/>
+      <c r="D20" s="11"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="4" t="s">
+      <c r="A21" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="B21" s="11" t="n">
+      <c r="B21" s="10" t="n">
         <f aca="false">B17-B11</f>
         <v>22330.77</v>
       </c>
-      <c r="C21" s="10" t="s">
+      <c r="C21" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="D21" s="12"/>
+      <c r="D21" s="11"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="6" t="s">
+      <c r="A23" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="B23" s="7"/>
-      <c r="C23" s="7"/>
-      <c r="D23" s="7"/>
+      <c r="B23" s="6"/>
+      <c r="C23" s="6"/>
+      <c r="D23" s="6"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="8" t="s">
+      <c r="A24" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="B24" s="8" t="s">
+      <c r="B24" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="C24" s="8" t="s">
+      <c r="C24" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="D24" s="8" t="s">
+      <c r="D24" s="7" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="4" t="s">
+      <c r="A25" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="B25" s="5" t="s">
+      <c r="B25" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="C25" s="10" t="s">
+      <c r="C25" s="9" t="s">
         <v>64</v>
       </c>
-      <c r="D25" s="10" t="s">
+      <c r="D25" s="9" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="6" t="s">
+      <c r="A27" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="B27" s="7"/>
-      <c r="C27" s="7"/>
-      <c r="D27" s="7"/>
+      <c r="B27" s="6"/>
+      <c r="C27" s="6"/>
+      <c r="D27" s="6"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="8" t="s">
+      <c r="A28" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="B28" s="8" t="s">
+      <c r="B28" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="C28" s="8" t="s">
+      <c r="C28" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="D28" s="8" t="s">
+      <c r="D28" s="7" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="4" t="s">
+      <c r="A29" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="B29" s="9" t="n">
+      <c r="B29" s="8" t="n">
         <v>6000</v>
       </c>
-      <c r="C29" s="10" t="s">
+      <c r="C29" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="D29" s="12"/>
+      <c r="D29" s="11"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="4" t="s">
+      <c r="A30" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="B30" s="9" t="n">
+      <c r="B30" s="8" t="n">
         <v>5000</v>
       </c>
-      <c r="C30" s="10" t="s">
+      <c r="C30" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="D30" s="12"/>
+      <c r="D30" s="11"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="4" t="s">
+      <c r="A31" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="B31" s="9" t="n">
+      <c r="B31" s="8" t="n">
         <v>2000</v>
       </c>
-      <c r="C31" s="10" t="s">
+      <c r="C31" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="D31" s="12"/>
+      <c r="D31" s="11"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="4" t="s">
+      <c r="A32" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="B32" s="11" t="n">
+      <c r="B32" s="10" t="n">
         <f aca="false">SUM(B29:B31)</f>
         <v>13000</v>
       </c>
-      <c r="C32" s="10" t="s">
+      <c r="C32" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="D32" s="12"/>
+      <c r="D32" s="11"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="4" t="s">
+      <c r="A33" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="B33" s="13" t="n">
+      <c r="B33" s="12" t="n">
         <f aca="false">B29/B32</f>
         <v>0.461538461538462</v>
       </c>
-      <c r="C33" s="10" t="s">
+      <c r="C33" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="D33" s="12"/>
+      <c r="D33" s="11"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="4" t="s">
+      <c r="A34" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="B34" s="13" t="n">
+      <c r="B34" s="12" t="n">
         <f aca="false">B30/B32</f>
         <v>0.384615384615385</v>
       </c>
-      <c r="C34" s="10" t="s">
+      <c r="C34" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="D34" s="12"/>
+      <c r="D34" s="11"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="4" t="s">
+      <c r="A35" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="B35" s="13" t="n">
+      <c r="B35" s="12" t="n">
         <f aca="false">B31/B32</f>
         <v>0.153846153846154</v>
       </c>
-      <c r="C35" s="10" t="s">
+      <c r="C35" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="D35" s="12"/>
+      <c r="D35" s="11"/>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="4" t="s">
+      <c r="A36" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="B36" s="5" t="s">
+      <c r="B36" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="C36" s="10" t="s">
+      <c r="C36" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="D36" s="10" t="s">
+      <c r="D36" s="9" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="6" t="s">
+      <c r="A38" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="B38" s="7"/>
-      <c r="C38" s="7"/>
-      <c r="D38" s="7"/>
+      <c r="B38" s="6"/>
+      <c r="C38" s="6"/>
+      <c r="D38" s="6"/>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="8" t="s">
+      <c r="A39" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="B39" s="8" t="s">
+      <c r="B39" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="C39" s="8" t="s">
+      <c r="C39" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="D39" s="8" t="s">
+      <c r="D39" s="7" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="4" t="s">
+      <c r="A40" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="B40" s="9" t="n">
+      <c r="B40" s="8" t="n">
         <v>878274</v>
       </c>
-      <c r="C40" s="10" t="s">
+      <c r="C40" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="D40" s="12"/>
+      <c r="D40" s="11"/>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A41" s="4" t="s">
+      <c r="A41" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="B41" s="9" t="n">
+      <c r="B41" s="8" t="n">
         <v>89230.77</v>
       </c>
-      <c r="C41" s="10" t="s">
+      <c r="C41" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="D41" s="12"/>
+      <c r="D41" s="11"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="4" t="s">
+      <c r="A42" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="B42" s="9" t="n">
+      <c r="B42" s="8" t="n">
         <v>111570.37</v>
       </c>
-      <c r="C42" s="10" t="s">
+      <c r="C42" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="D42" s="12"/>
+      <c r="D42" s="11"/>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A43" s="4" t="s">
+      <c r="A43" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="B43" s="9" t="n">
+      <c r="B43" s="8" t="n">
         <v>100000</v>
       </c>
-      <c r="C43" s="10" t="s">
+      <c r="C43" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="D43" s="12"/>
+      <c r="D43" s="11"/>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="4" t="s">
+      <c r="A44" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="B44" s="9" t="n">
+      <c r="B44" s="8" t="n">
         <v>83100</v>
       </c>
-      <c r="C44" s="10" t="s">
+      <c r="C44" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="D44" s="10" t="s">
+      <c r="D44" s="9" t="s">
         <v>83</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A45" s="14" t="s">
+      <c r="A45" s="13" t="s">
         <v>84</v>
       </c>
-      <c r="B45" s="15" t="n">
+      <c r="B45" s="14" t="n">
         <f aca="false">SUM(B40:B44)</f>
         <v>1262175.14</v>
       </c>
-      <c r="C45" s="16" t="s">
+      <c r="C45" s="15" t="s">
         <v>36</v>
       </c>
-      <c r="D45" s="17"/>
+      <c r="D45" s="16"/>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A46" s="4" t="s">
+      <c r="A46" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="B46" s="13" t="n">
+      <c r="B46" s="12" t="n">
         <f aca="false">B40/B45</f>
         <v>0.695841624641728</v>
       </c>
-      <c r="C46" s="10" t="s">
+      <c r="C46" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="D46" s="12"/>
+      <c r="D46" s="11"/>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A47" s="4" t="s">
+      <c r="A47" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="B47" s="13" t="n">
+      <c r="B47" s="12" t="n">
         <f aca="false">B41/B45</f>
         <v>0.0706960287619038</v>
       </c>
-      <c r="C47" s="10" t="s">
+      <c r="C47" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="D47" s="12"/>
+      <c r="D47" s="11"/>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A48" s="4" t="s">
+      <c r="A48" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="B48" s="13" t="n">
+      <c r="B48" s="12" t="n">
         <f aca="false">B42/B45</f>
         <v>0.0883953157245674</v>
       </c>
-      <c r="C48" s="10" t="s">
+      <c r="C48" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="D48" s="12"/>
+      <c r="D48" s="11"/>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A49" s="4" t="s">
+      <c r="A49" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="B49" s="13" t="n">
+      <c r="B49" s="12" t="n">
         <f aca="false">B43/B45</f>
         <v>0.0792283074122344</v>
       </c>
-      <c r="C49" s="10" t="s">
+      <c r="C49" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="D49" s="12"/>
+      <c r="D49" s="11"/>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A50" s="4" t="s">
+      <c r="A50" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="B50" s="13" t="n">
+      <c r="B50" s="12" t="n">
         <f aca="false">B44/B45</f>
         <v>0.0658387234595668</v>
       </c>
-      <c r="C50" s="10" t="s">
+      <c r="C50" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="D50" s="12"/>
+      <c r="D50" s="11"/>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A51" s="4" t="s">
+      <c r="A51" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="B51" s="5" t="s">
+      <c r="B51" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="C51" s="10" t="s">
+      <c r="C51" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="D51" s="10" t="s">
+      <c r="D51" s="9" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A53" s="6" t="s">
+      <c r="A53" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="B53" s="7"/>
-      <c r="C53" s="7"/>
-      <c r="D53" s="7"/>
+      <c r="B53" s="6"/>
+      <c r="C53" s="6"/>
+      <c r="D53" s="6"/>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A54" s="8" t="s">
+      <c r="A54" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="B54" s="8" t="s">
+      <c r="B54" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="C54" s="8" t="s">
+      <c r="C54" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="D54" s="8" t="s">
+      <c r="D54" s="7" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A55" s="4" t="s">
+      <c r="A55" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="B55" s="5" t="s">
+      <c r="B55" s="4" t="s">
         <v>94</v>
       </c>
-      <c r="C55" s="10" t="s">
+      <c r="C55" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="D55" s="10" t="s">
+      <c r="D55" s="9" t="s">
         <v>95</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A56" s="4" t="s">
+      <c r="A56" s="3" t="s">
         <v>96</v>
       </c>
-      <c r="B56" s="5" t="s">
+      <c r="B56" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="C56" s="10" t="s">
+      <c r="C56" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="D56" s="10" t="s">
+      <c r="D56" s="9" t="s">
         <v>98</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A58" s="6" t="s">
+      <c r="A58" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="B58" s="7"/>
-      <c r="C58" s="7"/>
-      <c r="D58" s="7"/>
+      <c r="B58" s="6"/>
+      <c r="C58" s="6"/>
+      <c r="D58" s="6"/>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A59" s="8" t="s">
+      <c r="A59" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="B59" s="8" t="s">
+      <c r="B59" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="C59" s="8" t="s">
+      <c r="C59" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="D59" s="8" t="s">
+      <c r="D59" s="7" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A60" s="4" t="s">
+      <c r="A60" s="3" t="s">
         <v>100</v>
       </c>
-      <c r="B60" s="9" t="n">
+      <c r="B60" s="8" t="n">
         <v>-215092</v>
       </c>
-      <c r="C60" s="10" t="s">
+      <c r="C60" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="D60" s="10" t="s">
+      <c r="D60" s="9" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A61" s="4" t="s">
+      <c r="A61" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="B61" s="5" t="s">
+      <c r="B61" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="C61" s="10" t="s">
+      <c r="C61" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="D61" s="10" t="s">
+      <c r="D61" s="9" t="s">
         <v>104</v>
       </c>
     </row>
@@ -2534,875 +2530,875 @@
   <dimension ref="A1:D79"/>
   <sheetFormatPr defaultColWidth="8.66796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="57.33"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="50"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="57.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="50"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="1" t="s">
         <v>105</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="6" t="s">
+      <c r="A3" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="B3" s="7"/>
-      <c r="C3" s="7"/>
-      <c r="D3" s="7"/>
+      <c r="B3" s="6"/>
+      <c r="C3" s="6"/>
+      <c r="D3" s="6"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="8" t="s">
+      <c r="A4" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="B4" s="8" t="s">
+      <c r="B4" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="C4" s="8" t="s">
+      <c r="C4" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="D4" s="8" t="s">
+      <c r="D4" s="7" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4" t="s">
+      <c r="A5" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="B5" s="9" t="n">
+      <c r="B5" s="8" t="n">
         <v>32500</v>
       </c>
-      <c r="C5" s="10" t="s">
+      <c r="C5" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="D5" s="10" t="s">
+      <c r="D5" s="9" t="s">
         <v>106</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4" t="s">
+      <c r="A6" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="B6" s="9" t="n">
+      <c r="B6" s="8" t="n">
         <v>80000</v>
       </c>
-      <c r="C6" s="10" t="s">
+      <c r="C6" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="D6" s="10" t="s">
+      <c r="D6" s="9" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="4" t="s">
+      <c r="A7" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="B7" s="11" t="n">
+      <c r="B7" s="10" t="n">
         <f aca="false">B6-B5</f>
         <v>47500</v>
       </c>
-      <c r="C7" s="10" t="s">
+      <c r="C7" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="D7" s="10" t="s">
+      <c r="D7" s="9" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="4" t="s">
+      <c r="A8" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="B8" s="9" t="n">
+      <c r="B8" s="8" t="n">
         <v>125000</v>
       </c>
-      <c r="C8" s="10" t="s">
+      <c r="C8" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="D8" s="10" t="s">
+      <c r="D8" s="9" t="s">
         <v>110</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="4" t="s">
+      <c r="A9" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="B9" s="9" t="n">
+      <c r="B9" s="8" t="n">
         <v>125000</v>
       </c>
-      <c r="C9" s="10" t="s">
+      <c r="C9" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="D9" s="12"/>
+      <c r="D9" s="11"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="4" t="s">
+      <c r="A10" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="B10" s="9" t="n">
+      <c r="B10" s="8" t="n">
         <v>175000</v>
       </c>
-      <c r="C10" s="10" t="s">
+      <c r="C10" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="D10" s="12"/>
+      <c r="D10" s="11"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="4" t="s">
+      <c r="A11" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="B11" s="11" t="n">
+      <c r="B11" s="10" t="n">
         <f aca="false">B8+B9</f>
         <v>250000</v>
       </c>
-      <c r="C11" s="10" t="s">
+      <c r="C11" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="D11" s="12"/>
+      <c r="D11" s="11"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="4" t="s">
+      <c r="A12" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="B12" s="11" t="n">
+      <c r="B12" s="10" t="n">
         <f aca="false">B8+B10</f>
         <v>300000</v>
       </c>
-      <c r="C12" s="10" t="s">
+      <c r="C12" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="D12" s="10" t="s">
+      <c r="D12" s="9" t="s">
         <v>111</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="4" t="s">
+      <c r="A13" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="B13" s="9" t="n">
+      <c r="B13" s="8" t="n">
         <v>54375</v>
       </c>
-      <c r="C13" s="10" t="s">
+      <c r="C13" s="9" t="s">
         <v>112</v>
       </c>
-      <c r="D13" s="12"/>
+      <c r="D13" s="11"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="4" t="s">
+      <c r="A14" s="3" t="s">
         <v>113</v>
       </c>
-      <c r="B14" s="9" t="n">
+      <c r="B14" s="8" t="n">
         <v>60000</v>
       </c>
-      <c r="C14" s="10" t="s">
+      <c r="C14" s="9" t="s">
         <v>112</v>
       </c>
-      <c r="D14" s="10" t="s">
+      <c r="D14" s="9" t="s">
         <v>114</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="4" t="s">
+      <c r="A15" s="3" t="s">
         <v>115</v>
       </c>
-      <c r="B15" s="9" t="n">
+      <c r="B15" s="8" t="n">
         <v>85000</v>
       </c>
-      <c r="C15" s="10" t="s">
+      <c r="C15" s="9" t="s">
         <v>112</v>
       </c>
-      <c r="D15" s="10" t="s">
+      <c r="D15" s="9" t="s">
         <v>116</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="4" t="s">
+      <c r="A16" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="B16" s="9" t="n">
+      <c r="B16" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="C16" s="10" t="s">
+      <c r="C16" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="D16" s="10" t="s">
+      <c r="D16" s="9" t="s">
         <v>117</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="4" t="s">
+      <c r="A17" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="B17" s="11" t="n">
+      <c r="B17" s="10" t="n">
         <f aca="false">SUM(B13:B16)</f>
         <v>199375</v>
       </c>
-      <c r="C17" s="10" t="s">
+      <c r="C17" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="D17" s="12"/>
+      <c r="D17" s="11"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="4" t="s">
+      <c r="A18" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="B18" s="11" t="n">
+      <c r="B18" s="10" t="n">
         <f aca="false">B17-B8</f>
         <v>74375</v>
       </c>
-      <c r="C18" s="10" t="s">
+      <c r="C18" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="D18" s="12"/>
+      <c r="D18" s="11"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="4" t="s">
+      <c r="A19" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="B19" s="11" t="n">
+      <c r="B19" s="10" t="n">
         <f aca="false">B17-B11</f>
         <v>-50625</v>
       </c>
-      <c r="C19" s="10" t="s">
+      <c r="C19" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="D19" s="12"/>
+      <c r="D19" s="11"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="4" t="s">
+      <c r="A20" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="B20" s="11" t="n">
+      <c r="B20" s="10" t="n">
         <f aca="false">B17-B12</f>
         <v>-100625</v>
       </c>
-      <c r="C20" s="10" t="s">
+      <c r="C20" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="D20" s="12"/>
+      <c r="D20" s="11"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="4" t="s">
+      <c r="A21" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="B21" s="11" t="n">
+      <c r="B21" s="10" t="n">
         <f aca="false">B18-B9</f>
         <v>-50625</v>
       </c>
-      <c r="C21" s="10" t="s">
+      <c r="C21" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="D21" s="10" t="s">
+      <c r="D21" s="9" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="4" t="s">
+      <c r="A22" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="B22" s="11" t="n">
+      <c r="B22" s="10" t="n">
         <f aca="false">B18-B10</f>
         <v>-100625</v>
       </c>
-      <c r="C22" s="10" t="s">
+      <c r="C22" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="D22" s="12"/>
+      <c r="D22" s="11"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="6" t="s">
+      <c r="A24" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="B24" s="7"/>
-      <c r="C24" s="7"/>
-      <c r="D24" s="7"/>
+      <c r="B24" s="6"/>
+      <c r="C24" s="6"/>
+      <c r="D24" s="6"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="8" t="s">
+      <c r="A25" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="B25" s="8" t="s">
+      <c r="B25" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="C25" s="8" t="s">
+      <c r="C25" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="D25" s="8" t="s">
+      <c r="D25" s="7" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="4" t="s">
+      <c r="A26" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="B26" s="5" t="s">
+      <c r="B26" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="C26" s="10" t="s">
+      <c r="C26" s="9" t="s">
         <v>64</v>
       </c>
-      <c r="D26" s="10" t="s">
+      <c r="D26" s="9" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="6" t="s">
+      <c r="A28" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="B28" s="7"/>
-      <c r="C28" s="7"/>
-      <c r="D28" s="7"/>
+      <c r="B28" s="6"/>
+      <c r="C28" s="6"/>
+      <c r="D28" s="6"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="8" t="s">
+      <c r="A29" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="B29" s="8" t="s">
+      <c r="B29" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="C29" s="8" t="s">
+      <c r="C29" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="D29" s="8" t="s">
+      <c r="D29" s="7" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="4" t="s">
+      <c r="A30" s="3" t="s">
         <v>119</v>
       </c>
-      <c r="B30" s="9" t="n">
+      <c r="B30" s="8" t="n">
         <v>60000</v>
       </c>
-      <c r="C30" s="10" t="s">
+      <c r="C30" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="D30" s="10" t="s">
+      <c r="D30" s="9" t="s">
         <v>120</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="4" t="s">
+      <c r="A31" s="3" t="s">
         <v>121</v>
       </c>
-      <c r="B31" s="9" t="n">
+      <c r="B31" s="8" t="n">
         <v>20000</v>
       </c>
-      <c r="C31" s="10" t="s">
+      <c r="C31" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="D31" s="12"/>
+      <c r="D31" s="11"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="4" t="s">
+      <c r="A32" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="B32" s="11" t="n">
+      <c r="B32" s="10" t="n">
         <f aca="false">SUM(B30:B31)</f>
         <v>80000</v>
       </c>
-      <c r="C32" s="10" t="s">
+      <c r="C32" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="D32" s="12"/>
+      <c r="D32" s="11"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="4" t="s">
+      <c r="A33" s="3" t="s">
         <v>122</v>
       </c>
-      <c r="B33" s="13" t="n">
+      <c r="B33" s="12" t="n">
         <f aca="false">B30/B32</f>
         <v>0.75</v>
       </c>
-      <c r="C33" s="10" t="s">
+      <c r="C33" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="D33" s="12"/>
+      <c r="D33" s="11"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="4" t="s">
+      <c r="A34" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="B34" s="13" t="n">
+      <c r="B34" s="12" t="n">
         <f aca="false">B31/B32</f>
         <v>0.25</v>
       </c>
-      <c r="C34" s="10" t="s">
+      <c r="C34" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="D34" s="12"/>
+      <c r="D34" s="11"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="4" t="s">
+      <c r="A35" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="B35" s="5" t="s">
+      <c r="B35" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="C35" s="10" t="s">
+      <c r="C35" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="D35" s="10" t="s">
+      <c r="D35" s="9" t="s">
         <v>124</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="6" t="s">
+      <c r="A37" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="B37" s="7"/>
-      <c r="C37" s="7"/>
-      <c r="D37" s="7"/>
+      <c r="B37" s="6"/>
+      <c r="C37" s="6"/>
+      <c r="D37" s="6"/>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="8" t="s">
+      <c r="A38" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="B38" s="8" t="s">
+      <c r="B38" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="C38" s="8" t="s">
+      <c r="C38" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="D38" s="8" t="s">
+      <c r="D38" s="7" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="4" t="s">
+      <c r="A39" s="3" t="s">
         <v>125</v>
       </c>
-      <c r="B39" s="9" t="n">
+      <c r="B39" s="8" t="n">
         <v>2196689</v>
       </c>
-      <c r="C39" s="10" t="s">
+      <c r="C39" s="9" t="s">
         <v>112</v>
       </c>
-      <c r="D39" s="12"/>
+      <c r="D39" s="11"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="4" t="s">
+      <c r="A40" s="3" t="s">
         <v>126</v>
       </c>
-      <c r="B40" s="18" t="n">
+      <c r="B40" s="17" t="n">
         <f aca="false">B60+B61</f>
         <v>1158832</v>
       </c>
-      <c r="C40" s="10" t="s">
+      <c r="C40" s="9" t="s">
         <v>112</v>
       </c>
-      <c r="D40" s="10" t="s">
+      <c r="D40" s="9" t="s">
         <v>127</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A41" s="4" t="s">
+      <c r="A41" s="3" t="s">
         <v>128</v>
       </c>
-      <c r="B41" s="18" t="n">
+      <c r="B41" s="17" t="n">
         <f aca="false">SUM(B52:B54)</f>
         <v>531793.35</v>
       </c>
-      <c r="C41" s="10" t="s">
+      <c r="C41" s="9" t="s">
         <v>112</v>
       </c>
-      <c r="D41" s="12"/>
+      <c r="D41" s="11"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="4" t="s">
+      <c r="A42" s="3" t="s">
         <v>129</v>
       </c>
-      <c r="B42" s="9" t="n">
+      <c r="B42" s="8" t="n">
         <v>139351.5</v>
       </c>
-      <c r="C42" s="10" t="s">
+      <c r="C42" s="9" t="s">
         <v>112</v>
       </c>
-      <c r="D42" s="12"/>
+      <c r="D42" s="11"/>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A43" s="4" t="s">
+      <c r="A43" s="3" t="s">
         <v>130</v>
       </c>
-      <c r="B43" s="9" t="n">
+      <c r="B43" s="8" t="n">
         <v>199375</v>
       </c>
-      <c r="C43" s="10" t="s">
+      <c r="C43" s="9" t="s">
         <v>112</v>
       </c>
-      <c r="D43" s="10" t="s">
+      <c r="D43" s="9" t="s">
         <v>131</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="14" t="s">
+      <c r="A44" s="13" t="s">
         <v>84</v>
       </c>
-      <c r="B44" s="15" t="n">
+      <c r="B44" s="14" t="n">
         <f aca="false">SUM(B39:B43)</f>
         <v>4226040.85</v>
       </c>
-      <c r="C44" s="16" t="s">
+      <c r="C44" s="15" t="s">
         <v>36</v>
       </c>
-      <c r="D44" s="17"/>
+      <c r="D44" s="16"/>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A45" s="4" t="s">
+      <c r="A45" s="3" t="s">
         <v>132</v>
       </c>
-      <c r="B45" s="13" t="n">
+      <c r="B45" s="12" t="n">
         <f aca="false">B39/B44</f>
         <v>0.519798335598199</v>
       </c>
-      <c r="C45" s="10" t="s">
+      <c r="C45" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="D45" s="12"/>
+      <c r="D45" s="11"/>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A46" s="4" t="s">
+      <c r="A46" s="3" t="s">
         <v>133</v>
       </c>
-      <c r="B46" s="13" t="n">
+      <c r="B46" s="12" t="n">
         <f aca="false">B40/B44</f>
         <v>0.274212209756562</v>
       </c>
-      <c r="C46" s="10" t="s">
+      <c r="C46" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="D46" s="12"/>
+      <c r="D46" s="11"/>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A47" s="4" t="s">
+      <c r="A47" s="3" t="s">
         <v>134</v>
       </c>
-      <c r="B47" s="13" t="n">
+      <c r="B47" s="12" t="n">
         <f aca="false">B41/B44</f>
         <v>0.125837247881785</v>
       </c>
-      <c r="C47" s="10" t="s">
+      <c r="C47" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="D47" s="12"/>
+      <c r="D47" s="11"/>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A48" s="4" t="s">
+      <c r="A48" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="B48" s="13" t="n">
+      <c r="B48" s="12" t="n">
         <f aca="false">B42/B44</f>
         <v>0.03297448012127</v>
       </c>
-      <c r="C48" s="10" t="s">
+      <c r="C48" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="D48" s="12"/>
+      <c r="D48" s="11"/>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A49" s="4" t="s">
+      <c r="A49" s="3" t="s">
         <v>135</v>
       </c>
-      <c r="B49" s="13" t="n">
+      <c r="B49" s="12" t="n">
         <f aca="false">B43/B44</f>
         <v>0.0471777266421833</v>
       </c>
-      <c r="C49" s="10" t="s">
+      <c r="C49" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="D49" s="12"/>
+      <c r="D49" s="11"/>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A51" s="3" t="s">
+      <c r="A51" s="2" t="s">
         <v>136</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A52" s="4" t="s">
+      <c r="A52" s="3" t="s">
         <v>137</v>
       </c>
-      <c r="B52" s="9" t="n">
+      <c r="B52" s="8" t="n">
         <v>348644</v>
       </c>
-      <c r="C52" s="10" t="s">
+      <c r="C52" s="9" t="s">
         <v>138</v>
       </c>
-      <c r="D52" s="12"/>
+      <c r="D52" s="11"/>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A53" s="4" t="s">
+      <c r="A53" s="3" t="s">
         <v>139</v>
       </c>
-      <c r="B53" s="9" t="n">
+      <c r="B53" s="8" t="n">
         <v>126980</v>
       </c>
-      <c r="C53" s="10" t="s">
+      <c r="C53" s="9" t="s">
         <v>138</v>
       </c>
-      <c r="D53" s="12"/>
+      <c r="D53" s="11"/>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A54" s="4" t="s">
+      <c r="A54" s="3" t="s">
         <v>140</v>
       </c>
-      <c r="B54" s="9" t="n">
+      <c r="B54" s="8" t="n">
         <v>56169.35</v>
       </c>
-      <c r="C54" s="10" t="s">
+      <c r="C54" s="9" t="s">
         <v>138</v>
       </c>
-      <c r="D54" s="12"/>
+      <c r="D54" s="11"/>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A55" s="4" t="s">
+      <c r="A55" s="3" t="s">
         <v>141</v>
       </c>
-      <c r="B55" s="13" t="n">
+      <c r="B55" s="12" t="n">
         <f aca="false">B52/B41</f>
         <v>0.655600526031399</v>
       </c>
-      <c r="C55" s="10" t="s">
+      <c r="C55" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="D55" s="12"/>
+      <c r="D55" s="11"/>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A56" s="4" t="s">
+      <c r="A56" s="3" t="s">
         <v>142</v>
       </c>
-      <c r="B56" s="13" t="n">
+      <c r="B56" s="12" t="n">
         <f aca="false">B53/B41</f>
         <v>0.238776961013145</v>
       </c>
-      <c r="C56" s="10" t="s">
+      <c r="C56" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="D56" s="12"/>
+      <c r="D56" s="11"/>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A57" s="4" t="s">
+      <c r="A57" s="3" t="s">
         <v>143</v>
       </c>
-      <c r="B57" s="13" t="n">
+      <c r="B57" s="12" t="n">
         <f aca="false">B54/B41</f>
         <v>0.105622512955455</v>
       </c>
-      <c r="C57" s="10" t="s">
+      <c r="C57" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="D57" s="12"/>
+      <c r="D57" s="11"/>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A59" s="3" t="s">
+      <c r="A59" s="2" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A60" s="4" t="s">
+      <c r="A60" s="3" t="s">
         <v>145</v>
       </c>
-      <c r="B60" s="9" t="n">
+      <c r="B60" s="8" t="n">
         <v>755018</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A61" s="4" t="s">
+      <c r="A61" s="3" t="s">
         <v>146</v>
       </c>
-      <c r="B61" s="9" t="n">
+      <c r="B61" s="8" t="n">
         <v>403814</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A62" s="4" t="s">
+      <c r="A62" s="3" t="s">
         <v>147</v>
       </c>
-      <c r="B62" s="13" t="n">
+      <c r="B62" s="12" t="n">
         <f aca="false">B60/B40</f>
         <v>0.651533613155315</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A63" s="4" t="s">
+      <c r="A63" s="3" t="s">
         <v>148</v>
       </c>
-      <c r="B63" s="13" t="n">
+      <c r="B63" s="12" t="n">
         <f aca="false">B61/B40</f>
         <v>0.348466386844685</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A64" s="4" t="s">
+      <c r="A64" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="B64" s="5" t="s">
+      <c r="B64" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="C64" s="10" t="s">
+      <c r="C64" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="D64" s="10" t="s">
+      <c r="D64" s="9" t="s">
         <v>149</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A66" s="6" t="s">
+      <c r="A66" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="B66" s="7"/>
-      <c r="C66" s="7"/>
-      <c r="D66" s="7"/>
+      <c r="B66" s="6"/>
+      <c r="C66" s="6"/>
+      <c r="D66" s="6"/>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A67" s="8" t="s">
+      <c r="A67" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="B67" s="8" t="s">
+      <c r="B67" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="C67" s="8" t="s">
+      <c r="C67" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="D67" s="8" t="s">
+      <c r="D67" s="7" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A68" s="4" t="s">
+      <c r="A68" s="3" t="s">
         <v>150</v>
       </c>
-      <c r="B68" s="5" t="s">
+      <c r="B68" s="4" t="s">
         <v>151</v>
       </c>
-      <c r="C68" s="10" t="s">
+      <c r="C68" s="9" t="s">
         <v>152</v>
       </c>
-      <c r="D68" s="10" t="s">
+      <c r="D68" s="9" t="s">
         <v>153</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A69" s="4" t="s">
+      <c r="A69" s="3" t="s">
         <v>154</v>
       </c>
-      <c r="B69" s="19" t="n">
+      <c r="B69" s="18" t="n">
         <f aca="true">DATE(2026,9,29)-TODAY()</f>
         <v>46</v>
       </c>
-      <c r="C69" s="10" t="s">
+      <c r="C69" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="D69" s="12"/>
+      <c r="D69" s="11"/>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A70" s="4" t="s">
+      <c r="A70" s="3" t="s">
         <v>155</v>
       </c>
-      <c r="B70" s="5" t="s">
+      <c r="B70" s="4" t="s">
         <v>156</v>
       </c>
-      <c r="C70" s="10" t="s">
+      <c r="C70" s="9" t="s">
         <v>152</v>
       </c>
-      <c r="D70" s="10" t="s">
+      <c r="D70" s="9" t="s">
         <v>157</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A71" s="4" t="s">
+      <c r="A71" s="3" t="s">
         <v>154</v>
       </c>
-      <c r="B71" s="19" t="n">
+      <c r="B71" s="18" t="n">
         <f aca="true">DATE(2026,8,26)-TODAY()</f>
         <v>12</v>
       </c>
-      <c r="C71" s="10" t="s">
+      <c r="C71" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="D71" s="10" t="s">
+      <c r="D71" s="9" t="s">
         <v>158</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A73" s="4" t="s">
+      <c r="A73" s="3" t="s">
         <v>96</v>
       </c>
-      <c r="B73" s="5" t="s">
+      <c r="B73" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="C73" s="10" t="s">
+      <c r="C73" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="D73" s="10" t="s">
+      <c r="D73" s="9" t="s">
         <v>159</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A75" s="6" t="s">
+      <c r="A75" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="B75" s="7"/>
-      <c r="C75" s="7"/>
-      <c r="D75" s="7"/>
+      <c r="B75" s="6"/>
+      <c r="C75" s="6"/>
+      <c r="D75" s="6"/>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A76" s="8" t="s">
+      <c r="A76" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="B76" s="8" t="s">
+      <c r="B76" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="C76" s="8" t="s">
+      <c r="C76" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="D76" s="8" t="s">
+      <c r="D76" s="7" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A77" s="4" t="s">
+      <c r="A77" s="3" t="s">
         <v>160</v>
       </c>
-      <c r="B77" s="9" t="n">
+      <c r="B77" s="8" t="n">
         <f aca="false">B40</f>
         <v>1158832</v>
       </c>
-      <c r="C77" s="10" t="s">
+      <c r="C77" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="D77" s="10" t="s">
+      <c r="D77" s="9" t="s">
         <v>161</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="32.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A78" s="4" t="s">
+      <c r="A78" s="3" t="s">
         <v>100</v>
       </c>
-      <c r="B78" s="9" t="n">
+      <c r="B78" s="8" t="n">
         <v>-162000</v>
       </c>
-      <c r="C78" s="10" t="s">
+      <c r="C78" s="9" t="s">
         <v>162</v>
       </c>
-      <c r="D78" s="10" t="s">
+      <c r="D78" s="9" t="s">
         <v>163</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="32.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A79" s="4" t="s">
+      <c r="A79" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="B79" s="5" t="s">
+      <c r="B79" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="C79" s="10" t="s">
+      <c r="C79" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="D79" s="10" t="s">
+      <c r="D79" s="9" t="s">
         <v>164</v>
       </c>
     </row>
@@ -3425,447 +3421,447 @@
   <dimension ref="A1:F35"/>
   <sheetFormatPr defaultColWidth="8.66796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="20" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="20" width="50.67"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="20" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="20" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="20" width="50"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="7" style="20" width="8.67"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="19" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="19" width="50.67"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="19" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="19" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="19" width="50"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="7" style="19" width="8.67"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="21" t="s">
+      <c r="A1" s="20" t="s">
         <v>165</v>
       </c>
-      <c r="B1" s="21"/>
-      <c r="C1" s="21"/>
-      <c r="D1" s="21"/>
-      <c r="E1" s="21"/>
-      <c r="F1" s="21"/>
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="20"/>
+      <c r="E1" s="20"/>
+      <c r="F1" s="20"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="22" t="s">
+      <c r="A2" s="21" t="s">
         <v>166</v>
       </c>
-      <c r="B2" s="22"/>
-      <c r="C2" s="22"/>
-      <c r="D2" s="22"/>
-      <c r="E2" s="22"/>
-      <c r="F2" s="22"/>
+      <c r="B2" s="21"/>
+      <c r="C2" s="21"/>
+      <c r="D2" s="21"/>
+      <c r="E2" s="21"/>
+      <c r="F2" s="21"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="23" t="s">
+      <c r="A4" s="22" t="s">
         <v>167</v>
       </c>
-      <c r="B4" s="23"/>
-      <c r="C4" s="23"/>
-      <c r="D4" s="23"/>
-      <c r="E4" s="23"/>
-      <c r="F4" s="23"/>
+      <c r="B4" s="22"/>
+      <c r="C4" s="22"/>
+      <c r="D4" s="22"/>
+      <c r="E4" s="22"/>
+      <c r="F4" s="22"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="24" t="s">
+      <c r="A5" s="23" t="s">
         <v>168</v>
       </c>
-      <c r="B5" s="24" t="s">
+      <c r="B5" s="23" t="s">
         <v>169</v>
       </c>
-      <c r="C5" s="24" t="s">
+      <c r="C5" s="23" t="s">
         <v>27</v>
       </c>
-      <c r="D5" s="24" t="s">
+      <c r="D5" s="23" t="s">
         <v>170</v>
       </c>
-      <c r="E5" s="24" t="s">
+      <c r="E5" s="23" t="s">
         <v>171</v>
       </c>
-      <c r="F5" s="24" t="s">
+      <c r="F5" s="23" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="25" t="s">
+      <c r="A6" s="24" t="s">
         <v>172</v>
       </c>
-      <c r="B6" s="26" t="str">
+      <c r="B6" s="25" t="str">
         <f aca="false">AMS!A41</f>
         <v>Fondo Monetario</v>
       </c>
-      <c r="C6" s="27" t="n">
+      <c r="C6" s="26" t="n">
         <f aca="false">AMS!B41</f>
         <v>89230.77</v>
       </c>
-      <c r="D6" s="28"/>
-      <c r="E6" s="29" t="s">
+      <c r="D6" s="27"/>
+      <c r="E6" s="28" t="s">
         <v>173</v>
       </c>
-      <c r="F6" s="28"/>
+      <c r="F6" s="27"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="25"/>
-      <c r="B7" s="26" t="str">
+      <c r="A7" s="24"/>
+      <c r="B7" s="25" t="str">
         <f aca="false">AMS!A44</f>
         <v>Liquidez (excluido FM)</v>
       </c>
-      <c r="C7" s="27" t="n">
+      <c r="C7" s="26" t="n">
         <f aca="false">AMS!B44</f>
         <v>83100</v>
       </c>
-      <c r="D7" s="28"/>
-      <c r="E7" s="29" t="s">
+      <c r="D7" s="27"/>
+      <c r="E7" s="28" t="s">
         <v>174</v>
       </c>
-      <c r="F7" s="28"/>
+      <c r="F7" s="27"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="30"/>
-      <c r="B8" s="31" t="s">
+      <c r="A8" s="29"/>
+      <c r="B8" s="30" t="s">
         <v>175</v>
       </c>
-      <c r="C8" s="32" t="n">
+      <c r="C8" s="31" t="n">
         <f aca="false">SUM(C6:C7)</f>
         <v>172330.77</v>
       </c>
-      <c r="D8" s="33" t="n">
+      <c r="D8" s="32" t="n">
         <f aca="false">C8/C$15</f>
         <v>0.136534752221471</v>
       </c>
-      <c r="E8" s="30"/>
-      <c r="F8" s="30"/>
+      <c r="E8" s="29"/>
+      <c r="F8" s="29"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="34" t="s">
+      <c r="A9" s="33" t="s">
         <v>176</v>
       </c>
-      <c r="B9" s="35" t="str">
+      <c r="B9" s="34" t="str">
         <f aca="false">AMS!A40</f>
         <v>SP500 (fondos indexados)</v>
       </c>
-      <c r="C9" s="36" t="n">
+      <c r="C9" s="35" t="n">
         <f aca="false">AMS!B40</f>
         <v>878274</v>
       </c>
-      <c r="D9" s="37"/>
-      <c r="E9" s="38" t="s">
+      <c r="D9" s="36"/>
+      <c r="E9" s="37" t="s">
         <v>177</v>
       </c>
-      <c r="F9" s="37"/>
+      <c r="F9" s="36"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="39"/>
-      <c r="B10" s="40" t="s">
+      <c r="A10" s="38"/>
+      <c r="B10" s="39" t="s">
         <v>178</v>
       </c>
-      <c r="C10" s="41" t="n">
+      <c r="C10" s="40" t="n">
         <f aca="false">C9</f>
         <v>878274</v>
       </c>
-      <c r="D10" s="42" t="n">
+      <c r="D10" s="41" t="n">
         <f aca="false">C10/C$15</f>
         <v>0.695841624641728</v>
       </c>
-      <c r="E10" s="39"/>
-      <c r="F10" s="39"/>
+      <c r="E10" s="38"/>
+      <c r="F10" s="38"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="43" t="s">
+      <c r="A11" s="42" t="s">
         <v>179</v>
       </c>
-      <c r="B11" s="44" t="str">
+      <c r="B11" s="43" t="str">
         <f aca="false">AMS!A42</f>
         <v>ETF</v>
       </c>
-      <c r="C11" s="45" t="n">
+      <c r="C11" s="44" t="n">
         <f aca="false">AMS!B42</f>
         <v>111570.37</v>
       </c>
-      <c r="D11" s="46"/>
-      <c r="E11" s="47" t="s">
+      <c r="D11" s="45"/>
+      <c r="E11" s="46" t="s">
         <v>180</v>
       </c>
-      <c r="F11" s="46"/>
+      <c r="F11" s="45"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="43"/>
-      <c r="B12" s="44" t="str">
+      <c r="A12" s="42"/>
+      <c r="B12" s="43" t="str">
         <f aca="false">AMS!A43</f>
         <v>Pisos</v>
       </c>
-      <c r="C12" s="45" t="n">
+      <c r="C12" s="44" t="n">
         <f aca="false">AMS!B43</f>
         <v>100000</v>
       </c>
-      <c r="D12" s="46"/>
-      <c r="E12" s="47" t="s">
+      <c r="D12" s="45"/>
+      <c r="E12" s="46" t="s">
         <v>181</v>
       </c>
-      <c r="F12" s="46"/>
+      <c r="F12" s="45"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="48"/>
-      <c r="B13" s="49" t="s">
+      <c r="A13" s="47"/>
+      <c r="B13" s="48" t="s">
         <v>182</v>
       </c>
-      <c r="C13" s="50" t="n">
+      <c r="C13" s="49" t="n">
         <f aca="false">SUM(C11:C12)</f>
         <v>211570.37</v>
       </c>
-      <c r="D13" s="51" t="n">
+      <c r="D13" s="50" t="n">
         <f aca="false">C13/C$15</f>
         <v>0.167623623136802</v>
       </c>
-      <c r="E13" s="48"/>
-      <c r="F13" s="48"/>
+      <c r="E13" s="47"/>
+      <c r="F13" s="47"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="52" t="s">
+      <c r="A15" s="51" t="s">
         <v>183</v>
       </c>
-      <c r="B15" s="52"/>
-      <c r="C15" s="53" t="n">
+      <c r="B15" s="51"/>
+      <c r="C15" s="52" t="n">
         <f aca="false">C8+C10+C13</f>
         <v>1262175.14</v>
       </c>
-      <c r="D15" s="54" t="n">
+      <c r="D15" s="53" t="n">
         <f aca="false">C15/C15</f>
         <v>1</v>
       </c>
-      <c r="E15" s="55"/>
-      <c r="F15" s="55"/>
+      <c r="E15" s="54"/>
+      <c r="F15" s="54"/>
     </row>
     <row r="16" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B16" s="56" t="s">
+      <c r="B16" s="55" t="s">
         <v>184</v>
       </c>
-      <c r="C16" s="57" t="n">
+      <c r="C16" s="56" t="n">
         <f aca="false">C15-AMS!B45</f>
         <v>0</v>
       </c>
-      <c r="F16" s="58" t="s">
+      <c r="F16" s="57" t="s">
         <v>185</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="23" t="s">
+    <row r="19" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="22" t="s">
         <v>186</v>
       </c>
-      <c r="B19" s="23"/>
-      <c r="C19" s="23"/>
-      <c r="D19" s="23"/>
-      <c r="E19" s="23"/>
-      <c r="F19" s="23"/>
+      <c r="B19" s="22"/>
+      <c r="C19" s="22"/>
+      <c r="D19" s="22"/>
+      <c r="E19" s="22"/>
+      <c r="F19" s="22"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="24" t="s">
+      <c r="A20" s="23" t="s">
         <v>168</v>
       </c>
-      <c r="B20" s="24" t="s">
+      <c r="B20" s="23" t="s">
         <v>169</v>
       </c>
-      <c r="C20" s="24" t="s">
+      <c r="C20" s="23" t="s">
         <v>27</v>
       </c>
-      <c r="D20" s="24" t="s">
+      <c r="D20" s="23" t="s">
         <v>170</v>
       </c>
-      <c r="E20" s="24" t="s">
+      <c r="E20" s="23" t="s">
         <v>171</v>
       </c>
-      <c r="F20" s="24" t="s">
+      <c r="F20" s="23" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="25" t="s">
+      <c r="A21" s="24" t="s">
         <v>172</v>
       </c>
-      <c r="B21" s="26" t="str">
+      <c r="B21" s="25" t="str">
         <f aca="false">AML!A43</f>
         <v>Liquidez + Depósitos (excluido FM)</v>
       </c>
-      <c r="C21" s="27" t="n">
+      <c r="C21" s="26" t="n">
         <f aca="false">AML!B43</f>
         <v>199375</v>
       </c>
-      <c r="D21" s="28"/>
-      <c r="E21" s="29" t="s">
+      <c r="D21" s="27"/>
+      <c r="E21" s="28" t="s">
         <v>187</v>
       </c>
-      <c r="F21" s="28"/>
+      <c r="F21" s="27"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="30"/>
-      <c r="B22" s="31" t="s">
+      <c r="A22" s="29"/>
+      <c r="B22" s="30" t="s">
         <v>175</v>
       </c>
-      <c r="C22" s="32" t="n">
+      <c r="C22" s="31" t="n">
         <f aca="false">C21</f>
         <v>199375</v>
       </c>
-      <c r="D22" s="33" t="n">
+      <c r="D22" s="32" t="n">
         <f aca="false">C22/C$30</f>
         <v>0.0471777266421833</v>
       </c>
-      <c r="E22" s="30"/>
-      <c r="F22" s="30"/>
+      <c r="E22" s="29"/>
+      <c r="F22" s="29"/>
     </row>
     <row r="23" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="34" t="s">
+      <c r="A23" s="33" t="s">
         <v>176</v>
       </c>
-      <c r="B23" s="35" t="str">
+      <c r="B23" s="34" t="str">
         <f aca="false">AML!A39</f>
         <v>Fondos RV</v>
       </c>
-      <c r="C23" s="36" t="n">
+      <c r="C23" s="35" t="n">
         <f aca="false">AML!B39</f>
         <v>2196689</v>
       </c>
-      <c r="D23" s="37"/>
-      <c r="E23" s="38" t="s">
+      <c r="D23" s="36"/>
+      <c r="E23" s="37" t="s">
         <v>188</v>
       </c>
-      <c r="F23" s="37"/>
+      <c r="F23" s="36"/>
     </row>
     <row r="24" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="34"/>
-      <c r="B24" s="35" t="str">
+      <c r="A24" s="33"/>
+      <c r="B24" s="34" t="str">
         <f aca="false">AML!A40</f>
         <v>Planes de Pensiones (Papá + Mamá)</v>
       </c>
-      <c r="C24" s="36" t="n">
+      <c r="C24" s="35" t="n">
         <f aca="false">AML!B40</f>
         <v>1158832</v>
       </c>
-      <c r="D24" s="37"/>
-      <c r="E24" s="38" t="s">
+      <c r="D24" s="36"/>
+      <c r="E24" s="37" t="s">
         <v>189</v>
       </c>
-      <c r="F24" s="59" t="s">
+      <c r="F24" s="58" t="s">
         <v>190</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="39"/>
-      <c r="B25" s="40" t="s">
+      <c r="A25" s="38"/>
+      <c r="B25" s="39" t="s">
         <v>178</v>
       </c>
-      <c r="C25" s="41" t="n">
+      <c r="C25" s="40" t="n">
         <f aca="false">SUM(C23:C24)</f>
         <v>3355521</v>
       </c>
-      <c r="D25" s="42" t="n">
+      <c r="D25" s="41" t="n">
         <f aca="false">C25/C$30</f>
         <v>0.794010545354762</v>
       </c>
-      <c r="E25" s="39"/>
-      <c r="F25" s="39"/>
+      <c r="E25" s="38"/>
+      <c r="F25" s="38"/>
     </row>
     <row r="26" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="43" t="s">
+      <c r="A26" s="42" t="s">
         <v>179</v>
       </c>
-      <c r="B26" s="44" t="str">
+      <c r="B26" s="43" t="str">
         <f aca="false">AML!A41</f>
         <v>Acciones (Iberdrola + BBVA + TEF)</v>
       </c>
-      <c r="C26" s="45" t="n">
+      <c r="C26" s="44" t="n">
         <f aca="false">AML!B41</f>
         <v>531793.35</v>
       </c>
-      <c r="D26" s="46"/>
-      <c r="E26" s="47" t="s">
+      <c r="D26" s="45"/>
+      <c r="E26" s="46" t="s">
         <v>191</v>
       </c>
-      <c r="F26" s="60" t="s">
+      <c r="F26" s="59" t="s">
         <v>192</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="43"/>
-      <c r="B27" s="44" t="str">
+      <c r="A27" s="42"/>
+      <c r="B27" s="43" t="str">
         <f aca="false">AML!A42</f>
         <v>ETF (Aristócratas)</v>
       </c>
-      <c r="C27" s="45" t="n">
+      <c r="C27" s="44" t="n">
         <f aca="false">AML!B42</f>
         <v>139351.5</v>
       </c>
-      <c r="D27" s="46"/>
-      <c r="E27" s="47" t="s">
+      <c r="D27" s="45"/>
+      <c r="E27" s="46" t="s">
         <v>193</v>
       </c>
-      <c r="F27" s="46"/>
+      <c r="F27" s="45"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="48"/>
-      <c r="B28" s="49" t="s">
+      <c r="A28" s="47"/>
+      <c r="B28" s="48" t="s">
         <v>182</v>
       </c>
-      <c r="C28" s="50" t="n">
+      <c r="C28" s="49" t="n">
         <f aca="false">SUM(C26:C27)</f>
         <v>671144.85</v>
       </c>
-      <c r="D28" s="51" t="n">
+      <c r="D28" s="50" t="n">
         <f aca="false">C28/C$30</f>
         <v>0.158811728003055</v>
       </c>
-      <c r="E28" s="48"/>
-      <c r="F28" s="48"/>
+      <c r="E28" s="47"/>
+      <c r="F28" s="47"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="52" t="s">
+      <c r="A30" s="51" t="s">
         <v>194</v>
       </c>
-      <c r="B30" s="52"/>
-      <c r="C30" s="53" t="n">
+      <c r="B30" s="51"/>
+      <c r="C30" s="52" t="n">
         <f aca="false">C22+C25+C28</f>
         <v>4226040.85</v>
       </c>
-      <c r="D30" s="54" t="n">
+      <c r="D30" s="53" t="n">
         <f aca="false">C30/C30</f>
         <v>1</v>
       </c>
-      <c r="E30" s="55"/>
-      <c r="F30" s="55"/>
+      <c r="E30" s="54"/>
+      <c r="F30" s="54"/>
     </row>
     <row r="31" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B31" s="56" t="s">
+      <c r="B31" s="55" t="s">
         <v>184</v>
       </c>
-      <c r="C31" s="57" t="n">
+      <c r="C31" s="56" t="n">
         <f aca="false">C30-AML!B44</f>
         <v>0</v>
       </c>
-      <c r="F31" s="58" t="s">
+      <c r="F31" s="57" t="s">
         <v>185</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="61" t="s">
+      <c r="A33" s="60" t="s">
         <v>195</v>
       </c>
-      <c r="B33" s="61"/>
-      <c r="C33" s="61"/>
-      <c r="D33" s="61"/>
-      <c r="E33" s="61"/>
-      <c r="F33" s="61"/>
+      <c r="B33" s="60"/>
+      <c r="C33" s="60"/>
+      <c r="D33" s="60"/>
+      <c r="E33" s="60"/>
+      <c r="F33" s="60"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="61"/>
-      <c r="B34" s="61"/>
-      <c r="C34" s="61"/>
-      <c r="D34" s="61"/>
-      <c r="E34" s="61"/>
-      <c r="F34" s="61"/>
+      <c r="A34" s="60"/>
+      <c r="B34" s="60"/>
+      <c r="C34" s="60"/>
+      <c r="D34" s="60"/>
+      <c r="E34" s="60"/>
+      <c r="F34" s="60"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="61"/>
-      <c r="B35" s="61"/>
-      <c r="C35" s="61"/>
-      <c r="D35" s="61"/>
-      <c r="E35" s="61"/>
-      <c r="F35" s="61"/>
+      <c r="A35" s="60"/>
+      <c r="B35" s="60"/>
+      <c r="C35" s="60"/>
+      <c r="D35" s="60"/>
+      <c r="E35" s="60"/>
+      <c r="F35" s="60"/>
     </row>
   </sheetData>
   <mergeCells count="11">
@@ -3899,550 +3895,550 @@
   <dimension ref="A1:H34"/>
   <sheetFormatPr defaultColWidth="8.66796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="20" width="42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="2" style="20" width="16"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="9" style="20" width="8.67"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="19" width="42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="2" style="19" width="16"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="9" style="19" width="8.67"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="21" t="s">
+      <c r="A1" s="20" t="s">
         <v>196</v>
       </c>
-      <c r="B1" s="21"/>
-      <c r="C1" s="21"/>
-      <c r="D1" s="21"/>
-      <c r="E1" s="21"/>
-      <c r="F1" s="21"/>
-      <c r="G1" s="21"/>
-      <c r="H1" s="21"/>
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="20"/>
+      <c r="E1" s="20"/>
+      <c r="F1" s="20"/>
+      <c r="G1" s="20"/>
+      <c r="H1" s="20"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="22" t="s">
+      <c r="A2" s="21" t="s">
         <v>197</v>
       </c>
-      <c r="B2" s="22"/>
-      <c r="C2" s="22"/>
-      <c r="D2" s="22"/>
-      <c r="E2" s="22"/>
-      <c r="F2" s="22"/>
-      <c r="G2" s="22"/>
-      <c r="H2" s="22"/>
+      <c r="B2" s="21"/>
+      <c r="C2" s="21"/>
+      <c r="D2" s="21"/>
+      <c r="E2" s="21"/>
+      <c r="F2" s="21"/>
+      <c r="G2" s="21"/>
+      <c r="H2" s="21"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="23" t="s">
+      <c r="A4" s="22" t="s">
         <v>198</v>
       </c>
-      <c r="B4" s="23"/>
-      <c r="C4" s="23"/>
-      <c r="D4" s="23"/>
-      <c r="E4" s="23"/>
-      <c r="F4" s="23"/>
-      <c r="G4" s="23"/>
-      <c r="H4" s="23"/>
+      <c r="B4" s="22"/>
+      <c r="C4" s="22"/>
+      <c r="D4" s="22"/>
+      <c r="E4" s="22"/>
+      <c r="F4" s="22"/>
+      <c r="G4" s="22"/>
+      <c r="H4" s="22"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="24" t="s">
+      <c r="A5" s="23" t="s">
         <v>26</v>
       </c>
-      <c r="B5" s="24" t="s">
+      <c r="B5" s="23" t="s">
         <v>27</v>
       </c>
-      <c r="C5" s="24" t="s">
+      <c r="C5" s="23" t="s">
         <v>28</v>
       </c>
-      <c r="D5" s="24" t="s">
+      <c r="D5" s="23" t="s">
         <v>29</v>
       </c>
-      <c r="E5" s="24"/>
-      <c r="F5" s="24"/>
-      <c r="G5" s="24"/>
-      <c r="H5" s="24"/>
+      <c r="E5" s="23"/>
+      <c r="F5" s="23"/>
+      <c r="G5" s="23"/>
+      <c r="H5" s="23"/>
     </row>
     <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="62" t="s">
+      <c r="A6" s="61" t="s">
         <v>199</v>
       </c>
-      <c r="B6" s="63" t="n">
+      <c r="B6" s="62" t="n">
         <v>46247</v>
       </c>
-      <c r="C6" s="64" t="s">
+      <c r="C6" s="63" t="s">
         <v>31</v>
       </c>
-      <c r="D6" s="65" t="s">
+      <c r="D6" s="64" t="s">
         <v>200</v>
       </c>
-      <c r="E6" s="65"/>
-      <c r="F6" s="65"/>
-      <c r="G6" s="65"/>
-      <c r="H6" s="65"/>
+      <c r="E6" s="64"/>
+      <c r="F6" s="64"/>
+      <c r="G6" s="64"/>
+      <c r="H6" s="64"/>
     </row>
     <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="62" t="s">
+      <c r="A7" s="61" t="s">
         <v>201</v>
       </c>
-      <c r="B7" s="66" t="n">
+      <c r="B7" s="65" t="n">
         <v>878274</v>
       </c>
-      <c r="C7" s="64" t="s">
+      <c r="C7" s="63" t="s">
         <v>31</v>
       </c>
-      <c r="D7" s="65" t="s">
+      <c r="D7" s="64" t="s">
         <v>202</v>
       </c>
-      <c r="E7" s="65"/>
-      <c r="F7" s="65"/>
-      <c r="G7" s="65"/>
-      <c r="H7" s="65"/>
+      <c r="E7" s="64"/>
+      <c r="F7" s="64"/>
+      <c r="G7" s="64"/>
+      <c r="H7" s="64"/>
     </row>
     <row r="8" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="62" t="s">
+      <c r="A8" s="61" t="s">
         <v>203</v>
       </c>
-      <c r="B8" s="66" t="n">
+      <c r="B8" s="65" t="n">
         <v>2196689</v>
       </c>
-      <c r="C8" s="64" t="s">
+      <c r="C8" s="63" t="s">
         <v>31</v>
       </c>
-      <c r="D8" s="65" t="s">
+      <c r="D8" s="64" t="s">
         <v>204</v>
       </c>
-      <c r="E8" s="65"/>
-      <c r="F8" s="65"/>
-      <c r="G8" s="65"/>
-      <c r="H8" s="65"/>
+      <c r="E8" s="64"/>
+      <c r="F8" s="64"/>
+      <c r="G8" s="64"/>
+      <c r="H8" s="64"/>
     </row>
     <row r="9" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="62" t="s">
+      <c r="A9" s="61" t="s">
         <v>205</v>
       </c>
-      <c r="B9" s="66" t="n">
+      <c r="B9" s="65" t="n">
         <v>1158833</v>
       </c>
-      <c r="C9" s="64" t="s">
+      <c r="C9" s="63" t="s">
         <v>31</v>
       </c>
-      <c r="D9" s="65" t="s">
+      <c r="D9" s="64" t="s">
         <v>206</v>
       </c>
-      <c r="E9" s="65"/>
-      <c r="F9" s="65"/>
-      <c r="G9" s="65"/>
-      <c r="H9" s="65"/>
+      <c r="E9" s="64"/>
+      <c r="F9" s="64"/>
+      <c r="G9" s="64"/>
+      <c r="H9" s="64"/>
     </row>
     <row r="10" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="67" t="s">
+      <c r="A10" s="66" t="s">
         <v>207</v>
       </c>
-      <c r="B10" s="68" t="n">
+      <c r="B10" s="67" t="n">
         <f aca="false">B8+B9</f>
         <v>3355522</v>
       </c>
-      <c r="C10" s="64" t="s">
+      <c r="C10" s="63" t="s">
         <v>36</v>
       </c>
-      <c r="D10" s="65" t="s">
+      <c r="D10" s="64" t="s">
         <v>208</v>
       </c>
-      <c r="E10" s="65"/>
-      <c r="F10" s="65"/>
-      <c r="G10" s="65"/>
-      <c r="H10" s="65"/>
+      <c r="E10" s="64"/>
+      <c r="F10" s="64"/>
+      <c r="G10" s="64"/>
+      <c r="H10" s="64"/>
     </row>
     <row r="12" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="23" t="s">
+      <c r="A12" s="22" t="s">
         <v>209</v>
       </c>
-      <c r="B12" s="23"/>
-      <c r="C12" s="23"/>
-      <c r="D12" s="23"/>
-      <c r="E12" s="23"/>
-      <c r="F12" s="23"/>
-      <c r="G12" s="23"/>
-      <c r="H12" s="23"/>
+      <c r="B12" s="22"/>
+      <c r="C12" s="22"/>
+      <c r="D12" s="22"/>
+      <c r="E12" s="22"/>
+      <c r="F12" s="22"/>
+      <c r="G12" s="22"/>
+      <c r="H12" s="22"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="24" t="s">
+      <c r="A13" s="23" t="s">
         <v>26</v>
       </c>
-      <c r="B13" s="24" t="s">
+      <c r="B13" s="23" t="s">
         <v>27</v>
       </c>
-      <c r="C13" s="24" t="s">
+      <c r="C13" s="23" t="s">
         <v>28</v>
       </c>
-      <c r="D13" s="24" t="s">
+      <c r="D13" s="23" t="s">
         <v>29</v>
       </c>
-      <c r="E13" s="24"/>
-      <c r="F13" s="24"/>
-      <c r="G13" s="24"/>
-      <c r="H13" s="24"/>
+      <c r="E13" s="23"/>
+      <c r="F13" s="23"/>
+      <c r="G13" s="23"/>
+      <c r="H13" s="23"/>
     </row>
     <row r="14" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="62" t="s">
+      <c r="A14" s="61" t="s">
         <v>210</v>
       </c>
-      <c r="B14" s="69" t="n">
+      <c r="B14" s="68" t="n">
         <v>0.07</v>
       </c>
-      <c r="C14" s="64" t="s">
+      <c r="C14" s="63" t="s">
         <v>31</v>
       </c>
-      <c r="D14" s="65" t="s">
+      <c r="D14" s="64" t="s">
         <v>211</v>
       </c>
-      <c r="E14" s="65"/>
-      <c r="F14" s="65"/>
-      <c r="G14" s="65"/>
-      <c r="H14" s="65"/>
+      <c r="E14" s="64"/>
+      <c r="F14" s="64"/>
+      <c r="G14" s="64"/>
+      <c r="H14" s="64"/>
     </row>
     <row r="15" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="62" t="s">
+      <c r="A15" s="61" t="s">
         <v>212</v>
       </c>
-      <c r="B15" s="69" t="n">
+      <c r="B15" s="68" t="n">
         <v>0.094</v>
       </c>
-      <c r="C15" s="64" t="s">
+      <c r="C15" s="63" t="s">
         <v>31</v>
       </c>
-      <c r="D15" s="65" t="s">
+      <c r="D15" s="64" t="s">
         <v>213</v>
       </c>
-      <c r="E15" s="65"/>
-      <c r="F15" s="65"/>
-      <c r="G15" s="65"/>
-      <c r="H15" s="65"/>
+      <c r="E15" s="64"/>
+      <c r="F15" s="64"/>
+      <c r="G15" s="64"/>
+      <c r="H15" s="64"/>
     </row>
     <row r="17" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="23" t="s">
+      <c r="A17" s="22" t="s">
         <v>214</v>
       </c>
-      <c r="B17" s="23"/>
-      <c r="C17" s="23"/>
-      <c r="D17" s="23"/>
-      <c r="E17" s="23"/>
-      <c r="F17" s="23"/>
-      <c r="G17" s="23"/>
-      <c r="H17" s="23"/>
+      <c r="B17" s="22"/>
+      <c r="C17" s="22"/>
+      <c r="D17" s="22"/>
+      <c r="E17" s="22"/>
+      <c r="F17" s="22"/>
+      <c r="G17" s="22"/>
+      <c r="H17" s="22"/>
     </row>
     <row r="18" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="24" t="s">
+      <c r="A18" s="23" t="s">
         <v>215</v>
       </c>
-      <c r="B18" s="24" t="s">
+      <c r="B18" s="23" t="s">
         <v>216</v>
       </c>
-      <c r="C18" s="24" t="s">
+      <c r="C18" s="23" t="s">
         <v>217</v>
       </c>
-      <c r="D18" s="70" t="s">
+      <c r="D18" s="69" t="s">
         <v>218</v>
       </c>
-      <c r="E18" s="71" t="s">
+      <c r="E18" s="70" t="s">
         <v>219</v>
       </c>
-      <c r="F18" s="24" t="s">
+      <c r="F18" s="23" t="s">
         <v>220</v>
       </c>
-      <c r="G18" s="24"/>
-      <c r="H18" s="24"/>
+      <c r="G18" s="23"/>
+      <c r="H18" s="23"/>
     </row>
     <row r="19" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="72" t="s">
+      <c r="A19" s="71" t="s">
         <v>221</v>
       </c>
-      <c r="B19" s="73" t="n">
+      <c r="B19" s="72" t="n">
         <f aca="false">DATE(YEAR($B$6)+5,MONTH($B$6),DAY($B$6))</f>
         <v>48073</v>
       </c>
-      <c r="C19" s="36" t="n">
+      <c r="C19" s="35" t="n">
         <f aca="false">$B$7*(1+$B$14)^5</f>
         <v>1231824.71872881</v>
       </c>
-      <c r="D19" s="74" t="n">
+      <c r="D19" s="73" t="n">
         <f aca="false">$B$7*(1+$B$15)^5</f>
         <v>1376311.17540442</v>
       </c>
-      <c r="E19" s="75" t="n">
+      <c r="E19" s="74" t="n">
         <f aca="false">$B$10*(1+$B$14)^5</f>
         <v>4706293.18850193</v>
       </c>
-      <c r="F19" s="36" t="n">
+      <c r="F19" s="35" t="n">
         <f aca="false">$B$10*(1+$B$15)^5</f>
         <v>5258316.22923529</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="72" t="s">
+      <c r="A20" s="71" t="s">
         <v>222</v>
       </c>
-      <c r="B20" s="73" t="n">
+      <c r="B20" s="72" t="n">
         <f aca="false">DATE(YEAR($B$6)+10,MONTH($B$6),DAY($B$6))</f>
         <v>49900</v>
       </c>
-      <c r="C20" s="36" t="n">
+      <c r="C20" s="35" t="n">
         <f aca="false">$B$7*(1+$B$14)^10</f>
         <v>1727697.89117214</v>
       </c>
-      <c r="D20" s="74" t="n">
+      <c r="D20" s="73" t="n">
         <f aca="false">$B$7*(1+$B$15)^10</f>
         <v>2156767.08127885</v>
       </c>
-      <c r="E20" s="75" t="n">
+      <c r="E20" s="74" t="n">
         <f aca="false">$B$10*(1+$B$14)^10</f>
         <v>6600819.656715</v>
       </c>
-      <c r="F20" s="36" t="n">
+      <c r="F20" s="35" t="n">
         <f aca="false">$B$10*(1+$B$15)^10</f>
         <v>8240115.71571852</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="72" t="s">
+      <c r="A21" s="71" t="s">
         <v>223</v>
       </c>
-      <c r="B21" s="73" t="n">
+      <c r="B21" s="72" t="n">
         <f aca="false">DATE(YEAR($B$6)+15,MONTH($B$6),DAY($B$6))</f>
         <v>51726</v>
       </c>
-      <c r="C21" s="36" t="n">
+      <c r="C21" s="35" t="n">
         <f aca="false">$B$7*(1+$B$14)^15</f>
         <v>2423185.66739022</v>
       </c>
-      <c r="D21" s="74" t="n">
+      <c r="D21" s="73" t="n">
         <f aca="false">$B$7*(1+$B$15)^15</f>
         <v>3379791.08650428</v>
       </c>
-      <c r="E21" s="75" t="n">
+      <c r="E21" s="74" t="n">
         <f aca="false">$B$10*(1+$B$14)^15</f>
         <v>9257991.03356421</v>
       </c>
-      <c r="F21" s="36" t="n">
+      <c r="F21" s="35" t="n">
         <f aca="false">$B$10*(1+$B$15)^15</f>
         <v>12912785.0148917</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="23" t="s">
+      <c r="A23" s="22" t="s">
         <v>224</v>
       </c>
-      <c r="B23" s="23"/>
-      <c r="C23" s="23"/>
-      <c r="D23" s="23"/>
-      <c r="E23" s="23"/>
-      <c r="F23" s="23"/>
-      <c r="G23" s="23"/>
-      <c r="H23" s="23"/>
+      <c r="B23" s="22"/>
+      <c r="C23" s="22"/>
+      <c r="D23" s="22"/>
+      <c r="E23" s="22"/>
+      <c r="F23" s="22"/>
+      <c r="G23" s="22"/>
+      <c r="H23" s="22"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="24" t="s">
+      <c r="A24" s="23" t="s">
         <v>225</v>
       </c>
-      <c r="B24" s="24" t="s">
+      <c r="B24" s="23" t="s">
         <v>226</v>
       </c>
-      <c r="C24" s="24" t="s">
+      <c r="C24" s="23" t="s">
         <v>227</v>
       </c>
-      <c r="D24" s="24" t="s">
+      <c r="D24" s="23" t="s">
         <v>228</v>
       </c>
-      <c r="E24" s="70" t="s">
+      <c r="E24" s="69" t="s">
         <v>229</v>
       </c>
-      <c r="F24" s="71" t="s">
+      <c r="F24" s="70" t="s">
         <v>230</v>
       </c>
-      <c r="G24" s="24" t="s">
+      <c r="G24" s="23" t="s">
         <v>231</v>
       </c>
-      <c r="H24" s="24" t="s">
+      <c r="H24" s="23" t="s">
         <v>232</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="76"/>
-      <c r="B25" s="77" t="str">
+      <c r="A25" s="75"/>
+      <c r="B25" s="76" t="str">
         <f aca="false">IF($A25="","",($A25-$B$6)/365.25)</f>
         <v/>
       </c>
-      <c r="C25" s="66"/>
-      <c r="D25" s="78" t="str">
+      <c r="C25" s="65"/>
+      <c r="D25" s="77" t="str">
         <f aca="false">IF($A25="","",$B$7*(1+$B$15)^$B25)</f>
         <v/>
       </c>
-      <c r="E25" s="79" t="str">
+      <c r="E25" s="78" t="str">
         <f aca="false">IF(OR($A25="",$C25=""),"",$C25-$D25)</f>
         <v/>
       </c>
-      <c r="F25" s="80"/>
-      <c r="G25" s="78" t="str">
+      <c r="F25" s="79"/>
+      <c r="G25" s="77" t="str">
         <f aca="false">IF($A25="","",$B$10*(1+$B$15)^$B25)</f>
         <v/>
       </c>
-      <c r="H25" s="81" t="str">
+      <c r="H25" s="80" t="str">
         <f aca="false">IF(OR($A25="",$F25=""),"",$F25-$G25)</f>
         <v/>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="76"/>
-      <c r="B26" s="77" t="str">
+      <c r="A26" s="75"/>
+      <c r="B26" s="76" t="str">
         <f aca="false">IF($A26="","",($A26-$B$6)/365.25)</f>
         <v/>
       </c>
-      <c r="C26" s="66"/>
-      <c r="D26" s="78" t="str">
+      <c r="C26" s="65"/>
+      <c r="D26" s="77" t="str">
         <f aca="false">IF($A26="","",$B$7*(1+$B$15)^$B26)</f>
         <v/>
       </c>
-      <c r="E26" s="79" t="str">
+      <c r="E26" s="78" t="str">
         <f aca="false">IF(OR($A26="",$C26=""),"",$C26-$D26)</f>
         <v/>
       </c>
-      <c r="F26" s="80"/>
-      <c r="G26" s="78" t="str">
+      <c r="F26" s="79"/>
+      <c r="G26" s="77" t="str">
         <f aca="false">IF($A26="","",$B$10*(1+$B$15)^$B26)</f>
         <v/>
       </c>
-      <c r="H26" s="81" t="str">
+      <c r="H26" s="80" t="str">
         <f aca="false">IF(OR($A26="",$F26=""),"",$F26-$G26)</f>
         <v/>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="76"/>
-      <c r="B27" s="77" t="str">
+      <c r="A27" s="75"/>
+      <c r="B27" s="76" t="str">
         <f aca="false">IF($A27="","",($A27-$B$6)/365.25)</f>
         <v/>
       </c>
-      <c r="C27" s="66"/>
-      <c r="D27" s="78" t="str">
+      <c r="C27" s="65"/>
+      <c r="D27" s="77" t="str">
         <f aca="false">IF($A27="","",$B$7*(1+$B$15)^$B27)</f>
         <v/>
       </c>
-      <c r="E27" s="79" t="str">
+      <c r="E27" s="78" t="str">
         <f aca="false">IF(OR($A27="",$C27=""),"",$C27-$D27)</f>
         <v/>
       </c>
-      <c r="F27" s="80"/>
-      <c r="G27" s="78" t="str">
+      <c r="F27" s="79"/>
+      <c r="G27" s="77" t="str">
         <f aca="false">IF($A27="","",$B$10*(1+$B$15)^$B27)</f>
         <v/>
       </c>
-      <c r="H27" s="81" t="str">
+      <c r="H27" s="80" t="str">
         <f aca="false">IF(OR($A27="",$F27=""),"",$F27-$G27)</f>
         <v/>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="76"/>
-      <c r="B28" s="77" t="str">
+      <c r="A28" s="75"/>
+      <c r="B28" s="76" t="str">
         <f aca="false">IF($A28="","",($A28-$B$6)/365.25)</f>
         <v/>
       </c>
-      <c r="C28" s="66"/>
-      <c r="D28" s="78" t="str">
+      <c r="C28" s="65"/>
+      <c r="D28" s="77" t="str">
         <f aca="false">IF($A28="","",$B$7*(1+$B$15)^$B28)</f>
         <v/>
       </c>
-      <c r="E28" s="79" t="str">
+      <c r="E28" s="78" t="str">
         <f aca="false">IF(OR($A28="",$C28=""),"",$C28-$D28)</f>
         <v/>
       </c>
-      <c r="F28" s="80"/>
-      <c r="G28" s="78" t="str">
+      <c r="F28" s="79"/>
+      <c r="G28" s="77" t="str">
         <f aca="false">IF($A28="","",$B$10*(1+$B$15)^$B28)</f>
         <v/>
       </c>
-      <c r="H28" s="81" t="str">
+      <c r="H28" s="80" t="str">
         <f aca="false">IF(OR($A28="",$F28=""),"",$F28-$G28)</f>
         <v/>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="76"/>
-      <c r="B29" s="77" t="str">
+      <c r="A29" s="75"/>
+      <c r="B29" s="76" t="str">
         <f aca="false">IF($A29="","",($A29-$B$6)/365.25)</f>
         <v/>
       </c>
-      <c r="C29" s="66"/>
-      <c r="D29" s="78" t="str">
+      <c r="C29" s="65"/>
+      <c r="D29" s="77" t="str">
         <f aca="false">IF($A29="","",$B$7*(1+$B$15)^$B29)</f>
         <v/>
       </c>
-      <c r="E29" s="79" t="str">
+      <c r="E29" s="78" t="str">
         <f aca="false">IF(OR($A29="",$C29=""),"",$C29-$D29)</f>
         <v/>
       </c>
-      <c r="F29" s="80"/>
-      <c r="G29" s="78" t="str">
+      <c r="F29" s="79"/>
+      <c r="G29" s="77" t="str">
         <f aca="false">IF($A29="","",$B$10*(1+$B$15)^$B29)</f>
         <v/>
       </c>
-      <c r="H29" s="81" t="str">
+      <c r="H29" s="80" t="str">
         <f aca="false">IF(OR($A29="",$F29=""),"",$F29-$G29)</f>
         <v/>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="76"/>
-      <c r="B30" s="77" t="str">
+      <c r="A30" s="75"/>
+      <c r="B30" s="76" t="str">
         <f aca="false">IF($A30="","",($A30-$B$6)/365.25)</f>
         <v/>
       </c>
-      <c r="C30" s="66"/>
-      <c r="D30" s="78" t="str">
+      <c r="C30" s="65"/>
+      <c r="D30" s="77" t="str">
         <f aca="false">IF($A30="","",$B$7*(1+$B$15)^$B30)</f>
         <v/>
       </c>
-      <c r="E30" s="79" t="str">
+      <c r="E30" s="78" t="str">
         <f aca="false">IF(OR($A30="",$C30=""),"",$C30-$D30)</f>
         <v/>
       </c>
-      <c r="F30" s="80"/>
-      <c r="G30" s="78" t="str">
+      <c r="F30" s="79"/>
+      <c r="G30" s="77" t="str">
         <f aca="false">IF($A30="","",$B$10*(1+$B$15)^$B30)</f>
         <v/>
       </c>
-      <c r="H30" s="81" t="str">
+      <c r="H30" s="80" t="str">
         <f aca="false">IF(OR($A30="",$F30=""),"",$F30-$G30)</f>
         <v/>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="61" t="s">
+      <c r="A32" s="60" t="s">
         <v>233</v>
       </c>
-      <c r="B32" s="61"/>
-      <c r="C32" s="61"/>
-      <c r="D32" s="61"/>
-      <c r="E32" s="61"/>
-      <c r="F32" s="61"/>
-      <c r="G32" s="61"/>
-      <c r="H32" s="61"/>
+      <c r="B32" s="60"/>
+      <c r="C32" s="60"/>
+      <c r="D32" s="60"/>
+      <c r="E32" s="60"/>
+      <c r="F32" s="60"/>
+      <c r="G32" s="60"/>
+      <c r="H32" s="60"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="61"/>
-      <c r="B33" s="61"/>
-      <c r="C33" s="61"/>
-      <c r="D33" s="61"/>
-      <c r="E33" s="61"/>
-      <c r="F33" s="61"/>
-      <c r="G33" s="61"/>
-      <c r="H33" s="61"/>
+      <c r="A33" s="60"/>
+      <c r="B33" s="60"/>
+      <c r="C33" s="60"/>
+      <c r="D33" s="60"/>
+      <c r="E33" s="60"/>
+      <c r="F33" s="60"/>
+      <c r="G33" s="60"/>
+      <c r="H33" s="60"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="61"/>
-      <c r="B34" s="61"/>
-      <c r="C34" s="61"/>
-      <c r="D34" s="61"/>
-      <c r="E34" s="61"/>
-      <c r="F34" s="61"/>
-      <c r="G34" s="61"/>
-      <c r="H34" s="61"/>
+      <c r="A34" s="60"/>
+      <c r="B34" s="60"/>
+      <c r="C34" s="60"/>
+      <c r="D34" s="60"/>
+      <c r="E34" s="60"/>
+      <c r="F34" s="60"/>
+      <c r="G34" s="60"/>
+      <c r="H34" s="60"/>
     </row>
   </sheetData>
   <mergeCells count="16">

</xml_diff>